<commit_message>
P35 pass 3: pilot report, owner questions, refreshed rebuild list and quality report
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/models/quality_report.xlsx
+++ b/Docs/models/quality_report.xlsx
@@ -3696,10 +3696,10 @@
         </is>
       </c>
       <c r="M23" t="n">
-        <v>0.038</v>
+        <v>0.039</v>
       </c>
       <c r="N23" t="n">
-        <v>0.065</v>
+        <v>0.066</v>
       </c>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="n">
@@ -6433,10 +6433,10 @@
         </is>
       </c>
       <c r="M42" t="n">
-        <v>0.047</v>
+        <v>0.046</v>
       </c>
       <c r="N42" t="n">
-        <v>0.056</v>
+        <v>0.055</v>
       </c>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="n">
@@ -6576,10 +6576,10 @@
         </is>
       </c>
       <c r="M43" t="n">
-        <v>0.092</v>
+        <v>0.091</v>
       </c>
       <c r="N43" t="n">
-        <v>0.113</v>
+        <v>0.112</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
@@ -6723,10 +6723,10 @@
         </is>
       </c>
       <c r="M44" t="n">
-        <v>0.043</v>
+        <v>0.042</v>
       </c>
       <c r="N44" t="n">
-        <v>0.048</v>
+        <v>0.047</v>
       </c>
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="n">
@@ -12312,10 +12312,10 @@
         </is>
       </c>
       <c r="M83" t="n">
-        <v>0.153</v>
+        <v>0.15</v>
       </c>
       <c r="N83" t="n">
-        <v>0.041</v>
+        <v>0.036</v>
       </c>
       <c r="O83" t="inlineStr">
         <is>
@@ -18400,7 +18400,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>17324</v>
+        <v>35714</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -18409,7 +18409,7 @@
       </c>
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="n">
-        <v>64.8</v>
+        <v>79.7</v>
       </c>
       <c r="H126" t="inlineStr">
         <is>
@@ -18421,84 +18421,76 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="J126" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
-      <c r="K126" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
+      <c r="J126" t="inlineStr"/>
+      <c r="K126" t="inlineStr"/>
       <c r="L126" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="M126" t="n">
-        <v>0.006</v>
+        <v>0.032</v>
       </c>
       <c r="N126" t="n">
-        <v>0</v>
+        <v>0.016</v>
       </c>
       <c r="O126" t="inlineStr"/>
       <c r="P126" t="n">
-        <v>1.5567</v>
+        <v>1.6225</v>
       </c>
       <c r="Q126" t="n">
-        <v>0.1032</v>
+        <v>0.1474</v>
       </c>
       <c r="R126" t="n">
-        <v>2.6663</v>
+        <v>3.4735</v>
       </c>
       <c r="S126" t="n">
-        <v>0.0142</v>
+        <v>0.0902</v>
       </c>
       <c r="T126" t="n">
-        <v>532</v>
+        <v>1084</v>
       </c>
       <c r="U126" t="n">
-        <v>105</v>
+        <v>225</v>
       </c>
       <c r="V126" t="n">
-        <v>0.4224</v>
+        <v>0.8565</v>
       </c>
       <c r="W126" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="X126" t="n">
-        <v>105</v>
+        <v>208</v>
       </c>
       <c r="Y126" t="n">
-        <v>409</v>
+        <v>857</v>
       </c>
       <c r="Z126" t="n">
-        <v>0.4224</v>
+        <v>0.7917999999999999</v>
       </c>
       <c r="AA126" t="n">
-        <v>1.6454</v>
+        <v>3.2625</v>
       </c>
       <c r="AB126" t="n">
-        <v>248.5773</v>
+        <v>262.6824</v>
       </c>
       <c r="AC126" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AD126" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="AE126" t="n">
-        <v>0.1413</v>
+        <v>0.1194</v>
       </c>
       <c r="AF126" t="n">
-        <v>0.9461000000000001</v>
+        <v>0.9728</v>
       </c>
       <c r="AG126" t="n">
-        <v>0.0856</v>
+        <v>0.096</v>
       </c>
       <c r="AH126" t="n">
-        <v>0.1568</v>
+        <v>0.1777</v>
       </c>
       <c r="AI126" t="n">
         <v>0</v>
@@ -18507,16 +18499,16 @@
         <v>1</v>
       </c>
       <c r="AK126" t="n">
-        <v>0.747</v>
+        <v>1</v>
       </c>
       <c r="AL126" t="n">
-        <v>0.717</v>
+        <v>0.9340000000000001</v>
       </c>
       <c r="AM126" t="n">
-        <v>0.244</v>
+        <v>0.495</v>
       </c>
       <c r="AN126" t="n">
-        <v>0.2</v>
+        <v>0.384</v>
       </c>
       <c r="AO126" t="n">
         <v>1</v>
@@ -19438,10 +19430,10 @@
         </is>
       </c>
       <c r="M133" t="n">
-        <v>0.136</v>
+        <v>0.135</v>
       </c>
       <c r="N133" t="n">
-        <v>0.109</v>
+        <v>0.107</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -19585,10 +19577,10 @@
         </is>
       </c>
       <c r="M134" t="n">
-        <v>0.025</v>
+        <v>0.026</v>
       </c>
       <c r="N134" t="n">
-        <v>0.025</v>
+        <v>0.026</v>
       </c>
       <c r="O134" t="inlineStr"/>
       <c r="P134" t="n">
@@ -23740,10 +23732,10 @@
         </is>
       </c>
       <c r="M163" t="n">
-        <v>0.478</v>
+        <v>0.485</v>
       </c>
       <c r="N163" t="n">
-        <v>0.394</v>
+        <v>0.407</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -26278,14 +26270,14 @@
         </is>
       </c>
       <c r="M181" t="n">
-        <v>0.385</v>
+        <v>0.374</v>
       </c>
       <c r="N181" t="n">
         <v>0.27</v>
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>zu23_technical</t>
+          <t>vbied</t>
         </is>
       </c>
       <c r="P181" t="n">
@@ -26384,7 +26376,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>4410</v>
+        <v>9052</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -26393,11 +26385,11 @@
       </c>
       <c r="F182" t="inlineStr"/>
       <c r="G182" t="n">
-        <v>54.4</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>Kém</t>
+          <t>Cần sửa</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -26405,105 +26397,97 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="J182" t="inlineStr">
-        <is>
-          <t>Tốt</t>
-        </is>
-      </c>
-      <c r="K182" t="inlineStr">
-        <is>
-          <t>Tốt</t>
-        </is>
-      </c>
+      <c r="J182" t="inlineStr"/>
+      <c r="K182" t="inlineStr"/>
       <c r="L182" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="M182" t="n">
-        <v>0.045</v>
+        <v>0.038</v>
       </c>
       <c r="N182" t="n">
-        <v>0.045</v>
+        <v>0</v>
       </c>
       <c r="O182" t="inlineStr"/>
       <c r="P182" t="n">
-        <v>1.3812</v>
+        <v>1.9512</v>
       </c>
       <c r="Q182" t="n">
-        <v>0.2285</v>
+        <v>0.252</v>
       </c>
       <c r="R182" t="n">
-        <v>8.3499</v>
+        <v>10.8497</v>
       </c>
       <c r="S182" t="n">
-        <v>0.0027</v>
+        <v>0.1039</v>
       </c>
       <c r="T182" t="n">
-        <v>118</v>
+        <v>264</v>
       </c>
       <c r="U182" t="n">
-        <v>64</v>
+        <v>117</v>
       </c>
       <c r="V182" t="n">
-        <v>0.384</v>
+        <v>0.522</v>
       </c>
       <c r="W182" t="n">
-        <v>21</v>
+        <v>72</v>
       </c>
       <c r="X182" t="n">
-        <v>55</v>
+        <v>106</v>
       </c>
       <c r="Y182" t="n">
-        <v>42</v>
+        <v>86</v>
       </c>
       <c r="Z182" t="n">
-        <v>0.33</v>
+        <v>0.4729</v>
       </c>
       <c r="AA182" t="n">
-        <v>0.252</v>
+        <v>0.3837</v>
       </c>
       <c r="AB182" t="n">
-        <v>166.6799</v>
+        <v>224.1503</v>
       </c>
       <c r="AC182" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="AD182" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="AE182" t="n">
-        <v>0.2958</v>
+        <v>0.147</v>
       </c>
       <c r="AF182" t="n">
-        <v>0.9728</v>
+        <v>0.8137</v>
       </c>
       <c r="AG182" t="n">
-        <v>0.0825</v>
+        <v>0.0415</v>
       </c>
       <c r="AH182" t="n">
-        <v>0.1179</v>
+        <v>0.06809999999999999</v>
       </c>
       <c r="AI182" t="n">
         <v>0</v>
       </c>
       <c r="AJ182" t="n">
-        <v>0.305</v>
+        <v>0.761</v>
       </c>
       <c r="AK182" t="n">
-        <v>0.963</v>
+        <v>1</v>
       </c>
       <c r="AL182" t="n">
-        <v>0.844</v>
+        <v>1</v>
       </c>
       <c r="AM182" t="n">
-        <v>0.504</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="AN182" t="n">
-        <v>0.306</v>
+        <v>0.456</v>
       </c>
       <c r="AO182" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="183">
@@ -31871,7 +31855,7 @@
         </is>
       </c>
       <c r="M220" t="n">
-        <v>0.591</v>
+        <v>0.59</v>
       </c>
       <c r="N220" t="n">
         <v>0.435</v>
@@ -32021,7 +32005,7 @@
         <v>0.029</v>
       </c>
       <c r="N221" t="n">
-        <v>0.029</v>
+        <v>0.03</v>
       </c>
       <c r="O221" t="inlineStr"/>
       <c r="P221" t="n">
@@ -32161,10 +32145,10 @@
         </is>
       </c>
       <c r="M222" t="n">
-        <v>0.092</v>
+        <v>0.089</v>
       </c>
       <c r="N222" t="n">
-        <v>0.029</v>
+        <v>0.024</v>
       </c>
       <c r="O222" t="inlineStr"/>
       <c r="P222" t="n">
@@ -33407,119 +33391,103 @@
         </is>
       </c>
       <c r="D231" t="n">
-        <v>1996</v>
+        <v>7436</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="F231" t="inlineStr">
-        <is>
-          <t>triangles_floor: 1996 (floor 2100, class 3000-5000) | parts: missing axles | own_geometry: 56% of triangles shared (most with rocket_technical) | not_single_block: 1 sloped face directions</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr"/>
       <c r="G231" t="n">
-        <v>77.7</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>Cần sửa</t>
+          <t>Tốt</t>
         </is>
       </c>
       <c r="I231" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="J231" t="inlineStr">
-        <is>
-          <t>Tốt</t>
-        </is>
-      </c>
-      <c r="K231" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr"/>
+      <c r="K231" t="inlineStr"/>
       <c r="L231" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="M231" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.019</v>
       </c>
       <c r="N231" t="n">
-        <v>0.394</v>
-      </c>
-      <c r="O231" t="inlineStr">
-        <is>
-          <t>rocket_technical</t>
-        </is>
-      </c>
+        <v>0.008</v>
+      </c>
+      <c r="O231" t="inlineStr"/>
       <c r="P231" t="n">
-        <v>1.3737</v>
+        <v>1.5041</v>
       </c>
       <c r="Q231" t="n">
-        <v>0.3416</v>
+        <v>0.362</v>
       </c>
       <c r="R231" t="n">
-        <v>12.0746</v>
+        <v>17.1551</v>
       </c>
       <c r="S231" t="n">
-        <v>0.009900000000000001</v>
+        <v>0.0007</v>
       </c>
       <c r="T231" t="n">
-        <v>45</v>
+        <v>272</v>
       </c>
       <c r="U231" t="n">
-        <v>25</v>
+        <v>93</v>
       </c>
       <c r="V231" t="n">
-        <v>0.4608</v>
+        <v>1.4347</v>
       </c>
       <c r="W231" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="X231" t="n">
-        <v>22</v>
+        <v>68</v>
       </c>
       <c r="Y231" t="n">
-        <v>13</v>
+        <v>181</v>
       </c>
       <c r="Z231" t="n">
-        <v>0.4055</v>
+        <v>1.0491</v>
       </c>
       <c r="AA231" t="n">
-        <v>0.2396</v>
+        <v>2.7923</v>
       </c>
       <c r="AB231" t="n">
-        <v>54.2563</v>
+        <v>64.8205</v>
       </c>
       <c r="AC231" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AD231" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="AE231" t="n">
-        <v>0.1246</v>
+        <v>0.117</v>
       </c>
       <c r="AF231" t="n">
-        <v>0.9987</v>
+        <v>0.8137</v>
       </c>
       <c r="AG231" t="n">
-        <v>0.1834</v>
+        <v>0.0433</v>
       </c>
       <c r="AH231" t="n">
-        <v>0.2533</v>
+        <v>0.2765</v>
       </c>
       <c r="AI231" t="n">
         <v>0</v>
       </c>
       <c r="AJ231" t="n">
-        <v>0.708</v>
+        <v>0.955</v>
       </c>
       <c r="AK231" t="n">
         <v>1</v>
@@ -33528,10 +33496,10 @@
         <v>1</v>
       </c>
       <c r="AM231" t="n">
-        <v>0.822</v>
+        <v>1</v>
       </c>
       <c r="AN231" t="n">
-        <v>0.573</v>
+        <v>1</v>
       </c>
       <c r="AO231" t="n">
         <v>0.5</v>

</xml_diff>

<commit_message>
Prompt 35 wave 1: joined report, full gate refresh (35/230 pass), gate prints UTF-8 on Windows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/models/quality_report.xlsx
+++ b/Docs/models/quality_report.xlsx
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>0.057</v>
+        <v>0.058</v>
       </c>
       <c r="O2" t="n">
         <v>0.126</v>
@@ -1731,10 +1731,10 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="O9" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="n">
@@ -2438,113 +2438,97 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>3388</v>
+        <v>7492</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>parts: missing axles | own_geometry: 65% of triangles shared (most with supply_truck)</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>70.09999999999999</v>
+        <v>92</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Cần sửa</t>
+          <t>Tốt</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Tốt</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N14" t="n">
-        <v>0.653</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="O14" t="n">
-        <v>0.497</v>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>supply_truck</t>
-        </is>
-      </c>
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="P14" t="inlineStr"/>
       <c r="Q14" t="n">
-        <v>1.767</v>
+        <v>1.8834</v>
       </c>
       <c r="R14" t="n">
-        <v>0.2324</v>
+        <v>0.2929</v>
       </c>
       <c r="S14" t="n">
-        <v>7.563</v>
+        <v>9.5406</v>
       </c>
       <c r="T14" t="n">
-        <v>0.0043</v>
+        <v>0.0074</v>
       </c>
       <c r="U14" t="n">
-        <v>136</v>
+        <v>261</v>
       </c>
       <c r="V14" t="n">
-        <v>39</v>
+        <v>112</v>
       </c>
       <c r="W14" t="n">
-        <v>0.2493</v>
+        <v>0.7023</v>
       </c>
       <c r="X14" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="Y14" t="n">
-        <v>115</v>
+        <v>167</v>
       </c>
       <c r="Z14" t="n">
-        <v>12</v>
+        <v>77</v>
       </c>
       <c r="AA14" t="n">
-        <v>0.735</v>
+        <v>1.0471</v>
       </c>
       <c r="AB14" t="n">
-        <v>0.0767</v>
+        <v>0.4828</v>
       </c>
       <c r="AC14" t="n">
-        <v>156.4595</v>
+        <v>159.4865</v>
       </c>
       <c r="AD14" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="AE14" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="AF14" t="n">
-        <v>0.15</v>
+        <v>0.1605</v>
       </c>
       <c r="AG14" t="n">
-        <v>0.9899</v>
+        <v>0.9641</v>
       </c>
       <c r="AH14" t="n">
-        <v>0.1091</v>
+        <v>0.089</v>
       </c>
       <c r="AI14" t="n">
-        <v>0.09470000000000001</v>
+        <v>0.1986</v>
       </c>
       <c r="AJ14" t="n">
         <v>0</v>
@@ -2553,16 +2537,16 @@
         <v>1</v>
       </c>
       <c r="AL14" t="n">
-        <v>0.869</v>
+        <v>1</v>
       </c>
       <c r="AM14" t="n">
-        <v>0.634</v>
+        <v>0.8</v>
       </c>
       <c r="AN14" t="n">
-        <v>0.445</v>
+        <v>1</v>
       </c>
       <c r="AO14" t="n">
-        <v>0.581</v>
+        <v>1</v>
       </c>
       <c r="AP14" t="n">
         <v>0.5</v>
@@ -2622,7 +2606,7 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="O15" t="n">
-        <v>0.01</v>
+        <v>0.011</v>
       </c>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="n">
@@ -2915,7 +2899,7 @@
         </is>
       </c>
       <c r="N17" t="n">
-        <v>0.038</v>
+        <v>0.036</v>
       </c>
       <c r="O17" t="n">
         <v>0.03</v>
@@ -3063,7 +3047,7 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>0.158</v>
+        <v>0.164</v>
       </c>
       <c r="O18" t="n">
         <v>0.186</v>
@@ -3363,7 +3347,7 @@
         </is>
       </c>
       <c r="N20" t="n">
-        <v>0.038</v>
+        <v>0.092</v>
       </c>
       <c r="O20" t="n">
         <v>0.098</v>
@@ -4987,12 +4971,16 @@
         </is>
       </c>
       <c r="N31" t="n">
-        <v>0.032</v>
+        <v>0.109</v>
       </c>
       <c r="O31" t="n">
         <v>0.043</v>
       </c>
-      <c r="P31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>mlrs</t>
+        </is>
+      </c>
       <c r="Q31" t="n">
         <v>1.5867</v>
       </c>
@@ -5423,7 +5411,7 @@
         </is>
       </c>
       <c r="N34" t="n">
-        <v>0.032</v>
+        <v>0.033</v>
       </c>
       <c r="O34" t="n">
         <v>0.082</v>
@@ -5559,10 +5547,10 @@
         </is>
       </c>
       <c r="N35" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="O35" t="n">
-        <v>0.163</v>
+        <v>0.156</v>
       </c>
       <c r="P35" t="inlineStr">
         <is>
@@ -6307,10 +6295,10 @@
         </is>
       </c>
       <c r="N40" t="n">
-        <v>0.054</v>
+        <v>0.059</v>
       </c>
       <c r="O40" t="n">
-        <v>0.016</v>
+        <v>0.023</v>
       </c>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="n">
@@ -7051,10 +7039,10 @@
         </is>
       </c>
       <c r="N45" t="n">
-        <v>0.031</v>
+        <v>0.032</v>
       </c>
       <c r="O45" t="n">
-        <v>0.031</v>
+        <v>0.032</v>
       </c>
       <c r="P45" t="inlineStr"/>
       <c r="Q45" t="n">
@@ -7199,7 +7187,7 @@
         </is>
       </c>
       <c r="N46" t="n">
-        <v>0.05</v>
+        <v>0.051</v>
       </c>
       <c r="O46" t="n">
         <v>0.052</v>
@@ -7495,10 +7483,10 @@
         </is>
       </c>
       <c r="N48" t="n">
-        <v>0.049</v>
+        <v>0.051</v>
       </c>
       <c r="O48" t="n">
-        <v>0.041</v>
+        <v>0.043</v>
       </c>
       <c r="P48" t="inlineStr"/>
       <c r="Q48" t="n">
@@ -7643,10 +7631,10 @@
         </is>
       </c>
       <c r="N49" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.09</v>
       </c>
       <c r="O49" t="n">
-        <v>0.026</v>
+        <v>0.034</v>
       </c>
       <c r="P49" t="inlineStr"/>
       <c r="Q49" t="n">
@@ -8194,113 +8182,101 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>2396</v>
+        <v>6956</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>parts: missing axles, stowage | own_geometry: 57% of triangles shared (most with shahed_truck) | not_single_block: 2 sloped face directions</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Cần sửa</t>
+          <t>Tốt</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>Tốt</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N53" t="n">
-        <v>0.5659999999999999</v>
+        <v>0.126</v>
       </c>
       <c r="O53" t="n">
-        <v>0.412</v>
+        <v>0.147</v>
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>shahed_truck</t>
+          <t>elite_mlrs</t>
         </is>
       </c>
       <c r="Q53" t="n">
-        <v>1.5892</v>
+        <v>1.5996</v>
       </c>
       <c r="R53" t="n">
-        <v>0.2156</v>
+        <v>0.2508</v>
       </c>
       <c r="S53" t="n">
-        <v>7.9092</v>
+        <v>7.775</v>
       </c>
       <c r="T53" t="n">
-        <v>0.013</v>
+        <v>0.0014</v>
       </c>
       <c r="U53" t="n">
-        <v>69</v>
+        <v>212</v>
       </c>
       <c r="V53" t="n">
-        <v>40</v>
+        <v>106</v>
       </c>
       <c r="W53" t="n">
-        <v>0.2978</v>
+        <v>0.6981000000000001</v>
       </c>
       <c r="X53" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="Y53" t="n">
-        <v>45</v>
+        <v>139</v>
       </c>
       <c r="Z53" t="n">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="AA53" t="n">
-        <v>0.335</v>
+        <v>0.9155</v>
       </c>
       <c r="AB53" t="n">
-        <v>0.0893</v>
+        <v>0.3622</v>
       </c>
       <c r="AC53" t="n">
-        <v>134.3258</v>
+        <v>151.8327</v>
       </c>
       <c r="AD53" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AE53" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="AF53" t="n">
-        <v>0.2071</v>
+        <v>0.1327</v>
       </c>
       <c r="AG53" t="n">
-        <v>0.9905</v>
+        <v>0.9634</v>
       </c>
       <c r="AH53" t="n">
-        <v>0.1341</v>
+        <v>0.07829999999999999</v>
       </c>
       <c r="AI53" t="n">
-        <v>0.2335</v>
+        <v>0.2107</v>
       </c>
       <c r="AJ53" t="n">
         <v>0</v>
@@ -8309,19 +8285,19 @@
         <v>1</v>
       </c>
       <c r="AL53" t="n">
-        <v>0.806</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="AM53" t="n">
-        <v>0.663</v>
+        <v>0.652</v>
       </c>
       <c r="AN53" t="n">
-        <v>0.531</v>
+        <v>1</v>
       </c>
       <c r="AO53" t="n">
-        <v>0.359</v>
+        <v>0.881</v>
       </c>
       <c r="AP53" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="54">
@@ -9131,10 +9107,10 @@
         </is>
       </c>
       <c r="N59" t="n">
-        <v>0.078</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="O59" t="n">
-        <v>0.04</v>
+        <v>0.042</v>
       </c>
       <c r="P59" t="inlineStr"/>
       <c r="Q59" t="n">
@@ -9863,10 +9839,10 @@
         </is>
       </c>
       <c r="N64" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="O64" t="n">
         <v>0.037</v>
-      </c>
-      <c r="O64" t="n">
-        <v>0.036</v>
       </c>
       <c r="P64" t="inlineStr"/>
       <c r="Q64" t="n">
@@ -10011,10 +9987,10 @@
         </is>
       </c>
       <c r="N65" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="O65" t="n">
         <v>0.025</v>
-      </c>
-      <c r="O65" t="n">
-        <v>0.024</v>
       </c>
       <c r="P65" t="inlineStr"/>
       <c r="Q65" t="n">
@@ -10751,10 +10727,10 @@
         </is>
       </c>
       <c r="N70" t="n">
-        <v>0.025</v>
+        <v>0.026</v>
       </c>
       <c r="O70" t="n">
-        <v>0.041</v>
+        <v>0.043</v>
       </c>
       <c r="P70" t="inlineStr"/>
       <c r="Q70" t="n">
@@ -11355,7 +11331,7 @@
         </is>
       </c>
       <c r="N74" t="n">
-        <v>0.895</v>
+        <v>0.9</v>
       </c>
       <c r="O74" t="n">
         <v>0.902</v>
@@ -11466,20 +11442,16 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>7288</v>
+        <v>10002</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>parts: missing mantlet, idler</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr"/>
       <c r="H75" t="n">
-        <v>94.3</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
@@ -11488,112 +11460,100 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K75" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
-      <c r="L75" t="inlineStr">
-        <is>
-          <t>Kém</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
       <c r="M75" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N75" t="n">
-        <v>0.864</v>
+        <v>0.019</v>
       </c>
       <c r="O75" t="n">
-        <v>0.914</v>
-      </c>
-      <c r="P75" t="inlineStr">
-        <is>
-          <t>twin_tank</t>
-        </is>
-      </c>
+        <v>0.017</v>
+      </c>
+      <c r="P75" t="inlineStr"/>
       <c r="Q75" t="n">
-        <v>1.3126</v>
+        <v>1.3279</v>
       </c>
       <c r="R75" t="n">
-        <v>0.2626</v>
+        <v>0.2652</v>
       </c>
       <c r="S75" t="n">
-        <v>8.7125</v>
+        <v>6.9078</v>
       </c>
       <c r="T75" t="n">
-        <v>0.0024</v>
+        <v>0.0004</v>
       </c>
       <c r="U75" t="n">
-        <v>165</v>
+        <v>341</v>
       </c>
       <c r="V75" t="n">
-        <v>68</v>
+        <v>105</v>
       </c>
       <c r="W75" t="n">
-        <v>0.4403</v>
+        <v>0.6904</v>
       </c>
       <c r="X75" t="n">
         <v>15</v>
       </c>
       <c r="Y75" t="n">
-        <v>104</v>
+        <v>220</v>
       </c>
       <c r="Z75" t="n">
-        <v>46</v>
+        <v>106</v>
       </c>
       <c r="AA75" t="n">
-        <v>0.6735</v>
+        <v>1.4466</v>
       </c>
       <c r="AB75" t="n">
-        <v>0.2979</v>
+        <v>0.697</v>
       </c>
       <c r="AC75" t="n">
-        <v>154.4276</v>
+        <v>152.0785</v>
       </c>
       <c r="AD75" t="n">
         <v>8</v>
       </c>
       <c r="AE75" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="AF75" t="n">
-        <v>0.1557</v>
+        <v>0.1744</v>
       </c>
       <c r="AG75" t="n">
-        <v>0.981</v>
+        <v>0.9261</v>
       </c>
       <c r="AH75" t="n">
-        <v>0.1065</v>
+        <v>0.06710000000000001</v>
       </c>
       <c r="AI75" t="n">
-        <v>0.2309</v>
+        <v>0.1618</v>
       </c>
       <c r="AJ75" t="n">
         <v>0</v>
       </c>
       <c r="AK75" t="n">
-        <v>0.799</v>
+        <v>0.838</v>
       </c>
       <c r="AL75" t="n">
         <v>1</v>
       </c>
       <c r="AM75" t="n">
-        <v>1</v>
+        <v>0.908</v>
       </c>
       <c r="AN75" t="n">
         <v>1</v>
       </c>
       <c r="AO75" t="n">
-        <v>0.954</v>
+        <v>1</v>
       </c>
       <c r="AP75" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="76">
@@ -11618,113 +11578,101 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>2692</v>
+        <v>7446</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>parts: missing axles, stowage | own_geometry: 87% of triangles shared (most with mlrs) | not_single_block: 2 sloped face directions</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr"/>
       <c r="H76" t="n">
-        <v>68</v>
+        <v>87.7</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Cần sửa</t>
+          <t>Tốt</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K76" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
-      <c r="L76" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" t="inlineStr"/>
       <c r="M76" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N76" t="n">
-        <v>0.866</v>
+        <v>0.152</v>
       </c>
       <c r="O76" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.177</v>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>mlrs</t>
+          <t>lancet_truck</t>
         </is>
       </c>
       <c r="Q76" t="n">
-        <v>1.6477</v>
+        <v>1.8438</v>
       </c>
       <c r="R76" t="n">
-        <v>0.1868</v>
+        <v>0.2143</v>
       </c>
       <c r="S76" t="n">
-        <v>6.4757</v>
+        <v>5.0479</v>
       </c>
       <c r="T76" t="n">
-        <v>0.0133</v>
+        <v>0.0241</v>
       </c>
       <c r="U76" t="n">
-        <v>75</v>
+        <v>219</v>
       </c>
       <c r="V76" t="n">
-        <v>37</v>
+        <v>104</v>
       </c>
       <c r="W76" t="n">
-        <v>0.2437</v>
+        <v>0.5588</v>
       </c>
       <c r="X76" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="Y76" t="n">
-        <v>49</v>
+        <v>108</v>
       </c>
       <c r="Z76" t="n">
-        <v>18</v>
+        <v>90</v>
       </c>
       <c r="AA76" t="n">
-        <v>0.3227</v>
+        <v>0.5803</v>
       </c>
       <c r="AB76" t="n">
-        <v>0.1186</v>
+        <v>0.4836</v>
       </c>
       <c r="AC76" t="n">
-        <v>151.8238</v>
+        <v>186.1109</v>
       </c>
       <c r="AD76" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="AE76" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="AF76" t="n">
-        <v>0.2156</v>
+        <v>0.1168</v>
       </c>
       <c r="AG76" t="n">
-        <v>0.99</v>
+        <v>0.981</v>
       </c>
       <c r="AH76" t="n">
-        <v>0.1044</v>
+        <v>0.106</v>
       </c>
       <c r="AI76" t="n">
-        <v>0.2069</v>
+        <v>0.1995</v>
       </c>
       <c r="AJ76" t="n">
         <v>0</v>
@@ -11733,16 +11681,16 @@
         <v>1</v>
       </c>
       <c r="AL76" t="n">
-        <v>0.699</v>
+        <v>0.801</v>
       </c>
       <c r="AM76" t="n">
-        <v>0.543</v>
+        <v>0.423</v>
       </c>
       <c r="AN76" t="n">
-        <v>0.435</v>
+        <v>0.997</v>
       </c>
       <c r="AO76" t="n">
-        <v>0.38</v>
+        <v>0.959</v>
       </c>
       <c r="AP76" t="n">
         <v>1</v>
@@ -12703,7 +12651,7 @@
         </is>
       </c>
       <c r="N83" t="n">
-        <v>0.151</v>
+        <v>0.163</v>
       </c>
       <c r="O83" t="n">
         <v>0.039</v>
@@ -12991,10 +12939,10 @@
         </is>
       </c>
       <c r="N85" t="n">
-        <v>0.033</v>
+        <v>0.034</v>
       </c>
       <c r="O85" t="n">
-        <v>0.063</v>
+        <v>0.064</v>
       </c>
       <c r="P85" t="inlineStr"/>
       <c r="Q85" t="n">
@@ -13139,10 +13087,10 @@
         </is>
       </c>
       <c r="N86" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="O86" t="n">
-        <v>0.076</v>
+        <v>0.081</v>
       </c>
       <c r="P86" t="inlineStr"/>
       <c r="Q86" t="n">
@@ -13562,7 +13510,7 @@
         <v>0.046</v>
       </c>
       <c r="O89" t="n">
-        <v>0.106</v>
+        <v>0.107</v>
       </c>
       <c r="P89" t="inlineStr">
         <is>
@@ -13847,14 +13795,14 @@
         </is>
       </c>
       <c r="N91" t="n">
-        <v>0.713</v>
+        <v>0.187</v>
       </c>
       <c r="O91" t="n">
-        <v>0.489</v>
+        <v>0.038</v>
       </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t>lancet_truck</t>
+          <t>artillery</t>
         </is>
       </c>
       <c r="Q91" t="n">
@@ -14295,10 +14243,10 @@
         </is>
       </c>
       <c r="N94" t="n">
-        <v>0.697</v>
+        <v>0.698</v>
       </c>
       <c r="O94" t="n">
-        <v>0.516</v>
+        <v>0.517</v>
       </c>
       <c r="P94" t="inlineStr">
         <is>
@@ -14447,7 +14395,7 @@
         </is>
       </c>
       <c r="N95" t="n">
-        <v>0.024</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="O95" t="n">
         <v>0.01</v>
@@ -14595,10 +14543,10 @@
         </is>
       </c>
       <c r="N96" t="n">
-        <v>0.091</v>
+        <v>0.09</v>
       </c>
       <c r="O96" t="n">
-        <v>0.047</v>
+        <v>0.046</v>
       </c>
       <c r="P96" t="inlineStr"/>
       <c r="Q96" t="n">
@@ -16075,10 +16023,10 @@
         </is>
       </c>
       <c r="N106" t="n">
-        <v>0.06</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="O106" t="n">
-        <v>0.026</v>
+        <v>0.031</v>
       </c>
       <c r="P106" t="inlineStr"/>
       <c r="Q106" t="n">
@@ -16807,7 +16755,7 @@
         </is>
       </c>
       <c r="N111" t="n">
-        <v>0.902</v>
+        <v>0.907</v>
       </c>
       <c r="O111" t="n">
         <v>0.925</v>
@@ -18583,10 +18531,10 @@
         </is>
       </c>
       <c r="N123" t="n">
-        <v>0.261</v>
+        <v>0.281</v>
       </c>
       <c r="O123" t="n">
-        <v>0.227</v>
+        <v>0.222</v>
       </c>
       <c r="P123" t="inlineStr">
         <is>
@@ -18887,10 +18835,10 @@
         </is>
       </c>
       <c r="N125" t="n">
-        <v>0.108</v>
+        <v>0.123</v>
       </c>
       <c r="O125" t="n">
-        <v>0.055</v>
+        <v>0.051</v>
       </c>
       <c r="P125" t="inlineStr">
         <is>
@@ -19027,10 +18975,10 @@
         </is>
       </c>
       <c r="N126" t="n">
-        <v>0.037</v>
+        <v>0.038</v>
       </c>
       <c r="O126" t="n">
-        <v>0.01</v>
+        <v>0.011</v>
       </c>
       <c r="P126" t="inlineStr"/>
       <c r="Q126" t="n">
@@ -19430,131 +19378,119 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>2314</v>
+        <v>7300</v>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G129" t="inlineStr">
-        <is>
-          <t>parts: missing axles | own_geometry: 79% of triangles shared (most with fpv_carrier)</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr"/>
       <c r="H129" t="n">
-        <v>62.9</v>
+        <v>94.3</v>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Cần sửa</t>
+          <t>Tốt</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K129" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
-      <c r="L129" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr"/>
+      <c r="L129" t="inlineStr"/>
       <c r="M129" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N129" t="n">
-        <v>0.787</v>
+        <v>0.139</v>
       </c>
       <c r="O129" t="n">
-        <v>0.548</v>
+        <v>0.183</v>
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>fpv_carrier</t>
+          <t>elite_mlrs</t>
         </is>
       </c>
       <c r="Q129" t="n">
-        <v>1.4003</v>
+        <v>1.8937</v>
       </c>
       <c r="R129" t="n">
-        <v>0.2033</v>
+        <v>0.2699</v>
       </c>
       <c r="S129" t="n">
-        <v>6.0347</v>
+        <v>7.4263</v>
       </c>
       <c r="T129" t="n">
-        <v>0.0237</v>
+        <v>0.029</v>
       </c>
       <c r="U129" t="n">
-        <v>68</v>
+        <v>237</v>
       </c>
       <c r="V129" t="n">
-        <v>35</v>
+        <v>97</v>
       </c>
       <c r="W129" t="n">
-        <v>0.2579</v>
+        <v>0.854</v>
       </c>
       <c r="X129" t="n">
+        <v>12</v>
+      </c>
+      <c r="Y129" t="n">
+        <v>122</v>
+      </c>
+      <c r="Z129" t="n">
+        <v>103</v>
+      </c>
+      <c r="AA129" t="n">
+        <v>1.0741</v>
+      </c>
+      <c r="AB129" t="n">
+        <v>0.9068000000000001</v>
+      </c>
+      <c r="AC129" t="n">
+        <v>113.5857</v>
+      </c>
+      <c r="AD129" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE129" t="n">
         <v>10</v>
       </c>
-      <c r="Y129" t="n">
-        <v>35</v>
-      </c>
-      <c r="Z129" t="n">
-        <v>23</v>
-      </c>
-      <c r="AA129" t="n">
-        <v>0.2579</v>
-      </c>
-      <c r="AB129" t="n">
-        <v>0.1695</v>
-      </c>
-      <c r="AC129" t="n">
-        <v>135.7238</v>
-      </c>
-      <c r="AD129" t="n">
-        <v>4</v>
-      </c>
-      <c r="AE129" t="n">
-        <v>9</v>
-      </c>
       <c r="AF129" t="n">
-        <v>0.3964</v>
+        <v>0.1712</v>
       </c>
       <c r="AG129" t="n">
-        <v>0.9987</v>
+        <v>0.9035</v>
       </c>
       <c r="AH129" t="n">
-        <v>0.1463</v>
+        <v>0.0655</v>
       </c>
       <c r="AI129" t="n">
-        <v>0.1625</v>
+        <v>0.2388</v>
       </c>
       <c r="AJ129" t="n">
         <v>0</v>
       </c>
       <c r="AK129" t="n">
-        <v>0.758</v>
+        <v>1</v>
       </c>
       <c r="AL129" t="n">
-        <v>0.76</v>
+        <v>1</v>
       </c>
       <c r="AM129" t="n">
-        <v>0.506</v>
+        <v>0.622</v>
       </c>
       <c r="AN129" t="n">
-        <v>0.46</v>
+        <v>1</v>
       </c>
       <c r="AO129" t="n">
-        <v>0.382</v>
+        <v>1</v>
       </c>
       <c r="AP129" t="n">
         <v>1</v>
@@ -20215,10 +20151,10 @@
         </is>
       </c>
       <c r="N134" t="n">
-        <v>0.026</v>
+        <v>0.028</v>
       </c>
       <c r="O134" t="n">
-        <v>0.026</v>
+        <v>0.028</v>
       </c>
       <c r="P134" t="inlineStr"/>
       <c r="Q134" t="n">
@@ -20811,7 +20747,7 @@
         </is>
       </c>
       <c r="N138" t="n">
-        <v>0.083</v>
+        <v>0.092</v>
       </c>
       <c r="O138" t="n">
         <v>0.067</v>
@@ -20955,14 +20891,14 @@
         </is>
       </c>
       <c r="N139" t="n">
-        <v>0.801</v>
+        <v>0.52</v>
       </c>
       <c r="O139" t="n">
-        <v>0.898</v>
+        <v>0.459</v>
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>elite_mbt</t>
+          <t>twin_tank</t>
         </is>
       </c>
       <c r="Q139" t="n">
@@ -21103,10 +21039,10 @@
         </is>
       </c>
       <c r="N140" t="n">
-        <v>0.064</v>
+        <v>0.065</v>
       </c>
       <c r="O140" t="n">
-        <v>0.107</v>
+        <v>0.109</v>
       </c>
       <c r="P140" t="inlineStr">
         <is>
@@ -21806,29 +21742,25 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>4914</v>
+        <v>6314</v>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G145" t="inlineStr">
-        <is>
-          <t>own_geometry: 40% of triangles shared (most with nlos_atgm_vehicle)</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr"/>
       <c r="H145" t="n">
-        <v>79.7</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>Cần sửa</t>
+          <t>Tốt</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K145" t="inlineStr"/>
@@ -21839,90 +21771,86 @@
         </is>
       </c>
       <c r="N145" t="n">
-        <v>0.397</v>
+        <v>0.066</v>
       </c>
       <c r="O145" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="P145" t="inlineStr">
-        <is>
-          <t>nlos_atgm_vehicle</t>
-        </is>
-      </c>
+        <v>0.032</v>
+      </c>
+      <c r="P145" t="inlineStr"/>
       <c r="Q145" t="n">
-        <v>1.6943</v>
+        <v>1.4051</v>
       </c>
       <c r="R145" t="n">
-        <v>0.2561</v>
+        <v>0.2127</v>
       </c>
       <c r="S145" t="n">
-        <v>11.6007</v>
+        <v>7.5174</v>
       </c>
       <c r="T145" t="n">
-        <v>0.0074</v>
+        <v>0.0034</v>
       </c>
       <c r="U145" t="n">
-        <v>144</v>
+        <v>194</v>
       </c>
       <c r="V145" t="n">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="W145" t="n">
-        <v>0.2871</v>
+        <v>0.6274</v>
       </c>
       <c r="X145" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="Y145" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Z145" t="n">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="AA145" t="n">
-        <v>0.6004</v>
+        <v>0.8218</v>
       </c>
       <c r="AB145" t="n">
-        <v>0.2153</v>
+        <v>0.7776</v>
       </c>
       <c r="AC145" t="n">
-        <v>153.2419</v>
+        <v>113.1663</v>
       </c>
       <c r="AD145" t="n">
         <v>6</v>
       </c>
       <c r="AE145" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AF145" t="n">
-        <v>0.3741</v>
+        <v>0.083</v>
       </c>
       <c r="AG145" t="n">
-        <v>0.9634</v>
+        <v>0.9288999999999999</v>
       </c>
       <c r="AH145" t="n">
-        <v>0.09130000000000001</v>
+        <v>0.06610000000000001</v>
       </c>
       <c r="AI145" t="n">
-        <v>0.09909999999999999</v>
+        <v>0.3119</v>
       </c>
       <c r="AJ145" t="n">
         <v>0</v>
       </c>
       <c r="AK145" t="n">
-        <v>1</v>
+        <v>0.768</v>
       </c>
       <c r="AL145" t="n">
-        <v>0.958</v>
+        <v>0.795</v>
       </c>
       <c r="AM145" t="n">
-        <v>0.972</v>
+        <v>0.63</v>
       </c>
       <c r="AN145" t="n">
-        <v>0.512</v>
+        <v>1</v>
       </c>
       <c r="AO145" t="n">
-        <v>0.702</v>
+        <v>1</v>
       </c>
       <c r="AP145" t="n">
         <v>0.5</v>
@@ -21991,10 +21919,10 @@
         </is>
       </c>
       <c r="N146" t="n">
-        <v>0.095</v>
+        <v>0.094</v>
       </c>
       <c r="O146" t="n">
-        <v>0.047</v>
+        <v>0.043</v>
       </c>
       <c r="P146" t="inlineStr"/>
       <c r="Q146" t="n">
@@ -22727,10 +22655,10 @@
         </is>
       </c>
       <c r="N151" t="n">
-        <v>0.075</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="O151" t="n">
-        <v>0.083</v>
+        <v>0.08</v>
       </c>
       <c r="P151" t="inlineStr"/>
       <c r="Q151" t="n">
@@ -22875,10 +22803,10 @@
         </is>
       </c>
       <c r="N152" t="n">
-        <v>0.062</v>
+        <v>0.06</v>
       </c>
       <c r="O152" t="n">
-        <v>0.068</v>
+        <v>0.066</v>
       </c>
       <c r="P152" t="inlineStr"/>
       <c r="Q152" t="n">
@@ -23023,10 +22951,10 @@
         </is>
       </c>
       <c r="N153" t="n">
-        <v>0.083</v>
+        <v>0.08</v>
       </c>
       <c r="O153" t="n">
-        <v>0.092</v>
+        <v>0.089</v>
       </c>
       <c r="P153" t="inlineStr"/>
       <c r="Q153" t="n">
@@ -23323,14 +23251,14 @@
         </is>
       </c>
       <c r="N155" t="n">
-        <v>0.867</v>
+        <v>0.117</v>
       </c>
       <c r="O155" t="n">
-        <v>0.944</v>
+        <v>0.021</v>
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>elite_mlrs</t>
+          <t>shahed_truck</t>
         </is>
       </c>
       <c r="Q155" t="n">
@@ -23619,10 +23547,10 @@
         </is>
       </c>
       <c r="N157" t="n">
-        <v>0.133</v>
+        <v>0.135</v>
       </c>
       <c r="O157" t="n">
-        <v>0.195</v>
+        <v>0.198</v>
       </c>
       <c r="P157" t="inlineStr">
         <is>
@@ -24219,14 +24147,14 @@
         </is>
       </c>
       <c r="N161" t="n">
-        <v>0.866</v>
+        <v>0.115</v>
       </c>
       <c r="O161" t="n">
-        <v>0.556</v>
+        <v>0.028</v>
       </c>
       <c r="P161" t="inlineStr">
         <is>
-          <t>smoke_carrier</t>
+          <t>command_vehicle</t>
         </is>
       </c>
       <c r="Q161" t="n">
@@ -24371,10 +24299,10 @@
         </is>
       </c>
       <c r="N162" t="n">
-        <v>0.128</v>
+        <v>0.129</v>
       </c>
       <c r="O162" t="n">
-        <v>0.152</v>
+        <v>0.154</v>
       </c>
       <c r="P162" t="inlineStr">
         <is>
@@ -24491,7 +24419,7 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>own_geometry: 48% of triangles shared (most with microwave_vehicle)</t>
+          <t>own_geometry: 32% of triangles shared (most with interceptor_drone_vehicle)</t>
         </is>
       </c>
       <c r="H163" t="n">
@@ -24515,14 +24443,14 @@
         </is>
       </c>
       <c r="N163" t="n">
-        <v>0.481</v>
+        <v>0.315</v>
       </c>
       <c r="O163" t="n">
-        <v>0.4</v>
+        <v>0.23</v>
       </c>
       <c r="P163" t="inlineStr">
         <is>
-          <t>microwave_vehicle</t>
+          <t>interceptor_drone_vehicle</t>
         </is>
       </c>
       <c r="Q163" t="n">
@@ -25395,10 +25323,10 @@
         </is>
       </c>
       <c r="N169" t="n">
-        <v>0.137</v>
+        <v>0.163</v>
       </c>
       <c r="O169" t="n">
-        <v>0.092</v>
+        <v>0.098</v>
       </c>
       <c r="P169" t="inlineStr">
         <is>
@@ -25535,7 +25463,7 @@
         </is>
       </c>
       <c r="N170" t="n">
-        <v>0.047</v>
+        <v>0.053</v>
       </c>
       <c r="O170" t="n">
         <v>0.037</v>
@@ -25683,10 +25611,10 @@
         </is>
       </c>
       <c r="N171" t="n">
-        <v>0.164</v>
+        <v>0.165</v>
       </c>
       <c r="O171" t="n">
-        <v>0.164</v>
+        <v>0.166</v>
       </c>
       <c r="P171" t="inlineStr">
         <is>
@@ -25983,7 +25911,7 @@
         </is>
       </c>
       <c r="N173" t="n">
-        <v>0.065</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="O173" t="n">
         <v>0.077</v>
@@ -26263,12 +26191,16 @@
         </is>
       </c>
       <c r="N175" t="n">
-        <v>0.095</v>
+        <v>0.117</v>
       </c>
       <c r="O175" t="n">
-        <v>0.007</v>
-      </c>
-      <c r="P175" t="inlineStr"/>
+        <v>0.004</v>
+      </c>
+      <c r="P175" t="inlineStr">
+        <is>
+          <t>radar_scout</t>
+        </is>
+      </c>
       <c r="Q175" t="n">
         <v>1.5917</v>
       </c>
@@ -26698,7 +26630,7 @@
         <v>0.007</v>
       </c>
       <c r="O178" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
       <c r="P178" t="inlineStr"/>
       <c r="Q178" t="n">
@@ -27135,16 +27067,12 @@
         </is>
       </c>
       <c r="N181" t="n">
-        <v>0.374</v>
+        <v>0.049</v>
       </c>
       <c r="O181" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="P181" t="inlineStr">
-        <is>
-          <t>vbied</t>
-        </is>
-      </c>
+        <v>0.022</v>
+      </c>
+      <c r="P181" t="inlineStr"/>
       <c r="Q181" t="n">
         <v>1.5169</v>
       </c>
@@ -27707,12 +27635,16 @@
         </is>
       </c>
       <c r="N185" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.126</v>
       </c>
       <c r="O185" t="n">
         <v>0.034</v>
       </c>
-      <c r="P185" t="inlineStr"/>
+      <c r="P185" t="inlineStr">
+        <is>
+          <t>mine_layer</t>
+        </is>
+      </c>
       <c r="Q185" t="n">
         <v>1.7226</v>
       </c>
@@ -28003,10 +27935,10 @@
         </is>
       </c>
       <c r="N187" t="n">
-        <v>0.075</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="O187" t="n">
-        <v>0.008</v>
+        <v>0.012</v>
       </c>
       <c r="P187" t="inlineStr"/>
       <c r="Q187" t="n">
@@ -28151,7 +28083,7 @@
         </is>
       </c>
       <c r="N188" t="n">
-        <v>0.03</v>
+        <v>0.028</v>
       </c>
       <c r="O188" t="n">
         <v>0.022</v>
@@ -28299,10 +28231,10 @@
         </is>
       </c>
       <c r="N189" t="n">
-        <v>0.032</v>
+        <v>0.031</v>
       </c>
       <c r="O189" t="n">
-        <v>0.032</v>
+        <v>0.031</v>
       </c>
       <c r="P189" t="inlineStr"/>
       <c r="Q189" t="n">
@@ -28595,14 +28527,14 @@
         </is>
       </c>
       <c r="N191" t="n">
-        <v>0.536</v>
+        <v>0.159</v>
       </c>
       <c r="O191" t="n">
-        <v>0.384</v>
+        <v>0.073</v>
       </c>
       <c r="P191" t="inlineStr">
         <is>
-          <t>counter_battery_radar</t>
+          <t>mlrs</t>
         </is>
       </c>
       <c r="Q191" t="n">
@@ -29339,7 +29271,7 @@
         </is>
       </c>
       <c r="N196" t="n">
-        <v>0.062</v>
+        <v>0.073</v>
       </c>
       <c r="O196" t="n">
         <v>0.053</v>
@@ -29779,10 +29711,10 @@
         </is>
       </c>
       <c r="N199" t="n">
-        <v>0.467</v>
+        <v>0.47</v>
       </c>
       <c r="O199" t="n">
-        <v>0.467</v>
+        <v>0.47</v>
       </c>
       <c r="P199" t="inlineStr">
         <is>
@@ -29931,14 +29863,14 @@
         </is>
       </c>
       <c r="N200" t="n">
-        <v>0.439</v>
+        <v>0.413</v>
       </c>
       <c r="O200" t="n">
-        <v>0.439</v>
+        <v>0.413</v>
       </c>
       <c r="P200" t="inlineStr">
         <is>
-          <t>swarm_carrier</t>
+          <t>transport_plane</t>
         </is>
       </c>
       <c r="Q200" t="n">
@@ -30042,20 +29974,16 @@
         </is>
       </c>
       <c r="E201" t="n">
-        <v>3698</v>
+        <v>8458</v>
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G201" t="inlineStr">
-        <is>
-          <t>parts: missing mantlet, idler, skirts, sight, roof_mg, stowage | own_geometry: 68% of triangles shared (most with mortar_carrier)</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr"/>
       <c r="H201" t="n">
-        <v>84.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="I201" t="inlineStr">
         <is>
@@ -30064,109 +29992,101 @@
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K201" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
-      <c r="L201" t="inlineStr">
-        <is>
-          <t>Kém</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K201" t="inlineStr"/>
+      <c r="L201" t="inlineStr"/>
       <c r="M201" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N201" t="n">
-        <v>0.676</v>
+        <v>0.06</v>
       </c>
       <c r="O201" t="n">
-        <v>0.345</v>
+        <v>0.113</v>
       </c>
       <c r="P201" t="inlineStr">
         <is>
-          <t>mortar_carrier</t>
+          <t>counter_battery_radar</t>
         </is>
       </c>
       <c r="Q201" t="n">
-        <v>1.255</v>
+        <v>1.5235</v>
       </c>
       <c r="R201" t="n">
-        <v>0.1728</v>
+        <v>0.2897</v>
       </c>
       <c r="S201" t="n">
-        <v>7.166</v>
+        <v>10.307</v>
       </c>
       <c r="T201" t="n">
-        <v>0.0103</v>
+        <v>0.1218</v>
       </c>
       <c r="U201" t="n">
-        <v>79</v>
+        <v>258</v>
       </c>
       <c r="V201" t="n">
-        <v>33</v>
+        <v>89</v>
       </c>
       <c r="W201" t="n">
-        <v>0.3919</v>
+        <v>0.8197</v>
       </c>
       <c r="X201" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="Y201" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="Z201" t="n">
-        <v>22</v>
+        <v>96</v>
       </c>
       <c r="AA201" t="n">
-        <v>0.5938</v>
+        <v>1.3816</v>
       </c>
       <c r="AB201" t="n">
-        <v>0.2613</v>
+        <v>0.8842</v>
       </c>
       <c r="AC201" t="n">
-        <v>84.1992</v>
+        <v>108.5706</v>
       </c>
       <c r="AD201" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="AE201" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="AF201" t="n">
-        <v>0.1557</v>
+        <v>0.1402</v>
       </c>
       <c r="AG201" t="n">
-        <v>0.9898</v>
+        <v>0.9041</v>
       </c>
       <c r="AH201" t="n">
-        <v>0.1404</v>
+        <v>0.07049999999999999</v>
       </c>
       <c r="AI201" t="n">
-        <v>0.1638</v>
+        <v>0.1528</v>
       </c>
       <c r="AJ201" t="n">
         <v>0</v>
       </c>
       <c r="AK201" t="n">
-        <v>0.652</v>
+        <v>1</v>
       </c>
       <c r="AL201" t="n">
-        <v>0.795</v>
+        <v>1</v>
       </c>
       <c r="AM201" t="n">
-        <v>0.9419999999999999</v>
+        <v>1</v>
       </c>
       <c r="AN201" t="n">
         <v>1</v>
       </c>
       <c r="AO201" t="n">
-        <v>0.839</v>
+        <v>1</v>
       </c>
       <c r="AP201" t="n">
         <v>1</v>
@@ -30223,7 +30143,7 @@
         </is>
       </c>
       <c r="N202" t="n">
-        <v>0.067</v>
+        <v>0.068</v>
       </c>
       <c r="O202" t="n">
         <v>0.022</v>
@@ -30823,10 +30743,10 @@
         </is>
       </c>
       <c r="N206" t="n">
-        <v>0.033</v>
+        <v>0.03</v>
       </c>
       <c r="O206" t="n">
-        <v>0.047</v>
+        <v>0.044</v>
       </c>
       <c r="P206" t="inlineStr"/>
       <c r="Q206" t="n">
@@ -31214,113 +31134,101 @@
         </is>
       </c>
       <c r="E209" t="n">
-        <v>2862</v>
+        <v>7494</v>
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G209" t="inlineStr">
-        <is>
-          <t>parts: missing axles | own_geometry: 77% of triangles shared (most with ammo_carrier)</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr"/>
       <c r="H209" t="n">
-        <v>72.09999999999999</v>
+        <v>87.8</v>
       </c>
       <c r="I209" t="inlineStr">
         <is>
-          <t>Cần sửa</t>
+          <t>Tốt</t>
         </is>
       </c>
       <c r="J209" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K209" t="inlineStr">
-        <is>
-          <t>Tốt</t>
-        </is>
-      </c>
-      <c r="L209" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K209" t="inlineStr"/>
+      <c r="L209" t="inlineStr"/>
       <c r="M209" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N209" t="n">
-        <v>0.774</v>
+        <v>0.119</v>
       </c>
       <c r="O209" t="n">
-        <v>0.643</v>
+        <v>0.156</v>
       </c>
       <c r="P209" t="inlineStr">
         <is>
-          <t>ammo_carrier</t>
+          <t>elite_mlrs</t>
         </is>
       </c>
       <c r="Q209" t="n">
-        <v>1.6189</v>
+        <v>1.6796</v>
       </c>
       <c r="R209" t="n">
-        <v>0.2297</v>
+        <v>0.2327</v>
       </c>
       <c r="S209" t="n">
-        <v>8.0054</v>
+        <v>7.7282</v>
       </c>
       <c r="T209" t="n">
-        <v>0.0029</v>
+        <v>0.0019</v>
       </c>
       <c r="U209" t="n">
-        <v>94</v>
+        <v>272</v>
       </c>
       <c r="V209" t="n">
-        <v>38</v>
+        <v>121</v>
       </c>
       <c r="W209" t="n">
-        <v>0.2995</v>
+        <v>0.8546</v>
       </c>
       <c r="X209" t="n">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="Y209" t="n">
-        <v>76</v>
+        <v>142</v>
       </c>
       <c r="Z209" t="n">
-        <v>11</v>
+        <v>109</v>
       </c>
       <c r="AA209" t="n">
-        <v>0.599</v>
+        <v>1.0029</v>
       </c>
       <c r="AB209" t="n">
-        <v>0.0867</v>
+        <v>0.7698</v>
       </c>
       <c r="AC209" t="n">
-        <v>126.8722</v>
+        <v>141.5894</v>
       </c>
       <c r="AD209" t="n">
         <v>4</v>
       </c>
       <c r="AE209" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="AF209" t="n">
-        <v>0.143</v>
+        <v>0.1557</v>
       </c>
       <c r="AG209" t="n">
-        <v>0.9987</v>
+        <v>0.9295</v>
       </c>
       <c r="AH209" t="n">
-        <v>0.1447</v>
+        <v>0.06660000000000001</v>
       </c>
       <c r="AI209" t="n">
-        <v>0.1537</v>
+        <v>0.176</v>
       </c>
       <c r="AJ209" t="n">
         <v>0</v>
@@ -31329,16 +31237,16 @@
         <v>1</v>
       </c>
       <c r="AL209" t="n">
-        <v>0.859</v>
+        <v>0.87</v>
       </c>
       <c r="AM209" t="n">
-        <v>0.671</v>
+        <v>0.648</v>
       </c>
       <c r="AN209" t="n">
-        <v>0.534</v>
+        <v>1</v>
       </c>
       <c r="AO209" t="n">
-        <v>0.5649999999999999</v>
+        <v>1</v>
       </c>
       <c r="AP209" t="n">
         <v>0.5</v>
@@ -31403,10 +31311,10 @@
         </is>
       </c>
       <c r="N210" t="n">
-        <v>0.025</v>
+        <v>0.024</v>
       </c>
       <c r="O210" t="n">
-        <v>0.032</v>
+        <v>0.031</v>
       </c>
       <c r="P210" t="inlineStr"/>
       <c r="Q210" t="n">
@@ -31510,20 +31418,16 @@
         </is>
       </c>
       <c r="E211" t="n">
-        <v>3464</v>
+        <v>4918</v>
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G211" t="inlineStr">
-        <is>
-          <t>parts: missing tail, intakes, exhaust, pylons, stores | own_geometry: 50% of triangles shared (most with sky_gunship)</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr"/>
       <c r="H211" t="n">
-        <v>95</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="I211" t="inlineStr">
         <is>
@@ -31532,91 +31436,79 @@
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K211" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
-      <c r="L211" t="inlineStr">
-        <is>
-          <t>Kém</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K211" t="inlineStr"/>
+      <c r="L211" t="inlineStr"/>
       <c r="M211" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N211" t="n">
-        <v>0.495</v>
+        <v>0</v>
       </c>
       <c r="O211" t="n">
-        <v>0.495</v>
-      </c>
-      <c r="P211" t="inlineStr">
-        <is>
-          <t>sky_gunship</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="P211" t="inlineStr"/>
       <c r="Q211" t="n">
-        <v>1.4849</v>
+        <v>1.6297</v>
       </c>
       <c r="R211" t="n">
-        <v>0.2364</v>
+        <v>0.1043</v>
       </c>
       <c r="S211" t="n">
-        <v>6.2107</v>
+        <v>3.0387</v>
       </c>
       <c r="T211" t="n">
-        <v>0.0031</v>
+        <v>0.0065</v>
       </c>
       <c r="U211" t="n">
-        <v>121</v>
+        <v>185</v>
       </c>
       <c r="V211" t="n">
-        <v>31</v>
+        <v>69</v>
       </c>
       <c r="W211" t="n">
-        <v>0.8401</v>
+        <v>1.7828</v>
       </c>
       <c r="X211" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Y211" t="n">
-        <v>35</v>
+        <v>63</v>
       </c>
       <c r="Z211" t="n">
-        <v>83</v>
+        <v>118</v>
       </c>
       <c r="AA211" t="n">
-        <v>0.9485</v>
+        <v>1.6278</v>
       </c>
       <c r="AB211" t="n">
-        <v>2.2494</v>
+        <v>3.0489</v>
       </c>
       <c r="AC211" t="n">
-        <v>36.899</v>
+        <v>38.7021</v>
       </c>
       <c r="AD211" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="AE211" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AF211" t="n">
-        <v>0.1557</v>
+        <v>0.2481</v>
       </c>
       <c r="AG211" t="n">
-        <v>1</v>
+        <v>0.9898</v>
       </c>
       <c r="AH211" t="n">
-        <v>0.1209</v>
+        <v>0.0944</v>
       </c>
       <c r="AI211" t="n">
-        <v>0.3523</v>
+        <v>0.1374</v>
       </c>
       <c r="AJ211" t="n">
         <v>0</v>
@@ -31625,10 +31517,10 @@
         <v>1</v>
       </c>
       <c r="AL211" t="n">
-        <v>1</v>
+        <v>0.742</v>
       </c>
       <c r="AM211" t="n">
-        <v>1</v>
+        <v>0.601</v>
       </c>
       <c r="AN211" t="n">
         <v>1</v>
@@ -32158,7 +32050,7 @@
         <v>0.026</v>
       </c>
       <c r="O215" t="n">
-        <v>0.055</v>
+        <v>0.054</v>
       </c>
       <c r="P215" t="inlineStr"/>
       <c r="Q215" t="n">
@@ -32303,7 +32195,7 @@
         </is>
       </c>
       <c r="N216" t="n">
-        <v>0.149</v>
+        <v>0.189</v>
       </c>
       <c r="O216" t="n">
         <v>0.103</v>
@@ -32595,7 +32487,7 @@
         </is>
       </c>
       <c r="N218" t="n">
-        <v>0.035</v>
+        <v>0.043</v>
       </c>
       <c r="O218" t="n">
         <v>0.08799999999999999</v>
@@ -32859,7 +32751,7 @@
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t>parts: missing mantlet, idler | own_geometry: 59% of triangles shared (most with elite_mbt)</t>
+          <t>parts: missing mantlet, idler | own_geometry: 52% of triangles shared (most with main_battle_tank)</t>
         </is>
       </c>
       <c r="H220" t="n">
@@ -32891,14 +32783,14 @@
         </is>
       </c>
       <c r="N220" t="n">
-        <v>0.59</v>
+        <v>0.522</v>
       </c>
       <c r="O220" t="n">
-        <v>0.435</v>
+        <v>0.408</v>
       </c>
       <c r="P220" t="inlineStr">
         <is>
-          <t>elite_mbt</t>
+          <t>main_battle_tank</t>
         </is>
       </c>
       <c r="Q220" t="n">
@@ -33043,10 +32935,10 @@
         </is>
       </c>
       <c r="N221" t="n">
-        <v>0.029</v>
+        <v>0.028</v>
       </c>
       <c r="O221" t="n">
-        <v>0.03</v>
+        <v>0.028</v>
       </c>
       <c r="P221" t="inlineStr"/>
       <c r="Q221" t="n">
@@ -33191,10 +33083,10 @@
         </is>
       </c>
       <c r="N222" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.083</v>
       </c>
       <c r="O222" t="n">
-        <v>0.021</v>
+        <v>0.016</v>
       </c>
       <c r="P222" t="inlineStr"/>
       <c r="Q222" t="n">
@@ -33298,131 +33190,115 @@
         </is>
       </c>
       <c r="E223" t="n">
-        <v>1574</v>
+        <v>4698</v>
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G223" t="inlineStr">
-        <is>
-          <t>triangles_floor: 1574 (floor 2100, class 3000-5000) | parts: missing axles, glass | own_geometry: 67% of triangles shared (most with rocket_technical) | not_single_block: 2 sloped face directions</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr"/>
       <c r="H223" t="n">
-        <v>59.7</v>
+        <v>86.2</v>
       </c>
       <c r="I223" t="inlineStr">
         <is>
-          <t>Kém</t>
+          <t>Tốt</t>
         </is>
       </c>
       <c r="J223" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K223" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
-      <c r="L223" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K223" t="inlineStr"/>
+      <c r="L223" t="inlineStr"/>
       <c r="M223" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N223" t="n">
-        <v>0.672</v>
+        <v>0.096</v>
       </c>
       <c r="O223" t="n">
-        <v>0.569</v>
-      </c>
-      <c r="P223" t="inlineStr">
-        <is>
-          <t>rocket_technical</t>
-        </is>
-      </c>
+        <v>0.027</v>
+      </c>
+      <c r="P223" t="inlineStr"/>
       <c r="Q223" t="n">
-        <v>1.36</v>
+        <v>1.3296</v>
       </c>
       <c r="R223" t="n">
-        <v>0.1279</v>
+        <v>0.315</v>
       </c>
       <c r="S223" t="n">
-        <v>4.3283</v>
+        <v>8.383800000000001</v>
       </c>
       <c r="T223" t="n">
-        <v>0.0122</v>
+        <v>0.0316</v>
       </c>
       <c r="U223" t="n">
-        <v>48</v>
+        <v>198</v>
       </c>
       <c r="V223" t="n">
-        <v>31</v>
+        <v>89</v>
       </c>
       <c r="W223" t="n">
-        <v>0.396</v>
+        <v>1.4631</v>
       </c>
       <c r="X223" t="n">
+        <v>32</v>
+      </c>
+      <c r="Y223" t="n">
+        <v>71</v>
+      </c>
+      <c r="Z223" t="n">
+        <v>95</v>
+      </c>
+      <c r="AA223" t="n">
+        <v>1.1672</v>
+      </c>
+      <c r="AB223" t="n">
+        <v>1.5617</v>
+      </c>
+      <c r="AC223" t="n">
+        <v>60.8313</v>
+      </c>
+      <c r="AD223" t="n">
         <v>12</v>
       </c>
-      <c r="Y223" t="n">
-        <v>28</v>
-      </c>
-      <c r="Z223" t="n">
-        <v>8</v>
-      </c>
-      <c r="AA223" t="n">
-        <v>0.3577</v>
-      </c>
-      <c r="AB223" t="n">
-        <v>0.1022</v>
-      </c>
-      <c r="AC223" t="n">
-        <v>78.2743</v>
-      </c>
-      <c r="AD223" t="n">
-        <v>2</v>
-      </c>
       <c r="AE223" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AF223" t="n">
-        <v>0.191</v>
+        <v>0.0785</v>
       </c>
       <c r="AG223" t="n">
-        <v>0.9996</v>
+        <v>0.8064</v>
       </c>
       <c r="AH223" t="n">
-        <v>0.1715</v>
+        <v>0.0339</v>
       </c>
       <c r="AI223" t="n">
-        <v>0.223</v>
+        <v>0.2941</v>
       </c>
       <c r="AJ223" t="n">
         <v>0</v>
       </c>
       <c r="AK223" t="n">
-        <v>0.6820000000000001</v>
+        <v>0.625</v>
       </c>
       <c r="AL223" t="n">
-        <v>0.478</v>
+        <v>1</v>
       </c>
       <c r="AM223" t="n">
-        <v>0.363</v>
+        <v>0.703</v>
       </c>
       <c r="AN223" t="n">
-        <v>0.706</v>
+        <v>1</v>
       </c>
       <c r="AO223" t="n">
-        <v>0.391</v>
+        <v>1</v>
       </c>
       <c r="AP223" t="n">
         <v>1</v>
@@ -33631,7 +33507,7 @@
         </is>
       </c>
       <c r="N225" t="n">
-        <v>0.404</v>
+        <v>0.405</v>
       </c>
       <c r="O225" t="n">
         <v>0.408</v>
@@ -33783,10 +33659,10 @@
         </is>
       </c>
       <c r="N226" t="n">
-        <v>0.474</v>
+        <v>0.473</v>
       </c>
       <c r="O226" t="n">
-        <v>0.474</v>
+        <v>0.473</v>
       </c>
       <c r="P226" t="inlineStr">
         <is>
@@ -33931,10 +33807,10 @@
         </is>
       </c>
       <c r="N227" t="n">
-        <v>0.018</v>
+        <v>0.022</v>
       </c>
       <c r="O227" t="n">
-        <v>0.018</v>
+        <v>0.022</v>
       </c>
       <c r="P227" t="inlineStr"/>
       <c r="Q227" t="n">
@@ -34079,7 +33955,7 @@
         </is>
       </c>
       <c r="N228" t="n">
-        <v>0.109</v>
+        <v>0.184</v>
       </c>
       <c r="O228" t="n">
         <v>0.153</v>
@@ -34223,7 +34099,7 @@
         </is>
       </c>
       <c r="N229" t="n">
-        <v>0.12</v>
+        <v>0.123</v>
       </c>
       <c r="O229" t="n">
         <v>0.143</v>
@@ -34375,10 +34251,10 @@
         </is>
       </c>
       <c r="N230" t="n">
-        <v>0.019</v>
+        <v>0.015</v>
       </c>
       <c r="O230" t="n">
-        <v>0.021</v>
+        <v>0.016</v>
       </c>
       <c r="P230" t="inlineStr"/>
       <c r="Q230" t="n">
@@ -34511,10 +34387,10 @@
         </is>
       </c>
       <c r="N231" t="n">
-        <v>0.018</v>
+        <v>0.027</v>
       </c>
       <c r="O231" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.013</v>
       </c>
       <c r="P231" t="inlineStr"/>
       <c r="Q231" t="n">

</xml_diff>

<commit_message>
P35 wave 8: full gate refresh (230 models, 112 pass every gate; the wave's 20 all pass)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/models/quality_report.xlsx
+++ b/Docs/models/quality_report.xlsx
@@ -679,10 +679,10 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>0.107</v>
+        <v>0.129</v>
       </c>
       <c r="O2" t="n">
-        <v>0.062</v>
+        <v>0.075</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -819,10 +819,10 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>0.066</v>
+        <v>0.068</v>
       </c>
       <c r="O3" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="n">
@@ -955,10 +955,10 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>0.106</v>
+        <v>0.149</v>
       </c>
       <c r="O4" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.064</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>0.003</v>
+        <v>0.005</v>
       </c>
       <c r="O5" t="n">
         <v>0.002</v>
@@ -1255,7 +1255,7 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>0.003</v>
+        <v>0.005</v>
       </c>
       <c r="O6" t="n">
         <v>0.002</v>
@@ -1531,10 +1531,10 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>0.128</v>
+        <v>0.129</v>
       </c>
       <c r="O8" t="n">
-        <v>0.076</v>
+        <v>0.077</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
@@ -1831,10 +1831,10 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>0.132</v>
+        <v>0.104</v>
       </c>
       <c r="O10" t="n">
-        <v>0.213</v>
+        <v>0.125</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
@@ -1979,10 +1979,10 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>0.152</v>
+        <v>0.118</v>
       </c>
       <c r="O11" t="n">
-        <v>0.15</v>
+        <v>0.067</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
@@ -2131,10 +2131,10 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>0.131</v>
+        <v>0.146</v>
       </c>
       <c r="O12" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.136</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
@@ -2419,10 +2419,10 @@
         </is>
       </c>
       <c r="N14" t="n">
+        <v>0.08400000000000001</v>
+      </c>
+      <c r="O14" t="n">
         <v>0.08500000000000001</v>
-      </c>
-      <c r="O14" t="n">
-        <v>0.08599999999999999</v>
       </c>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="n">
@@ -2691,7 +2691,7 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>0.091</v>
+        <v>0.09</v>
       </c>
       <c r="O16" t="n">
         <v>0.122</v>
@@ -2983,14 +2983,14 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>0.168</v>
+        <v>0.157</v>
       </c>
       <c r="O18" t="n">
-        <v>0.173</v>
+        <v>0.146</v>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>wheeled_gun</t>
+          <t>elite_aa</t>
         </is>
       </c>
       <c r="Q18" t="n">
@@ -3094,20 +3094,16 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>21954</v>
+        <v>26470</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>mounts: muzzles 5/7</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>81.8</v>
+        <v>89.5</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -3116,87 +3112,79 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>Tốt</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N19" t="n">
-        <v>0.063</v>
+        <v>0.028</v>
       </c>
       <c r="O19" t="n">
-        <v>0.064</v>
+        <v>0.034</v>
       </c>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="n">
-        <v>1.5102</v>
+        <v>1.6263</v>
       </c>
       <c r="R19" t="n">
-        <v>0.1927</v>
+        <v>0.2394</v>
       </c>
       <c r="S19" t="n">
-        <v>5.8484</v>
+        <v>7.8238</v>
       </c>
       <c r="T19" t="n">
-        <v>0.0068</v>
+        <v>0.06619999999999999</v>
       </c>
       <c r="U19" t="n">
-        <v>560</v>
+        <v>1086</v>
       </c>
       <c r="V19" t="n">
+        <v>124</v>
+      </c>
+      <c r="W19" t="n">
+        <v>2.0022</v>
+      </c>
+      <c r="X19" t="n">
+        <v>15</v>
+      </c>
+      <c r="Y19" t="n">
         <v>114</v>
       </c>
-      <c r="W19" t="n">
-        <v>1.965</v>
-      </c>
-      <c r="X19" t="n">
-        <v>6</v>
-      </c>
-      <c r="Y19" t="n">
-        <v>118</v>
-      </c>
       <c r="Z19" t="n">
-        <v>436</v>
+        <v>957</v>
       </c>
       <c r="AA19" t="n">
-        <v>2.0339</v>
+        <v>1.8407</v>
       </c>
       <c r="AB19" t="n">
-        <v>7.5152</v>
+        <v>15.4522</v>
       </c>
       <c r="AC19" t="n">
-        <v>58.0156</v>
+        <v>61.933</v>
       </c>
       <c r="AD19" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AE19" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AF19" t="n">
-        <v>0.2871</v>
+        <v>0.2786</v>
       </c>
       <c r="AG19" t="n">
-        <v>0.8216</v>
+        <v>0.8064</v>
       </c>
       <c r="AH19" t="n">
-        <v>0.0488</v>
+        <v>0.0351</v>
       </c>
       <c r="AI19" t="n">
-        <v>0.2472</v>
+        <v>0.0988</v>
       </c>
       <c r="AJ19" t="n">
         <v>0</v>
@@ -3211,13 +3199,13 @@
         <v>1</v>
       </c>
       <c r="AN19" t="n">
-        <v>0.695</v>
+        <v>0.708</v>
       </c>
       <c r="AO19" t="n">
-        <v>0.524</v>
+        <v>0.6909999999999999</v>
       </c>
       <c r="AP19" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -3271,10 +3259,10 @@
         </is>
       </c>
       <c r="N20" t="n">
-        <v>0.135</v>
+        <v>0.138</v>
       </c>
       <c r="O20" t="n">
-        <v>0.121</v>
+        <v>0.12</v>
       </c>
       <c r="P20" t="inlineStr">
         <is>
@@ -4119,10 +4107,10 @@
         </is>
       </c>
       <c r="N26" t="n">
-        <v>0.108</v>
+        <v>0.106</v>
       </c>
       <c r="O26" t="n">
-        <v>0.124</v>
+        <v>0.122</v>
       </c>
       <c r="P26" t="inlineStr">
         <is>
@@ -4259,10 +4247,10 @@
         </is>
       </c>
       <c r="N27" t="n">
-        <v>0.108</v>
+        <v>0.107</v>
       </c>
       <c r="O27" t="n">
-        <v>0.116</v>
+        <v>0.115</v>
       </c>
       <c r="P27" t="inlineStr">
         <is>
@@ -4407,7 +4395,7 @@
         </is>
       </c>
       <c r="N28" t="n">
-        <v>0.014</v>
+        <v>0.012</v>
       </c>
       <c r="O28" t="n">
         <v>0.015</v>
@@ -4691,10 +4679,10 @@
         </is>
       </c>
       <c r="N30" t="n">
-        <v>0.16</v>
+        <v>0.184</v>
       </c>
       <c r="O30" t="n">
-        <v>0.13</v>
+        <v>0.166</v>
       </c>
       <c r="P30" t="inlineStr">
         <is>
@@ -4843,14 +4831,14 @@
         </is>
       </c>
       <c r="N31" t="n">
-        <v>0.125</v>
+        <v>0.116</v>
       </c>
       <c r="O31" t="n">
-        <v>0.043</v>
+        <v>0.023</v>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>mlrs</t>
+          <t>shahed_truck</t>
         </is>
       </c>
       <c r="Q31" t="n">
@@ -5090,18 +5078,14 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>21610</v>
+        <v>25692</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>mounts: Mount_APS</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
         <v>99.59999999999999</v>
       </c>
@@ -5112,87 +5096,79 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>Tốt</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N33" t="n">
-        <v>0.024</v>
+        <v>0.021</v>
       </c>
       <c r="O33" t="n">
-        <v>0.032</v>
+        <v>0.025</v>
       </c>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="n">
-        <v>1.7429</v>
+        <v>1.8859</v>
       </c>
       <c r="R33" t="n">
-        <v>0.2544</v>
+        <v>0.1963</v>
       </c>
       <c r="S33" t="n">
-        <v>8.126099999999999</v>
+        <v>5.8834</v>
       </c>
       <c r="T33" t="n">
-        <v>0.025</v>
+        <v>0.0316</v>
       </c>
       <c r="U33" t="n">
-        <v>435</v>
+        <v>707</v>
       </c>
       <c r="V33" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W33" t="n">
-        <v>0.5488</v>
+        <v>0.4386</v>
       </c>
       <c r="X33" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="Y33" t="n">
-        <v>225</v>
+        <v>354</v>
       </c>
       <c r="Z33" t="n">
-        <v>187</v>
+        <v>333</v>
       </c>
       <c r="AA33" t="n">
-        <v>1.0737</v>
+        <v>1.2938</v>
       </c>
       <c r="AB33" t="n">
-        <v>0.8924</v>
+        <v>1.2171</v>
       </c>
       <c r="AC33" t="n">
-        <v>209.5465</v>
+        <v>273.6087</v>
       </c>
       <c r="AD33" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="AE33" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="AF33" t="n">
-        <v>0.2579</v>
+        <v>0.2702</v>
       </c>
       <c r="AG33" t="n">
-        <v>0.981</v>
+        <v>0.9041</v>
       </c>
       <c r="AH33" t="n">
-        <v>0.1092</v>
+        <v>0.062</v>
       </c>
       <c r="AI33" t="n">
-        <v>0.175</v>
+        <v>0.1884</v>
       </c>
       <c r="AJ33" t="n">
         <v>0</v>
@@ -5201,16 +5177,16 @@
         <v>1</v>
       </c>
       <c r="AL33" t="n">
-        <v>1</v>
+        <v>0.999</v>
       </c>
       <c r="AM33" t="n">
-        <v>1</v>
+        <v>0.977</v>
       </c>
       <c r="AN33" t="n">
         <v>1</v>
       </c>
       <c r="AO33" t="n">
-        <v>0.971</v>
+        <v>1</v>
       </c>
       <c r="AP33" t="n">
         <v>1</v>
@@ -5267,10 +5243,10 @@
         </is>
       </c>
       <c r="N34" t="n">
-        <v>0.028</v>
+        <v>0.027</v>
       </c>
       <c r="O34" t="n">
-        <v>0.043</v>
+        <v>0.039</v>
       </c>
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="n">
@@ -5403,10 +5379,10 @@
         </is>
       </c>
       <c r="N35" t="n">
-        <v>0.046</v>
+        <v>0.063</v>
       </c>
       <c r="O35" t="n">
-        <v>0.08</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="n">
@@ -6111,10 +6087,10 @@
         </is>
       </c>
       <c r="N40" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="O40" t="n">
-        <v>0.062</v>
+        <v>0.064</v>
       </c>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="n">
@@ -6250,7 +6226,7 @@
         <v>0.145</v>
       </c>
       <c r="O41" t="n">
-        <v>0.098</v>
+        <v>0.099</v>
       </c>
       <c r="P41" t="inlineStr">
         <is>
@@ -6550,7 +6526,7 @@
         <v>0.07199999999999999</v>
       </c>
       <c r="O43" t="n">
-        <v>0.078</v>
+        <v>0.077</v>
       </c>
       <c r="P43" t="inlineStr"/>
       <c r="Q43" t="n">
@@ -6695,10 +6671,10 @@
         </is>
       </c>
       <c r="N44" t="n">
-        <v>0.037</v>
+        <v>0.027</v>
       </c>
       <c r="O44" t="n">
-        <v>0.042</v>
+        <v>0.03</v>
       </c>
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="n">
@@ -6979,7 +6955,7 @@
         </is>
       </c>
       <c r="N46" t="n">
-        <v>0.04</v>
+        <v>0.041</v>
       </c>
       <c r="O46" t="n">
         <v>0.041</v>
@@ -7575,10 +7551,10 @@
         </is>
       </c>
       <c r="N50" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="O50" t="n">
         <v>0.046</v>
-      </c>
-      <c r="O50" t="n">
-        <v>0.047</v>
       </c>
       <c r="P50" t="inlineStr"/>
       <c r="Q50" t="n">
@@ -7719,10 +7695,10 @@
         </is>
       </c>
       <c r="N51" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
       <c r="O51" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
       <c r="P51" t="inlineStr"/>
       <c r="Q51" t="n">
@@ -7826,127 +7802,119 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>3084</v>
+        <v>6096</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>parts: missing glass</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr"/>
       <c r="H52" t="n">
-        <v>73.5</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Cần sửa</t>
+          <t>Tốt</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N52" t="n">
-        <v>0.056</v>
+        <v>0.145</v>
       </c>
       <c r="O52" t="n">
-        <v>0.036</v>
-      </c>
-      <c r="P52" t="inlineStr"/>
+        <v>0.082</v>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>mlrs</t>
+        </is>
+      </c>
       <c r="Q52" t="n">
-        <v>1.4013</v>
+        <v>1.5282</v>
       </c>
       <c r="R52" t="n">
-        <v>0.23</v>
+        <v>0.257</v>
       </c>
       <c r="S52" t="n">
-        <v>8.0418</v>
+        <v>8.3324</v>
       </c>
       <c r="T52" t="n">
-        <v>0.0182</v>
+        <v>0.0183</v>
       </c>
       <c r="U52" t="n">
-        <v>68</v>
+        <v>178</v>
       </c>
       <c r="V52" t="n">
-        <v>34</v>
+        <v>79</v>
       </c>
       <c r="W52" t="n">
-        <v>0.3577</v>
+        <v>1.0291</v>
       </c>
       <c r="X52" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Y52" t="n">
-        <v>39</v>
+        <v>79</v>
       </c>
       <c r="Z52" t="n">
-        <v>23</v>
+        <v>91</v>
       </c>
       <c r="AA52" t="n">
-        <v>0.4103</v>
+        <v>1.0291</v>
       </c>
       <c r="AB52" t="n">
-        <v>0.242</v>
+        <v>1.1854</v>
       </c>
       <c r="AC52" t="n">
-        <v>95.0425</v>
+        <v>76.76609999999999</v>
       </c>
       <c r="AD52" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AE52" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AF52" t="n">
-        <v>0.3709</v>
+        <v>0.3274</v>
       </c>
       <c r="AG52" t="n">
-        <v>1</v>
+        <v>0.981</v>
       </c>
       <c r="AH52" t="n">
-        <v>0.1933</v>
+        <v>0.0796</v>
       </c>
       <c r="AI52" t="n">
-        <v>0.2033</v>
+        <v>0.2369</v>
       </c>
       <c r="AJ52" t="n">
         <v>0</v>
       </c>
       <c r="AK52" t="n">
-        <v>0.76</v>
+        <v>1</v>
       </c>
       <c r="AL52" t="n">
-        <v>0.86</v>
+        <v>0.961</v>
       </c>
       <c r="AM52" t="n">
-        <v>0.674</v>
+        <v>0.698</v>
       </c>
       <c r="AN52" t="n">
-        <v>0.638</v>
+        <v>1</v>
       </c>
       <c r="AO52" t="n">
-        <v>0.579</v>
+        <v>1</v>
       </c>
       <c r="AP52" t="n">
         <v>1</v>
@@ -8003,7 +7971,7 @@
         </is>
       </c>
       <c r="N53" t="n">
-        <v>0.109</v>
+        <v>0.111</v>
       </c>
       <c r="O53" t="n">
         <v>0.12</v>
@@ -8439,16 +8407,12 @@
         </is>
       </c>
       <c r="N56" t="n">
-        <v>0.117</v>
+        <v>0.092</v>
       </c>
       <c r="O56" t="n">
-        <v>0.051</v>
-      </c>
-      <c r="P56" t="inlineStr">
-        <is>
-          <t>drone_hangar_b</t>
-        </is>
-      </c>
+        <v>0.053</v>
+      </c>
+      <c r="P56" t="inlineStr"/>
       <c r="Q56" t="n">
         <v>2.187</v>
       </c>
@@ -8591,10 +8555,10 @@
         </is>
       </c>
       <c r="N57" t="n">
-        <v>0.022</v>
+        <v>0.023</v>
       </c>
       <c r="O57" t="n">
-        <v>0.022</v>
+        <v>0.023</v>
       </c>
       <c r="P57" t="inlineStr"/>
       <c r="Q57" t="n">
@@ -8739,10 +8703,10 @@
         </is>
       </c>
       <c r="N58" t="n">
-        <v>0.399</v>
+        <v>0.396</v>
       </c>
       <c r="O58" t="n">
-        <v>0.195</v>
+        <v>0.191</v>
       </c>
       <c r="P58" t="inlineStr">
         <is>
@@ -8990,7 +8954,7 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>1556</v>
+        <v>3592</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
@@ -8999,102 +8963,94 @@
       </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="n">
-        <v>73.2</v>
+        <v>84.2</v>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Cần sửa</t>
+          <t>Tốt</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>Tốt</t>
-        </is>
-      </c>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>Tốt</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
       <c r="M60" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N60" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="O60" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="P60" t="inlineStr"/>
       <c r="Q60" t="n">
-        <v>1.5104</v>
+        <v>1.7243</v>
       </c>
       <c r="R60" t="n">
-        <v>0.2138</v>
+        <v>0.3205</v>
       </c>
       <c r="S60" t="n">
-        <v>9.2278</v>
+        <v>17.9992</v>
       </c>
       <c r="T60" t="n">
-        <v>0.0131</v>
+        <v>0.1447</v>
       </c>
       <c r="U60" t="n">
-        <v>50</v>
+        <v>397</v>
       </c>
       <c r="V60" t="n">
-        <v>45</v>
+        <v>110</v>
       </c>
       <c r="W60" t="n">
-        <v>0.5964</v>
+        <v>1.1714</v>
       </c>
       <c r="X60" t="n">
         <v>2</v>
       </c>
       <c r="Y60" t="n">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="Z60" t="n">
-        <v>24</v>
+        <v>346</v>
       </c>
       <c r="AA60" t="n">
-        <v>0.3181</v>
+        <v>0.5218</v>
       </c>
       <c r="AB60" t="n">
-        <v>0.3181</v>
+        <v>3.6845</v>
       </c>
       <c r="AC60" t="n">
-        <v>75.45480000000001</v>
+        <v>93.9062</v>
       </c>
       <c r="AD60" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="AE60" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="AF60" t="n">
-        <v>0.2687</v>
+        <v>0.2813</v>
       </c>
       <c r="AG60" t="n">
-        <v>0.8137</v>
+        <v>0.7985</v>
       </c>
       <c r="AH60" t="n">
-        <v>0.0429</v>
+        <v>0.0244</v>
       </c>
       <c r="AI60" t="n">
-        <v>0.374</v>
+        <v>0.297</v>
       </c>
       <c r="AJ60" t="n">
         <v>0</v>
       </c>
       <c r="AK60" t="n">
-        <v>0.322</v>
+        <v>0.458</v>
       </c>
       <c r="AL60" t="n">
         <v>1</v>
@@ -9106,7 +9062,7 @@
         <v>1</v>
       </c>
       <c r="AO60" t="n">
-        <v>0.342</v>
+        <v>0.849</v>
       </c>
       <c r="AP60" t="n">
         <v>1</v>
@@ -9134,127 +9090,115 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>2124</v>
+        <v>4340</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>ao_dust_wear: COLOR_0 p05 0.31 p95 0.81, worn 0.0%, dust +0.28</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr"/>
       <c r="H61" t="n">
-        <v>65.90000000000001</v>
+        <v>98.8</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Cần sửa</t>
+          <t>Tốt</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>Tốt</t>
-        </is>
-      </c>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>Tốt</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N61" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="O61" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="P61" t="inlineStr"/>
       <c r="Q61" t="n">
-        <v>2.1189</v>
+        <v>2.9043</v>
       </c>
       <c r="R61" t="n">
-        <v>0.1482</v>
+        <v>0.2157</v>
       </c>
       <c r="S61" t="n">
-        <v>4.144</v>
+        <v>9.415699999999999</v>
       </c>
       <c r="T61" t="n">
-        <v>0.029</v>
+        <v>0.1359</v>
       </c>
       <c r="U61" t="n">
-        <v>42</v>
+        <v>433</v>
       </c>
       <c r="V61" t="n">
-        <v>37</v>
+        <v>99</v>
       </c>
       <c r="W61" t="n">
-        <v>0.4574</v>
+        <v>1.6331</v>
       </c>
       <c r="X61" t="n">
         <v>11</v>
       </c>
       <c r="Y61" t="n">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="Z61" t="n">
-        <v>19</v>
+        <v>384</v>
       </c>
       <c r="AA61" t="n">
-        <v>0.1483</v>
+        <v>0.6268</v>
       </c>
       <c r="AB61" t="n">
-        <v>0.2349</v>
+        <v>6.3345</v>
       </c>
       <c r="AC61" t="n">
-        <v>80.9003</v>
+        <v>60.6206</v>
       </c>
       <c r="AD61" t="n">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="AE61" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="AF61" t="n">
-        <v>0.3075</v>
+        <v>0.3803</v>
       </c>
       <c r="AG61" t="n">
-        <v>0.8058</v>
+        <v>0.798</v>
       </c>
       <c r="AH61" t="n">
-        <v>0</v>
+        <v>0.0053</v>
       </c>
       <c r="AI61" t="n">
-        <v>0.2823</v>
+        <v>0.1605</v>
       </c>
       <c r="AJ61" t="n">
         <v>0</v>
       </c>
       <c r="AK61" t="n">
-        <v>0.707</v>
+        <v>1</v>
       </c>
       <c r="AL61" t="n">
-        <v>0.695</v>
+        <v>1</v>
       </c>
       <c r="AM61" t="n">
-        <v>0.479</v>
+        <v>1</v>
       </c>
       <c r="AN61" t="n">
-        <v>0.887</v>
+        <v>1</v>
       </c>
       <c r="AO61" t="n">
-        <v>0.195</v>
+        <v>0.919</v>
       </c>
       <c r="AP61" t="n">
         <v>1</v>
@@ -9455,10 +9399,10 @@
         </is>
       </c>
       <c r="N63" t="n">
-        <v>0.127</v>
+        <v>0.124</v>
       </c>
       <c r="O63" t="n">
-        <v>0.152</v>
+        <v>0.153</v>
       </c>
       <c r="P63" t="inlineStr">
         <is>
@@ -9595,10 +9539,10 @@
         </is>
       </c>
       <c r="N64" t="n">
-        <v>0.126</v>
+        <v>0.123</v>
       </c>
       <c r="O64" t="n">
-        <v>0.149</v>
+        <v>0.15</v>
       </c>
       <c r="P64" t="inlineStr">
         <is>
@@ -9735,10 +9679,10 @@
         </is>
       </c>
       <c r="N65" t="n">
-        <v>0.096</v>
+        <v>0.094</v>
       </c>
       <c r="O65" t="n">
-        <v>0.122</v>
+        <v>0.123</v>
       </c>
       <c r="P65" t="inlineStr">
         <is>
@@ -10035,10 +9979,10 @@
         </is>
       </c>
       <c r="N67" t="n">
-        <v>0.025</v>
+        <v>0.023</v>
       </c>
       <c r="O67" t="n">
-        <v>0.021</v>
+        <v>0.022</v>
       </c>
       <c r="P67" t="inlineStr"/>
       <c r="Q67" t="n">
@@ -10183,10 +10127,10 @@
         </is>
       </c>
       <c r="N68" t="n">
-        <v>0.119</v>
+        <v>0.2</v>
       </c>
       <c r="O68" t="n">
-        <v>0.083</v>
+        <v>0.168</v>
       </c>
       <c r="P68" t="inlineStr">
         <is>
@@ -10627,10 +10571,10 @@
         </is>
       </c>
       <c r="N71" t="n">
-        <v>0.147</v>
+        <v>0.152</v>
       </c>
       <c r="O71" t="n">
-        <v>0.195</v>
+        <v>0.206</v>
       </c>
       <c r="P71" t="inlineStr">
         <is>
@@ -10779,10 +10723,10 @@
         </is>
       </c>
       <c r="N72" t="n">
-        <v>0.156</v>
+        <v>0.155</v>
       </c>
       <c r="O72" t="n">
-        <v>0.267</v>
+        <v>0.265</v>
       </c>
       <c r="P72" t="inlineStr">
         <is>
@@ -11035,7 +10979,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>parts: missing mantlet, idler, stowage | own_geometry: 94% of triangles shared (most with heavy_tank)</t>
+          <t>parts: missing mantlet, idler, stowage</t>
         </is>
       </c>
       <c r="H74" t="n">
@@ -11067,16 +11011,12 @@
         </is>
       </c>
       <c r="N74" t="n">
-        <v>0.9360000000000001</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="O74" t="n">
-        <v>0.916</v>
-      </c>
-      <c r="P74" t="inlineStr">
-        <is>
-          <t>heavy_tank</t>
-        </is>
-      </c>
+        <v>0.082</v>
+      </c>
+      <c r="P74" t="inlineStr"/>
       <c r="Q74" t="n">
         <v>1.2415</v>
       </c>
@@ -11343,7 +11283,7 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>0.144</v>
+        <v>0.138</v>
       </c>
       <c r="O76" t="n">
         <v>0.155</v>
@@ -11495,12 +11435,16 @@
         </is>
       </c>
       <c r="N77" t="n">
-        <v>0.092</v>
+        <v>0.098</v>
       </c>
       <c r="O77" t="n">
-        <v>0.08699999999999999</v>
-      </c>
-      <c r="P77" t="inlineStr"/>
+        <v>0.103</v>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>elite_heavy_tank</t>
+        </is>
+      </c>
       <c r="Q77" t="n">
         <v>1.2432</v>
       </c>
@@ -11634,7 +11578,7 @@
         <v>0.112</v>
       </c>
       <c r="O78" t="n">
-        <v>0.174</v>
+        <v>0.176</v>
       </c>
       <c r="P78" t="inlineStr">
         <is>
@@ -11783,10 +11727,10 @@
         </is>
       </c>
       <c r="N79" t="n">
-        <v>0.077</v>
+        <v>0.039</v>
       </c>
       <c r="O79" t="n">
-        <v>0.096</v>
+        <v>0.062</v>
       </c>
       <c r="P79" t="inlineStr"/>
       <c r="Q79" t="n">
@@ -11927,10 +11871,10 @@
         </is>
       </c>
       <c r="N80" t="n">
-        <v>0.034</v>
+        <v>0.038</v>
       </c>
       <c r="O80" t="n">
-        <v>0.034</v>
+        <v>0.038</v>
       </c>
       <c r="P80" t="inlineStr"/>
       <c r="Q80" t="n">
@@ -12063,10 +12007,10 @@
         </is>
       </c>
       <c r="N81" t="n">
-        <v>0.089</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="O81" t="n">
-        <v>0.09</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="P81" t="inlineStr"/>
       <c r="Q81" t="n">
@@ -12207,10 +12151,10 @@
         </is>
       </c>
       <c r="N82" t="n">
-        <v>0.039</v>
+        <v>0.042</v>
       </c>
       <c r="O82" t="n">
-        <v>0.039</v>
+        <v>0.042</v>
       </c>
       <c r="P82" t="inlineStr"/>
       <c r="Q82" t="n">
@@ -12355,10 +12299,10 @@
         </is>
       </c>
       <c r="N83" t="n">
-        <v>0.172</v>
+        <v>0.189</v>
       </c>
       <c r="O83" t="n">
-        <v>0.026</v>
+        <v>0.01</v>
       </c>
       <c r="P83" t="inlineStr">
         <is>
@@ -12639,10 +12583,10 @@
         </is>
       </c>
       <c r="N85" t="n">
-        <v>0.022</v>
+        <v>0.021</v>
       </c>
       <c r="O85" t="n">
-        <v>0.037</v>
+        <v>0.036</v>
       </c>
       <c r="P85" t="inlineStr"/>
       <c r="Q85" t="n">
@@ -12775,10 +12719,10 @@
         </is>
       </c>
       <c r="N86" t="n">
-        <v>0.041</v>
+        <v>0.04</v>
       </c>
       <c r="O86" t="n">
-        <v>0.052</v>
+        <v>0.05</v>
       </c>
       <c r="P86" t="inlineStr"/>
       <c r="Q86" t="n">
@@ -12923,10 +12867,10 @@
         </is>
       </c>
       <c r="N87" t="n">
-        <v>0.036</v>
+        <v>0.024</v>
       </c>
       <c r="O87" t="n">
-        <v>0.038</v>
+        <v>0.025</v>
       </c>
       <c r="P87" t="inlineStr"/>
       <c r="Q87" t="n">
@@ -13195,10 +13139,10 @@
         </is>
       </c>
       <c r="N89" t="n">
-        <v>0.031</v>
+        <v>0.038</v>
       </c>
       <c r="O89" t="n">
-        <v>0.066</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="P89" t="inlineStr"/>
       <c r="Q89" t="n">
@@ -13467,12 +13411,16 @@
         </is>
       </c>
       <c r="N91" t="n">
-        <v>0.083</v>
+        <v>0.095</v>
       </c>
       <c r="O91" t="n">
-        <v>0.062</v>
-      </c>
-      <c r="P91" t="inlineStr"/>
+        <v>0.107</v>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>tank_destroyer</t>
+        </is>
+      </c>
       <c r="Q91" t="n">
         <v>1.4669</v>
       </c>
@@ -13615,10 +13563,10 @@
         </is>
       </c>
       <c r="N92" t="n">
-        <v>0.018</v>
+        <v>0.012</v>
       </c>
       <c r="O92" t="n">
-        <v>0.013</v>
+        <v>0.006</v>
       </c>
       <c r="P92" t="inlineStr"/>
       <c r="Q92" t="n">
@@ -13763,10 +13711,10 @@
         </is>
       </c>
       <c r="N93" t="n">
-        <v>0.039</v>
+        <v>0.074</v>
       </c>
       <c r="O93" t="n">
-        <v>0.039</v>
+        <v>0.074</v>
       </c>
       <c r="P93" t="inlineStr"/>
       <c r="Q93" t="n">
@@ -13899,10 +13847,10 @@
         </is>
       </c>
       <c r="N94" t="n">
-        <v>0.057</v>
+        <v>0.065</v>
       </c>
       <c r="O94" t="n">
-        <v>0.046</v>
+        <v>0.042</v>
       </c>
       <c r="P94" t="inlineStr"/>
       <c r="Q94" t="n">
@@ -14006,20 +13954,16 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>6342</v>
+        <v>7408</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G95" t="inlineStr">
-        <is>
-          <t>parts: missing stowage | not_single_block: 0 sloped face directions</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr"/>
       <c r="H95" t="n">
-        <v>87.5</v>
+        <v>95.8</v>
       </c>
       <c r="I95" t="inlineStr">
         <is>
@@ -14028,87 +13972,79 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K95" t="inlineStr">
-        <is>
-          <t>Tốt</t>
-        </is>
-      </c>
-      <c r="L95" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr"/>
       <c r="M95" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N95" t="n">
-        <v>0.067</v>
+        <v>0.063</v>
       </c>
       <c r="O95" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.055</v>
       </c>
       <c r="P95" t="inlineStr"/>
       <c r="Q95" t="n">
-        <v>1.7673</v>
+        <v>1.9846</v>
       </c>
       <c r="R95" t="n">
-        <v>0.3805</v>
+        <v>0.287</v>
       </c>
       <c r="S95" t="n">
-        <v>14.135</v>
+        <v>9.1074</v>
       </c>
       <c r="T95" t="n">
-        <v>0.0189</v>
+        <v>0.0495</v>
       </c>
       <c r="U95" t="n">
-        <v>179</v>
+        <v>271</v>
       </c>
       <c r="V95" t="n">
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="W95" t="n">
-        <v>0.4036</v>
+        <v>0.5856</v>
       </c>
       <c r="X95" t="n">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="Y95" t="n">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="Z95" t="n">
-        <v>34</v>
+        <v>130</v>
       </c>
       <c r="AA95" t="n">
-        <v>0.445</v>
+        <v>0.5794</v>
       </c>
       <c r="AB95" t="n">
-        <v>0.1759</v>
+        <v>0.8099</v>
       </c>
       <c r="AC95" t="n">
-        <v>193.2431</v>
+        <v>160.5099</v>
       </c>
       <c r="AD95" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AE95" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AF95" t="n">
-        <v>0.2828</v>
+        <v>0.3368</v>
       </c>
       <c r="AG95" t="n">
-        <v>0.9634</v>
+        <v>0.9641</v>
       </c>
       <c r="AH95" t="n">
-        <v>0.08939999999999999</v>
+        <v>0.0712</v>
       </c>
       <c r="AI95" t="n">
-        <v>0.0121</v>
+        <v>0.1257</v>
       </c>
       <c r="AJ95" t="n">
         <v>0</v>
@@ -14120,13 +14056,13 @@
         <v>1</v>
       </c>
       <c r="AM95" t="n">
-        <v>1</v>
+        <v>0.763</v>
       </c>
       <c r="AN95" t="n">
-        <v>0.72</v>
+        <v>1</v>
       </c>
       <c r="AO95" t="n">
-        <v>0.537</v>
+        <v>0.959</v>
       </c>
       <c r="AP95" t="n">
         <v>1</v>
@@ -14198,7 +14134,7 @@
         <v>0.09</v>
       </c>
       <c r="O96" t="n">
-        <v>0.047</v>
+        <v>0.048</v>
       </c>
       <c r="P96" t="inlineStr"/>
       <c r="Q96" t="n">
@@ -14343,10 +14279,10 @@
         </is>
       </c>
       <c r="N97" t="n">
-        <v>0.029</v>
+        <v>0.032</v>
       </c>
       <c r="O97" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.079</v>
       </c>
       <c r="P97" t="inlineStr"/>
       <c r="Q97" t="n">
@@ -14479,10 +14415,10 @@
         </is>
       </c>
       <c r="N98" t="n">
-        <v>0.037</v>
+        <v>0.03</v>
       </c>
       <c r="O98" t="n">
-        <v>0.038</v>
+        <v>0.03</v>
       </c>
       <c r="P98" t="inlineStr"/>
       <c r="Q98" t="n">
@@ -14615,10 +14551,10 @@
         </is>
       </c>
       <c r="N99" t="n">
-        <v>0.044</v>
+        <v>0.038</v>
       </c>
       <c r="O99" t="n">
-        <v>0.046</v>
+        <v>0.039</v>
       </c>
       <c r="P99" t="inlineStr"/>
       <c r="Q99" t="n">
@@ -14899,10 +14835,10 @@
         </is>
       </c>
       <c r="N101" t="n">
-        <v>0.045</v>
+        <v>0.041</v>
       </c>
       <c r="O101" t="n">
-        <v>0.075</v>
+        <v>0.068</v>
       </c>
       <c r="P101" t="inlineStr"/>
       <c r="Q101" t="n">
@@ -15047,10 +14983,10 @@
         </is>
       </c>
       <c r="N102" t="n">
-        <v>0.043</v>
+        <v>0.028</v>
       </c>
       <c r="O102" t="n">
-        <v>0.042</v>
+        <v>0.026</v>
       </c>
       <c r="P102" t="inlineStr"/>
       <c r="Q102" t="n">
@@ -15290,20 +15226,16 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>4660</v>
+        <v>5624</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G104" t="inlineStr">
-        <is>
-          <t>parts: missing stub_wings | mounts: Turret (main mount)</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr"/>
       <c r="H104" t="n">
-        <v>81.40000000000001</v>
+        <v>91.5</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
@@ -15312,87 +15244,79 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K104" t="inlineStr">
-        <is>
-          <t>Tốt</t>
-        </is>
-      </c>
-      <c r="L104" t="inlineStr">
-        <is>
-          <t>Kém</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr"/>
+      <c r="L104" t="inlineStr"/>
       <c r="M104" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N104" t="n">
-        <v>0.003</v>
+        <v>0.019</v>
       </c>
       <c r="O104" t="n">
-        <v>0.007</v>
+        <v>0.031</v>
       </c>
       <c r="P104" t="inlineStr"/>
       <c r="Q104" t="n">
-        <v>1.9707</v>
+        <v>2.0363</v>
       </c>
       <c r="R104" t="n">
-        <v>0.2215</v>
+        <v>0.2352</v>
       </c>
       <c r="S104" t="n">
-        <v>12.6976</v>
+        <v>13.3857</v>
       </c>
       <c r="T104" t="n">
-        <v>0.4948</v>
+        <v>0.2087</v>
       </c>
       <c r="U104" t="n">
-        <v>113</v>
+        <v>173</v>
       </c>
       <c r="V104" t="n">
+        <v>78</v>
+      </c>
+      <c r="W104" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="X104" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y104" t="n">
         <v>70</v>
       </c>
-      <c r="W104" t="n">
-        <v>1.7856</v>
-      </c>
-      <c r="X104" t="n">
-        <v>6</v>
-      </c>
-      <c r="Y104" t="n">
-        <v>50</v>
-      </c>
       <c r="Z104" t="n">
-        <v>57</v>
+        <v>99</v>
       </c>
       <c r="AA104" t="n">
-        <v>1.2754</v>
+        <v>1.5975</v>
       </c>
       <c r="AB104" t="n">
-        <v>1.4539</v>
+        <v>2.2593</v>
       </c>
       <c r="AC104" t="n">
-        <v>39.2036</v>
+        <v>43.8191</v>
       </c>
       <c r="AD104" t="n">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="AE104" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AF104" t="n">
-        <v>0.3912</v>
+        <v>0.3964</v>
       </c>
       <c r="AG104" t="n">
-        <v>0.9987</v>
+        <v>0.8143</v>
       </c>
       <c r="AH104" t="n">
-        <v>0.1373</v>
+        <v>0.0382</v>
       </c>
       <c r="AI104" t="n">
-        <v>0.1508</v>
+        <v>0.1716</v>
       </c>
       <c r="AJ104" t="n">
         <v>0</v>
@@ -15401,19 +15325,19 @@
         <v>1</v>
       </c>
       <c r="AL104" t="n">
-        <v>0.855</v>
+        <v>0.908</v>
       </c>
       <c r="AM104" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.727</v>
       </c>
       <c r="AN104" t="n">
-        <v>0.92</v>
+        <v>0.917</v>
       </c>
       <c r="AO104" t="n">
-        <v>0.655</v>
+        <v>0.909</v>
       </c>
       <c r="AP104" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="105">
@@ -15438,20 +15362,16 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>14164</v>
+        <v>18228</v>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G105" t="inlineStr">
-        <is>
-          <t>mounts: Mount_mg 1/2</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr"/>
       <c r="H105" t="n">
-        <v>100</v>
+        <v>97.8</v>
       </c>
       <c r="I105" t="inlineStr">
         <is>
@@ -15460,87 +15380,79 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K105" t="inlineStr">
-        <is>
-          <t>Tốt</t>
-        </is>
-      </c>
-      <c r="L105" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr"/>
+      <c r="L105" t="inlineStr"/>
       <c r="M105" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N105" t="n">
-        <v>0.037</v>
+        <v>0.038</v>
       </c>
       <c r="O105" t="n">
-        <v>0.039</v>
+        <v>0.038</v>
       </c>
       <c r="P105" t="inlineStr"/>
       <c r="Q105" t="n">
-        <v>1.7995</v>
+        <v>1.7701</v>
       </c>
       <c r="R105" t="n">
-        <v>0.1587</v>
+        <v>0.1702</v>
       </c>
       <c r="S105" t="n">
-        <v>4.6253</v>
+        <v>5.2517</v>
       </c>
       <c r="T105" t="n">
-        <v>0.017</v>
+        <v>0.0175</v>
       </c>
       <c r="U105" t="n">
-        <v>571</v>
+        <v>560</v>
       </c>
       <c r="V105" t="n">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="W105" t="n">
-        <v>0.4386</v>
+        <v>0.4153</v>
       </c>
       <c r="X105" t="n">
-        <v>26</v>
+        <v>48</v>
       </c>
       <c r="Y105" t="n">
-        <v>335</v>
+        <v>254</v>
       </c>
       <c r="Z105" t="n">
-        <v>210</v>
+        <v>258</v>
       </c>
       <c r="AA105" t="n">
-        <v>0.7693</v>
+        <v>0.5409</v>
       </c>
       <c r="AB105" t="n">
-        <v>0.4822</v>
+        <v>0.5494</v>
       </c>
       <c r="AC105" t="n">
-        <v>435.4758</v>
+        <v>469.5681</v>
       </c>
       <c r="AD105" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AE105" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="AF105" t="n">
-        <v>0.272</v>
+        <v>0.289</v>
       </c>
       <c r="AG105" t="n">
-        <v>1</v>
+        <v>0.9987</v>
       </c>
       <c r="AH105" t="n">
-        <v>0.0658</v>
+        <v>0.1165</v>
       </c>
       <c r="AI105" t="n">
-        <v>0.1662</v>
+        <v>0.17</v>
       </c>
       <c r="AJ105" t="n">
         <v>0</v>
@@ -15558,7 +15470,7 @@
         <v>1</v>
       </c>
       <c r="AO105" t="n">
-        <v>1</v>
+        <v>0.852</v>
       </c>
       <c r="AP105" t="n">
         <v>1</v>
@@ -15586,20 +15498,16 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>4524</v>
+        <v>7278</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G106" t="inlineStr">
-        <is>
-          <t>parts: missing axles, stowage | not_single_block: 0 sloped face directions</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr"/>
       <c r="H106" t="n">
-        <v>81.40000000000001</v>
+        <v>94.8</v>
       </c>
       <c r="I106" t="inlineStr">
         <is>
@@ -15608,87 +15516,83 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K106" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
-      <c r="L106" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr"/>
+      <c r="L106" t="inlineStr"/>
       <c r="M106" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N106" t="n">
-        <v>0.073</v>
+        <v>0.193</v>
       </c>
       <c r="O106" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="P106" t="inlineStr"/>
+        <v>0.161</v>
+      </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t>railgun_truck</t>
+        </is>
+      </c>
       <c r="Q106" t="n">
-        <v>1.6177</v>
+        <v>1.557</v>
       </c>
       <c r="R106" t="n">
-        <v>0.2201</v>
+        <v>0.2557</v>
       </c>
       <c r="S106" t="n">
-        <v>8.0215</v>
+        <v>8.3492</v>
       </c>
       <c r="T106" t="n">
-        <v>0.0012</v>
+        <v>0.0331</v>
       </c>
       <c r="U106" t="n">
-        <v>104</v>
+        <v>214</v>
       </c>
       <c r="V106" t="n">
-        <v>39</v>
+        <v>86</v>
       </c>
       <c r="W106" t="n">
-        <v>0.4282</v>
+        <v>0.7277</v>
       </c>
       <c r="X106" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="Y106" t="n">
-        <v>66</v>
+        <v>119</v>
       </c>
       <c r="Z106" t="n">
-        <v>36</v>
+        <v>83</v>
       </c>
       <c r="AA106" t="n">
-        <v>0.7246</v>
+        <v>1.0069</v>
       </c>
       <c r="AB106" t="n">
-        <v>0.3952</v>
+        <v>0.7023</v>
       </c>
       <c r="AC106" t="n">
-        <v>91.08459999999999</v>
+        <v>118.1813</v>
       </c>
       <c r="AD106" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AE106" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="AF106" t="n">
-        <v>0.1876</v>
+        <v>0.1354</v>
       </c>
       <c r="AG106" t="n">
-        <v>0.9898</v>
+        <v>0.9553</v>
       </c>
       <c r="AH106" t="n">
-        <v>0.1028</v>
+        <v>0.077</v>
       </c>
       <c r="AI106" t="n">
-        <v>0.1645</v>
+        <v>0.1459</v>
       </c>
       <c r="AJ106" t="n">
         <v>0</v>
@@ -15697,19 +15601,19 @@
         <v>1</v>
       </c>
       <c r="AL106" t="n">
-        <v>0.823</v>
+        <v>0.956</v>
       </c>
       <c r="AM106" t="n">
-        <v>0.672</v>
+        <v>0.7</v>
       </c>
       <c r="AN106" t="n">
-        <v>0.764</v>
+        <v>1</v>
       </c>
       <c r="AO106" t="n">
-        <v>0.915</v>
+        <v>1</v>
       </c>
       <c r="AP106" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107">
@@ -15775,7 +15679,7 @@
         </is>
       </c>
       <c r="N107" t="n">
-        <v>0.01</v>
+        <v>0.013</v>
       </c>
       <c r="O107" t="n">
         <v>0.006</v>
@@ -15914,7 +15818,7 @@
         <v>0.034</v>
       </c>
       <c r="O108" t="n">
-        <v>0.043</v>
+        <v>0.04</v>
       </c>
       <c r="P108" t="inlineStr"/>
       <c r="Q108" t="n">
@@ -16210,11 +16114,11 @@
         <v>0.112</v>
       </c>
       <c r="O110" t="n">
-        <v>0.059</v>
+        <v>0.061</v>
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t>heavy_tank</t>
+          <t>rocket_technical</t>
         </is>
       </c>
       <c r="Q110" t="n">
@@ -16318,20 +16222,16 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>5662</v>
+        <v>9296</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G111" t="inlineStr">
-        <is>
-          <t>parts: missing mantlet, idler, stowage</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr"/>
       <c r="H111" t="n">
-        <v>81.2</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="I111" t="inlineStr">
         <is>
@@ -16340,112 +16240,104 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K111" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
-      <c r="L111" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr"/>
+      <c r="L111" t="inlineStr"/>
       <c r="M111" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N111" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.196</v>
       </c>
       <c r="O111" t="n">
-        <v>0.929</v>
+        <v>0.112</v>
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t>elite_heavy_tank</t>
+          <t>wheeled_gun</t>
         </is>
       </c>
       <c r="Q111" t="n">
-        <v>1.2365</v>
+        <v>1.3777</v>
       </c>
       <c r="R111" t="n">
-        <v>0.2224</v>
+        <v>0.3103</v>
       </c>
       <c r="S111" t="n">
-        <v>5.9899</v>
+        <v>9.206099999999999</v>
       </c>
       <c r="T111" t="n">
-        <v>0.0005</v>
+        <v>0.0019</v>
       </c>
       <c r="U111" t="n">
-        <v>130</v>
+        <v>263</v>
       </c>
       <c r="V111" t="n">
-        <v>48</v>
+        <v>82</v>
       </c>
       <c r="W111" t="n">
-        <v>0.3781</v>
+        <v>0.5348000000000001</v>
       </c>
       <c r="X111" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="Y111" t="n">
-        <v>87</v>
+        <v>166</v>
       </c>
       <c r="Z111" t="n">
-        <v>37</v>
+        <v>82</v>
       </c>
       <c r="AA111" t="n">
-        <v>0.6853</v>
+        <v>1.0826</v>
       </c>
       <c r="AB111" t="n">
-        <v>0.2914</v>
+        <v>0.5348000000000001</v>
       </c>
       <c r="AC111" t="n">
-        <v>126.9564</v>
+        <v>153.336</v>
       </c>
       <c r="AD111" t="n">
         <v>7</v>
       </c>
       <c r="AE111" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AF111" t="n">
-        <v>0.2193</v>
+        <v>0.1329</v>
       </c>
       <c r="AG111" t="n">
-        <v>0.9467</v>
+        <v>0.9375</v>
       </c>
       <c r="AH111" t="n">
-        <v>0.0936</v>
+        <v>0.0745</v>
       </c>
       <c r="AI111" t="n">
-        <v>0.2397</v>
+        <v>0.2128</v>
       </c>
       <c r="AJ111" t="n">
         <v>0</v>
       </c>
       <c r="AK111" t="n">
-        <v>0.605</v>
+        <v>0.966</v>
       </c>
       <c r="AL111" t="n">
         <v>1</v>
       </c>
       <c r="AM111" t="n">
-        <v>0.788</v>
+        <v>1</v>
       </c>
       <c r="AN111" t="n">
         <v>1</v>
       </c>
       <c r="AO111" t="n">
-        <v>0.951</v>
+        <v>1</v>
       </c>
       <c r="AP111" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="112">
@@ -16499,10 +16391,10 @@
         </is>
       </c>
       <c r="N112" t="n">
-        <v>0.13</v>
+        <v>0.131</v>
       </c>
       <c r="O112" t="n">
-        <v>0.061</v>
+        <v>0.062</v>
       </c>
       <c r="P112" t="inlineStr">
         <is>
@@ -16651,10 +16543,10 @@
         </is>
       </c>
       <c r="N113" t="n">
-        <v>0.049</v>
+        <v>0.055</v>
       </c>
       <c r="O113" t="n">
-        <v>0.054</v>
+        <v>0.061</v>
       </c>
       <c r="P113" t="inlineStr"/>
       <c r="Q113" t="n">
@@ -16787,7 +16679,7 @@
         </is>
       </c>
       <c r="N114" t="n">
-        <v>0.124</v>
+        <v>0.125</v>
       </c>
       <c r="O114" t="n">
         <v>0.049</v>
@@ -16927,10 +16819,10 @@
         </is>
       </c>
       <c r="N115" t="n">
-        <v>0.025</v>
+        <v>0.028</v>
       </c>
       <c r="O115" t="n">
-        <v>0.036</v>
+        <v>0.037</v>
       </c>
       <c r="P115" t="inlineStr"/>
       <c r="Q115" t="n">
@@ -17199,10 +17091,10 @@
         </is>
       </c>
       <c r="N117" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="O117" t="n">
         <v>0.031</v>
-      </c>
-      <c r="O117" t="n">
-        <v>0.028</v>
       </c>
       <c r="P117" t="inlineStr"/>
       <c r="Q117" t="n">
@@ -17783,10 +17675,10 @@
         </is>
       </c>
       <c r="N121" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="O121" t="n">
-        <v>0.135</v>
+        <v>0.13</v>
       </c>
       <c r="P121" t="inlineStr">
         <is>
@@ -17923,10 +17815,10 @@
         </is>
       </c>
       <c r="N122" t="n">
-        <v>0.057</v>
+        <v>0.062</v>
       </c>
       <c r="O122" t="n">
-        <v>0.059</v>
+        <v>0.063</v>
       </c>
       <c r="P122" t="inlineStr"/>
       <c r="Q122" t="n">
@@ -18063,10 +17955,10 @@
         </is>
       </c>
       <c r="N123" t="n">
-        <v>0.282</v>
+        <v>0.277</v>
       </c>
       <c r="O123" t="n">
-        <v>0.224</v>
+        <v>0.222</v>
       </c>
       <c r="P123" t="inlineStr">
         <is>
@@ -18215,12 +18107,16 @@
         </is>
       </c>
       <c r="N124" t="n">
-        <v>0.043</v>
+        <v>0.08</v>
       </c>
       <c r="O124" t="n">
-        <v>0.057</v>
-      </c>
-      <c r="P124" t="inlineStr"/>
+        <v>0.106</v>
+      </c>
+      <c r="P124" t="inlineStr">
+        <is>
+          <t>glide_bomber</t>
+        </is>
+      </c>
       <c r="Q124" t="n">
         <v>1.3602</v>
       </c>
@@ -18363,14 +18259,14 @@
         </is>
       </c>
       <c r="N125" t="n">
-        <v>0.131</v>
+        <v>0.141</v>
       </c>
       <c r="O125" t="n">
-        <v>0.049</v>
+        <v>0.059</v>
       </c>
       <c r="P125" t="inlineStr">
         <is>
-          <t>wheeled_gun</t>
+          <t>scout_jeep</t>
         </is>
       </c>
       <c r="Q125" t="n">
@@ -18619,7 +18515,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>mounts: Mount_APS | own_geometry: 38% of triangles shared (most with rail_supergun)</t>
+          <t>mounts: Mount_APS | own_geometry: 42% of triangles shared (most with rail_supergun)</t>
         </is>
       </c>
       <c r="H127" t="n">
@@ -18651,10 +18547,10 @@
         </is>
       </c>
       <c r="N127" t="n">
-        <v>0.384</v>
+        <v>0.416</v>
       </c>
       <c r="O127" t="n">
-        <v>0.384</v>
+        <v>0.416</v>
       </c>
       <c r="P127" t="inlineStr">
         <is>
@@ -18803,10 +18699,10 @@
         </is>
       </c>
       <c r="N128" t="n">
-        <v>0.03</v>
+        <v>0.011</v>
       </c>
       <c r="O128" t="n">
-        <v>0.03</v>
+        <v>0.011</v>
       </c>
       <c r="P128" t="inlineStr"/>
       <c r="Q128" t="n">
@@ -18939,10 +18835,10 @@
         </is>
       </c>
       <c r="N129" t="n">
-        <v>0.125</v>
+        <v>0.137</v>
       </c>
       <c r="O129" t="n">
-        <v>0.151</v>
+        <v>0.148</v>
       </c>
       <c r="P129" t="inlineStr">
         <is>
@@ -19231,10 +19127,10 @@
         </is>
       </c>
       <c r="N131" t="n">
-        <v>0.035</v>
+        <v>0.036</v>
       </c>
       <c r="O131" t="n">
-        <v>0.048</v>
+        <v>0.049</v>
       </c>
       <c r="P131" t="inlineStr"/>
       <c r="Q131" t="n">
@@ -19367,7 +19263,7 @@
         </is>
       </c>
       <c r="N132" t="n">
-        <v>0.051</v>
+        <v>0.052</v>
       </c>
       <c r="O132" t="n">
         <v>0.07199999999999999</v>
@@ -19503,10 +19399,10 @@
         </is>
       </c>
       <c r="N133" t="n">
-        <v>0.115</v>
+        <v>0.116</v>
       </c>
       <c r="O133" t="n">
-        <v>0.049</v>
+        <v>0.05</v>
       </c>
       <c r="P133" t="inlineStr">
         <is>
@@ -19614,20 +19510,16 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>26744</v>
+        <v>24358</v>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G134" t="inlineStr">
-        <is>
-          <t>mounts: Mount_APS</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr"/>
       <c r="H134" t="n">
-        <v>100</v>
+        <v>98.8</v>
       </c>
       <c r="I134" t="inlineStr">
         <is>
@@ -19636,87 +19528,79 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K134" t="inlineStr">
-        <is>
-          <t>Tốt</t>
-        </is>
-      </c>
-      <c r="L134" t="inlineStr">
-        <is>
-          <t>Kém</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr"/>
+      <c r="L134" t="inlineStr"/>
       <c r="M134" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N134" t="n">
-        <v>0.066</v>
+        <v>0.012</v>
       </c>
       <c r="O134" t="n">
-        <v>0.066</v>
+        <v>0.013</v>
       </c>
       <c r="P134" t="inlineStr"/>
       <c r="Q134" t="n">
-        <v>1.4831</v>
+        <v>1.4244</v>
       </c>
       <c r="R134" t="n">
-        <v>0.1241</v>
+        <v>0.113</v>
       </c>
       <c r="S134" t="n">
-        <v>2.8214</v>
+        <v>2.3977</v>
       </c>
       <c r="T134" t="n">
-        <v>0.0299</v>
+        <v>0.0148</v>
       </c>
       <c r="U134" t="n">
-        <v>612</v>
+        <v>576</v>
       </c>
       <c r="V134" t="n">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="W134" t="n">
-        <v>1.9009</v>
+        <v>1.8387</v>
       </c>
       <c r="X134" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="Y134" t="n">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="Z134" t="n">
-        <v>511</v>
+        <v>474</v>
       </c>
       <c r="AA134" t="n">
-        <v>1.4958</v>
+        <v>1.3752</v>
       </c>
       <c r="AB134" t="n">
-        <v>7.9619</v>
+        <v>7.324</v>
       </c>
       <c r="AC134" t="n">
-        <v>64.18089999999999</v>
+        <v>64.7183</v>
       </c>
       <c r="AD134" t="n">
         <v>8</v>
       </c>
       <c r="AE134" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="AF134" t="n">
-        <v>0.2958</v>
+        <v>0.2871</v>
       </c>
       <c r="AG134" t="n">
-        <v>0.8784</v>
+        <v>0.9288999999999999</v>
       </c>
       <c r="AH134" t="n">
-        <v>0.0543</v>
+        <v>0.0667</v>
       </c>
       <c r="AI134" t="n">
-        <v>0.1468</v>
+        <v>0.2334</v>
       </c>
       <c r="AJ134" t="n">
         <v>0</v>
@@ -19734,7 +19618,7 @@
         <v>1</v>
       </c>
       <c r="AO134" t="n">
-        <v>1</v>
+        <v>0.92</v>
       </c>
       <c r="AP134" t="n">
         <v>1</v>
@@ -19803,10 +19687,10 @@
         </is>
       </c>
       <c r="N135" t="n">
-        <v>0.034</v>
+        <v>0.031</v>
       </c>
       <c r="O135" t="n">
-        <v>0.01</v>
+        <v>0.008</v>
       </c>
       <c r="P135" t="inlineStr"/>
       <c r="Q135" t="n">
@@ -19939,7 +19823,7 @@
         </is>
       </c>
       <c r="N136" t="n">
-        <v>0.107</v>
+        <v>0.136</v>
       </c>
       <c r="O136" t="n">
         <v>0.141</v>
@@ -20079,10 +19963,10 @@
         </is>
       </c>
       <c r="N137" t="n">
-        <v>0.06</v>
+        <v>0.062</v>
       </c>
       <c r="O137" t="n">
-        <v>0.074</v>
+        <v>0.076</v>
       </c>
       <c r="P137" t="inlineStr"/>
       <c r="Q137" t="n">
@@ -20227,12 +20111,16 @@
         </is>
       </c>
       <c r="N138" t="n">
-        <v>0.098</v>
+        <v>0.1</v>
       </c>
       <c r="O138" t="n">
         <v>0.067</v>
       </c>
-      <c r="P138" t="inlineStr"/>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>heavy_rocket_artillery</t>
+        </is>
+      </c>
       <c r="Q138" t="n">
         <v>1.7364</v>
       </c>
@@ -20371,10 +20259,10 @@
         </is>
       </c>
       <c r="N139" t="n">
-        <v>0.137</v>
+        <v>0.106</v>
       </c>
       <c r="O139" t="n">
-        <v>0.14</v>
+        <v>0.143</v>
       </c>
       <c r="P139" t="inlineStr">
         <is>
@@ -20630,20 +20518,16 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>11476</v>
+        <v>9284</v>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G141" t="inlineStr">
-        <is>
-          <t>mounts: muzzles 7/9</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr"/>
       <c r="H141" t="n">
-        <v>99.3</v>
+        <v>100</v>
       </c>
       <c r="I141" t="inlineStr">
         <is>
@@ -20652,19 +20536,11 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K141" t="inlineStr">
-        <is>
-          <t>Tốt</t>
-        </is>
-      </c>
-      <c r="L141" t="inlineStr">
-        <is>
-          <t>Kém</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr"/>
+      <c r="L141" t="inlineStr"/>
       <c r="M141" t="inlineStr">
         <is>
           <t>NA</t>
@@ -20674,65 +20550,65 @@
         <v>0.023</v>
       </c>
       <c r="O141" t="n">
-        <v>0.036</v>
+        <v>0.047</v>
       </c>
       <c r="P141" t="inlineStr"/>
       <c r="Q141" t="n">
-        <v>2.1645</v>
+        <v>2.0243</v>
       </c>
       <c r="R141" t="n">
-        <v>0.1704</v>
+        <v>0.1431</v>
       </c>
       <c r="S141" t="n">
-        <v>5.1398</v>
+        <v>3.7013</v>
       </c>
       <c r="T141" t="n">
-        <v>0.0304</v>
+        <v>0.0423</v>
       </c>
       <c r="U141" t="n">
-        <v>313</v>
+        <v>342</v>
       </c>
       <c r="V141" t="n">
-        <v>98</v>
+        <v>74</v>
       </c>
       <c r="W141" t="n">
-        <v>1.5899</v>
+        <v>1.4579</v>
       </c>
       <c r="X141" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="Y141" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="Z141" t="n">
-        <v>230</v>
+        <v>259</v>
       </c>
       <c r="AA141" t="n">
-        <v>1.1843</v>
+        <v>1.4776</v>
       </c>
       <c r="AB141" t="n">
-        <v>3.7315</v>
+        <v>5.1026</v>
       </c>
       <c r="AC141" t="n">
-        <v>61.6379</v>
+        <v>50.7585</v>
       </c>
       <c r="AD141" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="AE141" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="AF141" t="n">
-        <v>0.3225</v>
+        <v>0.3182</v>
       </c>
       <c r="AG141" t="n">
-        <v>0.8457</v>
+        <v>0.9295</v>
       </c>
       <c r="AH141" t="n">
-        <v>0.0509</v>
+        <v>0.0708</v>
       </c>
       <c r="AI141" t="n">
-        <v>0.0978</v>
+        <v>0.1279</v>
       </c>
       <c r="AJ141" t="n">
         <v>0</v>
@@ -20750,7 +20626,7 @@
         <v>1</v>
       </c>
       <c r="AO141" t="n">
-        <v>0.954</v>
+        <v>1</v>
       </c>
       <c r="AP141" t="n">
         <v>1</v>
@@ -20819,7 +20695,7 @@
         </is>
       </c>
       <c r="N142" t="n">
-        <v>0.028</v>
+        <v>0.032</v>
       </c>
       <c r="O142" t="n">
         <v>0.021</v>
@@ -20967,7 +20843,7 @@
         </is>
       </c>
       <c r="N143" t="n">
-        <v>0.028</v>
+        <v>0.032</v>
       </c>
       <c r="O143" t="n">
         <v>0.022</v>
@@ -21103,10 +20979,10 @@
         </is>
       </c>
       <c r="N144" t="n">
-        <v>0.076</v>
+        <v>0.075</v>
       </c>
       <c r="O144" t="n">
-        <v>0.131</v>
+        <v>0.13</v>
       </c>
       <c r="P144" t="inlineStr">
         <is>
@@ -21243,10 +21119,10 @@
         </is>
       </c>
       <c r="N145" t="n">
-        <v>0.063</v>
+        <v>0.062</v>
       </c>
       <c r="O145" t="n">
-        <v>0.028</v>
+        <v>0.025</v>
       </c>
       <c r="P145" t="inlineStr"/>
       <c r="Q145" t="n">
@@ -21379,10 +21255,10 @@
         </is>
       </c>
       <c r="N146" t="n">
-        <v>0.122</v>
+        <v>0.124</v>
       </c>
       <c r="O146" t="n">
-        <v>0.144</v>
+        <v>0.146</v>
       </c>
       <c r="P146" t="inlineStr">
         <is>
@@ -22243,7 +22119,7 @@
         </is>
       </c>
       <c r="N152" t="n">
-        <v>0.093</v>
+        <v>0.092</v>
       </c>
       <c r="O152" t="n">
         <v>0.097</v>
@@ -22379,10 +22255,10 @@
         </is>
       </c>
       <c r="N153" t="n">
-        <v>0.094</v>
+        <v>0.093</v>
       </c>
       <c r="O153" t="n">
-        <v>0.099</v>
+        <v>0.097</v>
       </c>
       <c r="P153" t="inlineStr"/>
       <c r="Q153" t="n">
@@ -22527,10 +22403,10 @@
         </is>
       </c>
       <c r="N154" t="n">
-        <v>0.165</v>
+        <v>0.159</v>
       </c>
       <c r="O154" t="n">
-        <v>0.062</v>
+        <v>0.054</v>
       </c>
       <c r="P154" t="inlineStr">
         <is>
@@ -22638,113 +22514,101 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>2652</v>
+        <v>7472</v>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G155" t="inlineStr">
-        <is>
-          <t>parts: missing axles, stowage | not_single_block: 2 sloped face directions</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr"/>
       <c r="H155" t="n">
-        <v>74.8</v>
+        <v>96.5</v>
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>Cần sửa</t>
+          <t>Tốt</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K155" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
-      <c r="L155" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr"/>
+      <c r="L155" t="inlineStr"/>
       <c r="M155" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N155" t="n">
-        <v>0.115</v>
+        <v>0.134</v>
       </c>
       <c r="O155" t="n">
-        <v>0.017</v>
+        <v>0.05</v>
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>shahed_truck</t>
+          <t>wheeled_gun</t>
         </is>
       </c>
       <c r="Q155" t="n">
-        <v>1.6477</v>
+        <v>1.6725</v>
       </c>
       <c r="R155" t="n">
-        <v>0.2085</v>
+        <v>0.2892</v>
       </c>
       <c r="S155" t="n">
-        <v>7.5905</v>
+        <v>9.145799999999999</v>
       </c>
       <c r="T155" t="n">
-        <v>0.0133</v>
+        <v>0.0185</v>
       </c>
       <c r="U155" t="n">
-        <v>73</v>
+        <v>243</v>
       </c>
       <c r="V155" t="n">
-        <v>36</v>
+        <v>99</v>
       </c>
       <c r="W155" t="n">
-        <v>0.3138</v>
+        <v>0.6909999999999999</v>
       </c>
       <c r="X155" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="Y155" t="n">
-        <v>47</v>
+        <v>118</v>
       </c>
       <c r="Z155" t="n">
-        <v>18</v>
+        <v>107</v>
       </c>
       <c r="AA155" t="n">
-        <v>0.4097</v>
+        <v>0.8236</v>
       </c>
       <c r="AB155" t="n">
-        <v>0.1569</v>
+        <v>0.7468</v>
       </c>
       <c r="AC155" t="n">
-        <v>114.714</v>
+        <v>143.2745</v>
       </c>
       <c r="AD155" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AE155" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AF155" t="n">
-        <v>0.2345</v>
+        <v>0.1244</v>
       </c>
       <c r="AG155" t="n">
-        <v>0.981</v>
+        <v>0.8302</v>
       </c>
       <c r="AH155" t="n">
-        <v>0.1113</v>
+        <v>0.051</v>
       </c>
       <c r="AI155" t="n">
-        <v>0.1836</v>
+        <v>0.1366</v>
       </c>
       <c r="AJ155" t="n">
         <v>0</v>
@@ -22753,16 +22617,16 @@
         <v>1</v>
       </c>
       <c r="AL155" t="n">
-        <v>0.779</v>
+        <v>1</v>
       </c>
       <c r="AM155" t="n">
-        <v>0.636</v>
+        <v>0.766</v>
       </c>
       <c r="AN155" t="n">
-        <v>0.5600000000000001</v>
+        <v>1</v>
       </c>
       <c r="AO155" t="n">
-        <v>0.489</v>
+        <v>1</v>
       </c>
       <c r="AP155" t="n">
         <v>1</v>
@@ -22790,7 +22654,7 @@
         </is>
       </c>
       <c r="E156" t="n">
-        <v>23256</v>
+        <v>25402</v>
       </c>
       <c r="F156" t="inlineStr">
         <is>
@@ -22799,7 +22663,7 @@
       </c>
       <c r="G156" t="inlineStr"/>
       <c r="H156" t="n">
-        <v>94.59999999999999</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="I156" t="inlineStr">
         <is>
@@ -22811,84 +22675,76 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="K156" t="inlineStr">
-        <is>
-          <t>Tốt</t>
-        </is>
-      </c>
-      <c r="L156" t="inlineStr">
-        <is>
-          <t>Kém</t>
-        </is>
-      </c>
+      <c r="K156" t="inlineStr"/>
+      <c r="L156" t="inlineStr"/>
       <c r="M156" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N156" t="n">
-        <v>0.008</v>
+        <v>0.033</v>
       </c>
       <c r="O156" t="n">
-        <v>0.008</v>
+        <v>0.059</v>
       </c>
       <c r="P156" t="inlineStr"/>
       <c r="Q156" t="n">
-        <v>1.7675</v>
+        <v>2.3291</v>
       </c>
       <c r="R156" t="n">
-        <v>0.2369</v>
+        <v>0.1607</v>
       </c>
       <c r="S156" t="n">
-        <v>6.9288</v>
+        <v>4.4634</v>
       </c>
       <c r="T156" t="n">
-        <v>0.0007</v>
+        <v>0.0376</v>
       </c>
       <c r="U156" t="n">
-        <v>574</v>
+        <v>799</v>
       </c>
       <c r="V156" t="n">
-        <v>139</v>
+        <v>110</v>
       </c>
       <c r="W156" t="n">
-        <v>0.4978</v>
+        <v>0.4184</v>
       </c>
       <c r="X156" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="Y156" t="n">
-        <v>270</v>
+        <v>369</v>
       </c>
       <c r="Z156" t="n">
-        <v>280</v>
+        <v>404</v>
       </c>
       <c r="AA156" t="n">
-        <v>0.967</v>
+        <v>1.4034</v>
       </c>
       <c r="AB156" t="n">
-        <v>1.0028</v>
+        <v>1.5365</v>
       </c>
       <c r="AC156" t="n">
-        <v>279.2178</v>
+        <v>262.9279</v>
       </c>
       <c r="AD156" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AE156" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="AF156" t="n">
-        <v>0.3228</v>
+        <v>0.3037</v>
       </c>
       <c r="AG156" t="n">
-        <v>0.9898</v>
+        <v>0.8194</v>
       </c>
       <c r="AH156" t="n">
-        <v>0.09</v>
+        <v>0.0466</v>
       </c>
       <c r="AI156" t="n">
-        <v>0.1401</v>
+        <v>0.153</v>
       </c>
       <c r="AJ156" t="n">
         <v>0</v>
@@ -22897,19 +22753,19 @@
         <v>1</v>
       </c>
       <c r="AL156" t="n">
-        <v>1</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="AM156" t="n">
-        <v>1</v>
+        <v>0.741</v>
       </c>
       <c r="AN156" t="n">
-        <v>1</v>
+        <v>0.999</v>
       </c>
       <c r="AO156" t="n">
-        <v>0.974</v>
+        <v>1</v>
       </c>
       <c r="AP156" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="157">
@@ -23115,10 +22971,10 @@
         </is>
       </c>
       <c r="N158" t="n">
-        <v>0.003</v>
+        <v>0.005</v>
       </c>
       <c r="O158" t="n">
-        <v>0.007</v>
+        <v>0.011</v>
       </c>
       <c r="P158" t="inlineStr"/>
       <c r="Q158" t="n">
@@ -23251,10 +23107,10 @@
         </is>
       </c>
       <c r="N159" t="n">
-        <v>0.028</v>
+        <v>0.04</v>
       </c>
       <c r="O159" t="n">
-        <v>0.046</v>
+        <v>0.041</v>
       </c>
       <c r="P159" t="inlineStr"/>
       <c r="Q159" t="n">
@@ -23387,10 +23243,10 @@
         </is>
       </c>
       <c r="N160" t="n">
-        <v>0.02</v>
+        <v>0.025</v>
       </c>
       <c r="O160" t="n">
-        <v>0.021</v>
+        <v>0.027</v>
       </c>
       <c r="P160" t="inlineStr"/>
       <c r="Q160" t="n">
@@ -23523,10 +23379,10 @@
         </is>
       </c>
       <c r="N161" t="n">
-        <v>0.08</v>
+        <v>0.081</v>
       </c>
       <c r="O161" t="n">
-        <v>0.182</v>
+        <v>0.179</v>
       </c>
       <c r="P161" t="inlineStr">
         <is>
@@ -23675,10 +23531,10 @@
         </is>
       </c>
       <c r="N162" t="n">
-        <v>0.182</v>
+        <v>0.195</v>
       </c>
       <c r="O162" t="n">
-        <v>0.181</v>
+        <v>0.186</v>
       </c>
       <c r="P162" t="inlineStr">
         <is>
@@ -23795,7 +23651,7 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>own_geometry: 31% of triangles shared (most with interceptor_drone_vehicle)</t>
+          <t>own_geometry: 32% of triangles shared (most with interceptor_drone_vehicle)</t>
         </is>
       </c>
       <c r="H163" t="n">
@@ -23819,7 +23675,7 @@
         </is>
       </c>
       <c r="N163" t="n">
-        <v>0.311</v>
+        <v>0.319</v>
       </c>
       <c r="O163" t="n">
         <v>0.231</v>
@@ -23967,10 +23823,10 @@
         </is>
       </c>
       <c r="N164" t="n">
-        <v>0.054</v>
+        <v>0.018</v>
       </c>
       <c r="O164" t="n">
-        <v>0.057</v>
+        <v>0.02</v>
       </c>
       <c r="P164" t="inlineStr"/>
       <c r="Q164" t="n">
@@ -24115,10 +23971,10 @@
         </is>
       </c>
       <c r="N165" t="n">
-        <v>0.314</v>
+        <v>0.349</v>
       </c>
       <c r="O165" t="n">
-        <v>0.314</v>
+        <v>0.349</v>
       </c>
       <c r="P165" t="inlineStr">
         <is>
@@ -24554,7 +24410,7 @@
         <v>0.016</v>
       </c>
       <c r="O168" t="n">
-        <v>0.127</v>
+        <v>0.133</v>
       </c>
       <c r="P168" t="inlineStr">
         <is>
@@ -24662,7 +24518,7 @@
         </is>
       </c>
       <c r="E169" t="n">
-        <v>3362</v>
+        <v>5352</v>
       </c>
       <c r="F169" t="inlineStr">
         <is>
@@ -24671,16 +24527,16 @@
       </c>
       <c r="G169" t="inlineStr"/>
       <c r="H169" t="n">
-        <v>78.5</v>
+        <v>93</v>
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>Cần sửa</t>
+          <t>Tốt</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K169" t="inlineStr"/>
@@ -24691,90 +24547,90 @@
         </is>
       </c>
       <c r="N169" t="n">
-        <v>0.148</v>
+        <v>0.157</v>
       </c>
       <c r="O169" t="n">
-        <v>0.065</v>
+        <v>0.095</v>
       </c>
       <c r="P169" t="inlineStr">
         <is>
-          <t>interceptor_drone_vehicle</t>
+          <t>wheeled_gun</t>
         </is>
       </c>
       <c r="Q169" t="n">
-        <v>1.3921</v>
+        <v>1.4029</v>
       </c>
       <c r="R169" t="n">
-        <v>0.2321</v>
+        <v>0.2677</v>
       </c>
       <c r="S169" t="n">
-        <v>7.931</v>
+        <v>11.0392</v>
       </c>
       <c r="T169" t="n">
-        <v>0.0324</v>
+        <v>0.0107</v>
       </c>
       <c r="U169" t="n">
-        <v>74</v>
+        <v>153</v>
       </c>
       <c r="V169" t="n">
-        <v>35</v>
+        <v>69</v>
       </c>
       <c r="W169" t="n">
-        <v>0.4757</v>
+        <v>0.8947000000000001</v>
       </c>
       <c r="X169" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="Y169" t="n">
-        <v>35</v>
+        <v>63</v>
       </c>
       <c r="Z169" t="n">
-        <v>20</v>
+        <v>82</v>
       </c>
       <c r="AA169" t="n">
-        <v>0.4757</v>
+        <v>0.8169</v>
       </c>
       <c r="AB169" t="n">
-        <v>0.2718</v>
+        <v>1.0632</v>
       </c>
       <c r="AC169" t="n">
-        <v>73.5825</v>
+        <v>77.1247</v>
       </c>
       <c r="AD169" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="AE169" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="AF169" t="n">
-        <v>0.4103</v>
+        <v>0.2828</v>
       </c>
       <c r="AG169" t="n">
-        <v>0.9987</v>
+        <v>0.9816</v>
       </c>
       <c r="AH169" t="n">
-        <v>0.1887</v>
+        <v>0.11</v>
       </c>
       <c r="AI169" t="n">
-        <v>0.1771</v>
+        <v>0.2713</v>
       </c>
       <c r="AJ169" t="n">
         <v>0</v>
       </c>
       <c r="AK169" t="n">
-        <v>0.743</v>
+        <v>0.763</v>
       </c>
       <c r="AL169" t="n">
-        <v>0.868</v>
+        <v>1</v>
       </c>
       <c r="AM169" t="n">
-        <v>0.665</v>
+        <v>0.925</v>
       </c>
       <c r="AN169" t="n">
-        <v>0.848</v>
+        <v>1</v>
       </c>
       <c r="AO169" t="n">
-        <v>0.662</v>
+        <v>1</v>
       </c>
       <c r="AP169" t="n">
         <v>1</v>
@@ -24831,7 +24687,7 @@
         </is>
       </c>
       <c r="N170" t="n">
-        <v>0.054</v>
+        <v>0.043</v>
       </c>
       <c r="O170" t="n">
         <v>0.01</v>
@@ -25131,10 +24987,10 @@
         </is>
       </c>
       <c r="N172" t="n">
-        <v>0.052</v>
+        <v>0.055</v>
       </c>
       <c r="O172" t="n">
-        <v>0.059</v>
+        <v>0.063</v>
       </c>
       <c r="P172" t="inlineStr"/>
       <c r="Q172" t="n">
@@ -25238,20 +25094,16 @@
         </is>
       </c>
       <c r="E173" t="n">
-        <v>2924</v>
+        <v>7482</v>
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G173" t="inlineStr">
-        <is>
-          <t>parts: missing axles, stowage | not_single_block: 0 sloped face directions</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr"/>
       <c r="H173" t="n">
-        <v>80.59999999999999</v>
+        <v>97.3</v>
       </c>
       <c r="I173" t="inlineStr">
         <is>
@@ -25260,87 +25112,83 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K173" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
-      <c r="L173" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr"/>
+      <c r="L173" t="inlineStr"/>
       <c r="M173" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N173" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.137</v>
       </c>
       <c r="O173" t="n">
-        <v>0.075</v>
-      </c>
-      <c r="P173" t="inlineStr"/>
+        <v>0.146</v>
+      </c>
+      <c r="P173" t="inlineStr">
+        <is>
+          <t>heavy_aa</t>
+        </is>
+      </c>
       <c r="Q173" t="n">
-        <v>1.7966</v>
+        <v>1.9139</v>
       </c>
       <c r="R173" t="n">
-        <v>0.2535</v>
+        <v>0.3113</v>
       </c>
       <c r="S173" t="n">
-        <v>8.043200000000001</v>
+        <v>9.812200000000001</v>
       </c>
       <c r="T173" t="n">
-        <v>0.0195</v>
+        <v>0.0276</v>
       </c>
       <c r="U173" t="n">
-        <v>82</v>
+        <v>237</v>
       </c>
       <c r="V173" t="n">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="W173" t="n">
-        <v>0.3422</v>
+        <v>0.6568000000000001</v>
       </c>
       <c r="X173" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Y173" t="n">
-        <v>63</v>
+        <v>157</v>
       </c>
       <c r="Z173" t="n">
-        <v>10</v>
+        <v>72</v>
       </c>
       <c r="AA173" t="n">
-        <v>0.634</v>
+        <v>1.322</v>
       </c>
       <c r="AB173" t="n">
-        <v>0.1006</v>
+        <v>0.6063</v>
       </c>
       <c r="AC173" t="n">
-        <v>99.3706</v>
+        <v>118.761</v>
       </c>
       <c r="AD173" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AE173" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="AF173" t="n">
-        <v>0.2539</v>
+        <v>0.1221</v>
       </c>
       <c r="AG173" t="n">
         <v>1</v>
       </c>
       <c r="AH173" t="n">
-        <v>0.2349</v>
+        <v>0.112</v>
       </c>
       <c r="AI173" t="n">
-        <v>0.2996</v>
+        <v>0.2348</v>
       </c>
       <c r="AJ173" t="n">
         <v>0</v>
@@ -25349,16 +25197,16 @@
         <v>1</v>
       </c>
       <c r="AL173" t="n">
-        <v>0.948</v>
+        <v>1</v>
       </c>
       <c r="AM173" t="n">
-        <v>0.674</v>
+        <v>0.822</v>
       </c>
       <c r="AN173" t="n">
-        <v>0.61</v>
+        <v>1</v>
       </c>
       <c r="AO173" t="n">
-        <v>0.606</v>
+        <v>1</v>
       </c>
       <c r="AP173" t="n">
         <v>1</v>
@@ -25423,12 +25271,16 @@
         </is>
       </c>
       <c r="N174" t="n">
-        <v>0.049</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="O174" t="n">
-        <v>0.075</v>
-      </c>
-      <c r="P174" t="inlineStr"/>
+        <v>0.107</v>
+      </c>
+      <c r="P174" t="inlineStr">
+        <is>
+          <t>aps_tank</t>
+        </is>
+      </c>
       <c r="Q174" t="n">
         <v>1.3585</v>
       </c>
@@ -25559,14 +25411,14 @@
         </is>
       </c>
       <c r="N175" t="n">
-        <v>0.113</v>
+        <v>0.123</v>
       </c>
       <c r="O175" t="n">
-        <v>0.006</v>
+        <v>0.026</v>
       </c>
       <c r="P175" t="inlineStr">
         <is>
-          <t>radar_scout</t>
+          <t>scout_jeep_hd</t>
         </is>
       </c>
       <c r="Q175" t="n">
@@ -25699,10 +25551,10 @@
         </is>
       </c>
       <c r="N176" t="n">
-        <v>0.025</v>
+        <v>0.018</v>
       </c>
       <c r="O176" t="n">
-        <v>0.026</v>
+        <v>0.017</v>
       </c>
       <c r="P176" t="inlineStr"/>
       <c r="Q176" t="n">
@@ -25838,7 +25690,7 @@
         <v>0.045</v>
       </c>
       <c r="O177" t="n">
-        <v>0.053</v>
+        <v>0.052</v>
       </c>
       <c r="P177" t="inlineStr"/>
       <c r="Q177" t="n">
@@ -26078,7 +25930,7 @@
         </is>
       </c>
       <c r="E179" t="n">
-        <v>2302</v>
+        <v>5224</v>
       </c>
       <c r="F179" t="inlineStr">
         <is>
@@ -26087,7 +25939,7 @@
       </c>
       <c r="G179" t="inlineStr"/>
       <c r="H179" t="n">
-        <v>81.7</v>
+        <v>99.3</v>
       </c>
       <c r="I179" t="inlineStr">
         <is>
@@ -26099,94 +25951,82 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="K179" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
-      <c r="L179" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
+      <c r="K179" t="inlineStr"/>
+      <c r="L179" t="inlineStr"/>
       <c r="M179" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N179" t="n">
-        <v>0.123</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="O179" t="n">
-        <v>0.127</v>
-      </c>
-      <c r="P179" t="inlineStr">
-        <is>
-          <t>airborne_light_tank</t>
-        </is>
-      </c>
+        <v>0.098</v>
+      </c>
+      <c r="P179" t="inlineStr"/>
       <c r="Q179" t="n">
-        <v>1.2965</v>
+        <v>1.4659</v>
       </c>
       <c r="R179" t="n">
-        <v>0.2336</v>
+        <v>0.2764</v>
       </c>
       <c r="S179" t="n">
-        <v>9.3042</v>
+        <v>9.6251</v>
       </c>
       <c r="T179" t="n">
-        <v>0.0005</v>
+        <v>0.0041</v>
       </c>
       <c r="U179" t="n">
-        <v>47</v>
+        <v>145</v>
       </c>
       <c r="V179" t="n">
-        <v>27</v>
+        <v>72</v>
       </c>
       <c r="W179" t="n">
-        <v>0.3375</v>
+        <v>0.6133999999999999</v>
       </c>
       <c r="X179" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="Y179" t="n">
-        <v>29</v>
+        <v>77</v>
       </c>
       <c r="Z179" t="n">
-        <v>13</v>
+        <v>54</v>
       </c>
       <c r="AA179" t="n">
-        <v>0.3625</v>
+        <v>0.656</v>
       </c>
       <c r="AB179" t="n">
-        <v>0.1625</v>
+        <v>0.46</v>
       </c>
       <c r="AC179" t="n">
-        <v>80.0048</v>
+        <v>117.3831</v>
       </c>
       <c r="AD179" t="n">
+        <v>8</v>
+      </c>
+      <c r="AE179" t="n">
         <v>10</v>
       </c>
-      <c r="AE179" t="n">
-        <v>7</v>
-      </c>
       <c r="AF179" t="n">
-        <v>0.7073</v>
+        <v>0.4338</v>
       </c>
       <c r="AG179" t="n">
-        <v>0.9898</v>
+        <v>0.8216</v>
       </c>
       <c r="AH179" t="n">
-        <v>0.1723</v>
+        <v>0.0499</v>
       </c>
       <c r="AI179" t="n">
-        <v>0.0539</v>
+        <v>0.1704</v>
       </c>
       <c r="AJ179" t="n">
         <v>0</v>
       </c>
       <c r="AK179" t="n">
-        <v>0.758</v>
+        <v>1</v>
       </c>
       <c r="AL179" t="n">
         <v>1</v>
@@ -26198,10 +26038,10 @@
         <v>1</v>
       </c>
       <c r="AO179" t="n">
-        <v>0.517</v>
+        <v>0.95</v>
       </c>
       <c r="AP179" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="180">
@@ -26255,14 +26095,14 @@
         </is>
       </c>
       <c r="N180" t="n">
-        <v>0.091</v>
+        <v>0.153</v>
       </c>
       <c r="O180" t="n">
-        <v>0.103</v>
+        <v>0.102</v>
       </c>
       <c r="P180" t="inlineStr">
         <is>
-          <t>armored_bulldozer</t>
+          <t>mlrs</t>
         </is>
       </c>
       <c r="Q180" t="n">
@@ -26407,10 +26247,10 @@
         </is>
       </c>
       <c r="N181" t="n">
-        <v>0.118</v>
+        <v>0.123</v>
       </c>
       <c r="O181" t="n">
-        <v>0.02</v>
+        <v>0.008</v>
       </c>
       <c r="P181" t="inlineStr">
         <is>
@@ -26547,10 +26387,10 @@
         </is>
       </c>
       <c r="N182" t="n">
-        <v>0.121</v>
+        <v>0.122</v>
       </c>
       <c r="O182" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.073</v>
       </c>
       <c r="P182" t="inlineStr">
         <is>
@@ -26687,10 +26527,10 @@
         </is>
       </c>
       <c r="N183" t="n">
-        <v>0.127</v>
+        <v>0.128</v>
       </c>
       <c r="O183" t="n">
-        <v>0.077</v>
+        <v>0.079</v>
       </c>
       <c r="P183" t="inlineStr">
         <is>
@@ -26827,10 +26667,10 @@
         </is>
       </c>
       <c r="N184" t="n">
-        <v>0.125</v>
+        <v>0.126</v>
       </c>
       <c r="O184" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="P184" t="inlineStr">
         <is>
@@ -26967,10 +26807,10 @@
         </is>
       </c>
       <c r="N185" t="n">
-        <v>0.113</v>
+        <v>0.11</v>
       </c>
       <c r="O185" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.061</v>
       </c>
       <c r="P185" t="inlineStr">
         <is>
@@ -27107,10 +26947,10 @@
         </is>
       </c>
       <c r="N186" t="n">
-        <v>0.02</v>
+        <v>0.022</v>
       </c>
       <c r="O186" t="n">
-        <v>0.033</v>
+        <v>0.038</v>
       </c>
       <c r="P186" t="inlineStr"/>
       <c r="Q186" t="n">
@@ -27255,12 +27095,16 @@
         </is>
       </c>
       <c r="N187" t="n">
-        <v>0.092</v>
+        <v>0.108</v>
       </c>
       <c r="O187" t="n">
-        <v>0.008999999999999999</v>
-      </c>
-      <c r="P187" t="inlineStr"/>
+        <v>0.013</v>
+      </c>
+      <c r="P187" t="inlineStr">
+        <is>
+          <t>iron_beam</t>
+        </is>
+      </c>
       <c r="Q187" t="n">
         <v>1.4631</v>
       </c>
@@ -27403,10 +27247,10 @@
         </is>
       </c>
       <c r="N188" t="n">
-        <v>0.315</v>
+        <v>0.345</v>
       </c>
       <c r="O188" t="n">
-        <v>0.308</v>
+        <v>0.339</v>
       </c>
       <c r="P188" t="inlineStr">
         <is>
@@ -27555,14 +27399,14 @@
         </is>
       </c>
       <c r="N189" t="n">
-        <v>0.223</v>
+        <v>0.244</v>
       </c>
       <c r="O189" t="n">
-        <v>0.223</v>
+        <v>0.244</v>
       </c>
       <c r="P189" t="inlineStr">
         <is>
-          <t>leviathan</t>
+          <t>kraken</t>
         </is>
       </c>
       <c r="Q189" t="n">
@@ -27695,7 +27539,7 @@
         </is>
       </c>
       <c r="N190" t="n">
-        <v>0.093</v>
+        <v>0.095</v>
       </c>
       <c r="O190" t="n">
         <v>0.133</v>
@@ -27847,14 +27691,14 @@
         </is>
       </c>
       <c r="N191" t="n">
-        <v>0.16</v>
+        <v>0.157</v>
       </c>
       <c r="O191" t="n">
-        <v>0.073</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="P191" t="inlineStr">
         <is>
-          <t>mlrs</t>
+          <t>ballistic_launcher</t>
         </is>
       </c>
       <c r="Q191" t="n">
@@ -27999,10 +27843,10 @@
         </is>
       </c>
       <c r="N192" t="n">
-        <v>0.027</v>
+        <v>0.04</v>
       </c>
       <c r="O192" t="n">
-        <v>0.036</v>
+        <v>0.062</v>
       </c>
       <c r="P192" t="inlineStr"/>
       <c r="Q192" t="n">
@@ -28135,10 +27979,10 @@
         </is>
       </c>
       <c r="N193" t="n">
-        <v>0.039</v>
+        <v>0.016</v>
       </c>
       <c r="O193" t="n">
-        <v>0.05</v>
+        <v>0.016</v>
       </c>
       <c r="P193" t="inlineStr"/>
       <c r="Q193" t="n">
@@ -28271,10 +28115,10 @@
         </is>
       </c>
       <c r="N194" t="n">
-        <v>0.021</v>
+        <v>0.031</v>
       </c>
       <c r="O194" t="n">
-        <v>0.024</v>
+        <v>0.039</v>
       </c>
       <c r="P194" t="inlineStr"/>
       <c r="Q194" t="n">
@@ -28555,10 +28399,10 @@
         </is>
       </c>
       <c r="N196" t="n">
-        <v>0.054</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="O196" t="n">
-        <v>0.135</v>
+        <v>0.149</v>
       </c>
       <c r="P196" t="inlineStr">
         <is>
@@ -28695,10 +28539,10 @@
         </is>
       </c>
       <c r="N197" t="n">
-        <v>0.119</v>
+        <v>0.118</v>
       </c>
       <c r="O197" t="n">
-        <v>0.025</v>
+        <v>0.023</v>
       </c>
       <c r="P197" t="inlineStr">
         <is>
@@ -28843,10 +28687,10 @@
         </is>
       </c>
       <c r="N198" t="n">
-        <v>0.037</v>
+        <v>0.038</v>
       </c>
       <c r="O198" t="n">
-        <v>0.038</v>
+        <v>0.039</v>
       </c>
       <c r="P198" t="inlineStr"/>
       <c r="Q198" t="n">
@@ -28979,10 +28823,10 @@
         </is>
       </c>
       <c r="N199" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="O199" t="n">
         <v>0.036</v>
-      </c>
-      <c r="O199" t="n">
-        <v>0.038</v>
       </c>
       <c r="P199" t="inlineStr"/>
       <c r="Q199" t="n">
@@ -29115,10 +28959,10 @@
         </is>
       </c>
       <c r="N200" t="n">
-        <v>0.021</v>
+        <v>0.025</v>
       </c>
       <c r="O200" t="n">
-        <v>0.022</v>
+        <v>0.025</v>
       </c>
       <c r="P200" t="inlineStr"/>
       <c r="Q200" t="n">
@@ -29391,10 +29235,10 @@
         </is>
       </c>
       <c r="N202" t="n">
-        <v>0.073</v>
+        <v>0.078</v>
       </c>
       <c r="O202" t="n">
-        <v>0.025</v>
+        <v>0.008</v>
       </c>
       <c r="P202" t="inlineStr"/>
       <c r="Q202" t="n">
@@ -29527,10 +29371,10 @@
         </is>
       </c>
       <c r="N203" t="n">
-        <v>0.011</v>
+        <v>0.007</v>
       </c>
       <c r="O203" t="n">
-        <v>0.007</v>
+        <v>0.003</v>
       </c>
       <c r="P203" t="inlineStr"/>
       <c r="Q203" t="n">
@@ -29959,7 +29803,7 @@
         </is>
       </c>
       <c r="N206" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
       <c r="O206" t="n">
         <v>0.001</v>
@@ -30095,7 +29939,7 @@
         </is>
       </c>
       <c r="N207" t="n">
-        <v>0.018</v>
+        <v>0.014</v>
       </c>
       <c r="O207" t="n">
         <v>0.031</v>
@@ -30231,10 +30075,10 @@
         </is>
       </c>
       <c r="N208" t="n">
-        <v>0.019</v>
+        <v>0.027</v>
       </c>
       <c r="O208" t="n">
-        <v>0.024</v>
+        <v>0.02</v>
       </c>
       <c r="P208" t="inlineStr"/>
       <c r="Q208" t="n">
@@ -30367,10 +30211,10 @@
         </is>
       </c>
       <c r="N209" t="n">
-        <v>0.115</v>
+        <v>0.114</v>
       </c>
       <c r="O209" t="n">
-        <v>0.135</v>
+        <v>0.134</v>
       </c>
       <c r="P209" t="inlineStr">
         <is>
@@ -30515,7 +30359,7 @@
         </is>
       </c>
       <c r="N210" t="n">
-        <v>0.024</v>
+        <v>0.025</v>
       </c>
       <c r="O210" t="n">
         <v>0.029</v>
@@ -30787,7 +30631,7 @@
         </is>
       </c>
       <c r="N212" t="n">
-        <v>0.104</v>
+        <v>0.143</v>
       </c>
       <c r="O212" t="n">
         <v>0.16</v>
@@ -30939,10 +30783,10 @@
         </is>
       </c>
       <c r="N213" t="n">
-        <v>0.035</v>
+        <v>0.031</v>
       </c>
       <c r="O213" t="n">
-        <v>0.033</v>
+        <v>0.029</v>
       </c>
       <c r="P213" t="inlineStr"/>
       <c r="Q213" t="n">
@@ -31075,10 +30919,10 @@
         </is>
       </c>
       <c r="N214" t="n">
-        <v>0.113</v>
+        <v>0.114</v>
       </c>
       <c r="O214" t="n">
-        <v>0.09</v>
+        <v>0.094</v>
       </c>
       <c r="P214" t="inlineStr">
         <is>
@@ -31215,16 +31059,12 @@
         </is>
       </c>
       <c r="N215" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="O215" t="n">
         <v>0.05</v>
       </c>
-      <c r="O215" t="n">
-        <v>0.105</v>
-      </c>
-      <c r="P215" t="inlineStr">
-        <is>
-          <t>twin_tank</t>
-        </is>
-      </c>
+      <c r="P215" t="inlineStr"/>
       <c r="Q215" t="n">
         <v>1.4213</v>
       </c>
@@ -31355,10 +31195,10 @@
         </is>
       </c>
       <c r="N216" t="n">
-        <v>0.115</v>
+        <v>0.118</v>
       </c>
       <c r="O216" t="n">
-        <v>0.223</v>
+        <v>0.228</v>
       </c>
       <c r="P216" t="inlineStr">
         <is>
@@ -31495,10 +31335,10 @@
         </is>
       </c>
       <c r="N217" t="n">
-        <v>0.06</v>
+        <v>0.082</v>
       </c>
       <c r="O217" t="n">
-        <v>0.031</v>
+        <v>0.033</v>
       </c>
       <c r="P217" t="inlineStr"/>
       <c r="Q217" t="n">
@@ -31631,10 +31471,10 @@
         </is>
       </c>
       <c r="N218" t="n">
-        <v>0.108</v>
+        <v>0.106</v>
       </c>
       <c r="O218" t="n">
-        <v>0.078</v>
+        <v>0.075</v>
       </c>
       <c r="P218" t="inlineStr">
         <is>
@@ -31783,10 +31623,10 @@
         </is>
       </c>
       <c r="N219" t="n">
-        <v>0.006</v>
+        <v>0.004</v>
       </c>
       <c r="O219" t="n">
-        <v>0.008</v>
+        <v>0.004</v>
       </c>
       <c r="P219" t="inlineStr"/>
       <c r="Q219" t="n">
@@ -31919,10 +31759,10 @@
         </is>
       </c>
       <c r="N220" t="n">
-        <v>0.157</v>
+        <v>0.175</v>
       </c>
       <c r="O220" t="n">
-        <v>0.14</v>
+        <v>0.142</v>
       </c>
       <c r="P220" t="inlineStr">
         <is>
@@ -32059,10 +31899,10 @@
         </is>
       </c>
       <c r="N221" t="n">
-        <v>0.036</v>
+        <v>0.037</v>
       </c>
       <c r="O221" t="n">
-        <v>0.045</v>
+        <v>0.046</v>
       </c>
       <c r="P221" t="inlineStr"/>
       <c r="Q221" t="n">
@@ -32207,10 +32047,10 @@
         </is>
       </c>
       <c r="N222" t="n">
-        <v>0.03</v>
+        <v>0.024</v>
       </c>
       <c r="O222" t="n">
-        <v>0.008</v>
+        <v>0.013</v>
       </c>
       <c r="P222" t="inlineStr"/>
       <c r="Q222" t="n">
@@ -32343,12 +32183,16 @@
         </is>
       </c>
       <c r="N223" t="n">
-        <v>0.099</v>
+        <v>0.123</v>
       </c>
       <c r="O223" t="n">
-        <v>0.027</v>
-      </c>
-      <c r="P223" t="inlineStr"/>
+        <v>0.019</v>
+      </c>
+      <c r="P223" t="inlineStr">
+        <is>
+          <t>elite_mlrs</t>
+        </is>
+      </c>
       <c r="Q223" t="n">
         <v>1.3296</v>
       </c>
@@ -32483,10 +32327,10 @@
         </is>
       </c>
       <c r="N224" t="n">
-        <v>0.011</v>
+        <v>0.008</v>
       </c>
       <c r="O224" t="n">
-        <v>0.017</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="P224" t="inlineStr"/>
       <c r="Q224" t="n">
@@ -32891,10 +32735,10 @@
         </is>
       </c>
       <c r="N227" t="n">
-        <v>0.01</v>
+        <v>0.008</v>
       </c>
       <c r="O227" t="n">
-        <v>0.014</v>
+        <v>0.011</v>
       </c>
       <c r="P227" t="inlineStr"/>
       <c r="Q227" t="n">
@@ -32998,131 +32842,119 @@
         </is>
       </c>
       <c r="E228" t="n">
-        <v>3058</v>
+        <v>7178</v>
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="G228" t="inlineStr">
-        <is>
-          <t>parts: missing axles, glass, stowage</t>
-        </is>
-      </c>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr"/>
       <c r="H228" t="n">
-        <v>70.59999999999999</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="I228" t="inlineStr">
         <is>
-          <t>Cần sửa</t>
+          <t>Tốt</t>
         </is>
       </c>
       <c r="J228" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K228" t="inlineStr">
-        <is>
-          <t>Tốt</t>
-        </is>
-      </c>
-      <c r="L228" t="inlineStr">
-        <is>
-          <t>Cần sửa</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K228" t="inlineStr"/>
+      <c r="L228" t="inlineStr"/>
       <c r="M228" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="N228" t="n">
-        <v>0.166</v>
+        <v>0.295</v>
       </c>
       <c r="O228" t="n">
-        <v>0.097</v>
+        <v>0.027</v>
       </c>
       <c r="P228" t="inlineStr">
         <is>
-          <t>elite_tank_destroyer</t>
+          <t>heavy_tank</t>
         </is>
       </c>
       <c r="Q228" t="n">
-        <v>1.2332</v>
+        <v>1.4696</v>
       </c>
       <c r="R228" t="n">
-        <v>0.2359</v>
+        <v>0.2793</v>
       </c>
       <c r="S228" t="n">
-        <v>8.099299999999999</v>
+        <v>11.039</v>
       </c>
       <c r="T228" t="n">
-        <v>0.016</v>
+        <v>0.0195</v>
       </c>
       <c r="U228" t="n">
-        <v>65</v>
+        <v>160</v>
       </c>
       <c r="V228" t="n">
-        <v>36</v>
+        <v>71</v>
       </c>
       <c r="W228" t="n">
-        <v>0.4493</v>
+        <v>1.0002</v>
       </c>
       <c r="X228" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Y228" t="n">
-        <v>30</v>
+        <v>69</v>
       </c>
       <c r="Z228" t="n">
-        <v>29</v>
+        <v>86</v>
       </c>
       <c r="AA228" t="n">
-        <v>0.3744</v>
+        <v>0.9721</v>
       </c>
       <c r="AB228" t="n">
-        <v>0.362</v>
+        <v>1.2115</v>
       </c>
       <c r="AC228" t="n">
-        <v>80.1208</v>
+        <v>70.9836</v>
       </c>
       <c r="AD228" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="AE228" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="AF228" t="n">
-        <v>0.2109</v>
+        <v>0.129</v>
       </c>
       <c r="AG228" t="n">
-        <v>0.99</v>
+        <v>0.9816</v>
       </c>
       <c r="AH228" t="n">
-        <v>0.1508</v>
+        <v>0.1013</v>
       </c>
       <c r="AI228" t="n">
-        <v>0.2294</v>
+        <v>0.2437</v>
       </c>
       <c r="AJ228" t="n">
         <v>0</v>
       </c>
       <c r="AK228" t="n">
-        <v>0.442</v>
+        <v>0.89</v>
       </c>
       <c r="AL228" t="n">
-        <v>0.882</v>
+        <v>1</v>
       </c>
       <c r="AM228" t="n">
-        <v>0.679</v>
+        <v>0.925</v>
       </c>
       <c r="AN228" t="n">
-        <v>0.801</v>
+        <v>1</v>
       </c>
       <c r="AO228" t="n">
-        <v>0.677</v>
+        <v>1</v>
       </c>
       <c r="AP228" t="n">
         <v>1</v>
@@ -33183,7 +33015,7 @@
         </is>
       </c>
       <c r="N229" t="n">
-        <v>0.123</v>
+        <v>0.124</v>
       </c>
       <c r="O229" t="n">
         <v>0.146</v>
@@ -33323,10 +33155,10 @@
         </is>
       </c>
       <c r="N230" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="O230" t="n">
-        <v>0.11</v>
+        <v>0.104</v>
       </c>
       <c r="P230" t="inlineStr">
         <is>
@@ -33463,10 +33295,10 @@
         </is>
       </c>
       <c r="N231" t="n">
-        <v>0.032</v>
+        <v>0.031</v>
       </c>
       <c r="O231" t="n">
-        <v>0.024</v>
+        <v>0.018</v>
       </c>
       <c r="P231" t="inlineStr"/>
       <c r="Q231" t="n">

</xml_diff>

<commit_message>
P35: final report Docs/models/REBUILD_REPORT.md (section 10), full gate refresh after the owner fixes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/models/quality_report.xlsx
+++ b/Docs/models/quality_report.xlsx
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>9256</v>
+        <v>10648</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -2616,7 +2616,7 @@
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>85.8</v>
+        <v>95</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -2636,10 +2636,10 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>0.096</v>
+        <v>0.046</v>
       </c>
       <c r="O16" t="n">
-        <v>0.127</v>
+        <v>0.104</v>
       </c>
       <c r="P16" t="inlineStr">
         <is>
@@ -2647,73 +2647,73 @@
         </is>
       </c>
       <c r="Q16" t="n">
-        <v>1.3317</v>
+        <v>1.3994</v>
       </c>
       <c r="R16" t="n">
-        <v>0.1701</v>
+        <v>0.2015</v>
       </c>
       <c r="S16" t="n">
-        <v>3.9951</v>
+        <v>5.6118</v>
       </c>
       <c r="T16" t="n">
-        <v>0.0396</v>
+        <v>0.0086</v>
       </c>
       <c r="U16" t="n">
-        <v>288</v>
+        <v>371</v>
       </c>
       <c r="V16" t="n">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="W16" t="n">
-        <v>0.5717</v>
+        <v>0.6569</v>
       </c>
       <c r="X16" t="n">
         <v>11</v>
       </c>
       <c r="Y16" t="n">
-        <v>137</v>
+        <v>196</v>
       </c>
       <c r="Z16" t="n">
-        <v>140</v>
+        <v>164</v>
       </c>
       <c r="AA16" t="n">
-        <v>0.9107</v>
+        <v>1.3995</v>
       </c>
       <c r="AB16" t="n">
-        <v>0.9307</v>
+        <v>1.171</v>
       </c>
       <c r="AC16" t="n">
-        <v>150.4287</v>
+        <v>140.0463</v>
       </c>
       <c r="AD16" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AE16" t="n">
         <v>8</v>
       </c>
       <c r="AF16" t="n">
-        <v>0.2036</v>
+        <v>0.1218</v>
       </c>
       <c r="AG16" t="n">
-        <v>0.8867</v>
+        <v>0.8222</v>
       </c>
       <c r="AH16" t="n">
-        <v>0.06469999999999999</v>
+        <v>0.0482</v>
       </c>
       <c r="AI16" t="n">
-        <v>0.2211</v>
+        <v>0.2121</v>
       </c>
       <c r="AJ16" t="n">
         <v>0</v>
       </c>
       <c r="AK16" t="n">
-        <v>0.848</v>
+        <v>1</v>
       </c>
       <c r="AL16" t="n">
-        <v>0.782</v>
+        <v>0.927</v>
       </c>
       <c r="AM16" t="n">
-        <v>0.525</v>
+        <v>0.738</v>
       </c>
       <c r="AN16" t="n">
         <v>1</v>
@@ -2918,10 +2918,10 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>0.006</v>
+        <v>0.011</v>
       </c>
       <c r="O18" t="n">
-        <v>0.012</v>
+        <v>0.031</v>
       </c>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="n">
@@ -3192,10 +3192,10 @@
         </is>
       </c>
       <c r="N20" t="n">
-        <v>0.112</v>
+        <v>0.101</v>
       </c>
       <c r="O20" t="n">
-        <v>0.094</v>
+        <v>0.097</v>
       </c>
       <c r="P20" t="inlineStr">
         <is>
@@ -4880,10 +4880,10 @@
         </is>
       </c>
       <c r="N32" t="n">
-        <v>0.044</v>
+        <v>0.043</v>
       </c>
       <c r="O32" t="n">
-        <v>0.065</v>
+        <v>0.063</v>
       </c>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="n">
@@ -6266,10 +6266,10 @@
         </is>
       </c>
       <c r="N42" t="n">
-        <v>0.074</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="O42" t="n">
-        <v>0.076</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="n">
@@ -6403,10 +6403,10 @@
         </is>
       </c>
       <c r="N43" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.068</v>
       </c>
       <c r="O43" t="n">
-        <v>0.074</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="P43" t="inlineStr"/>
       <c r="Q43" t="n">
@@ -6540,10 +6540,10 @@
         </is>
       </c>
       <c r="N44" t="n">
-        <v>0.074</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="O44" t="n">
-        <v>0.073</v>
+        <v>0.068</v>
       </c>
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="n">
@@ -6814,7 +6814,7 @@
         </is>
       </c>
       <c r="N46" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="O46" t="n">
         <v>0.127</v>
@@ -7239,10 +7239,10 @@
         </is>
       </c>
       <c r="N49" t="n">
-        <v>0.165</v>
+        <v>0.161</v>
       </c>
       <c r="O49" t="n">
-        <v>0.166</v>
+        <v>0.159</v>
       </c>
       <c r="P49" t="inlineStr">
         <is>
@@ -7793,10 +7793,10 @@
         </is>
       </c>
       <c r="N53" t="n">
-        <v>0.122</v>
+        <v>0.121</v>
       </c>
       <c r="O53" t="n">
-        <v>0.127</v>
+        <v>0.126</v>
       </c>
       <c r="P53" t="inlineStr">
         <is>
@@ -10449,7 +10449,7 @@
         <v>0.122</v>
       </c>
       <c r="O72" t="n">
-        <v>0.132</v>
+        <v>0.134</v>
       </c>
       <c r="P72" t="inlineStr">
         <is>
@@ -10724,7 +10724,7 @@
         </is>
       </c>
       <c r="N74" t="n">
-        <v>0.096</v>
+        <v>0.095</v>
       </c>
       <c r="O74" t="n">
         <v>0.062</v>
@@ -10861,10 +10861,10 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>0.06</v>
+        <v>0.061</v>
       </c>
       <c r="O75" t="n">
-        <v>0.044</v>
+        <v>0.045</v>
       </c>
       <c r="P75" t="inlineStr"/>
       <c r="Q75" t="n">
@@ -11139,10 +11139,10 @@
         </is>
       </c>
       <c r="N77" t="n">
-        <v>0.103</v>
+        <v>0.104</v>
       </c>
       <c r="O77" t="n">
-        <v>0.105</v>
+        <v>0.107</v>
       </c>
       <c r="P77" t="inlineStr">
         <is>
@@ -12420,7 +12420,7 @@
         </is>
       </c>
       <c r="N86" t="n">
-        <v>0.051</v>
+        <v>0.054</v>
       </c>
       <c r="O86" t="n">
         <v>0.076</v>
@@ -12835,10 +12835,10 @@
         </is>
       </c>
       <c r="N89" t="n">
-        <v>0.039</v>
+        <v>0.04</v>
       </c>
       <c r="O89" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.074</v>
       </c>
       <c r="P89" t="inlineStr"/>
       <c r="Q89" t="n">
@@ -13661,10 +13661,10 @@
         </is>
       </c>
       <c r="N95" t="n">
-        <v>0.078</v>
+        <v>0.077</v>
       </c>
       <c r="O95" t="n">
-        <v>0.057</v>
+        <v>0.055</v>
       </c>
       <c r="P95" t="inlineStr"/>
       <c r="Q95" t="n">
@@ -17282,7 +17282,7 @@
         <v>0.118</v>
       </c>
       <c r="O121" t="n">
-        <v>0.175</v>
+        <v>0.174</v>
       </c>
       <c r="P121" t="inlineStr">
         <is>
@@ -19495,10 +19495,10 @@
         </is>
       </c>
       <c r="N137" t="n">
-        <v>0.057</v>
+        <v>0.056</v>
       </c>
       <c r="O137" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.067</v>
       </c>
       <c r="P137" t="inlineStr"/>
       <c r="Q137" t="n">
@@ -20762,10 +20762,10 @@
         </is>
       </c>
       <c r="N146" t="n">
-        <v>0.139</v>
+        <v>0.14</v>
       </c>
       <c r="O146" t="n">
-        <v>0.176</v>
+        <v>0.178</v>
       </c>
       <c r="P146" t="inlineStr">
         <is>
@@ -22987,7 +22987,7 @@
         <v>0.075</v>
       </c>
       <c r="O162" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="P162" t="inlineStr"/>
       <c r="Q162" t="n">
@@ -24514,7 +24514,7 @@
         <v>0.164</v>
       </c>
       <c r="O173" t="n">
-        <v>0.152</v>
+        <v>0.151</v>
       </c>
       <c r="P173" t="inlineStr">
         <is>
@@ -25619,10 +25619,10 @@
         </is>
       </c>
       <c r="N181" t="n">
-        <v>0.092</v>
+        <v>0.09</v>
       </c>
       <c r="O181" t="n">
-        <v>0.073</v>
+        <v>0.068</v>
       </c>
       <c r="P181" t="inlineStr"/>
       <c r="Q181" t="n">
@@ -27577,7 +27577,7 @@
         </is>
       </c>
       <c r="N195" t="n">
-        <v>0.031</v>
+        <v>0.016</v>
       </c>
       <c r="O195" t="n">
         <v>0.014</v>
@@ -29938,7 +29938,7 @@
         </is>
       </c>
       <c r="N212" t="n">
-        <v>0.17</v>
+        <v>0.173</v>
       </c>
       <c r="O212" t="n">
         <v>0.222</v>
@@ -30357,10 +30357,10 @@
         </is>
       </c>
       <c r="N215" t="n">
-        <v>0.037</v>
+        <v>0.038</v>
       </c>
       <c r="O215" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="P215" t="inlineStr"/>
       <c r="Q215" t="n">

</xml_diff>

<commit_message>
P35 GLB size: quantise all 518 GLBs (KHR_mesh_quantization), 168.4 -> 131.3 MiB (+6.6 % vs 01f7312b); baseline accepted, gate refreshed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/models/quality_report.xlsx
+++ b/Docs/models/quality_report.xlsx
@@ -2147,7 +2147,7 @@
         <v>0.0568</v>
       </c>
       <c r="AI12" t="n">
-        <v>0.2422</v>
+        <v>0.2423</v>
       </c>
       <c r="AJ12" t="n">
         <v>0</v>
@@ -4086,7 +4086,7 @@
         <v>19</v>
       </c>
       <c r="AF26" t="n">
-        <v>0.3617</v>
+        <v>0.3616</v>
       </c>
       <c r="AG26" t="n">
         <v>0.8702</v>
@@ -10370,7 +10370,7 @@
         <v>0.0668</v>
       </c>
       <c r="AI71" t="n">
-        <v>0.2466</v>
+        <v>0.2467</v>
       </c>
       <c r="AJ71" t="n">
         <v>0</v>
@@ -11622,7 +11622,7 @@
         <v>19</v>
       </c>
       <c r="AF80" t="n">
-        <v>0.356</v>
+        <v>0.3561</v>
       </c>
       <c r="AG80" t="n">
         <v>1</v>
@@ -11908,7 +11908,7 @@
         <v>19</v>
       </c>
       <c r="AF82" t="n">
-        <v>0.356</v>
+        <v>0.3561</v>
       </c>
       <c r="AG82" t="n">
         <v>0.9987</v>
@@ -13576,7 +13576,7 @@
         <v>9</v>
       </c>
       <c r="AF94" t="n">
-        <v>0.122</v>
+        <v>0.1219</v>
       </c>
       <c r="AG94" t="n">
         <v>0.9119</v>
@@ -14265,7 +14265,7 @@
         <v>15</v>
       </c>
       <c r="AF99" t="n">
-        <v>0.3854</v>
+        <v>0.3853</v>
       </c>
       <c r="AG99" t="n">
         <v>0.9547</v>
@@ -15255,7 +15255,7 @@
         <v>0.1354</v>
       </c>
       <c r="AG106" t="n">
-        <v>0.9553</v>
+        <v>0.9554</v>
       </c>
       <c r="AH106" t="n">
         <v>0.077</v>
@@ -15802,7 +15802,7 @@
         <v>10</v>
       </c>
       <c r="AF110" t="n">
-        <v>0.1118</v>
+        <v>0.1117</v>
       </c>
       <c r="AG110" t="n">
         <v>0.9387</v>
@@ -16373,7 +16373,7 @@
         <v>0.3293</v>
       </c>
       <c r="AG114" t="n">
-        <v>0.9553</v>
+        <v>0.9554</v>
       </c>
       <c r="AH114" t="n">
         <v>0.0779</v>
@@ -18578,7 +18578,7 @@
         <v>12</v>
       </c>
       <c r="AF130" t="n">
-        <v>0.1497</v>
+        <v>0.1498</v>
       </c>
       <c r="AG130" t="n">
         <v>0.8058</v>
@@ -24801,7 +24801,7 @@
         <v>1.5917</v>
       </c>
       <c r="R175" t="n">
-        <v>0.3986</v>
+        <v>0.3983</v>
       </c>
       <c r="S175" t="n">
         <v>19.4316</v>
@@ -27073,7 +27073,7 @@
         <v>11</v>
       </c>
       <c r="AF191" t="n">
-        <v>0.1697</v>
+        <v>0.1698</v>
       </c>
       <c r="AG191" t="n">
         <v>0.9566</v>
@@ -27629,7 +27629,7 @@
         <v>12</v>
       </c>
       <c r="AF195" t="n">
-        <v>0.361</v>
+        <v>0.3609</v>
       </c>
       <c r="AG195" t="n">
         <v>1</v>
@@ -28058,7 +28058,7 @@
         <v>12</v>
       </c>
       <c r="AF198" t="n">
-        <v>0.356</v>
+        <v>0.3561</v>
       </c>
       <c r="AG198" t="n">
         <v>1</v>
@@ -32355,7 +32355,7 @@
         <v>13</v>
       </c>
       <c r="AF229" t="n">
-        <v>0.1746</v>
+        <v>0.1747</v>
       </c>
       <c r="AG229" t="n">
         <v>0.9628</v>

</xml_diff>

<commit_message>
Play-test 13 (lane B): FPV carrier redrawn as a protected drone truck
Bonneted 6x6, launch station with open lids and armed quadcopters, relay mast, EW;
7452 tris, soft 99.7. DECISIONS + CHANGELOG for lane B models.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/models/quality_report.xlsx
+++ b/Docs/models/quality_report.xlsx
@@ -6463,10 +6463,8 @@
           <t>ballistic_launcher</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>7454</t>
-        </is>
+      <c r="E31" t="n">
+        <v>7454</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -6474,10 +6472,8 @@
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>81.5</t>
-        </is>
+      <c r="H31" t="n">
+        <v>81.5</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -6496,150 +6492,94 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>0.107</t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>0.084</t>
-        </is>
+      <c r="N31" t="n">
+        <v>0.107</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0.08500000000000001</v>
       </c>
       <c r="P31" t="inlineStr">
         <is>
           <t>long_sam</t>
         </is>
       </c>
-      <c r="Q31" t="inlineStr">
-        <is>
-          <t>1.3156</t>
-        </is>
-      </c>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>0.405</t>
-        </is>
-      </c>
-      <c r="S31" t="inlineStr">
-        <is>
-          <t>11.3406</t>
-        </is>
-      </c>
-      <c r="T31" t="inlineStr">
-        <is>
-          <t>0.0309</t>
-        </is>
-      </c>
-      <c r="U31" t="inlineStr">
-        <is>
-          <t>226</t>
-        </is>
-      </c>
-      <c r="V31" t="inlineStr">
-        <is>
-          <t>79</t>
-        </is>
-      </c>
-      <c r="W31" t="inlineStr">
-        <is>
-          <t>0.6075</t>
-        </is>
-      </c>
-      <c r="X31" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="Y31" t="inlineStr">
-        <is>
-          <t>121</t>
-        </is>
-      </c>
-      <c r="Z31" t="inlineStr">
-        <is>
-          <t>89</t>
-        </is>
-      </c>
-      <c r="AA31" t="inlineStr">
-        <is>
-          <t>0.9305</t>
-        </is>
-      </c>
-      <c r="AB31" t="inlineStr">
-        <is>
-          <t>0.6845</t>
-        </is>
-      </c>
-      <c r="AC31" t="inlineStr">
-        <is>
-          <t>130.0313</t>
-        </is>
-      </c>
-      <c r="AD31" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="AE31" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="AF31" t="inlineStr">
-        <is>
-          <t>0.1674</t>
-        </is>
-      </c>
-      <c r="AG31" t="inlineStr">
-        <is>
-          <t>0.9381</t>
-        </is>
-      </c>
-      <c r="AH31" t="inlineStr">
-        <is>
-          <t>0.0656</t>
-        </is>
-      </c>
-      <c r="AI31" t="inlineStr">
-        <is>
-          <t>0.0596</t>
-        </is>
-      </c>
-      <c r="AJ31" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AK31" t="inlineStr">
-        <is>
-          <t>0.446</t>
-        </is>
-      </c>
-      <c r="AL31" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AM31" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AN31" t="inlineStr">
-        <is>
-          <t>0.901</t>
-        </is>
-      </c>
-      <c r="AO31" t="inlineStr">
-        <is>
-          <t>0.821</t>
-        </is>
-      </c>
-      <c r="AP31" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="Q31" t="n">
+        <v>1.3156</v>
+      </c>
+      <c r="R31" t="n">
+        <v>0.405</v>
+      </c>
+      <c r="S31" t="n">
+        <v>11.3406</v>
+      </c>
+      <c r="T31" t="n">
+        <v>0.0309</v>
+      </c>
+      <c r="U31" t="n">
+        <v>226</v>
+      </c>
+      <c r="V31" t="n">
+        <v>79</v>
+      </c>
+      <c r="W31" t="n">
+        <v>0.6075</v>
+      </c>
+      <c r="X31" t="n">
+        <v>16</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>121</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>89</v>
+      </c>
+      <c r="AA31" t="n">
+        <v>0.9305</v>
+      </c>
+      <c r="AB31" t="n">
+        <v>0.6845</v>
+      </c>
+      <c r="AC31" t="n">
+        <v>130.0313</v>
+      </c>
+      <c r="AD31" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>11</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>0.1674</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>0.9381</v>
+      </c>
+      <c r="AH31" t="n">
+        <v>0.06560000000000001</v>
+      </c>
+      <c r="AI31" t="n">
+        <v>0.0596</v>
+      </c>
+      <c r="AJ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK31" t="n">
+        <v>0.446</v>
+      </c>
+      <c r="AL31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN31" t="n">
+        <v>0.901</v>
+      </c>
+      <c r="AO31" t="n">
+        <v>0.821</v>
+      </c>
+      <c r="AP31" t="n">
+        <v>1</v>
       </c>
       <c r="AQ31" t="inlineStr"/>
     </row>
@@ -16827,10 +16767,8 @@
           <t>fibre_fpv_carrier</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>6364</t>
-        </is>
+      <c r="E83" t="n">
+        <v>6364</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
@@ -16838,10 +16776,8 @@
         </is>
       </c>
       <c r="G83" t="inlineStr"/>
-      <c r="H83" t="inlineStr">
-        <is>
-          <t>90.5</t>
-        </is>
+      <c r="H83" t="n">
+        <v>90.5</v>
       </c>
       <c r="I83" t="inlineStr">
         <is>
@@ -16860,150 +16796,94 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N83" t="inlineStr">
-        <is>
-          <t>0.14</t>
-        </is>
-      </c>
-      <c r="O83" t="inlineStr">
-        <is>
-          <t>0.066</t>
-        </is>
+      <c r="N83" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="O83" t="n">
+        <v>0.066</v>
       </c>
       <c r="P83" t="inlineStr">
         <is>
           <t>missile_boat</t>
         </is>
       </c>
-      <c r="Q83" t="inlineStr">
-        <is>
-          <t>1.7341</t>
-        </is>
-      </c>
-      <c r="R83" t="inlineStr">
-        <is>
-          <t>0.2622</t>
-        </is>
-      </c>
-      <c r="S83" t="inlineStr">
-        <is>
-          <t>10.3585</t>
-        </is>
-      </c>
-      <c r="T83" t="inlineStr">
-        <is>
-          <t>0.015</t>
-        </is>
-      </c>
-      <c r="U83" t="inlineStr">
-        <is>
-          <t>226</t>
-        </is>
-      </c>
-      <c r="V83" t="inlineStr">
-        <is>
-          <t>74</t>
-        </is>
-      </c>
-      <c r="W83" t="inlineStr">
-        <is>
-          <t>1.0259</t>
-        </is>
-      </c>
-      <c r="X83" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="Y83" t="inlineStr">
-        <is>
-          <t>78</t>
-        </is>
-      </c>
-      <c r="Z83" t="inlineStr">
-        <is>
-          <t>137</t>
-        </is>
-      </c>
-      <c r="AA83" t="inlineStr">
-        <is>
-          <t>1.0813</t>
-        </is>
-      </c>
-      <c r="AB83" t="inlineStr">
-        <is>
-          <t>1.8992</t>
-        </is>
-      </c>
-      <c r="AC83" t="inlineStr">
-        <is>
-          <t>72.1347</t>
-        </is>
-      </c>
-      <c r="AD83" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="AE83" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="AF83" t="inlineStr">
-        <is>
-          <t>0.0847</t>
-        </is>
-      </c>
-      <c r="AG83" t="inlineStr">
-        <is>
-          <t>0.8143</t>
-        </is>
-      </c>
-      <c r="AH83" t="inlineStr">
-        <is>
-          <t>0.0459</t>
-        </is>
-      </c>
-      <c r="AI83" t="inlineStr">
-        <is>
-          <t>0.3254</t>
-        </is>
-      </c>
-      <c r="AJ83" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AK83" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AL83" t="inlineStr">
-        <is>
-          <t>0.87</t>
-        </is>
-      </c>
-      <c r="AM83" t="inlineStr">
-        <is>
-          <t>0.794</t>
-        </is>
-      </c>
-      <c r="AN83" t="inlineStr">
-        <is>
-          <t>0.874</t>
-        </is>
-      </c>
-      <c r="AO83" t="inlineStr">
-        <is>
-          <t>0.868</t>
-        </is>
-      </c>
-      <c r="AP83" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="Q83" t="n">
+        <v>1.7341</v>
+      </c>
+      <c r="R83" t="n">
+        <v>0.2622</v>
+      </c>
+      <c r="S83" t="n">
+        <v>10.3585</v>
+      </c>
+      <c r="T83" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="U83" t="n">
+        <v>226</v>
+      </c>
+      <c r="V83" t="n">
+        <v>74</v>
+      </c>
+      <c r="W83" t="n">
+        <v>1.0259</v>
+      </c>
+      <c r="X83" t="n">
+        <v>11</v>
+      </c>
+      <c r="Y83" t="n">
+        <v>78</v>
+      </c>
+      <c r="Z83" t="n">
+        <v>137</v>
+      </c>
+      <c r="AA83" t="n">
+        <v>1.0813</v>
+      </c>
+      <c r="AB83" t="n">
+        <v>1.8992</v>
+      </c>
+      <c r="AC83" t="n">
+        <v>72.1347</v>
+      </c>
+      <c r="AD83" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE83" t="n">
+        <v>12</v>
+      </c>
+      <c r="AF83" t="n">
+        <v>0.0847</v>
+      </c>
+      <c r="AG83" t="n">
+        <v>0.8143</v>
+      </c>
+      <c r="AH83" t="n">
+        <v>0.0459</v>
+      </c>
+      <c r="AI83" t="n">
+        <v>0.3254</v>
+      </c>
+      <c r="AJ83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK83" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL83" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="AM83" t="n">
+        <v>0.794</v>
+      </c>
+      <c r="AN83" t="n">
+        <v>0.874</v>
+      </c>
+      <c r="AO83" t="n">
+        <v>0.868</v>
+      </c>
+      <c r="AP83" t="n">
+        <v>1</v>
       </c>
       <c r="AQ83" t="inlineStr"/>
     </row>
@@ -18427,10 +18307,8 @@
           <t>fpv_carrier</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>7310</t>
-        </is>
+      <c r="E91" t="n">
+        <v>7452</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -18438,19 +18316,17 @@
         </is>
       </c>
       <c r="G91" t="inlineStr"/>
-      <c r="H91" t="inlineStr">
-        <is>
-          <t>76.4</t>
-        </is>
+      <c r="H91" t="n">
+        <v>99.7</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>Cần sửa</t>
+          <t>Tốt</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K91" t="inlineStr"/>
@@ -18460,150 +18336,94 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N91" t="inlineStr">
-        <is>
-          <t>0.102</t>
-        </is>
-      </c>
-      <c r="O91" t="inlineStr">
-        <is>
-          <t>0.099</t>
-        </is>
+      <c r="N91" t="n">
+        <v>0.122</v>
+      </c>
+      <c r="O91" t="n">
+        <v>0.064</v>
       </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t>nlos_atgm_vehicle</t>
-        </is>
-      </c>
-      <c r="Q91" t="inlineStr">
-        <is>
-          <t>1.4669</t>
-        </is>
-      </c>
-      <c r="R91" t="inlineStr">
-        <is>
-          <t>0.1982</t>
-        </is>
-      </c>
-      <c r="S91" t="inlineStr">
-        <is>
-          <t>5.2146</t>
-        </is>
-      </c>
-      <c r="T91" t="inlineStr">
-        <is>
-          <t>0.0866</t>
-        </is>
-      </c>
-      <c r="U91" t="inlineStr">
-        <is>
-          <t>331</t>
-        </is>
-      </c>
-      <c r="V91" t="inlineStr">
-        <is>
-          <t>73</t>
-        </is>
-      </c>
-      <c r="W91" t="inlineStr">
-        <is>
-          <t>0.5266</t>
-        </is>
-      </c>
-      <c r="X91" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="Y91" t="inlineStr">
-        <is>
-          <t>108</t>
-        </is>
-      </c>
-      <c r="Z91" t="inlineStr">
-        <is>
-          <t>217</t>
-        </is>
-      </c>
-      <c r="AA91" t="inlineStr">
-        <is>
-          <t>0.7791</t>
-        </is>
-      </c>
-      <c r="AB91" t="inlineStr">
-        <is>
-          <t>1.5655</t>
-        </is>
-      </c>
-      <c r="AC91" t="inlineStr">
-        <is>
-          <t>138.6153</t>
-        </is>
-      </c>
-      <c r="AD91" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="AE91" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="AF91" t="inlineStr">
-        <is>
-          <t>0.0963</t>
-        </is>
-      </c>
-      <c r="AG91" t="inlineStr">
-        <is>
-          <t>0.8137</t>
-        </is>
-      </c>
-      <c r="AH91" t="inlineStr">
-        <is>
-          <t>0.0445</t>
-        </is>
-      </c>
-      <c r="AI91" t="inlineStr">
-        <is>
-          <t>0.2097</t>
-        </is>
-      </c>
-      <c r="AJ91" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AK91" t="inlineStr">
-        <is>
-          <t>0.66</t>
-        </is>
-      </c>
-      <c r="AL91" t="inlineStr">
-        <is>
-          <t>0.828</t>
-        </is>
-      </c>
-      <c r="AM91" t="inlineStr">
-        <is>
-          <t>0.627</t>
-        </is>
-      </c>
-      <c r="AN91" t="inlineStr">
-        <is>
-          <t>0.781</t>
-        </is>
-      </c>
-      <c r="AO91" t="inlineStr">
-        <is>
-          <t>0.831</t>
-        </is>
-      </c>
-      <c r="AP91" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+          <t>shahed_truck</t>
+        </is>
+      </c>
+      <c r="Q91" t="n">
+        <v>1.7823</v>
+      </c>
+      <c r="R91" t="n">
+        <v>0.3323</v>
+      </c>
+      <c r="S91" t="n">
+        <v>12.8724</v>
+      </c>
+      <c r="T91" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="U91" t="n">
+        <v>301</v>
+      </c>
+      <c r="V91" t="n">
+        <v>124</v>
+      </c>
+      <c r="W91" t="n">
+        <v>0.9233</v>
+      </c>
+      <c r="X91" t="n">
+        <v>17</v>
+      </c>
+      <c r="Y91" t="n">
+        <v>151</v>
+      </c>
+      <c r="Z91" t="n">
+        <v>133</v>
+      </c>
+      <c r="AA91" t="n">
+        <v>1.1244</v>
+      </c>
+      <c r="AB91" t="n">
+        <v>0.9903</v>
+      </c>
+      <c r="AC91" t="n">
+        <v>134.2973</v>
+      </c>
+      <c r="AD91" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE91" t="n">
+        <v>11</v>
+      </c>
+      <c r="AF91" t="n">
+        <v>0.1354</v>
+      </c>
+      <c r="AG91" t="n">
+        <v>0.8305</v>
+      </c>
+      <c r="AH91" t="n">
+        <v>0.0504</v>
+      </c>
+      <c r="AI91" t="n">
+        <v>0.1935</v>
+      </c>
+      <c r="AJ91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK91" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL91" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM91" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN91" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO91" t="n">
+        <v>0.977</v>
+      </c>
+      <c r="AP91" t="n">
+        <v>1</v>
       </c>
       <c r="AQ91" t="inlineStr"/>
     </row>
@@ -19446,10 +19266,10 @@
         </is>
       </c>
       <c r="N96" t="n">
-        <v>0.15</v>
+        <v>0.154</v>
       </c>
       <c r="O96" t="n">
-        <v>0.149</v>
+        <v>0.147</v>
       </c>
       <c r="P96" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Play-test 13 follow-up (lane B): Inferno 125 mm thermobaric gun turret
The glacis TOS rocket box (Mount_rocket) is now a small cast casemate turret with a
short heavy 125 mm barrel and Muzzle_rocket at its mouth; the thermo part wrecks as a turret.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/models/quality_report.xlsx
+++ b/Docs/models/quality_report.xlsx
@@ -6463,8 +6463,10 @@
           <t>ballistic_launcher</t>
         </is>
       </c>
-      <c r="E31" t="n">
-        <v>7454</v>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>7454</t>
+        </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -6472,8 +6474,10 @@
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" t="n">
-        <v>81.5</v>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>81.5</t>
+        </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -6492,94 +6496,150 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N31" t="n">
-        <v>0.107</v>
-      </c>
-      <c r="O31" t="n">
-        <v>0.08500000000000001</v>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>0.107</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>0.085</t>
+        </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
           <t>long_sam</t>
         </is>
       </c>
-      <c r="Q31" t="n">
-        <v>1.3156</v>
-      </c>
-      <c r="R31" t="n">
-        <v>0.405</v>
-      </c>
-      <c r="S31" t="n">
-        <v>11.3406</v>
-      </c>
-      <c r="T31" t="n">
-        <v>0.0309</v>
-      </c>
-      <c r="U31" t="n">
-        <v>226</v>
-      </c>
-      <c r="V31" t="n">
-        <v>79</v>
-      </c>
-      <c r="W31" t="n">
-        <v>0.6075</v>
-      </c>
-      <c r="X31" t="n">
-        <v>16</v>
-      </c>
-      <c r="Y31" t="n">
-        <v>121</v>
-      </c>
-      <c r="Z31" t="n">
-        <v>89</v>
-      </c>
-      <c r="AA31" t="n">
-        <v>0.9305</v>
-      </c>
-      <c r="AB31" t="n">
-        <v>0.6845</v>
-      </c>
-      <c r="AC31" t="n">
-        <v>130.0313</v>
-      </c>
-      <c r="AD31" t="n">
-        <v>4</v>
-      </c>
-      <c r="AE31" t="n">
-        <v>11</v>
-      </c>
-      <c r="AF31" t="n">
-        <v>0.1674</v>
-      </c>
-      <c r="AG31" t="n">
-        <v>0.9381</v>
-      </c>
-      <c r="AH31" t="n">
-        <v>0.06560000000000001</v>
-      </c>
-      <c r="AI31" t="n">
-        <v>0.0596</v>
-      </c>
-      <c r="AJ31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK31" t="n">
-        <v>0.446</v>
-      </c>
-      <c r="AL31" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM31" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN31" t="n">
-        <v>0.901</v>
-      </c>
-      <c r="AO31" t="n">
-        <v>0.821</v>
-      </c>
-      <c r="AP31" t="n">
-        <v>1</v>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>1.3156</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>0.405</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>11.3406</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>0.0309</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>226</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>0.6075</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>121</t>
+        </is>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>0.9305</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>0.6845</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>130.0313</t>
+        </is>
+      </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE31" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="AF31" t="inlineStr">
+        <is>
+          <t>0.1674</t>
+        </is>
+      </c>
+      <c r="AG31" t="inlineStr">
+        <is>
+          <t>0.9381</t>
+        </is>
+      </c>
+      <c r="AH31" t="inlineStr">
+        <is>
+          <t>0.0656</t>
+        </is>
+      </c>
+      <c r="AI31" t="inlineStr">
+        <is>
+          <t>0.0596</t>
+        </is>
+      </c>
+      <c r="AJ31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK31" t="inlineStr">
+        <is>
+          <t>0.446</t>
+        </is>
+      </c>
+      <c r="AL31" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AM31" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN31" t="inlineStr">
+        <is>
+          <t>0.901</t>
+        </is>
+      </c>
+      <c r="AO31" t="inlineStr">
+        <is>
+          <t>0.821</t>
+        </is>
+      </c>
+      <c r="AP31" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
       <c r="AQ31" t="inlineStr"/>
     </row>
@@ -7002,10 +7062,8 @@
           <t>behemoth_inferno</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>23648</t>
-        </is>
+      <c r="E34" t="n">
+        <v>25710</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -7013,10 +7071,8 @@
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>84.3</t>
-        </is>
+      <c r="H34" t="n">
+        <v>86.3</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -7035,146 +7091,90 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>0.029</t>
-        </is>
-      </c>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t>0.042</t>
-        </is>
+      <c r="N34" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="O34" t="n">
+        <v>0.07199999999999999</v>
       </c>
       <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>1.5796</t>
-        </is>
-      </c>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>0.2017</t>
-        </is>
-      </c>
-      <c r="S34" t="inlineStr">
-        <is>
-          <t>6.0238</t>
-        </is>
-      </c>
-      <c r="T34" t="inlineStr">
-        <is>
-          <t>0.0014</t>
-        </is>
-      </c>
-      <c r="U34" t="inlineStr">
-        <is>
-          <t>557</t>
-        </is>
-      </c>
-      <c r="V34" t="inlineStr">
-        <is>
-          <t>94</t>
-        </is>
-      </c>
-      <c r="W34" t="inlineStr">
-        <is>
-          <t>0.5399</t>
-        </is>
-      </c>
-      <c r="X34" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="Y34" t="inlineStr">
-        <is>
-          <t>133</t>
-        </is>
-      </c>
-      <c r="Z34" t="inlineStr">
-        <is>
-          <t>403</t>
-        </is>
-      </c>
-      <c r="AA34" t="inlineStr">
-        <is>
-          <t>0.7638</t>
-        </is>
-      </c>
-      <c r="AB34" t="inlineStr">
-        <is>
-          <t>2.3145</t>
-        </is>
-      </c>
-      <c r="AC34" t="inlineStr">
-        <is>
-          <t>174.1199</t>
-        </is>
-      </c>
-      <c r="AD34" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="AE34" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="AF34" t="inlineStr">
-        <is>
-          <t>0.1029</t>
-        </is>
-      </c>
-      <c r="AG34" t="inlineStr">
-        <is>
-          <t>0.8064</t>
-        </is>
-      </c>
-      <c r="AH34" t="inlineStr">
-        <is>
-          <t>0.0383</t>
-        </is>
-      </c>
-      <c r="AI34" t="inlineStr">
-        <is>
-          <t>0.3075</t>
-        </is>
-      </c>
-      <c r="AJ34" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AK34" t="inlineStr">
-        <is>
-          <t>0.729</t>
-        </is>
-      </c>
-      <c r="AL34" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AM34" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AN34" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AO34" t="inlineStr">
-        <is>
-          <t>0.741</t>
-        </is>
-      </c>
-      <c r="AP34" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="Q34" t="n">
+        <v>1.6315</v>
+      </c>
+      <c r="R34" t="n">
+        <v>0.2035</v>
+      </c>
+      <c r="S34" t="n">
+        <v>6.2328</v>
+      </c>
+      <c r="T34" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="U34" t="n">
+        <v>564</v>
+      </c>
+      <c r="V34" t="n">
+        <v>116</v>
+      </c>
+      <c r="W34" t="n">
+        <v>0.6538</v>
+      </c>
+      <c r="X34" t="n">
+        <v>21</v>
+      </c>
+      <c r="Y34" t="n">
+        <v>148</v>
+      </c>
+      <c r="Z34" t="n">
+        <v>395</v>
+      </c>
+      <c r="AA34" t="n">
+        <v>0.8342000000000001</v>
+      </c>
+      <c r="AB34" t="n">
+        <v>2.2263</v>
+      </c>
+      <c r="AC34" t="n">
+        <v>177.4261</v>
+      </c>
+      <c r="AD34" t="n">
+        <v>21</v>
+      </c>
+      <c r="AE34" t="n">
+        <v>14</v>
+      </c>
+      <c r="AF34" t="n">
+        <v>0.1031</v>
+      </c>
+      <c r="AG34" t="n">
+        <v>0.8143</v>
+      </c>
+      <c r="AH34" t="n">
+        <v>0.0452</v>
+      </c>
+      <c r="AI34" t="n">
+        <v>0.2847</v>
+      </c>
+      <c r="AJ34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK34" t="n">
+        <v>0.794</v>
+      </c>
+      <c r="AL34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO34" t="n">
+        <v>0.764</v>
+      </c>
+      <c r="AP34" t="n">
+        <v>0.5</v>
       </c>
       <c r="AQ34" t="inlineStr"/>
     </row>
@@ -16767,8 +16767,10 @@
           <t>fibre_fpv_carrier</t>
         </is>
       </c>
-      <c r="E83" t="n">
-        <v>6364</v>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>6364</t>
+        </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
@@ -16776,8 +16778,10 @@
         </is>
       </c>
       <c r="G83" t="inlineStr"/>
-      <c r="H83" t="n">
-        <v>90.5</v>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>90.5</t>
+        </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
@@ -16796,94 +16800,150 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N83" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="O83" t="n">
-        <v>0.066</v>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>0.11</t>
+        </is>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>0.066</t>
+        </is>
       </c>
       <c r="P83" t="inlineStr">
         <is>
           <t>missile_boat</t>
         </is>
       </c>
-      <c r="Q83" t="n">
-        <v>1.7341</v>
-      </c>
-      <c r="R83" t="n">
-        <v>0.2622</v>
-      </c>
-      <c r="S83" t="n">
-        <v>10.3585</v>
-      </c>
-      <c r="T83" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="U83" t="n">
-        <v>226</v>
-      </c>
-      <c r="V83" t="n">
-        <v>74</v>
-      </c>
-      <c r="W83" t="n">
-        <v>1.0259</v>
-      </c>
-      <c r="X83" t="n">
-        <v>11</v>
-      </c>
-      <c r="Y83" t="n">
-        <v>78</v>
-      </c>
-      <c r="Z83" t="n">
-        <v>137</v>
-      </c>
-      <c r="AA83" t="n">
-        <v>1.0813</v>
-      </c>
-      <c r="AB83" t="n">
-        <v>1.8992</v>
-      </c>
-      <c r="AC83" t="n">
-        <v>72.1347</v>
-      </c>
-      <c r="AD83" t="n">
-        <v>4</v>
-      </c>
-      <c r="AE83" t="n">
-        <v>12</v>
-      </c>
-      <c r="AF83" t="n">
-        <v>0.0847</v>
-      </c>
-      <c r="AG83" t="n">
-        <v>0.8143</v>
-      </c>
-      <c r="AH83" t="n">
-        <v>0.0459</v>
-      </c>
-      <c r="AI83" t="n">
-        <v>0.3254</v>
-      </c>
-      <c r="AJ83" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK83" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL83" t="n">
-        <v>0.87</v>
-      </c>
-      <c r="AM83" t="n">
-        <v>0.794</v>
-      </c>
-      <c r="AN83" t="n">
-        <v>0.874</v>
-      </c>
-      <c r="AO83" t="n">
-        <v>0.868</v>
-      </c>
-      <c r="AP83" t="n">
-        <v>1</v>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>1.7341</t>
+        </is>
+      </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>0.2622</t>
+        </is>
+      </c>
+      <c r="S83" t="inlineStr">
+        <is>
+          <t>10.3585</t>
+        </is>
+      </c>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>0.015</t>
+        </is>
+      </c>
+      <c r="U83" t="inlineStr">
+        <is>
+          <t>226</t>
+        </is>
+      </c>
+      <c r="V83" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="W83" t="inlineStr">
+        <is>
+          <t>1.0259</t>
+        </is>
+      </c>
+      <c r="X83" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="Y83" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="Z83" t="inlineStr">
+        <is>
+          <t>137</t>
+        </is>
+      </c>
+      <c r="AA83" t="inlineStr">
+        <is>
+          <t>1.0813</t>
+        </is>
+      </c>
+      <c r="AB83" t="inlineStr">
+        <is>
+          <t>1.8992</t>
+        </is>
+      </c>
+      <c r="AC83" t="inlineStr">
+        <is>
+          <t>72.1347</t>
+        </is>
+      </c>
+      <c r="AD83" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE83" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="AF83" t="inlineStr">
+        <is>
+          <t>0.0847</t>
+        </is>
+      </c>
+      <c r="AG83" t="inlineStr">
+        <is>
+          <t>0.8143</t>
+        </is>
+      </c>
+      <c r="AH83" t="inlineStr">
+        <is>
+          <t>0.0459</t>
+        </is>
+      </c>
+      <c r="AI83" t="inlineStr">
+        <is>
+          <t>0.3254</t>
+        </is>
+      </c>
+      <c r="AJ83" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK83" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AL83" t="inlineStr">
+        <is>
+          <t>0.87</t>
+        </is>
+      </c>
+      <c r="AM83" t="inlineStr">
+        <is>
+          <t>0.794</t>
+        </is>
+      </c>
+      <c r="AN83" t="inlineStr">
+        <is>
+          <t>0.874</t>
+        </is>
+      </c>
+      <c r="AO83" t="inlineStr">
+        <is>
+          <t>0.868</t>
+        </is>
+      </c>
+      <c r="AP83" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
       <c r="AQ83" t="inlineStr"/>
     </row>
@@ -18307,8 +18367,10 @@
           <t>fpv_carrier</t>
         </is>
       </c>
-      <c r="E91" t="n">
-        <v>7452</v>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>7452</t>
+        </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -18316,8 +18378,10 @@
         </is>
       </c>
       <c r="G91" t="inlineStr"/>
-      <c r="H91" t="n">
-        <v>99.7</v>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>99.7</t>
+        </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
@@ -18336,94 +18400,150 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N91" t="n">
-        <v>0.122</v>
-      </c>
-      <c r="O91" t="n">
-        <v>0.064</v>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>0.122</t>
+        </is>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>0.064</t>
+        </is>
       </c>
       <c r="P91" t="inlineStr">
         <is>
           <t>shahed_truck</t>
         </is>
       </c>
-      <c r="Q91" t="n">
-        <v>1.7823</v>
-      </c>
-      <c r="R91" t="n">
-        <v>0.3323</v>
-      </c>
-      <c r="S91" t="n">
-        <v>12.8724</v>
-      </c>
-      <c r="T91" t="n">
-        <v>0.031</v>
-      </c>
-      <c r="U91" t="n">
-        <v>301</v>
-      </c>
-      <c r="V91" t="n">
-        <v>124</v>
-      </c>
-      <c r="W91" t="n">
-        <v>0.9233</v>
-      </c>
-      <c r="X91" t="n">
-        <v>17</v>
-      </c>
-      <c r="Y91" t="n">
-        <v>151</v>
-      </c>
-      <c r="Z91" t="n">
-        <v>133</v>
-      </c>
-      <c r="AA91" t="n">
-        <v>1.1244</v>
-      </c>
-      <c r="AB91" t="n">
-        <v>0.9903</v>
-      </c>
-      <c r="AC91" t="n">
-        <v>134.2973</v>
-      </c>
-      <c r="AD91" t="n">
-        <v>4</v>
-      </c>
-      <c r="AE91" t="n">
-        <v>11</v>
-      </c>
-      <c r="AF91" t="n">
-        <v>0.1354</v>
-      </c>
-      <c r="AG91" t="n">
-        <v>0.8305</v>
-      </c>
-      <c r="AH91" t="n">
-        <v>0.0504</v>
-      </c>
-      <c r="AI91" t="n">
-        <v>0.1935</v>
-      </c>
-      <c r="AJ91" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK91" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL91" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM91" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN91" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO91" t="n">
-        <v>0.977</v>
-      </c>
-      <c r="AP91" t="n">
-        <v>1</v>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>1.7823</t>
+        </is>
+      </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>0.3323</t>
+        </is>
+      </c>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t>12.8724</t>
+        </is>
+      </c>
+      <c r="T91" t="inlineStr">
+        <is>
+          <t>0.031</t>
+        </is>
+      </c>
+      <c r="U91" t="inlineStr">
+        <is>
+          <t>301</t>
+        </is>
+      </c>
+      <c r="V91" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
+      </c>
+      <c r="W91" t="inlineStr">
+        <is>
+          <t>0.9233</t>
+        </is>
+      </c>
+      <c r="X91" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="Y91" t="inlineStr">
+        <is>
+          <t>151</t>
+        </is>
+      </c>
+      <c r="Z91" t="inlineStr">
+        <is>
+          <t>133</t>
+        </is>
+      </c>
+      <c r="AA91" t="inlineStr">
+        <is>
+          <t>1.1244</t>
+        </is>
+      </c>
+      <c r="AB91" t="inlineStr">
+        <is>
+          <t>0.9903</t>
+        </is>
+      </c>
+      <c r="AC91" t="inlineStr">
+        <is>
+          <t>134.2973</t>
+        </is>
+      </c>
+      <c r="AD91" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE91" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="AF91" t="inlineStr">
+        <is>
+          <t>0.1354</t>
+        </is>
+      </c>
+      <c r="AG91" t="inlineStr">
+        <is>
+          <t>0.8305</t>
+        </is>
+      </c>
+      <c r="AH91" t="inlineStr">
+        <is>
+          <t>0.0504</t>
+        </is>
+      </c>
+      <c r="AI91" t="inlineStr">
+        <is>
+          <t>0.1935</t>
+        </is>
+      </c>
+      <c r="AJ91" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK91" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AL91" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AM91" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN91" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO91" t="inlineStr">
+        <is>
+          <t>0.977</t>
+        </is>
+      </c>
+      <c r="AP91" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
       <c r="AQ91" t="inlineStr"/>
     </row>
@@ -19236,8 +19356,10 @@
           <t>ground_cruise_missile_vehicle</t>
         </is>
       </c>
-      <c r="E96" t="n">
-        <v>5726</v>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>5726</t>
+        </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
@@ -19245,8 +19367,10 @@
         </is>
       </c>
       <c r="G96" t="inlineStr"/>
-      <c r="H96" t="n">
-        <v>88.09999999999999</v>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>88.1</t>
+        </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
@@ -19265,94 +19389,150 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N96" t="n">
-        <v>0.154</v>
-      </c>
-      <c r="O96" t="n">
-        <v>0.147</v>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>0.154</t>
+        </is>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>0.147</t>
+        </is>
       </c>
       <c r="P96" t="inlineStr">
         <is>
           <t>heavy_rocket_artillery</t>
         </is>
       </c>
-      <c r="Q96" t="n">
-        <v>1.6344</v>
-      </c>
-      <c r="R96" t="n">
-        <v>0.226</v>
-      </c>
-      <c r="S96" t="n">
-        <v>8.8756</v>
-      </c>
-      <c r="T96" t="n">
-        <v>0.0503</v>
-      </c>
-      <c r="U96" t="n">
-        <v>190</v>
-      </c>
-      <c r="V96" t="n">
-        <v>84</v>
-      </c>
-      <c r="W96" t="n">
-        <v>0.5851</v>
-      </c>
-      <c r="X96" t="n">
-        <v>13</v>
-      </c>
-      <c r="Y96" t="n">
-        <v>115</v>
-      </c>
-      <c r="Z96" t="n">
-        <v>62</v>
-      </c>
-      <c r="AA96" t="n">
-        <v>0.8011</v>
-      </c>
-      <c r="AB96" t="n">
-        <v>0.4319</v>
-      </c>
-      <c r="AC96" t="n">
-        <v>143.5559</v>
-      </c>
-      <c r="AD96" t="n">
-        <v>4</v>
-      </c>
-      <c r="AE96" t="n">
-        <v>10</v>
-      </c>
-      <c r="AF96" t="n">
-        <v>0.195</v>
-      </c>
-      <c r="AG96" t="n">
-        <v>0.9473</v>
-      </c>
-      <c r="AH96" t="n">
-        <v>0.0747</v>
-      </c>
-      <c r="AI96" t="n">
-        <v>0.1334</v>
-      </c>
-      <c r="AJ96" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK96" t="n">
-        <v>0.897</v>
-      </c>
-      <c r="AL96" t="n">
-        <v>0.944</v>
-      </c>
-      <c r="AM96" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN96" t="n">
-        <v>0.868</v>
-      </c>
-      <c r="AO96" t="n">
-        <v>0.609</v>
-      </c>
-      <c r="AP96" t="n">
-        <v>1</v>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>1.6344</t>
+        </is>
+      </c>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>0.226</t>
+        </is>
+      </c>
+      <c r="S96" t="inlineStr">
+        <is>
+          <t>8.8756</t>
+        </is>
+      </c>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t>0.0503</t>
+        </is>
+      </c>
+      <c r="U96" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+      <c r="V96" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="W96" t="inlineStr">
+        <is>
+          <t>0.5851</t>
+        </is>
+      </c>
+      <c r="X96" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="Y96" t="inlineStr">
+        <is>
+          <t>115</t>
+        </is>
+      </c>
+      <c r="Z96" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="AA96" t="inlineStr">
+        <is>
+          <t>0.8011</t>
+        </is>
+      </c>
+      <c r="AB96" t="inlineStr">
+        <is>
+          <t>0.4319</t>
+        </is>
+      </c>
+      <c r="AC96" t="inlineStr">
+        <is>
+          <t>143.5559</t>
+        </is>
+      </c>
+      <c r="AD96" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE96" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AF96" t="inlineStr">
+        <is>
+          <t>0.195</t>
+        </is>
+      </c>
+      <c r="AG96" t="inlineStr">
+        <is>
+          <t>0.9473</t>
+        </is>
+      </c>
+      <c r="AH96" t="inlineStr">
+        <is>
+          <t>0.0747</t>
+        </is>
+      </c>
+      <c r="AI96" t="inlineStr">
+        <is>
+          <t>0.1334</t>
+        </is>
+      </c>
+      <c r="AJ96" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK96" t="inlineStr">
+        <is>
+          <t>0.897</t>
+        </is>
+      </c>
+      <c r="AL96" t="inlineStr">
+        <is>
+          <t>0.944</t>
+        </is>
+      </c>
+      <c r="AM96" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN96" t="inlineStr">
+        <is>
+          <t>0.868</t>
+        </is>
+      </c>
+      <c r="AO96" t="inlineStr">
+        <is>
+          <t>0.609</t>
+        </is>
+      </c>
+      <c r="AP96" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
       <c r="AQ96" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Play-test 13 follow-up (lane B): Behemoth hull-gun shells leave the gun
Mount 6 (now 120 mm shells) is the third missile-slot mount: Muzzle_missile.002 at the
hull gun's second barrel; adds the mb_pt13_followup wrapper (registered last).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/models/quality_report.xlsx
+++ b/Docs/models/quality_report.xlsx
@@ -6865,10 +6865,8 @@
           <t>behemoth mara_behemoth behemoth_mk0</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>25692</t>
-        </is>
+      <c r="E33" t="n">
+        <v>25692</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -6876,10 +6874,8 @@
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>93.2</t>
-        </is>
+      <c r="H33" t="n">
+        <v>93.2</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -6898,146 +6894,90 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>0.023</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>0.03</t>
-        </is>
+      <c r="N33" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="O33" t="n">
+        <v>0.03</v>
       </c>
       <c r="P33" t="inlineStr"/>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>1.8859</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>0.1963</t>
-        </is>
-      </c>
-      <c r="S33" t="inlineStr">
-        <is>
-          <t>5.8834</t>
-        </is>
-      </c>
-      <c r="T33" t="inlineStr">
-        <is>
-          <t>0.0316</t>
-        </is>
-      </c>
-      <c r="U33" t="inlineStr">
-        <is>
-          <t>707</t>
-        </is>
-      </c>
-      <c r="V33" t="inlineStr">
-        <is>
-          <t>120</t>
-        </is>
-      </c>
-      <c r="W33" t="inlineStr">
-        <is>
-          <t>0.4386</t>
-        </is>
-      </c>
-      <c r="X33" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="Y33" t="inlineStr">
-        <is>
-          <t>354</t>
-        </is>
-      </c>
-      <c r="Z33" t="inlineStr">
-        <is>
-          <t>333</t>
-        </is>
-      </c>
-      <c r="AA33" t="inlineStr">
-        <is>
-          <t>1.2938</t>
-        </is>
-      </c>
-      <c r="AB33" t="inlineStr">
-        <is>
-          <t>1.2171</t>
-        </is>
-      </c>
-      <c r="AC33" t="inlineStr">
-        <is>
-          <t>273.6087</t>
-        </is>
-      </c>
-      <c r="AD33" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="AE33" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="AF33" t="inlineStr">
-        <is>
-          <t>0.2702</t>
-        </is>
-      </c>
-      <c r="AG33" t="inlineStr">
-        <is>
-          <t>0.9041</t>
-        </is>
-      </c>
-      <c r="AH33" t="inlineStr">
-        <is>
-          <t>0.062</t>
-        </is>
-      </c>
-      <c r="AI33" t="inlineStr">
-        <is>
-          <t>0.1884</t>
-        </is>
-      </c>
-      <c r="AJ33" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AK33" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AL33" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AM33" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AN33" t="inlineStr">
-        <is>
-          <t>0.83</t>
-        </is>
-      </c>
-      <c r="AO33" t="inlineStr">
-        <is>
-          <t>0.77</t>
-        </is>
-      </c>
-      <c r="AP33" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="Q33" t="n">
+        <v>1.8859</v>
+      </c>
+      <c r="R33" t="n">
+        <v>0.1963</v>
+      </c>
+      <c r="S33" t="n">
+        <v>5.8834</v>
+      </c>
+      <c r="T33" t="n">
+        <v>0.0316</v>
+      </c>
+      <c r="U33" t="n">
+        <v>707</v>
+      </c>
+      <c r="V33" t="n">
+        <v>120</v>
+      </c>
+      <c r="W33" t="n">
+        <v>0.4386</v>
+      </c>
+      <c r="X33" t="n">
+        <v>20</v>
+      </c>
+      <c r="Y33" t="n">
+        <v>354</v>
+      </c>
+      <c r="Z33" t="n">
+        <v>333</v>
+      </c>
+      <c r="AA33" t="n">
+        <v>1.2938</v>
+      </c>
+      <c r="AB33" t="n">
+        <v>1.2171</v>
+      </c>
+      <c r="AC33" t="n">
+        <v>273.6087</v>
+      </c>
+      <c r="AD33" t="n">
+        <v>8</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>12</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>0.2702</v>
+      </c>
+      <c r="AG33" t="n">
+        <v>0.9041</v>
+      </c>
+      <c r="AH33" t="n">
+        <v>0.062</v>
+      </c>
+      <c r="AI33" t="n">
+        <v>0.1884</v>
+      </c>
+      <c r="AJ33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN33" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="AO33" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="AP33" t="n">
+        <v>1</v>
       </c>
       <c r="AQ33" t="inlineStr"/>
     </row>
@@ -7062,8 +7002,10 @@
           <t>behemoth_inferno</t>
         </is>
       </c>
-      <c r="E34" t="n">
-        <v>25710</v>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>25710</t>
+        </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -7071,8 +7013,10 @@
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" t="n">
-        <v>86.3</v>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>86.3</t>
+        </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -7091,90 +7035,146 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N34" t="n">
-        <v>0.048</v>
-      </c>
-      <c r="O34" t="n">
-        <v>0.07199999999999999</v>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>0.048</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>0.072</t>
+        </is>
       </c>
       <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="n">
-        <v>1.6315</v>
-      </c>
-      <c r="R34" t="n">
-        <v>0.2035</v>
-      </c>
-      <c r="S34" t="n">
-        <v>6.2328</v>
-      </c>
-      <c r="T34" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="U34" t="n">
-        <v>564</v>
-      </c>
-      <c r="V34" t="n">
-        <v>116</v>
-      </c>
-      <c r="W34" t="n">
-        <v>0.6538</v>
-      </c>
-      <c r="X34" t="n">
-        <v>21</v>
-      </c>
-      <c r="Y34" t="n">
-        <v>148</v>
-      </c>
-      <c r="Z34" t="n">
-        <v>395</v>
-      </c>
-      <c r="AA34" t="n">
-        <v>0.8342000000000001</v>
-      </c>
-      <c r="AB34" t="n">
-        <v>2.2263</v>
-      </c>
-      <c r="AC34" t="n">
-        <v>177.4261</v>
-      </c>
-      <c r="AD34" t="n">
-        <v>21</v>
-      </c>
-      <c r="AE34" t="n">
-        <v>14</v>
-      </c>
-      <c r="AF34" t="n">
-        <v>0.1031</v>
-      </c>
-      <c r="AG34" t="n">
-        <v>0.8143</v>
-      </c>
-      <c r="AH34" t="n">
-        <v>0.0452</v>
-      </c>
-      <c r="AI34" t="n">
-        <v>0.2847</v>
-      </c>
-      <c r="AJ34" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK34" t="n">
-        <v>0.794</v>
-      </c>
-      <c r="AL34" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM34" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN34" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO34" t="n">
-        <v>0.764</v>
-      </c>
-      <c r="AP34" t="n">
-        <v>0.5</v>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>1.6315</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>0.2035</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>6.2328</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>0.005</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>564</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>116</t>
+        </is>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>0.6538</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>148</t>
+        </is>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>395</t>
+        </is>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>0.8342</t>
+        </is>
+      </c>
+      <c r="AB34" t="inlineStr">
+        <is>
+          <t>2.2263</t>
+        </is>
+      </c>
+      <c r="AC34" t="inlineStr">
+        <is>
+          <t>177.4261</t>
+        </is>
+      </c>
+      <c r="AD34" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="AE34" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="AF34" t="inlineStr">
+        <is>
+          <t>0.1031</t>
+        </is>
+      </c>
+      <c r="AG34" t="inlineStr">
+        <is>
+          <t>0.8143</t>
+        </is>
+      </c>
+      <c r="AH34" t="inlineStr">
+        <is>
+          <t>0.0452</t>
+        </is>
+      </c>
+      <c r="AI34" t="inlineStr">
+        <is>
+          <t>0.2847</t>
+        </is>
+      </c>
+      <c r="AJ34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK34" t="inlineStr">
+        <is>
+          <t>0.794</t>
+        </is>
+      </c>
+      <c r="AL34" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AM34" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN34" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO34" t="inlineStr">
+        <is>
+          <t>0.764</t>
+        </is>
+      </c>
+      <c r="AP34" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
       </c>
       <c r="AQ34" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Play-test 14 wave M2: train cars, Ixion weapons, Harpy wings, Daedalus
Juggernaut +3 / Nemesis +2 cars (re-centred, data length and part places), Ixion 30 mm,
Kornet x2, Grad pack (+ data weapons), Harpy stub wings with its guns and launchers, Daedalus 5x.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/models/quality_report.xlsx
+++ b/Docs/models/quality_report.xlsx
@@ -4047,10 +4047,8 @@
           <t>armored_train</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>26470</t>
-        </is>
+      <c r="E19" t="n">
+        <v>51170</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4058,10 +4056,8 @@
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>95.5</t>
-        </is>
+      <c r="H19" t="n">
+        <v>92.3</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -4080,146 +4076,90 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>0.036</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>0.044</t>
-        </is>
+      <c r="N19" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0.046</v>
       </c>
       <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>1.6263</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>0.2394</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>7.8238</t>
-        </is>
-      </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>0.0662</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>1086</t>
-        </is>
-      </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>124</t>
-        </is>
-      </c>
-      <c r="W19" t="inlineStr">
-        <is>
-          <t>2.0022</t>
-        </is>
-      </c>
-      <c r="X19" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="Y19" t="inlineStr">
-        <is>
-          <t>114</t>
-        </is>
-      </c>
-      <c r="Z19" t="inlineStr">
-        <is>
-          <t>957</t>
-        </is>
-      </c>
-      <c r="AA19" t="inlineStr">
-        <is>
-          <t>1.8407</t>
-        </is>
-      </c>
-      <c r="AB19" t="inlineStr">
-        <is>
-          <t>15.4522</t>
-        </is>
-      </c>
-      <c r="AC19" t="inlineStr">
-        <is>
-          <t>61.933</t>
-        </is>
-      </c>
-      <c r="AD19" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="AE19" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="AF19" t="inlineStr">
-        <is>
-          <t>0.2786</t>
-        </is>
-      </c>
-      <c r="AG19" t="inlineStr">
-        <is>
-          <t>0.8064</t>
-        </is>
-      </c>
-      <c r="AH19" t="inlineStr">
-        <is>
-          <t>0.0351</t>
-        </is>
-      </c>
-      <c r="AI19" t="inlineStr">
-        <is>
-          <t>0.0988</t>
-        </is>
-      </c>
-      <c r="AJ19" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AK19" t="inlineStr">
-        <is>
-          <t>0.972</t>
-        </is>
-      </c>
-      <c r="AL19" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AM19" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AN19" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AO19" t="inlineStr">
-        <is>
-          <t>0.747</t>
-        </is>
-      </c>
-      <c r="AP19" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="Q19" t="n">
+        <v>1.4469</v>
+      </c>
+      <c r="R19" t="n">
+        <v>0.2401</v>
+      </c>
+      <c r="S19" t="n">
+        <v>7.8832</v>
+      </c>
+      <c r="T19" t="n">
+        <v>0.0604</v>
+      </c>
+      <c r="U19" t="n">
+        <v>2162</v>
+      </c>
+      <c r="V19" t="n">
+        <v>179</v>
+      </c>
+      <c r="W19" t="n">
+        <v>5.472</v>
+      </c>
+      <c r="X19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>146</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>2016</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>4.4632</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>61.6293</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>32.7117</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>20</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>0.2702</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>0.8058</v>
+      </c>
+      <c r="AH19" t="n">
+        <v>0.0319</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>0.1293</v>
+      </c>
+      <c r="AJ19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK19" t="n">
+        <v>0.694</v>
+      </c>
+      <c r="AL19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP19" t="n">
+        <v>1</v>
       </c>
       <c r="AQ19" t="inlineStr"/>
     </row>
@@ -6865,8 +6805,10 @@
           <t>bastion_mk0</t>
         </is>
       </c>
-      <c r="E33" t="n">
-        <v>35481</v>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>35481</t>
+        </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -6874,8 +6816,10 @@
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
-      <c r="H33" t="n">
-        <v>100</v>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -6894,90 +6838,146 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N33" t="n">
-        <v>0.013</v>
-      </c>
-      <c r="O33" t="n">
-        <v>0.013</v>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>0.013</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>0.013</t>
+        </is>
       </c>
       <c r="P33" t="inlineStr"/>
-      <c r="Q33" t="n">
-        <v>1.7964</v>
-      </c>
-      <c r="R33" t="n">
-        <v>0.1892</v>
-      </c>
-      <c r="S33" t="n">
-        <v>5.2398</v>
-      </c>
-      <c r="T33" t="n">
-        <v>0.0255</v>
-      </c>
-      <c r="U33" t="n">
-        <v>1291</v>
-      </c>
-      <c r="V33" t="n">
-        <v>149</v>
-      </c>
-      <c r="W33" t="n">
-        <v>0.6503</v>
-      </c>
-      <c r="X33" t="n">
-        <v>25</v>
-      </c>
-      <c r="Y33" t="n">
-        <v>420</v>
-      </c>
-      <c r="Z33" t="n">
-        <v>846</v>
-      </c>
-      <c r="AA33" t="n">
-        <v>1.8331</v>
-      </c>
-      <c r="AB33" t="n">
-        <v>3.6924</v>
-      </c>
-      <c r="AC33" t="n">
-        <v>229.1202</v>
-      </c>
-      <c r="AD33" t="n">
-        <v>4</v>
-      </c>
-      <c r="AE33" t="n">
-        <v>17</v>
-      </c>
-      <c r="AF33" t="n">
-        <v>0.2307</v>
-      </c>
-      <c r="AG33" t="n">
-        <v>0.8064</v>
-      </c>
-      <c r="AH33" t="n">
-        <v>0.0348</v>
-      </c>
-      <c r="AI33" t="n">
-        <v>0.1637</v>
-      </c>
-      <c r="AJ33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK33" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL33" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM33" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN33" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO33" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP33" t="n">
-        <v>1</v>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>1.7964</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>0.1892</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>5.2398</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>0.0255</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>1291</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>149</t>
+        </is>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>0.6503</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>420</t>
+        </is>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>846</t>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>1.8331</t>
+        </is>
+      </c>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>3.6924</t>
+        </is>
+      </c>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>229.1202</t>
+        </is>
+      </c>
+      <c r="AD33" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE33" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="AF33" t="inlineStr">
+        <is>
+          <t>0.2307</t>
+        </is>
+      </c>
+      <c r="AG33" t="inlineStr">
+        <is>
+          <t>0.8064</t>
+        </is>
+      </c>
+      <c r="AH33" t="inlineStr">
+        <is>
+          <t>0.0348</t>
+        </is>
+      </c>
+      <c r="AI33" t="inlineStr">
+        <is>
+          <t>0.1637</t>
+        </is>
+      </c>
+      <c r="AJ33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK33" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AL33" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AM33" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN33" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO33" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AP33" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
       <c r="AQ33" t="inlineStr"/>
     </row>
@@ -7199,8 +7199,10 @@
           <t>behemoth_inferno</t>
         </is>
       </c>
-      <c r="E35" t="n">
-        <v>33342</v>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>33342</t>
+        </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -7208,8 +7210,10 @@
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" t="n">
-        <v>96.40000000000001</v>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>96.4</t>
+        </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -7228,90 +7232,146 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N35" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="O35" t="n">
-        <v>0.037</v>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>0.037</t>
+        </is>
       </c>
       <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="n">
-        <v>1.6967</v>
-      </c>
-      <c r="R35" t="n">
-        <v>0.181</v>
-      </c>
-      <c r="S35" t="n">
-        <v>5.1447</v>
-      </c>
-      <c r="T35" t="n">
-        <v>0.0703</v>
-      </c>
-      <c r="U35" t="n">
-        <v>965</v>
-      </c>
-      <c r="V35" t="n">
-        <v>155</v>
-      </c>
-      <c r="W35" t="n">
-        <v>0.5468</v>
-      </c>
-      <c r="X35" t="n">
-        <v>18</v>
-      </c>
-      <c r="Y35" t="n">
-        <v>419</v>
-      </c>
-      <c r="Z35" t="n">
-        <v>528</v>
-      </c>
-      <c r="AA35" t="n">
-        <v>1.4781</v>
-      </c>
-      <c r="AB35" t="n">
-        <v>1.8627</v>
-      </c>
-      <c r="AC35" t="n">
-        <v>283.4649</v>
-      </c>
-      <c r="AD35" t="n">
-        <v>8</v>
-      </c>
-      <c r="AE35" t="n">
-        <v>16</v>
-      </c>
-      <c r="AF35" t="n">
-        <v>0.2401</v>
-      </c>
-      <c r="AG35" t="n">
-        <v>0.8137</v>
-      </c>
-      <c r="AH35" t="n">
-        <v>0.0431</v>
-      </c>
-      <c r="AI35" t="n">
-        <v>0.1747</v>
-      </c>
-      <c r="AJ35" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK35" t="n">
-        <v>0.876</v>
-      </c>
-      <c r="AL35" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM35" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN35" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO35" t="n">
-        <v>0.967</v>
-      </c>
-      <c r="AP35" t="n">
-        <v>1</v>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>1.6967</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>0.181</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>5.1447</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>0.0703</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>965</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>155</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>0.5468</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>419</t>
+        </is>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>528</t>
+        </is>
+      </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>1.4781</t>
+        </is>
+      </c>
+      <c r="AB35" t="inlineStr">
+        <is>
+          <t>1.8627</t>
+        </is>
+      </c>
+      <c r="AC35" t="inlineStr">
+        <is>
+          <t>283.4649</t>
+        </is>
+      </c>
+      <c r="AD35" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AE35" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="AF35" t="inlineStr">
+        <is>
+          <t>0.2401</t>
+        </is>
+      </c>
+      <c r="AG35" t="inlineStr">
+        <is>
+          <t>0.8137</t>
+        </is>
+      </c>
+      <c r="AH35" t="inlineStr">
+        <is>
+          <t>0.0431</t>
+        </is>
+      </c>
+      <c r="AI35" t="inlineStr">
+        <is>
+          <t>0.1747</t>
+        </is>
+      </c>
+      <c r="AJ35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK35" t="inlineStr">
+        <is>
+          <t>0.876</t>
+        </is>
+      </c>
+      <c r="AL35" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AM35" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN35" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO35" t="inlineStr">
+        <is>
+          <t>0.967</t>
+        </is>
+      </c>
+      <c r="AP35" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
       <c r="AQ35" t="inlineStr"/>
     </row>
@@ -11726,10 +11786,8 @@
           <t>daedalus</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>13190</t>
-        </is>
+      <c r="E58" t="n">
+        <v>28160</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -11737,10 +11795,8 @@
         </is>
       </c>
       <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>83.1</t>
-        </is>
+      <c r="H58" t="n">
+        <v>86.40000000000001</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
@@ -11759,146 +11815,90 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N58" t="inlineStr">
-        <is>
-          <t>0.048</t>
-        </is>
-      </c>
-      <c r="O58" t="inlineStr">
-        <is>
-          <t>0.065</t>
-        </is>
+      <c r="N58" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="O58" t="n">
+        <v>0.017</v>
       </c>
       <c r="P58" t="inlineStr"/>
-      <c r="Q58" t="inlineStr">
-        <is>
-          <t>1.5856</t>
-        </is>
-      </c>
-      <c r="R58" t="inlineStr">
-        <is>
-          <t>0.1309</t>
-        </is>
-      </c>
-      <c r="S58" t="inlineStr">
-        <is>
-          <t>2.9722</t>
-        </is>
-      </c>
-      <c r="T58" t="inlineStr">
-        <is>
-          <t>0.0243</t>
-        </is>
-      </c>
-      <c r="U58" t="inlineStr">
-        <is>
-          <t>511</t>
-        </is>
-      </c>
-      <c r="V58" t="inlineStr">
-        <is>
-          <t>148</t>
-        </is>
-      </c>
-      <c r="W58" t="inlineStr">
-        <is>
-          <t>1.2109</t>
-        </is>
-      </c>
-      <c r="X58" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="Y58" t="inlineStr">
-        <is>
-          <t>125</t>
-        </is>
-      </c>
-      <c r="Z58" t="inlineStr">
-        <is>
-          <t>378</t>
-        </is>
-      </c>
-      <c r="AA58" t="inlineStr">
-        <is>
-          <t>1.0228</t>
-        </is>
-      </c>
-      <c r="AB58" t="inlineStr">
-        <is>
-          <t>3.0928</t>
-        </is>
-      </c>
-      <c r="AC58" t="inlineStr">
-        <is>
-          <t>122.219</t>
-        </is>
-      </c>
-      <c r="AD58" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="AE58" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AF58" t="inlineStr">
-        <is>
-          <t>0.3091</t>
-        </is>
-      </c>
-      <c r="AG58" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AH58" t="inlineStr">
-        <is>
-          <t>0.1444</t>
-        </is>
-      </c>
-      <c r="AI58" t="inlineStr">
-        <is>
-          <t>0.0512</t>
-        </is>
-      </c>
-      <c r="AJ58" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AK58" t="inlineStr">
-        <is>
-          <t>0.736</t>
-        </is>
-      </c>
-      <c r="AL58" t="inlineStr">
-        <is>
-          <t>0.866</t>
-        </is>
-      </c>
-      <c r="AM58" t="inlineStr">
-        <is>
-          <t>0.622</t>
-        </is>
-      </c>
-      <c r="AN58" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AO58" t="inlineStr">
-        <is>
-          <t>0.823</t>
-        </is>
-      </c>
-      <c r="AP58" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="Q58" t="n">
+        <v>1.4197</v>
+      </c>
+      <c r="R58" t="n">
+        <v>0.1861</v>
+      </c>
+      <c r="S58" t="n">
+        <v>5.1808</v>
+      </c>
+      <c r="T58" t="n">
+        <v>0.0362</v>
+      </c>
+      <c r="U58" t="n">
+        <v>1134</v>
+      </c>
+      <c r="V58" t="n">
+        <v>275</v>
+      </c>
+      <c r="W58" t="n">
+        <v>1.8311</v>
+      </c>
+      <c r="X58" t="n">
+        <v>16</v>
+      </c>
+      <c r="Y58" t="n">
+        <v>181</v>
+      </c>
+      <c r="Z58" t="n">
+        <v>937</v>
+      </c>
+      <c r="AA58" t="n">
+        <v>1.2052</v>
+      </c>
+      <c r="AB58" t="n">
+        <v>6.2391</v>
+      </c>
+      <c r="AC58" t="n">
+        <v>150.1808</v>
+      </c>
+      <c r="AD58" t="n">
+        <v>23</v>
+      </c>
+      <c r="AE58" t="n">
+        <v>14</v>
+      </c>
+      <c r="AF58" t="n">
+        <v>0.2193</v>
+      </c>
+      <c r="AG58" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH58" t="n">
+        <v>0.1705</v>
+      </c>
+      <c r="AI58" t="n">
+        <v>0.0733</v>
+      </c>
+      <c r="AJ58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK58" t="n">
+        <v>0.528</v>
+      </c>
+      <c r="AL58" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM58" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN58" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO58" t="n">
+        <v>0.881</v>
+      </c>
+      <c r="AP58" t="n">
+        <v>1</v>
       </c>
       <c r="AQ58" t="inlineStr"/>
     </row>
@@ -16904,8 +16904,10 @@
           <t>fenrir</t>
         </is>
       </c>
-      <c r="E84" t="n">
-        <v>30712</v>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>30712</t>
+        </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -16913,8 +16915,10 @@
         </is>
       </c>
       <c r="G84" t="inlineStr"/>
-      <c r="H84" t="n">
-        <v>94.59999999999999</v>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>94.6</t>
+        </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
@@ -16933,90 +16937,146 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N84" t="n">
-        <v>0.008999999999999999</v>
-      </c>
-      <c r="O84" t="n">
-        <v>0.03</v>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>0.009</t>
+        </is>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>0.03</t>
+        </is>
       </c>
       <c r="P84" t="inlineStr"/>
-      <c r="Q84" t="n">
-        <v>1.6233</v>
-      </c>
-      <c r="R84" t="n">
-        <v>0.1887</v>
-      </c>
-      <c r="S84" t="n">
-        <v>6.3611</v>
-      </c>
-      <c r="T84" t="n">
-        <v>0.08169999999999999</v>
-      </c>
-      <c r="U84" t="n">
-        <v>942</v>
-      </c>
-      <c r="V84" t="n">
-        <v>143</v>
-      </c>
-      <c r="W84" t="n">
-        <v>0.863</v>
-      </c>
-      <c r="X84" t="n">
-        <v>23</v>
-      </c>
-      <c r="Y84" t="n">
-        <v>349</v>
-      </c>
-      <c r="Z84" t="n">
-        <v>570</v>
-      </c>
-      <c r="AA84" t="n">
-        <v>2.1061</v>
-      </c>
-      <c r="AB84" t="n">
-        <v>3.4397</v>
-      </c>
-      <c r="AC84" t="n">
-        <v>165.7105</v>
-      </c>
-      <c r="AD84" t="n">
-        <v>7</v>
-      </c>
-      <c r="AE84" t="n">
-        <v>18</v>
-      </c>
-      <c r="AF84" t="n">
-        <v>0.2661</v>
-      </c>
-      <c r="AG84" t="n">
-        <v>0.8143</v>
-      </c>
-      <c r="AH84" t="n">
-        <v>0.0443</v>
-      </c>
-      <c r="AI84" t="n">
-        <v>0.1231</v>
-      </c>
-      <c r="AJ84" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK84" t="n">
-        <v>0.784</v>
-      </c>
-      <c r="AL84" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM84" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN84" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO84" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP84" t="n">
-        <v>1</v>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>1.6233</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>0.1887</t>
+        </is>
+      </c>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>6.3611</t>
+        </is>
+      </c>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t>0.0817</t>
+        </is>
+      </c>
+      <c r="U84" t="inlineStr">
+        <is>
+          <t>942</t>
+        </is>
+      </c>
+      <c r="V84" t="inlineStr">
+        <is>
+          <t>143</t>
+        </is>
+      </c>
+      <c r="W84" t="inlineStr">
+        <is>
+          <t>0.863</t>
+        </is>
+      </c>
+      <c r="X84" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="Y84" t="inlineStr">
+        <is>
+          <t>349</t>
+        </is>
+      </c>
+      <c r="Z84" t="inlineStr">
+        <is>
+          <t>570</t>
+        </is>
+      </c>
+      <c r="AA84" t="inlineStr">
+        <is>
+          <t>2.1061</t>
+        </is>
+      </c>
+      <c r="AB84" t="inlineStr">
+        <is>
+          <t>3.4397</t>
+        </is>
+      </c>
+      <c r="AC84" t="inlineStr">
+        <is>
+          <t>165.7105</t>
+        </is>
+      </c>
+      <c r="AD84" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AE84" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="AF84" t="inlineStr">
+        <is>
+          <t>0.2661</t>
+        </is>
+      </c>
+      <c r="AG84" t="inlineStr">
+        <is>
+          <t>0.8143</t>
+        </is>
+      </c>
+      <c r="AH84" t="inlineStr">
+        <is>
+          <t>0.0443</t>
+        </is>
+      </c>
+      <c r="AI84" t="inlineStr">
+        <is>
+          <t>0.1231</t>
+        </is>
+      </c>
+      <c r="AJ84" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK84" t="inlineStr">
+        <is>
+          <t>0.784</t>
+        </is>
+      </c>
+      <c r="AL84" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AM84" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN84" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO84" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AP84" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
       <c r="AQ84" t="inlineStr"/>
     </row>
@@ -18247,8 +18307,10 @@
           <t>fortress_bastion</t>
         </is>
       </c>
-      <c r="E91" t="n">
-        <v>56092</v>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>56092</t>
+        </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -18256,8 +18318,10 @@
         </is>
       </c>
       <c r="G91" t="inlineStr"/>
-      <c r="H91" t="n">
-        <v>100</v>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
@@ -18276,90 +18340,146 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N91" t="n">
-        <v>0.029</v>
-      </c>
-      <c r="O91" t="n">
-        <v>0.042</v>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>0.029</t>
+        </is>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>0.042</t>
+        </is>
       </c>
       <c r="P91" t="inlineStr"/>
-      <c r="Q91" t="n">
-        <v>1.8452</v>
-      </c>
-      <c r="R91" t="n">
-        <v>0.1728</v>
-      </c>
-      <c r="S91" t="n">
-        <v>5.887</v>
-      </c>
-      <c r="T91" t="n">
-        <v>0.034</v>
-      </c>
-      <c r="U91" t="n">
-        <v>1609</v>
-      </c>
-      <c r="V91" t="n">
-        <v>183</v>
-      </c>
-      <c r="W91" t="n">
-        <v>1.2447</v>
-      </c>
-      <c r="X91" t="n">
-        <v>6</v>
-      </c>
-      <c r="Y91" t="n">
-        <v>261</v>
-      </c>
-      <c r="Z91" t="n">
-        <v>1342</v>
-      </c>
-      <c r="AA91" t="n">
-        <v>1.7752</v>
-      </c>
-      <c r="AB91" t="n">
-        <v>9.1275</v>
-      </c>
-      <c r="AC91" t="n">
-        <v>147.0282</v>
-      </c>
-      <c r="AD91" t="n">
-        <v>6</v>
-      </c>
-      <c r="AE91" t="n">
-        <v>19</v>
-      </c>
-      <c r="AF91" t="n">
-        <v>0.2389</v>
-      </c>
-      <c r="AG91" t="n">
-        <v>0.8867</v>
-      </c>
-      <c r="AH91" t="n">
-        <v>0.0626</v>
-      </c>
-      <c r="AI91" t="n">
-        <v>0.1999</v>
-      </c>
-      <c r="AJ91" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK91" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL91" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM91" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN91" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO91" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP91" t="n">
-        <v>1</v>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>1.8452</t>
+        </is>
+      </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>0.1728</t>
+        </is>
+      </c>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t>5.887</t>
+        </is>
+      </c>
+      <c r="T91" t="inlineStr">
+        <is>
+          <t>0.034</t>
+        </is>
+      </c>
+      <c r="U91" t="inlineStr">
+        <is>
+          <t>1609</t>
+        </is>
+      </c>
+      <c r="V91" t="inlineStr">
+        <is>
+          <t>183</t>
+        </is>
+      </c>
+      <c r="W91" t="inlineStr">
+        <is>
+          <t>1.2447</t>
+        </is>
+      </c>
+      <c r="X91" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="Y91" t="inlineStr">
+        <is>
+          <t>261</t>
+        </is>
+      </c>
+      <c r="Z91" t="inlineStr">
+        <is>
+          <t>1342</t>
+        </is>
+      </c>
+      <c r="AA91" t="inlineStr">
+        <is>
+          <t>1.7752</t>
+        </is>
+      </c>
+      <c r="AB91" t="inlineStr">
+        <is>
+          <t>9.1275</t>
+        </is>
+      </c>
+      <c r="AC91" t="inlineStr">
+        <is>
+          <t>147.0282</t>
+        </is>
+      </c>
+      <c r="AD91" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AE91" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="AF91" t="inlineStr">
+        <is>
+          <t>0.2389</t>
+        </is>
+      </c>
+      <c r="AG91" t="inlineStr">
+        <is>
+          <t>0.8867</t>
+        </is>
+      </c>
+      <c r="AH91" t="inlineStr">
+        <is>
+          <t>0.0626</t>
+        </is>
+      </c>
+      <c r="AI91" t="inlineStr">
+        <is>
+          <t>0.1999</t>
+        </is>
+      </c>
+      <c r="AJ91" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK91" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AL91" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AM91" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN91" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO91" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AP91" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
       <c r="AQ91" t="inlineStr"/>
     </row>
@@ -25564,10 +25684,8 @@
           <t>ixion</t>
         </is>
       </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>36022</t>
-        </is>
+      <c r="E128" t="n">
+        <v>40940</v>
       </c>
       <c r="F128" t="inlineStr">
         <is>
@@ -25575,10 +25693,8 @@
         </is>
       </c>
       <c r="G128" t="inlineStr"/>
-      <c r="H128" t="inlineStr">
-        <is>
-          <t>89.2</t>
-        </is>
+      <c r="H128" t="n">
+        <v>90.7</v>
       </c>
       <c r="I128" t="inlineStr">
         <is>
@@ -25597,146 +25713,90 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N128" t="inlineStr">
-        <is>
-          <t>0.027</t>
-        </is>
-      </c>
-      <c r="O128" t="inlineStr">
-        <is>
-          <t>0.012</t>
-        </is>
+      <c r="N128" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="O128" t="n">
+        <v>0.024</v>
       </c>
       <c r="P128" t="inlineStr"/>
-      <c r="Q128" t="inlineStr">
-        <is>
-          <t>1.6346</t>
-        </is>
-      </c>
-      <c r="R128" t="inlineStr">
-        <is>
-          <t>0.1507</t>
-        </is>
-      </c>
-      <c r="S128" t="inlineStr">
-        <is>
-          <t>4.1563</t>
-        </is>
-      </c>
-      <c r="T128" t="inlineStr">
-        <is>
-          <t>0.0453</t>
-        </is>
-      </c>
-      <c r="U128" t="inlineStr">
-        <is>
-          <t>1098</t>
-        </is>
-      </c>
-      <c r="V128" t="inlineStr">
-        <is>
-          <t>227</t>
-        </is>
-      </c>
-      <c r="W128" t="inlineStr">
-        <is>
-          <t>0.8627</t>
-        </is>
-      </c>
-      <c r="X128" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="Y128" t="inlineStr">
-        <is>
-          <t>206</t>
-        </is>
-      </c>
-      <c r="Z128" t="inlineStr">
-        <is>
-          <t>873</t>
-        </is>
-      </c>
-      <c r="AA128" t="inlineStr">
-        <is>
-          <t>0.7829</t>
-        </is>
-      </c>
-      <c r="AB128" t="inlineStr">
-        <is>
-          <t>3.318</t>
-        </is>
-      </c>
-      <c r="AC128" t="inlineStr">
-        <is>
-          <t>263.1129</t>
-        </is>
-      </c>
-      <c r="AD128" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="AE128" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="AF128" t="inlineStr">
-        <is>
-          <t>0.1194</t>
-        </is>
-      </c>
-      <c r="AG128" t="inlineStr">
-        <is>
-          <t>0.9728</t>
-        </is>
-      </c>
-      <c r="AH128" t="inlineStr">
-        <is>
-          <t>0.0974</t>
-        </is>
-      </c>
-      <c r="AI128" t="inlineStr">
-        <is>
-          <t>0.1793</t>
-        </is>
-      </c>
-      <c r="AJ128" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AK128" t="inlineStr">
-        <is>
-          <t>0.798</t>
-        </is>
-      </c>
-      <c r="AL128" t="inlineStr">
-        <is>
-          <t>0.996</t>
-        </is>
-      </c>
-      <c r="AM128" t="inlineStr">
-        <is>
-          <t>0.87</t>
-        </is>
-      </c>
-      <c r="AN128" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AO128" t="inlineStr">
-        <is>
-          <t>0.747</t>
-        </is>
-      </c>
-      <c r="AP128" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="Q128" t="n">
+        <v>1.6385</v>
+      </c>
+      <c r="R128" t="n">
+        <v>0.1559</v>
+      </c>
+      <c r="S128" t="n">
+        <v>4.4752</v>
+      </c>
+      <c r="T128" t="n">
+        <v>0.0453</v>
+      </c>
+      <c r="U128" t="n">
+        <v>1228</v>
+      </c>
+      <c r="V128" t="n">
+        <v>261</v>
+      </c>
+      <c r="W128" t="n">
+        <v>0.9692</v>
+      </c>
+      <c r="X128" t="n">
+        <v>19</v>
+      </c>
+      <c r="Y128" t="n">
+        <v>233</v>
+      </c>
+      <c r="Z128" t="n">
+        <v>976</v>
+      </c>
+      <c r="AA128" t="n">
+        <v>0.8652</v>
+      </c>
+      <c r="AB128" t="n">
+        <v>3.6242</v>
+      </c>
+      <c r="AC128" t="n">
+        <v>269.3027</v>
+      </c>
+      <c r="AD128" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE128" t="n">
+        <v>17</v>
+      </c>
+      <c r="AF128" t="n">
+        <v>0.1219</v>
+      </c>
+      <c r="AG128" t="n">
+        <v>0.9634</v>
+      </c>
+      <c r="AH128" t="n">
+        <v>0.08790000000000001</v>
+      </c>
+      <c r="AI128" t="n">
+        <v>0.1761</v>
+      </c>
+      <c r="AJ128" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK128" t="n">
+        <v>0.803</v>
+      </c>
+      <c r="AL128" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM128" t="n">
+        <v>0.9370000000000001</v>
+      </c>
+      <c r="AN128" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO128" t="n">
+        <v>0.774</v>
+      </c>
+      <c r="AP128" t="n">
+        <v>1</v>
       </c>
       <c r="AQ128" t="inlineStr"/>
     </row>
@@ -28559,10 +28619,8 @@
           <t>mega_gunship</t>
         </is>
       </c>
-      <c r="E143" t="inlineStr">
-        <is>
-          <t>9284</t>
-        </is>
+      <c r="E143" t="n">
+        <v>26228</v>
       </c>
       <c r="F143" t="inlineStr">
         <is>
@@ -28570,10 +28628,8 @@
         </is>
       </c>
       <c r="G143" t="inlineStr"/>
-      <c r="H143" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
+      <c r="H143" t="n">
+        <v>100</v>
       </c>
       <c r="I143" t="inlineStr">
         <is>
@@ -28592,146 +28648,90 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N143" t="inlineStr">
-        <is>
-          <t>0.023</t>
-        </is>
-      </c>
-      <c r="O143" t="inlineStr">
-        <is>
-          <t>0.047</t>
-        </is>
+      <c r="N143" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="O143" t="n">
+        <v>0.028</v>
       </c>
       <c r="P143" t="inlineStr"/>
-      <c r="Q143" t="inlineStr">
-        <is>
-          <t>2.0243</t>
-        </is>
-      </c>
-      <c r="R143" t="inlineStr">
-        <is>
-          <t>0.1431</t>
-        </is>
-      </c>
-      <c r="S143" t="inlineStr">
-        <is>
-          <t>3.7013</t>
-        </is>
-      </c>
-      <c r="T143" t="inlineStr">
-        <is>
-          <t>0.0423</t>
-        </is>
-      </c>
-      <c r="U143" t="inlineStr">
-        <is>
-          <t>342</t>
-        </is>
-      </c>
-      <c r="V143" t="inlineStr">
-        <is>
-          <t>74</t>
-        </is>
-      </c>
-      <c r="W143" t="inlineStr">
-        <is>
-          <t>1.4579</t>
-        </is>
-      </c>
-      <c r="X143" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="Y143" t="inlineStr">
-        <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="Z143" t="inlineStr">
-        <is>
-          <t>259</t>
-        </is>
-      </c>
-      <c r="AA143" t="inlineStr">
-        <is>
-          <t>1.4776</t>
-        </is>
-      </c>
-      <c r="AB143" t="inlineStr">
-        <is>
-          <t>5.1026</t>
-        </is>
-      </c>
-      <c r="AC143" t="inlineStr">
-        <is>
-          <t>50.7585</t>
-        </is>
-      </c>
-      <c r="AD143" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="AE143" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="AF143" t="inlineStr">
-        <is>
-          <t>0.3182</t>
-        </is>
-      </c>
-      <c r="AG143" t="inlineStr">
-        <is>
-          <t>0.9295</t>
-        </is>
-      </c>
-      <c r="AH143" t="inlineStr">
-        <is>
-          <t>0.0708</t>
-        </is>
-      </c>
-      <c r="AI143" t="inlineStr">
-        <is>
-          <t>0.1279</t>
-        </is>
-      </c>
-      <c r="AJ143" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AK143" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AL143" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AM143" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AN143" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AO143" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AP143" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="Q143" t="n">
+        <v>2.2986</v>
+      </c>
+      <c r="R143" t="n">
+        <v>0.2102</v>
+      </c>
+      <c r="S143" t="n">
+        <v>7.0814</v>
+      </c>
+      <c r="T143" t="n">
+        <v>0.0353</v>
+      </c>
+      <c r="U143" t="n">
+        <v>966</v>
+      </c>
+      <c r="V143" t="n">
+        <v>167</v>
+      </c>
+      <c r="W143" t="n">
+        <v>2.4484</v>
+      </c>
+      <c r="X143" t="n">
+        <v>18</v>
+      </c>
+      <c r="Y143" t="n">
+        <v>121</v>
+      </c>
+      <c r="Z143" t="n">
+        <v>827</v>
+      </c>
+      <c r="AA143" t="n">
+        <v>1.774</v>
+      </c>
+      <c r="AB143" t="n">
+        <v>12.1245</v>
+      </c>
+      <c r="AC143" t="n">
+        <v>68.2092</v>
+      </c>
+      <c r="AD143" t="n">
+        <v>14</v>
+      </c>
+      <c r="AE143" t="n">
+        <v>12</v>
+      </c>
+      <c r="AF143" t="n">
+        <v>0.2915</v>
+      </c>
+      <c r="AG143" t="n">
+        <v>0.8137</v>
+      </c>
+      <c r="AH143" t="n">
+        <v>0.0393</v>
+      </c>
+      <c r="AI143" t="n">
+        <v>0.06320000000000001</v>
+      </c>
+      <c r="AJ143" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK143" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL143" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM143" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN143" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO143" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP143" t="n">
+        <v>1</v>
       </c>
       <c r="AQ143" t="inlineStr"/>
     </row>
@@ -31554,8 +31554,10 @@
           <t>mobile_fortress</t>
         </is>
       </c>
-      <c r="E158" t="n">
-        <v>55236</v>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>55236</t>
+        </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
@@ -31563,8 +31565,10 @@
         </is>
       </c>
       <c r="G158" t="inlineStr"/>
-      <c r="H158" t="n">
-        <v>100</v>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
       </c>
       <c r="I158" t="inlineStr">
         <is>
@@ -31583,90 +31587,146 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N158" t="n">
-        <v>0.014</v>
-      </c>
-      <c r="O158" t="n">
-        <v>0.033</v>
+      <c r="N158" t="inlineStr">
+        <is>
+          <t>0.014</t>
+        </is>
+      </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>0.033</t>
+        </is>
       </c>
       <c r="P158" t="inlineStr"/>
-      <c r="Q158" t="n">
-        <v>2.4311</v>
-      </c>
-      <c r="R158" t="n">
-        <v>0.2018</v>
-      </c>
-      <c r="S158" t="n">
-        <v>6.0667</v>
-      </c>
-      <c r="T158" t="n">
-        <v>0.199</v>
-      </c>
-      <c r="U158" t="n">
-        <v>1550</v>
-      </c>
-      <c r="V158" t="n">
-        <v>159</v>
-      </c>
-      <c r="W158" t="n">
-        <v>0.7494</v>
-      </c>
-      <c r="X158" t="n">
-        <v>19</v>
-      </c>
-      <c r="Y158" t="n">
-        <v>471</v>
-      </c>
-      <c r="Z158" t="n">
-        <v>1060</v>
-      </c>
-      <c r="AA158" t="n">
-        <v>2.2199</v>
-      </c>
-      <c r="AB158" t="n">
-        <v>4.996</v>
-      </c>
-      <c r="AC158" t="n">
-        <v>212.1676</v>
-      </c>
-      <c r="AD158" t="n">
-        <v>8</v>
-      </c>
-      <c r="AE158" t="n">
-        <v>18</v>
-      </c>
-      <c r="AF158" t="n">
-        <v>0.2828</v>
-      </c>
-      <c r="AG158" t="n">
-        <v>0.8137</v>
-      </c>
-      <c r="AH158" t="n">
-        <v>0.0368</v>
-      </c>
-      <c r="AI158" t="n">
-        <v>0.1436</v>
-      </c>
-      <c r="AJ158" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK158" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL158" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM158" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN158" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO158" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP158" t="n">
-        <v>1</v>
+      <c r="Q158" t="inlineStr">
+        <is>
+          <t>2.4311</t>
+        </is>
+      </c>
+      <c r="R158" t="inlineStr">
+        <is>
+          <t>0.2018</t>
+        </is>
+      </c>
+      <c r="S158" t="inlineStr">
+        <is>
+          <t>6.0667</t>
+        </is>
+      </c>
+      <c r="T158" t="inlineStr">
+        <is>
+          <t>0.199</t>
+        </is>
+      </c>
+      <c r="U158" t="inlineStr">
+        <is>
+          <t>1550</t>
+        </is>
+      </c>
+      <c r="V158" t="inlineStr">
+        <is>
+          <t>159</t>
+        </is>
+      </c>
+      <c r="W158" t="inlineStr">
+        <is>
+          <t>0.7494</t>
+        </is>
+      </c>
+      <c r="X158" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="Y158" t="inlineStr">
+        <is>
+          <t>471</t>
+        </is>
+      </c>
+      <c r="Z158" t="inlineStr">
+        <is>
+          <t>1060</t>
+        </is>
+      </c>
+      <c r="AA158" t="inlineStr">
+        <is>
+          <t>2.2199</t>
+        </is>
+      </c>
+      <c r="AB158" t="inlineStr">
+        <is>
+          <t>4.996</t>
+        </is>
+      </c>
+      <c r="AC158" t="inlineStr">
+        <is>
+          <t>212.1676</t>
+        </is>
+      </c>
+      <c r="AD158" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AE158" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="AF158" t="inlineStr">
+        <is>
+          <t>0.2828</t>
+        </is>
+      </c>
+      <c r="AG158" t="inlineStr">
+        <is>
+          <t>0.8137</t>
+        </is>
+      </c>
+      <c r="AH158" t="inlineStr">
+        <is>
+          <t>0.0368</t>
+        </is>
+      </c>
+      <c r="AI158" t="inlineStr">
+        <is>
+          <t>0.1436</t>
+        </is>
+      </c>
+      <c r="AJ158" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK158" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AL158" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AM158" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN158" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO158" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AP158" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
       <c r="AQ158" t="inlineStr"/>
     </row>
@@ -33078,10 +33138,8 @@
           <t>nuke_train</t>
         </is>
       </c>
-      <c r="E166" t="inlineStr">
-        <is>
-          <t>28910</t>
-        </is>
+      <c r="E166" t="n">
+        <v>40684</v>
       </c>
       <c r="F166" t="inlineStr">
         <is>
@@ -33089,10 +33147,8 @@
         </is>
       </c>
       <c r="G166" t="inlineStr"/>
-      <c r="H166" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
+      <c r="H166" t="n">
+        <v>92.90000000000001</v>
       </c>
       <c r="I166" t="inlineStr">
         <is>
@@ -33111,146 +33167,90 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N166" t="inlineStr">
-        <is>
-          <t>0.025</t>
-        </is>
-      </c>
-      <c r="O166" t="inlineStr">
-        <is>
-          <t>0.021</t>
-        </is>
+      <c r="N166" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="O166" t="n">
+        <v>0.026</v>
       </c>
       <c r="P166" t="inlineStr"/>
-      <c r="Q166" t="inlineStr">
-        <is>
-          <t>1.665</t>
-        </is>
-      </c>
-      <c r="R166" t="inlineStr">
-        <is>
-          <t>0.2098</t>
-        </is>
-      </c>
-      <c r="S166" t="inlineStr">
-        <is>
-          <t>6.5246</t>
-        </is>
-      </c>
-      <c r="T166" t="inlineStr">
-        <is>
-          <t>0.0309</t>
-        </is>
-      </c>
-      <c r="U166" t="inlineStr">
-        <is>
-          <t>932</t>
-        </is>
-      </c>
-      <c r="V166" t="inlineStr">
-        <is>
-          <t>176</t>
-        </is>
-      </c>
-      <c r="W166" t="inlineStr">
-        <is>
-          <t>5.0666</t>
-        </is>
-      </c>
-      <c r="X166" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="Y166" t="inlineStr">
-        <is>
-          <t>143</t>
-        </is>
-      </c>
-      <c r="Z166" t="inlineStr">
-        <is>
-          <t>787</t>
-        </is>
-      </c>
-      <c r="AA166" t="inlineStr">
-        <is>
-          <t>4.1166</t>
-        </is>
-      </c>
-      <c r="AB166" t="inlineStr">
-        <is>
-          <t>22.6558</t>
-        </is>
-      </c>
-      <c r="AC166" t="inlineStr">
-        <is>
-          <t>34.7373</t>
-        </is>
-      </c>
-      <c r="AD166" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="AE166" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="AF166" t="inlineStr">
-        <is>
-          <t>0.1654</t>
-        </is>
-      </c>
-      <c r="AG166" t="inlineStr">
-        <is>
-          <t>0.8342</t>
-        </is>
-      </c>
-      <c r="AH166" t="inlineStr">
-        <is>
-          <t>0.0511</t>
-        </is>
-      </c>
-      <c r="AI166" t="inlineStr">
-        <is>
-          <t>0.1228</t>
-        </is>
-      </c>
-      <c r="AJ166" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AK166" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AL166" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AM166" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AN166" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AO166" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AP166" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="Q166" t="n">
+        <v>1.4212</v>
+      </c>
+      <c r="R166" t="n">
+        <v>0.2061</v>
+      </c>
+      <c r="S166" t="n">
+        <v>6.3189</v>
+      </c>
+      <c r="T166" t="n">
+        <v>0.0532</v>
+      </c>
+      <c r="U166" t="n">
+        <v>1353</v>
+      </c>
+      <c r="V166" t="n">
+        <v>191</v>
+      </c>
+      <c r="W166" t="n">
+        <v>8.174899999999999</v>
+      </c>
+      <c r="X166" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y166" t="n">
+        <v>151</v>
+      </c>
+      <c r="Z166" t="n">
+        <v>1202</v>
+      </c>
+      <c r="AA166" t="n">
+        <v>6.4629</v>
+      </c>
+      <c r="AB166" t="n">
+        <v>51.4465</v>
+      </c>
+      <c r="AC166" t="n">
+        <v>23.3641</v>
+      </c>
+      <c r="AD166" t="n">
+        <v>8</v>
+      </c>
+      <c r="AE166" t="n">
+        <v>19</v>
+      </c>
+      <c r="AF166" t="n">
+        <v>0.1622</v>
+      </c>
+      <c r="AG166" t="n">
+        <v>0.8222</v>
+      </c>
+      <c r="AH166" t="n">
+        <v>0.0489</v>
+      </c>
+      <c r="AI166" t="n">
+        <v>0.1116</v>
+      </c>
+      <c r="AJ166" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK166" t="n">
+        <v>0.716</v>
+      </c>
+      <c r="AL166" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM166" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN166" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO166" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP166" t="n">
+        <v>1</v>
       </c>
       <c r="AQ166" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Play-test 14 wave M5: EW jammer, Laser AA, command vehicle, jet redrawn
Wheeled gun's turret cut to Centauro proportion; wheeled units under 7,500 tris.
Builder Tools/blender/mb_pt14_m5.py; DECISIONS "Play-test 14 model wave M5".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/models/quality_report.xlsx
+++ b/Docs/models/quality_report.xlsx
@@ -10841,10 +10841,8 @@
           <t>command_vehicle</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>6096</t>
-        </is>
+      <c r="E53" t="n">
+        <v>6494</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -10852,10 +10850,8 @@
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>92.7</t>
-        </is>
+      <c r="H53" t="n">
+        <v>95</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
@@ -10874,150 +10870,90 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N53" t="inlineStr">
-        <is>
-          <t>0.141</t>
-        </is>
-      </c>
-      <c r="O53" t="inlineStr">
-        <is>
-          <t>0.099</t>
-        </is>
-      </c>
-      <c r="P53" t="inlineStr">
-        <is>
-          <t>mlrs</t>
-        </is>
-      </c>
-      <c r="Q53" t="inlineStr">
-        <is>
-          <t>1.5282</t>
-        </is>
-      </c>
-      <c r="R53" t="inlineStr">
-        <is>
-          <t>0.257</t>
-        </is>
-      </c>
-      <c r="S53" t="inlineStr">
-        <is>
-          <t>8.3324</t>
-        </is>
-      </c>
-      <c r="T53" t="inlineStr">
-        <is>
-          <t>0.0183</t>
-        </is>
-      </c>
-      <c r="U53" t="inlineStr">
-        <is>
-          <t>178</t>
-        </is>
-      </c>
-      <c r="V53" t="inlineStr">
-        <is>
-          <t>79</t>
-        </is>
-      </c>
-      <c r="W53" t="inlineStr">
-        <is>
-          <t>1.0291</t>
-        </is>
-      </c>
-      <c r="X53" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="Y53" t="inlineStr">
-        <is>
-          <t>79</t>
-        </is>
-      </c>
-      <c r="Z53" t="inlineStr">
-        <is>
-          <t>91</t>
-        </is>
-      </c>
-      <c r="AA53" t="inlineStr">
-        <is>
-          <t>1.0291</t>
-        </is>
-      </c>
-      <c r="AB53" t="inlineStr">
-        <is>
-          <t>1.1854</t>
-        </is>
-      </c>
-      <c r="AC53" t="inlineStr">
-        <is>
-          <t>76.7661</t>
-        </is>
-      </c>
-      <c r="AD53" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="AE53" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="AF53" t="inlineStr">
-        <is>
-          <t>0.3274</t>
-        </is>
-      </c>
-      <c r="AG53" t="inlineStr">
-        <is>
-          <t>0.981</t>
-        </is>
-      </c>
-      <c r="AH53" t="inlineStr">
-        <is>
-          <t>0.0796</t>
-        </is>
-      </c>
-      <c r="AI53" t="inlineStr">
-        <is>
-          <t>0.2369</t>
-        </is>
-      </c>
-      <c r="AJ53" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AK53" t="inlineStr">
-        <is>
-          <t>0.747</t>
-        </is>
-      </c>
-      <c r="AL53" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AM53" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AN53" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AO53" t="inlineStr">
-        <is>
-          <t>0.937</t>
-        </is>
-      </c>
-      <c r="AP53" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N53" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="O53" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="n">
+        <v>1.5719</v>
+      </c>
+      <c r="R53" t="n">
+        <v>0.3086</v>
+      </c>
+      <c r="S53" t="n">
+        <v>10.3072</v>
+      </c>
+      <c r="T53" t="n">
+        <v>0.104</v>
+      </c>
+      <c r="U53" t="n">
+        <v>203</v>
+      </c>
+      <c r="V53" t="n">
+        <v>100</v>
+      </c>
+      <c r="W53" t="n">
+        <v>1.1986</v>
+      </c>
+      <c r="X53" t="n">
+        <v>11</v>
+      </c>
+      <c r="Y53" t="n">
+        <v>96</v>
+      </c>
+      <c r="Z53" t="n">
+        <v>96</v>
+      </c>
+      <c r="AA53" t="n">
+        <v>1.1507</v>
+      </c>
+      <c r="AB53" t="n">
+        <v>1.1507</v>
+      </c>
+      <c r="AC53" t="n">
+        <v>83.4303</v>
+      </c>
+      <c r="AD53" t="n">
+        <v>11</v>
+      </c>
+      <c r="AE53" t="n">
+        <v>13</v>
+      </c>
+      <c r="AF53" t="n">
+        <v>0.2915</v>
+      </c>
+      <c r="AG53" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="AH53" t="n">
+        <v>0.0704</v>
+      </c>
+      <c r="AI53" t="n">
+        <v>0.1767</v>
+      </c>
+      <c r="AJ53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK53" t="n">
+        <v>0.8090000000000001</v>
+      </c>
+      <c r="AL53" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM53" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN53" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO53" t="n">
+        <v>0.989</v>
+      </c>
+      <c r="AP53" t="n">
+        <v>1</v>
       </c>
       <c r="AQ53" t="inlineStr"/>
     </row>
@@ -16220,10 +16156,8 @@
           <t>ew_jammer</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>7428</t>
-        </is>
+      <c r="E80" t="n">
+        <v>7472</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -16231,10 +16165,8 @@
         </is>
       </c>
       <c r="G80" t="inlineStr"/>
-      <c r="H80" t="inlineStr">
-        <is>
-          <t>92.9</t>
-        </is>
+      <c r="H80" t="n">
+        <v>95.09999999999999</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
@@ -16253,150 +16185,90 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N80" t="inlineStr">
-        <is>
-          <t>0.202</t>
-        </is>
-      </c>
-      <c r="O80" t="inlineStr">
-        <is>
-          <t>0.274</t>
-        </is>
-      </c>
-      <c r="P80" t="inlineStr">
-        <is>
-          <t>river_patrol_boat</t>
-        </is>
-      </c>
-      <c r="Q80" t="inlineStr">
-        <is>
-          <t>1.6814</t>
-        </is>
-      </c>
-      <c r="R80" t="inlineStr">
-        <is>
-          <t>0.2136</t>
-        </is>
-      </c>
-      <c r="S80" t="inlineStr">
-        <is>
-          <t>6.2409</t>
-        </is>
-      </c>
-      <c r="T80" t="inlineStr">
-        <is>
-          <t>0.0118</t>
-        </is>
-      </c>
-      <c r="U80" t="inlineStr">
-        <is>
-          <t>241</t>
-        </is>
-      </c>
-      <c r="V80" t="inlineStr">
-        <is>
-          <t>93</t>
-        </is>
-      </c>
-      <c r="W80" t="inlineStr">
-        <is>
-          <t>0.7498</t>
-        </is>
-      </c>
-      <c r="X80" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="Y80" t="inlineStr">
-        <is>
-          <t>138</t>
-        </is>
-      </c>
-      <c r="Z80" t="inlineStr">
-        <is>
-          <t>94</t>
-        </is>
-      </c>
-      <c r="AA80" t="inlineStr">
-        <is>
-          <t>1.1126</t>
-        </is>
-      </c>
-      <c r="AB80" t="inlineStr">
-        <is>
-          <t>0.7579</t>
-        </is>
-      </c>
-      <c r="AC80" t="inlineStr">
-        <is>
-          <t>124.0319</t>
-        </is>
-      </c>
-      <c r="AD80" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="AE80" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="AF80" t="inlineStr">
-        <is>
-          <t>0.1354</t>
-        </is>
-      </c>
-      <c r="AG80" t="inlineStr">
-        <is>
-          <t>0.9118</t>
-        </is>
-      </c>
-      <c r="AH80" t="inlineStr">
-        <is>
-          <t>0.0602</t>
-        </is>
-      </c>
-      <c r="AI80" t="inlineStr">
-        <is>
-          <t>0.0402</t>
-        </is>
-      </c>
-      <c r="AJ80" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AK80" t="inlineStr">
-        <is>
-          <t>0.963</t>
-        </is>
-      </c>
-      <c r="AL80" t="inlineStr">
-        <is>
-          <t>0.892</t>
-        </is>
-      </c>
-      <c r="AM80" t="inlineStr">
-        <is>
-          <t>0.75</t>
-        </is>
-      </c>
-      <c r="AN80" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AO80" t="inlineStr">
-        <is>
-          <t>0.944</t>
-        </is>
-      </c>
-      <c r="AP80" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N80" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="O80" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="P80" t="inlineStr"/>
+      <c r="Q80" t="n">
+        <v>1.6109</v>
+      </c>
+      <c r="R80" t="n">
+        <v>0.2792</v>
+      </c>
+      <c r="S80" t="n">
+        <v>9.6951</v>
+      </c>
+      <c r="T80" t="n">
+        <v>0.0303</v>
+      </c>
+      <c r="U80" t="n">
+        <v>297</v>
+      </c>
+      <c r="V80" t="n">
+        <v>117</v>
+      </c>
+      <c r="W80" t="n">
+        <v>0.7806</v>
+      </c>
+      <c r="X80" t="n">
+        <v>16</v>
+      </c>
+      <c r="Y80" t="n">
+        <v>185</v>
+      </c>
+      <c r="Z80" t="n">
+        <v>96</v>
+      </c>
+      <c r="AA80" t="n">
+        <v>1.2342</v>
+      </c>
+      <c r="AB80" t="n">
+        <v>0.6405</v>
+      </c>
+      <c r="AC80" t="n">
+        <v>149.8923</v>
+      </c>
+      <c r="AD80" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE80" t="n">
+        <v>11</v>
+      </c>
+      <c r="AF80" t="n">
+        <v>0.2428</v>
+      </c>
+      <c r="AG80" t="n">
+        <v>0.9125</v>
+      </c>
+      <c r="AH80" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="AI80" t="n">
+        <v>0.0409</v>
+      </c>
+      <c r="AJ80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK80" t="n">
+        <v>0.864</v>
+      </c>
+      <c r="AL80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN80" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO80" t="n">
+        <v>0.898</v>
+      </c>
+      <c r="AP80" t="n">
+        <v>1</v>
       </c>
       <c r="AQ80" t="inlineStr"/>
     </row>
@@ -24413,8 +24285,10 @@
           <t>hydra</t>
         </is>
       </c>
-      <c r="E121" t="n">
-        <v>14952</v>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>14952</t>
+        </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
@@ -24422,8 +24296,10 @@
         </is>
       </c>
       <c r="G121" t="inlineStr"/>
-      <c r="H121" t="n">
-        <v>99.5</v>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>99.5</t>
+        </is>
       </c>
       <c r="I121" t="inlineStr">
         <is>
@@ -24442,90 +24318,146 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N121" t="n">
-        <v>0.018</v>
-      </c>
-      <c r="O121" t="n">
-        <v>0.015</v>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>0.018</t>
+        </is>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>0.015</t>
+        </is>
       </c>
       <c r="P121" t="inlineStr"/>
-      <c r="Q121" t="n">
-        <v>1.2769</v>
-      </c>
-      <c r="R121" t="n">
-        <v>0.0906</v>
-      </c>
-      <c r="S121" t="n">
-        <v>1.7553</v>
-      </c>
-      <c r="T121" t="n">
-        <v>0.0364</v>
-      </c>
-      <c r="U121" t="n">
-        <v>346</v>
-      </c>
-      <c r="V121" t="n">
-        <v>67</v>
-      </c>
-      <c r="W121" t="n">
-        <v>1.7618</v>
-      </c>
-      <c r="X121" t="n">
-        <v>13</v>
-      </c>
-      <c r="Y121" t="n">
-        <v>57</v>
-      </c>
-      <c r="Z121" t="n">
-        <v>276</v>
-      </c>
-      <c r="AA121" t="n">
-        <v>1.4988</v>
-      </c>
-      <c r="AB121" t="n">
-        <v>7.2576</v>
-      </c>
-      <c r="AC121" t="n">
-        <v>38.0293</v>
-      </c>
-      <c r="AD121" t="n">
-        <v>40</v>
-      </c>
-      <c r="AE121" t="n">
-        <v>9</v>
-      </c>
-      <c r="AF121" t="n">
-        <v>0.2493</v>
-      </c>
-      <c r="AG121" t="n">
-        <v>0.8058</v>
-      </c>
-      <c r="AH121" t="n">
-        <v>0.0247</v>
-      </c>
-      <c r="AI121" t="n">
-        <v>0.1362</v>
-      </c>
-      <c r="AJ121" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK121" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL121" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM121" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN121" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO121" t="n">
-        <v>0.965</v>
-      </c>
-      <c r="AP121" t="n">
-        <v>1</v>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t>1.2769</t>
+        </is>
+      </c>
+      <c r="R121" t="inlineStr">
+        <is>
+          <t>0.0906</t>
+        </is>
+      </c>
+      <c r="S121" t="inlineStr">
+        <is>
+          <t>1.7553</t>
+        </is>
+      </c>
+      <c r="T121" t="inlineStr">
+        <is>
+          <t>0.0364</t>
+        </is>
+      </c>
+      <c r="U121" t="inlineStr">
+        <is>
+          <t>346</t>
+        </is>
+      </c>
+      <c r="V121" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="W121" t="inlineStr">
+        <is>
+          <t>1.7618</t>
+        </is>
+      </c>
+      <c r="X121" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="Y121" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="Z121" t="inlineStr">
+        <is>
+          <t>276</t>
+        </is>
+      </c>
+      <c r="AA121" t="inlineStr">
+        <is>
+          <t>1.4988</t>
+        </is>
+      </c>
+      <c r="AB121" t="inlineStr">
+        <is>
+          <t>7.2576</t>
+        </is>
+      </c>
+      <c r="AC121" t="inlineStr">
+        <is>
+          <t>38.0293</t>
+        </is>
+      </c>
+      <c r="AD121" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="AE121" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="AF121" t="inlineStr">
+        <is>
+          <t>0.2493</t>
+        </is>
+      </c>
+      <c r="AG121" t="inlineStr">
+        <is>
+          <t>0.8058</t>
+        </is>
+      </c>
+      <c r="AH121" t="inlineStr">
+        <is>
+          <t>0.0247</t>
+        </is>
+      </c>
+      <c r="AI121" t="inlineStr">
+        <is>
+          <t>0.1362</t>
+        </is>
+      </c>
+      <c r="AJ121" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK121" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AL121" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AM121" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN121" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO121" t="inlineStr">
+        <is>
+          <t>0.965</t>
+        </is>
+      </c>
+      <c r="AP121" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
       <c r="AQ121" t="inlineStr"/>
     </row>
@@ -25547,10 +25479,8 @@
           <t>iron_beam</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>6718</t>
-        </is>
+      <c r="E127" t="n">
+        <v>7244</v>
       </c>
       <c r="F127" t="inlineStr">
         <is>
@@ -25558,10 +25488,8 @@
         </is>
       </c>
       <c r="G127" t="inlineStr"/>
-      <c r="H127" t="inlineStr">
-        <is>
-          <t>91.2</t>
-        </is>
+      <c r="H127" t="n">
+        <v>89</v>
       </c>
       <c r="I127" t="inlineStr">
         <is>
@@ -25580,146 +25508,90 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N127" t="inlineStr">
-        <is>
-          <t>0.095</t>
-        </is>
-      </c>
-      <c r="O127" t="inlineStr">
-        <is>
-          <t>0.098</t>
-        </is>
+      <c r="N127" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="O127" t="n">
+        <v>0.033</v>
       </c>
       <c r="P127" t="inlineStr"/>
-      <c r="Q127" t="inlineStr">
-        <is>
-          <t>1.5439</t>
-        </is>
-      </c>
-      <c r="R127" t="inlineStr">
-        <is>
-          <t>0.2706</t>
-        </is>
-      </c>
-      <c r="S127" t="inlineStr">
-        <is>
-          <t>9.6281</t>
-        </is>
-      </c>
-      <c r="T127" t="inlineStr">
-        <is>
-          <t>0.0404</t>
-        </is>
-      </c>
-      <c r="U127" t="inlineStr">
-        <is>
-          <t>184</t>
-        </is>
-      </c>
-      <c r="V127" t="inlineStr">
-        <is>
-          <t>76</t>
-        </is>
-      </c>
-      <c r="W127" t="inlineStr">
-        <is>
-          <t>0.6969</t>
-        </is>
-      </c>
-      <c r="X127" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="Y127" t="inlineStr">
-        <is>
-          <t>114</t>
-        </is>
-      </c>
-      <c r="Z127" t="inlineStr">
-        <is>
-          <t>62</t>
-        </is>
-      </c>
-      <c r="AA127" t="inlineStr">
-        <is>
-          <t>1.0453</t>
-        </is>
-      </c>
-      <c r="AB127" t="inlineStr">
-        <is>
-          <t>0.5685</t>
-        </is>
-      </c>
-      <c r="AC127" t="inlineStr">
-        <is>
-          <t>109.0591</t>
-        </is>
-      </c>
-      <c r="AD127" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="AE127" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AF127" t="inlineStr">
-        <is>
-          <t>0.1694</t>
-        </is>
-      </c>
-      <c r="AG127" t="inlineStr">
-        <is>
-          <t>0.956</t>
-        </is>
-      </c>
-      <c r="AH127" t="inlineStr">
-        <is>
-          <t>0.0837</t>
-        </is>
-      </c>
-      <c r="AI127" t="inlineStr">
-        <is>
-          <t>0.1243</t>
-        </is>
-      </c>
-      <c r="AJ127" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AK127" t="inlineStr">
-        <is>
-          <t>0.769</t>
-        </is>
-      </c>
-      <c r="AL127" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AM127" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AN127" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AO127" t="inlineStr">
-        <is>
-          <t>0.797</t>
-        </is>
-      </c>
-      <c r="AP127" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="Q127" t="n">
+        <v>1.422</v>
+      </c>
+      <c r="R127" t="n">
+        <v>0.2886</v>
+      </c>
+      <c r="S127" t="n">
+        <v>9.959199999999999</v>
+      </c>
+      <c r="T127" t="n">
+        <v>0.0107</v>
+      </c>
+      <c r="U127" t="n">
+        <v>255</v>
+      </c>
+      <c r="V127" t="n">
+        <v>99</v>
+      </c>
+      <c r="W127" t="n">
+        <v>0.8507</v>
+      </c>
+      <c r="X127" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y127" t="n">
+        <v>167</v>
+      </c>
+      <c r="Z127" t="n">
+        <v>82</v>
+      </c>
+      <c r="AA127" t="n">
+        <v>1.4351</v>
+      </c>
+      <c r="AB127" t="n">
+        <v>0.7047</v>
+      </c>
+      <c r="AC127" t="n">
+        <v>116.369</v>
+      </c>
+      <c r="AD127" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE127" t="n">
+        <v>11</v>
+      </c>
+      <c r="AF127" t="n">
+        <v>0.2426</v>
+      </c>
+      <c r="AG127" t="n">
+        <v>0.9381</v>
+      </c>
+      <c r="AH127" t="n">
+        <v>0.0717</v>
+      </c>
+      <c r="AI127" t="n">
+        <v>0.1298</v>
+      </c>
+      <c r="AJ127" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK127" t="n">
+        <v>0.597</v>
+      </c>
+      <c r="AL127" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM127" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN127" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO127" t="n">
+        <v>0.9379999999999999</v>
+      </c>
+      <c r="AP127" t="n">
+        <v>1</v>
       </c>
       <c r="AQ127" t="inlineStr"/>
     </row>
@@ -25941,8 +25813,10 @@
           <t>kraken</t>
         </is>
       </c>
-      <c r="E129" t="n">
-        <v>61644</v>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>61644</t>
+        </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
@@ -25950,8 +25824,10 @@
         </is>
       </c>
       <c r="G129" t="inlineStr"/>
-      <c r="H129" t="n">
-        <v>100</v>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
@@ -25970,94 +25846,150 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N129" t="n">
-        <v>0.107</v>
-      </c>
-      <c r="O129" t="n">
-        <v>0.102</v>
+      <c r="N129" t="inlineStr">
+        <is>
+          <t>0.107</t>
+        </is>
+      </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>0.102</t>
+        </is>
       </c>
       <c r="P129" t="inlineStr">
         <is>
           <t>leviathan</t>
         </is>
       </c>
-      <c r="Q129" t="n">
-        <v>1.2757</v>
-      </c>
-      <c r="R129" t="n">
-        <v>0.1255</v>
-      </c>
-      <c r="S129" t="n">
-        <v>3.2459</v>
-      </c>
-      <c r="T129" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="U129" t="n">
-        <v>1624</v>
-      </c>
-      <c r="V129" t="n">
-        <v>224</v>
-      </c>
-      <c r="W129" t="n">
-        <v>2.501</v>
-      </c>
-      <c r="X129" t="n">
-        <v>26</v>
-      </c>
-      <c r="Y129" t="n">
-        <v>169</v>
-      </c>
-      <c r="Z129" t="n">
-        <v>1429</v>
-      </c>
-      <c r="AA129" t="n">
-        <v>1.8869</v>
-      </c>
-      <c r="AB129" t="n">
-        <v>15.9553</v>
-      </c>
-      <c r="AC129" t="n">
-        <v>89.5626</v>
-      </c>
-      <c r="AD129" t="n">
-        <v>4</v>
-      </c>
-      <c r="AE129" t="n">
-        <v>17</v>
-      </c>
-      <c r="AF129" t="n">
-        <v>0.2705</v>
-      </c>
-      <c r="AG129" t="n">
-        <v>0.8731</v>
-      </c>
-      <c r="AH129" t="n">
-        <v>0.0611</v>
-      </c>
-      <c r="AI129" t="n">
-        <v>0.0731</v>
-      </c>
-      <c r="AJ129" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK129" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL129" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM129" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN129" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO129" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP129" t="n">
-        <v>1</v>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>1.2757</t>
+        </is>
+      </c>
+      <c r="R129" t="inlineStr">
+        <is>
+          <t>0.1255</t>
+        </is>
+      </c>
+      <c r="S129" t="inlineStr">
+        <is>
+          <t>3.2459</t>
+        </is>
+      </c>
+      <c r="T129" t="inlineStr">
+        <is>
+          <t>0.045</t>
+        </is>
+      </c>
+      <c r="U129" t="inlineStr">
+        <is>
+          <t>1624</t>
+        </is>
+      </c>
+      <c r="V129" t="inlineStr">
+        <is>
+          <t>224</t>
+        </is>
+      </c>
+      <c r="W129" t="inlineStr">
+        <is>
+          <t>2.501</t>
+        </is>
+      </c>
+      <c r="X129" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="Y129" t="inlineStr">
+        <is>
+          <t>169</t>
+        </is>
+      </c>
+      <c r="Z129" t="inlineStr">
+        <is>
+          <t>1429</t>
+        </is>
+      </c>
+      <c r="AA129" t="inlineStr">
+        <is>
+          <t>1.8869</t>
+        </is>
+      </c>
+      <c r="AB129" t="inlineStr">
+        <is>
+          <t>15.9553</t>
+        </is>
+      </c>
+      <c r="AC129" t="inlineStr">
+        <is>
+          <t>89.5626</t>
+        </is>
+      </c>
+      <c r="AD129" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE129" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="AF129" t="inlineStr">
+        <is>
+          <t>0.2705</t>
+        </is>
+      </c>
+      <c r="AG129" t="inlineStr">
+        <is>
+          <t>0.8731</t>
+        </is>
+      </c>
+      <c r="AH129" t="inlineStr">
+        <is>
+          <t>0.0611</t>
+        </is>
+      </c>
+      <c r="AI129" t="inlineStr">
+        <is>
+          <t>0.0731</t>
+        </is>
+      </c>
+      <c r="AJ129" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK129" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AL129" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AM129" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN129" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO129" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AP129" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
       <c r="AQ129" t="inlineStr"/>
     </row>
@@ -27276,8 +27208,10 @@
           <t>leviathan</t>
         </is>
       </c>
-      <c r="E136" t="n">
-        <v>62916</v>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>62916</t>
+        </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
@@ -27285,8 +27219,10 @@
         </is>
       </c>
       <c r="G136" t="inlineStr"/>
-      <c r="H136" t="n">
-        <v>97.09999999999999</v>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>97.1</t>
+        </is>
       </c>
       <c r="I136" t="inlineStr">
         <is>
@@ -27305,94 +27241,150 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N136" t="n">
-        <v>0.101</v>
-      </c>
-      <c r="O136" t="n">
-        <v>0.098</v>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t>0.101</t>
+        </is>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>0.098</t>
+        </is>
       </c>
       <c r="P136" t="inlineStr">
         <is>
           <t>kraken</t>
         </is>
       </c>
-      <c r="Q136" t="n">
-        <v>1.4776</v>
-      </c>
-      <c r="R136" t="n">
-        <v>0.1626</v>
-      </c>
-      <c r="S136" t="n">
-        <v>4.2655</v>
-      </c>
-      <c r="T136" t="n">
-        <v>0.0925</v>
-      </c>
-      <c r="U136" t="n">
-        <v>1425</v>
-      </c>
-      <c r="V136" t="n">
-        <v>228</v>
-      </c>
-      <c r="W136" t="n">
-        <v>2.0871</v>
-      </c>
-      <c r="X136" t="n">
-        <v>34</v>
-      </c>
-      <c r="Y136" t="n">
-        <v>125</v>
-      </c>
-      <c r="Z136" t="n">
-        <v>1266</v>
-      </c>
-      <c r="AA136" t="n">
-        <v>1.1443</v>
-      </c>
-      <c r="AB136" t="n">
-        <v>11.5891</v>
-      </c>
-      <c r="AC136" t="n">
-        <v>109.2404</v>
-      </c>
-      <c r="AD136" t="n">
-        <v>4</v>
-      </c>
-      <c r="AE136" t="n">
-        <v>19</v>
-      </c>
-      <c r="AF136" t="n">
-        <v>0.2426</v>
-      </c>
-      <c r="AG136" t="n">
-        <v>0.8649</v>
-      </c>
-      <c r="AH136" t="n">
-        <v>0.0598</v>
-      </c>
-      <c r="AI136" t="n">
-        <v>0.1438</v>
-      </c>
-      <c r="AJ136" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK136" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL136" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM136" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN136" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO136" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="AP136" t="n">
-        <v>1</v>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>1.4776</t>
+        </is>
+      </c>
+      <c r="R136" t="inlineStr">
+        <is>
+          <t>0.1626</t>
+        </is>
+      </c>
+      <c r="S136" t="inlineStr">
+        <is>
+          <t>4.2655</t>
+        </is>
+      </c>
+      <c r="T136" t="inlineStr">
+        <is>
+          <t>0.0925</t>
+        </is>
+      </c>
+      <c r="U136" t="inlineStr">
+        <is>
+          <t>1425</t>
+        </is>
+      </c>
+      <c r="V136" t="inlineStr">
+        <is>
+          <t>228</t>
+        </is>
+      </c>
+      <c r="W136" t="inlineStr">
+        <is>
+          <t>2.0871</t>
+        </is>
+      </c>
+      <c r="X136" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="Y136" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="Z136" t="inlineStr">
+        <is>
+          <t>1266</t>
+        </is>
+      </c>
+      <c r="AA136" t="inlineStr">
+        <is>
+          <t>1.1443</t>
+        </is>
+      </c>
+      <c r="AB136" t="inlineStr">
+        <is>
+          <t>11.5891</t>
+        </is>
+      </c>
+      <c r="AC136" t="inlineStr">
+        <is>
+          <t>109.2404</t>
+        </is>
+      </c>
+      <c r="AD136" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AE136" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="AF136" t="inlineStr">
+        <is>
+          <t>0.2426</t>
+        </is>
+      </c>
+      <c r="AG136" t="inlineStr">
+        <is>
+          <t>0.8649</t>
+        </is>
+      </c>
+      <c r="AH136" t="inlineStr">
+        <is>
+          <t>0.0598</t>
+        </is>
+      </c>
+      <c r="AI136" t="inlineStr">
+        <is>
+          <t>0.1438</t>
+        </is>
+      </c>
+      <c r="AJ136" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK136" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AL136" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AM136" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN136" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO136" t="inlineStr">
+        <is>
+          <t>0.81</t>
+        </is>
+      </c>
+      <c r="AP136" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
       <c r="AQ136" t="inlineStr"/>
     </row>
@@ -33403,8 +33395,10 @@
           <t>nyx</t>
         </is>
       </c>
-      <c r="E167" t="n">
-        <v>17624</v>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>17624</t>
+        </is>
       </c>
       <c r="F167" t="inlineStr">
         <is>
@@ -33412,8 +33406,10 @@
         </is>
       </c>
       <c r="G167" t="inlineStr"/>
-      <c r="H167" t="n">
-        <v>90.3</v>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>90.3</t>
+        </is>
       </c>
       <c r="I167" t="inlineStr">
         <is>
@@ -33432,90 +33428,146 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N167" t="n">
-        <v>0.067</v>
-      </c>
-      <c r="O167" t="n">
-        <v>0.073</v>
+      <c r="N167" t="inlineStr">
+        <is>
+          <t>0.067</t>
+        </is>
+      </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>0.073</t>
+        </is>
       </c>
       <c r="P167" t="inlineStr"/>
-      <c r="Q167" t="n">
-        <v>1.3153</v>
-      </c>
-      <c r="R167" t="n">
-        <v>0.0975</v>
-      </c>
-      <c r="S167" t="n">
-        <v>2.1729</v>
-      </c>
-      <c r="T167" t="n">
-        <v>0.0342</v>
-      </c>
-      <c r="U167" t="n">
-        <v>513</v>
-      </c>
-      <c r="V167" t="n">
-        <v>108</v>
-      </c>
-      <c r="W167" t="n">
-        <v>1.2423</v>
-      </c>
-      <c r="X167" t="n">
-        <v>23</v>
-      </c>
-      <c r="Y167" t="n">
-        <v>114</v>
-      </c>
-      <c r="Z167" t="n">
-        <v>376</v>
-      </c>
-      <c r="AA167" t="n">
-        <v>1.3113</v>
-      </c>
-      <c r="AB167" t="n">
-        <v>4.3252</v>
-      </c>
-      <c r="AC167" t="n">
-        <v>86.93340000000001</v>
-      </c>
-      <c r="AD167" t="n">
-        <v>8</v>
-      </c>
-      <c r="AE167" t="n">
-        <v>15</v>
-      </c>
-      <c r="AF167" t="n">
-        <v>0.2918</v>
-      </c>
-      <c r="AG167" t="n">
-        <v>0.9288999999999999</v>
-      </c>
-      <c r="AH167" t="n">
-        <v>0.09470000000000001</v>
-      </c>
-      <c r="AI167" t="n">
-        <v>0.1551</v>
-      </c>
-      <c r="AJ167" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK167" t="n">
-        <v>0.874</v>
-      </c>
-      <c r="AL167" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM167" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN167" t="n">
-        <v>0.845</v>
-      </c>
-      <c r="AO167" t="n">
-        <v>0.772</v>
-      </c>
-      <c r="AP167" t="n">
-        <v>1</v>
+      <c r="Q167" t="inlineStr">
+        <is>
+          <t>1.3153</t>
+        </is>
+      </c>
+      <c r="R167" t="inlineStr">
+        <is>
+          <t>0.0975</t>
+        </is>
+      </c>
+      <c r="S167" t="inlineStr">
+        <is>
+          <t>2.1729</t>
+        </is>
+      </c>
+      <c r="T167" t="inlineStr">
+        <is>
+          <t>0.0342</t>
+        </is>
+      </c>
+      <c r="U167" t="inlineStr">
+        <is>
+          <t>513</t>
+        </is>
+      </c>
+      <c r="V167" t="inlineStr">
+        <is>
+          <t>108</t>
+        </is>
+      </c>
+      <c r="W167" t="inlineStr">
+        <is>
+          <t>1.2423</t>
+        </is>
+      </c>
+      <c r="X167" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="Y167" t="inlineStr">
+        <is>
+          <t>114</t>
+        </is>
+      </c>
+      <c r="Z167" t="inlineStr">
+        <is>
+          <t>376</t>
+        </is>
+      </c>
+      <c r="AA167" t="inlineStr">
+        <is>
+          <t>1.3113</t>
+        </is>
+      </c>
+      <c r="AB167" t="inlineStr">
+        <is>
+          <t>4.3252</t>
+        </is>
+      </c>
+      <c r="AC167" t="inlineStr">
+        <is>
+          <t>86.9334</t>
+        </is>
+      </c>
+      <c r="AD167" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AE167" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="AF167" t="inlineStr">
+        <is>
+          <t>0.2918</t>
+        </is>
+      </c>
+      <c r="AG167" t="inlineStr">
+        <is>
+          <t>0.9289</t>
+        </is>
+      </c>
+      <c r="AH167" t="inlineStr">
+        <is>
+          <t>0.0947</t>
+        </is>
+      </c>
+      <c r="AI167" t="inlineStr">
+        <is>
+          <t>0.1551</t>
+        </is>
+      </c>
+      <c r="AJ167" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK167" t="inlineStr">
+        <is>
+          <t>0.874</t>
+        </is>
+      </c>
+      <c r="AL167" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AM167" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN167" t="inlineStr">
+        <is>
+          <t>0.845</t>
+        </is>
+      </c>
+      <c r="AO167" t="inlineStr">
+        <is>
+          <t>0.772</t>
+        </is>
+      </c>
+      <c r="AP167" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
       <c r="AQ167" t="inlineStr"/>
     </row>
@@ -37934,8 +37986,10 @@
           <t>scylla</t>
         </is>
       </c>
-      <c r="E190" t="n">
-        <v>27262</v>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>27262</t>
+        </is>
       </c>
       <c r="F190" t="inlineStr">
         <is>
@@ -37943,8 +37997,10 @@
         </is>
       </c>
       <c r="G190" t="inlineStr"/>
-      <c r="H190" t="n">
-        <v>95.40000000000001</v>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>95.4</t>
+        </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
@@ -37963,90 +38019,146 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N190" t="n">
-        <v>0.024</v>
-      </c>
-      <c r="O190" t="n">
-        <v>0.029</v>
+      <c r="N190" t="inlineStr">
+        <is>
+          <t>0.024</t>
+        </is>
+      </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>0.029</t>
+        </is>
       </c>
       <c r="P190" t="inlineStr"/>
-      <c r="Q190" t="n">
-        <v>1.5907</v>
-      </c>
-      <c r="R190" t="n">
-        <v>0.1453</v>
-      </c>
-      <c r="S190" t="n">
-        <v>4.2883</v>
-      </c>
-      <c r="T190" t="n">
-        <v>0.026</v>
-      </c>
-      <c r="U190" t="n">
-        <v>681</v>
-      </c>
-      <c r="V190" t="n">
-        <v>132</v>
-      </c>
-      <c r="W190" t="n">
-        <v>1.3895</v>
-      </c>
-      <c r="X190" t="n">
-        <v>22</v>
-      </c>
-      <c r="Y190" t="n">
-        <v>103</v>
-      </c>
-      <c r="Z190" t="n">
-        <v>556</v>
-      </c>
-      <c r="AA190" t="n">
-        <v>1.0842</v>
-      </c>
-      <c r="AB190" t="n">
-        <v>5.8526</v>
-      </c>
-      <c r="AC190" t="n">
-        <v>95.001</v>
-      </c>
-      <c r="AD190" t="n">
-        <v>10</v>
-      </c>
-      <c r="AE190" t="n">
-        <v>15</v>
-      </c>
-      <c r="AF190" t="n">
-        <v>0.2786</v>
-      </c>
-      <c r="AG190" t="n">
-        <v>0.9041</v>
-      </c>
-      <c r="AH190" t="n">
-        <v>0.0605</v>
-      </c>
-      <c r="AI190" t="n">
-        <v>0.1652</v>
-      </c>
-      <c r="AJ190" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK190" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL190" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM190" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN190" t="n">
-        <v>0.921</v>
-      </c>
-      <c r="AO190" t="n">
-        <v>0.796</v>
-      </c>
-      <c r="AP190" t="n">
-        <v>1</v>
+      <c r="Q190" t="inlineStr">
+        <is>
+          <t>1.5907</t>
+        </is>
+      </c>
+      <c r="R190" t="inlineStr">
+        <is>
+          <t>0.1453</t>
+        </is>
+      </c>
+      <c r="S190" t="inlineStr">
+        <is>
+          <t>4.2883</t>
+        </is>
+      </c>
+      <c r="T190" t="inlineStr">
+        <is>
+          <t>0.026</t>
+        </is>
+      </c>
+      <c r="U190" t="inlineStr">
+        <is>
+          <t>681</t>
+        </is>
+      </c>
+      <c r="V190" t="inlineStr">
+        <is>
+          <t>132</t>
+        </is>
+      </c>
+      <c r="W190" t="inlineStr">
+        <is>
+          <t>1.3895</t>
+        </is>
+      </c>
+      <c r="X190" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="Y190" t="inlineStr">
+        <is>
+          <t>103</t>
+        </is>
+      </c>
+      <c r="Z190" t="inlineStr">
+        <is>
+          <t>556</t>
+        </is>
+      </c>
+      <c r="AA190" t="inlineStr">
+        <is>
+          <t>1.0842</t>
+        </is>
+      </c>
+      <c r="AB190" t="inlineStr">
+        <is>
+          <t>5.8526</t>
+        </is>
+      </c>
+      <c r="AC190" t="inlineStr">
+        <is>
+          <t>95.001</t>
+        </is>
+      </c>
+      <c r="AD190" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AE190" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="AF190" t="inlineStr">
+        <is>
+          <t>0.2786</t>
+        </is>
+      </c>
+      <c r="AG190" t="inlineStr">
+        <is>
+          <t>0.9041</t>
+        </is>
+      </c>
+      <c r="AH190" t="inlineStr">
+        <is>
+          <t>0.0605</t>
+        </is>
+      </c>
+      <c r="AI190" t="inlineStr">
+        <is>
+          <t>0.1652</t>
+        </is>
+      </c>
+      <c r="AJ190" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK190" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AL190" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AM190" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN190" t="inlineStr">
+        <is>
+          <t>0.921</t>
+        </is>
+      </c>
+      <c r="AO190" t="inlineStr">
+        <is>
+          <t>0.796</t>
+        </is>
+      </c>
+      <c r="AP190" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
       <c r="AQ190" t="inlineStr"/>
     </row>
@@ -41472,10 +41584,8 @@
           <t>stealth_naval_strike</t>
         </is>
       </c>
-      <c r="E208" t="inlineStr">
-        <is>
-          <t>3662</t>
-        </is>
+      <c r="E208" t="n">
+        <v>6704</v>
       </c>
       <c r="F208" t="inlineStr">
         <is>
@@ -41483,10 +41593,8 @@
         </is>
       </c>
       <c r="G208" t="inlineStr"/>
-      <c r="H208" t="inlineStr">
-        <is>
-          <t>77.0</t>
-        </is>
+      <c r="H208" t="n">
+        <v>73.90000000000001</v>
       </c>
       <c r="I208" t="inlineStr">
         <is>
@@ -41505,146 +41613,90 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N208" t="inlineStr">
-        <is>
-          <t>0.063</t>
-        </is>
-      </c>
-      <c r="O208" t="inlineStr">
-        <is>
-          <t>0.065</t>
-        </is>
+      <c r="N208" t="n">
+        <v>0</v>
+      </c>
+      <c r="O208" t="n">
+        <v>0</v>
       </c>
       <c r="P208" t="inlineStr"/>
-      <c r="Q208" t="inlineStr">
-        <is>
-          <t>1.0731</t>
-        </is>
-      </c>
-      <c r="R208" t="inlineStr">
-        <is>
-          <t>0.1616</t>
-        </is>
-      </c>
-      <c r="S208" t="inlineStr">
-        <is>
-          <t>2.5064</t>
-        </is>
-      </c>
-      <c r="T208" t="inlineStr">
-        <is>
-          <t>0.0077</t>
-        </is>
-      </c>
-      <c r="U208" t="inlineStr">
-        <is>
-          <t>199</t>
-        </is>
-      </c>
-      <c r="V208" t="inlineStr">
-        <is>
-          <t>67</t>
-        </is>
-      </c>
-      <c r="W208" t="inlineStr">
-        <is>
-          <t>1.836</t>
-        </is>
-      </c>
-      <c r="X208" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="Y208" t="inlineStr">
-        <is>
-          <t>96</t>
-        </is>
-      </c>
-      <c r="Z208" t="inlineStr">
-        <is>
-          <t>82</t>
-        </is>
-      </c>
-      <c r="AA208" t="inlineStr">
-        <is>
-          <t>2.6307</t>
-        </is>
-      </c>
-      <c r="AB208" t="inlineStr">
-        <is>
-          <t>2.2471</t>
-        </is>
-      </c>
-      <c r="AC208" t="inlineStr">
-        <is>
-          <t>36.4921</t>
-        </is>
-      </c>
-      <c r="AD208" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="AE208" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AF208" t="inlineStr">
-        <is>
-          <t>0.262</t>
-        </is>
-      </c>
-      <c r="AG208" t="inlineStr">
-        <is>
-          <t>0.8301</t>
-        </is>
-      </c>
-      <c r="AH208" t="inlineStr">
-        <is>
-          <t>0.0501</t>
-        </is>
-      </c>
-      <c r="AI208" t="inlineStr">
-        <is>
-          <t>0.0595</t>
-        </is>
-      </c>
-      <c r="AJ208" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AK208" t="inlineStr">
-        <is>
-          <t>0.172</t>
-        </is>
-      </c>
-      <c r="AL208" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AM208" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AN208" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AO208" t="inlineStr">
-        <is>
-          <t>0.845</t>
-        </is>
-      </c>
-      <c r="AP208" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="Q208" t="n">
+        <v>1.0784</v>
+      </c>
+      <c r="R208" t="n">
+        <v>0.137</v>
+      </c>
+      <c r="S208" t="n">
+        <v>3.1341</v>
+      </c>
+      <c r="T208" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="U208" t="n">
+        <v>231</v>
+      </c>
+      <c r="V208" t="n">
+        <v>89</v>
+      </c>
+      <c r="W208" t="n">
+        <v>1.8954</v>
+      </c>
+      <c r="X208" t="n">
+        <v>10</v>
+      </c>
+      <c r="Y208" t="n">
+        <v>63</v>
+      </c>
+      <c r="Z208" t="n">
+        <v>158</v>
+      </c>
+      <c r="AA208" t="n">
+        <v>1.3417</v>
+      </c>
+      <c r="AB208" t="n">
+        <v>3.3648</v>
+      </c>
+      <c r="AC208" t="n">
+        <v>46.9564</v>
+      </c>
+      <c r="AD208" t="n">
+        <v>12</v>
+      </c>
+      <c r="AE208" t="n">
+        <v>9</v>
+      </c>
+      <c r="AF208" t="n">
+        <v>0.4338</v>
+      </c>
+      <c r="AG208" t="n">
+        <v>0.8216</v>
+      </c>
+      <c r="AH208" t="n">
+        <v>0.0486</v>
+      </c>
+      <c r="AI208" t="n">
+        <v>0.1024</v>
+      </c>
+      <c r="AJ208" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK208" t="n">
+        <v>0.184</v>
+      </c>
+      <c r="AL208" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM208" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN208" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO208" t="n">
+        <v>0.953</v>
+      </c>
+      <c r="AP208" t="n">
+        <v>0.5</v>
       </c>
       <c r="AQ208" t="inlineStr"/>
     </row>
@@ -46039,10 +46091,8 @@
           <t>wheeled_gun</t>
         </is>
       </c>
-      <c r="E231" t="inlineStr">
-        <is>
-          <t>7178</t>
-        </is>
+      <c r="E231" t="n">
+        <v>7190</v>
       </c>
       <c r="F231" t="inlineStr">
         <is>
@@ -46050,10 +46100,8 @@
         </is>
       </c>
       <c r="G231" t="inlineStr"/>
-      <c r="H231" t="inlineStr">
-        <is>
-          <t>90.3</t>
-        </is>
+      <c r="H231" t="n">
+        <v>91.09999999999999</v>
       </c>
       <c r="I231" t="inlineStr">
         <is>
@@ -46072,150 +46120,90 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N231" t="inlineStr">
-        <is>
-          <t>0.227</t>
-        </is>
-      </c>
-      <c r="O231" t="inlineStr">
-        <is>
-          <t>0.021</t>
-        </is>
-      </c>
-      <c r="P231" t="inlineStr">
-        <is>
-          <t>heavy_tank</t>
-        </is>
-      </c>
-      <c r="Q231" t="inlineStr">
-        <is>
-          <t>1.4696</t>
-        </is>
-      </c>
-      <c r="R231" t="inlineStr">
-        <is>
-          <t>0.2793</t>
-        </is>
-      </c>
-      <c r="S231" t="inlineStr">
-        <is>
-          <t>11.039</t>
-        </is>
-      </c>
-      <c r="T231" t="inlineStr">
-        <is>
-          <t>0.0195</t>
-        </is>
-      </c>
-      <c r="U231" t="inlineStr">
-        <is>
-          <t>160</t>
-        </is>
-      </c>
-      <c r="V231" t="inlineStr">
-        <is>
-          <t>71</t>
-        </is>
-      </c>
-      <c r="W231" t="inlineStr">
-        <is>
-          <t>1.0002</t>
-        </is>
-      </c>
-      <c r="X231" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="Y231" t="inlineStr">
-        <is>
-          <t>69</t>
-        </is>
-      </c>
-      <c r="Z231" t="inlineStr">
-        <is>
-          <t>86</t>
-        </is>
-      </c>
-      <c r="AA231" t="inlineStr">
-        <is>
-          <t>0.9721</t>
-        </is>
-      </c>
-      <c r="AB231" t="inlineStr">
-        <is>
-          <t>1.2115</t>
-        </is>
-      </c>
-      <c r="AC231" t="inlineStr">
-        <is>
-          <t>70.9836</t>
-        </is>
-      </c>
-      <c r="AD231" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="AE231" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="AF231" t="inlineStr">
-        <is>
-          <t>0.129</t>
-        </is>
-      </c>
-      <c r="AG231" t="inlineStr">
-        <is>
-          <t>0.9816</t>
-        </is>
-      </c>
-      <c r="AH231" t="inlineStr">
-        <is>
-          <t>0.1013</t>
-        </is>
-      </c>
-      <c r="AI231" t="inlineStr">
-        <is>
-          <t>0.2437</t>
-        </is>
-      </c>
-      <c r="AJ231" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AK231" t="inlineStr">
-        <is>
-          <t>0.664</t>
-        </is>
-      </c>
-      <c r="AL231" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AM231" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AN231" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AO231" t="inlineStr">
-        <is>
-          <t>0.913</t>
-        </is>
-      </c>
-      <c r="AP231" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="N231" t="n">
+        <v>0.057</v>
+      </c>
+      <c r="O231" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="P231" t="inlineStr"/>
+      <c r="Q231" t="n">
+        <v>1.4551</v>
+      </c>
+      <c r="R231" t="n">
+        <v>0.3137</v>
+      </c>
+      <c r="S231" t="n">
+        <v>10.5824</v>
+      </c>
+      <c r="T231" t="n">
+        <v>0.0363</v>
+      </c>
+      <c r="U231" t="n">
+        <v>216</v>
+      </c>
+      <c r="V231" t="n">
+        <v>97</v>
+      </c>
+      <c r="W231" t="n">
+        <v>1.3837</v>
+      </c>
+      <c r="X231" t="n">
+        <v>8</v>
+      </c>
+      <c r="Y231" t="n">
+        <v>87</v>
+      </c>
+      <c r="Z231" t="n">
+        <v>121</v>
+      </c>
+      <c r="AA231" t="n">
+        <v>1.2411</v>
+      </c>
+      <c r="AB231" t="n">
+        <v>1.7261</v>
+      </c>
+      <c r="AC231" t="n">
+        <v>70.10129999999999</v>
+      </c>
+      <c r="AD231" t="n">
+        <v>8</v>
+      </c>
+      <c r="AE231" t="n">
+        <v>13</v>
+      </c>
+      <c r="AF231" t="n">
+        <v>0.2305</v>
+      </c>
+      <c r="AG231" t="n">
+        <v>0.9399</v>
+      </c>
+      <c r="AH231" t="n">
+        <v>0.0774</v>
+      </c>
+      <c r="AI231" t="n">
+        <v>0.1858</v>
+      </c>
+      <c r="AJ231" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK231" t="n">
+        <v>0.644</v>
+      </c>
+      <c r="AL231" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM231" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN231" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO231" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP231" t="n">
+        <v>1</v>
       </c>
       <c r="AQ231" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Play-test 14 wave R3: bespoke weapons on the five ground bosses
Jotunn, Bastion, Bastion Mk.0, Fenrir, Inferno: own turrets, barrels, launchers, flak, radars, hatches (mb_pt14_r3.py).
Pivots unchanged; no data change. DECISIONS 'Play-test 14 boss redraw R3 (lane models)'.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/models/quality_report.xlsx
+++ b/Docs/models/quality_report.xlsx
@@ -4475,7 +4475,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>35481</t>
+          <t>39357</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -4508,49 +4508,49 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>0.014</t>
+          <t>0.011</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>0.014</t>
+          <t>0.007</t>
         </is>
       </c>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>1.7964</t>
+          <t>1.8338</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>0.1892</t>
+          <t>0.187</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>5.2398</t>
+          <t>4.9846</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>0.0255</t>
+          <t>0.0351</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr">
         <is>
-          <t>1291</t>
+          <t>1455</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>156</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>0.6503</t>
+          <t>0.687</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
@@ -4560,27 +4560,27 @@
       </c>
       <c r="Z21" t="inlineStr">
         <is>
-          <t>420</t>
+          <t>425</t>
         </is>
       </c>
       <c r="AA21" t="inlineStr">
         <is>
-          <t>846</t>
+          <t>1005</t>
         </is>
       </c>
       <c r="AB21" t="inlineStr">
         <is>
-          <t>1.8331</t>
+          <t>1.8717</t>
         </is>
       </c>
       <c r="AC21" t="inlineStr">
         <is>
-          <t>3.6924</t>
+          <t>4.426</t>
         </is>
       </c>
       <c r="AD21" t="inlineStr">
         <is>
-          <t>229.1202</t>
+          <t>227.0654</t>
         </is>
       </c>
       <c r="AE21" t="inlineStr">
@@ -4595,22 +4595,22 @@
       </c>
       <c r="AG21" t="inlineStr">
         <is>
-          <t>0.2307</t>
+          <t>0.242</t>
         </is>
       </c>
       <c r="AH21" t="inlineStr">
         <is>
-          <t>0.8064</t>
+          <t>0.8058</t>
         </is>
       </c>
       <c r="AI21" t="inlineStr">
         <is>
-          <t>0.0348</t>
+          <t>0.0299</t>
         </is>
       </c>
       <c r="AJ21" t="inlineStr">
         <is>
-          <t>0.1637</t>
+          <t>0.136</t>
         </is>
       </c>
       <c r="AK21" t="inlineStr">
@@ -4869,7 +4869,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>33342</t>
+          <t>38564</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -4880,7 +4880,7 @@
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
-          <t>96.4</t>
+          <t>96.6</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -4902,49 +4902,49 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>0.02</t>
+          <t>0.008</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>0.036</t>
+          <t>0.014</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>1.6967</t>
+          <t>1.6981</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>0.181</t>
+          <t>0.1894</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>5.1447</t>
+          <t>5.0411</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.0703</t>
+          <t>0.0603</t>
         </is>
       </c>
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr">
         <is>
-          <t>965</t>
+          <t>1048</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>174</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.5468</t>
+          <t>0.6036</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
@@ -4954,27 +4954,27 @@
       </c>
       <c r="Z23" t="inlineStr">
         <is>
-          <t>419</t>
+          <t>438</t>
         </is>
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>528</t>
+          <t>592</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
         <is>
-          <t>1.4781</t>
+          <t>1.5195</t>
         </is>
       </c>
       <c r="AC23" t="inlineStr">
         <is>
-          <t>1.8627</t>
+          <t>2.0538</t>
         </is>
       </c>
       <c r="AD23" t="inlineStr">
         <is>
-          <t>283.4649</t>
+          <t>288.2473</t>
         </is>
       </c>
       <c r="AE23" t="inlineStr">
@@ -4989,7 +4989,7 @@
       </c>
       <c r="AG23" t="inlineStr">
         <is>
-          <t>0.2401</t>
+          <t>0.2459</t>
         </is>
       </c>
       <c r="AH23" t="inlineStr">
@@ -4999,12 +4999,12 @@
       </c>
       <c r="AI23" t="inlineStr">
         <is>
-          <t>0.0431</t>
+          <t>0.0421</t>
         </is>
       </c>
       <c r="AJ23" t="inlineStr">
         <is>
-          <t>0.1747</t>
+          <t>0.1583</t>
         </is>
       </c>
       <c r="AK23" t="inlineStr">
@@ -5014,7 +5014,7 @@
       </c>
       <c r="AL23" t="inlineStr">
         <is>
-          <t>0.876</t>
+          <t>0.878</t>
         </is>
       </c>
       <c r="AM23" t="inlineStr">
@@ -5034,7 +5034,7 @@
       </c>
       <c r="AP23" t="inlineStr">
         <is>
-          <t>0.967</t>
+          <t>0.98</t>
         </is>
       </c>
       <c r="AQ23" t="inlineStr">
@@ -12049,7 +12049,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>30712</t>
+          <t>33588</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -12060,7 +12060,7 @@
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
-          <t>94.6</t>
+          <t>95.7</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -12082,28 +12082,28 @@
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>0.008</t>
+          <t>0.005</t>
         </is>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>0.027</t>
+          <t>0.016</t>
         </is>
       </c>
       <c r="P59" t="inlineStr"/>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>1.6233</t>
+          <t>1.6573</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>0.1887</t>
+          <t>0.2028</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>6.3611</t>
+          <t>6.56</t>
         </is>
       </c>
       <c r="T59" t="inlineStr">
@@ -12114,17 +12114,17 @@
       <c r="U59" t="inlineStr"/>
       <c r="V59" t="inlineStr">
         <is>
-          <t>942</t>
+          <t>1034</t>
         </is>
       </c>
       <c r="W59" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>169</t>
         </is>
       </c>
       <c r="X59" t="inlineStr">
         <is>
-          <t>0.863</t>
+          <t>1.0114</t>
         </is>
       </c>
       <c r="Y59" t="inlineStr">
@@ -12134,27 +12134,27 @@
       </c>
       <c r="Z59" t="inlineStr">
         <is>
-          <t>349</t>
+          <t>386</t>
         </is>
       </c>
       <c r="AA59" t="inlineStr">
         <is>
-          <t>570</t>
+          <t>625</t>
         </is>
       </c>
       <c r="AB59" t="inlineStr">
         <is>
-          <t>2.1061</t>
+          <t>2.31</t>
         </is>
       </c>
       <c r="AC59" t="inlineStr">
         <is>
-          <t>3.4397</t>
+          <t>3.7402</t>
         </is>
       </c>
       <c r="AD59" t="inlineStr">
         <is>
-          <t>165.7105</t>
+          <t>167.1012</t>
         </is>
       </c>
       <c r="AE59" t="inlineStr">
@@ -12169,22 +12169,22 @@
       </c>
       <c r="AG59" t="inlineStr">
         <is>
-          <t>0.2661</t>
+          <t>0.2708</t>
         </is>
       </c>
       <c r="AH59" t="inlineStr">
         <is>
-          <t>0.8143</t>
+          <t>0.8137</t>
         </is>
       </c>
       <c r="AI59" t="inlineStr">
         <is>
-          <t>0.0443</t>
+          <t>0.0397</t>
         </is>
       </c>
       <c r="AJ59" t="inlineStr">
         <is>
-          <t>0.1231</t>
+          <t>0.1313</t>
         </is>
       </c>
       <c r="AK59" t="inlineStr">
@@ -12194,7 +12194,7 @@
       </c>
       <c r="AL59" t="inlineStr">
         <is>
-          <t>0.784</t>
+          <t>0.826</t>
         </is>
       </c>
       <c r="AM59" t="inlineStr">
@@ -13249,10 +13249,8 @@
           <t>fortress_bastion</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>56092</t>
-        </is>
+      <c r="E65" t="n">
+        <v>60706</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
@@ -13260,10 +13258,8 @@
         </is>
       </c>
       <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
+      <c r="H65" t="n">
+        <v>100</v>
       </c>
       <c r="I65" t="inlineStr">
         <is>
@@ -13282,147 +13278,91 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N65" t="inlineStr">
-        <is>
-          <t>0.028</t>
-        </is>
-      </c>
-      <c r="O65" t="inlineStr">
-        <is>
-          <t>0.039</t>
-        </is>
+      <c r="N65" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="O65" t="n">
+        <v>0.007</v>
       </c>
       <c r="P65" t="inlineStr"/>
-      <c r="Q65" t="inlineStr">
-        <is>
-          <t>1.8452</t>
-        </is>
-      </c>
-      <c r="R65" t="inlineStr">
-        <is>
-          <t>0.1728</t>
-        </is>
-      </c>
-      <c r="S65" t="inlineStr">
-        <is>
-          <t>5.887</t>
-        </is>
-      </c>
-      <c r="T65" t="inlineStr">
-        <is>
-          <t>0.034</t>
-        </is>
+      <c r="Q65" t="n">
+        <v>1.8343</v>
+      </c>
+      <c r="R65" t="n">
+        <v>0.1876</v>
+      </c>
+      <c r="S65" t="n">
+        <v>6.4327</v>
+      </c>
+      <c r="T65" t="n">
+        <v>0.0201</v>
       </c>
       <c r="U65" t="inlineStr"/>
-      <c r="V65" t="inlineStr">
-        <is>
-          <t>1609</t>
-        </is>
-      </c>
-      <c r="W65" t="inlineStr">
-        <is>
-          <t>183</t>
-        </is>
-      </c>
-      <c r="X65" t="inlineStr">
-        <is>
-          <t>1.2447</t>
-        </is>
-      </c>
-      <c r="Y65" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="Z65" t="inlineStr">
-        <is>
-          <t>261</t>
-        </is>
-      </c>
-      <c r="AA65" t="inlineStr">
-        <is>
-          <t>1342</t>
-        </is>
-      </c>
-      <c r="AB65" t="inlineStr">
-        <is>
-          <t>1.7752</t>
-        </is>
-      </c>
-      <c r="AC65" t="inlineStr">
-        <is>
-          <t>9.1275</t>
-        </is>
-      </c>
-      <c r="AD65" t="inlineStr">
-        <is>
-          <t>147.0282</t>
-        </is>
-      </c>
-      <c r="AE65" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="AF65" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="AG65" t="inlineStr">
-        <is>
-          <t>0.2389</t>
-        </is>
-      </c>
-      <c r="AH65" t="inlineStr">
-        <is>
-          <t>0.8867</t>
-        </is>
-      </c>
-      <c r="AI65" t="inlineStr">
-        <is>
-          <t>0.0626</t>
-        </is>
-      </c>
-      <c r="AJ65" t="inlineStr">
-        <is>
-          <t>0.1999</t>
-        </is>
-      </c>
-      <c r="AK65" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AL65" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AM65" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AN65" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AO65" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AP65" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AQ65" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="V65" t="n">
+        <v>1683</v>
+      </c>
+      <c r="W65" t="n">
+        <v>201</v>
+      </c>
+      <c r="X65" t="n">
+        <v>1.345</v>
+      </c>
+      <c r="Y65" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z65" t="n">
+        <v>270</v>
+      </c>
+      <c r="AA65" t="n">
+        <v>1407</v>
+      </c>
+      <c r="AB65" t="n">
+        <v>1.8068</v>
+      </c>
+      <c r="AC65" t="n">
+        <v>9.4152</v>
+      </c>
+      <c r="AD65" t="n">
+        <v>149.4394</v>
+      </c>
+      <c r="AE65" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF65" t="n">
+        <v>20</v>
+      </c>
+      <c r="AG65" t="n">
+        <v>0.2462</v>
+      </c>
+      <c r="AH65" t="n">
+        <v>0.8778</v>
+      </c>
+      <c r="AI65" t="n">
+        <v>0.0586</v>
+      </c>
+      <c r="AJ65" t="n">
+        <v>0.1967</v>
+      </c>
+      <c r="AK65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL65" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM65" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN65" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO65" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP65" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ65" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="66">
@@ -18254,8 +18194,10 @@
           <t>icarus_mk0</t>
         </is>
       </c>
-      <c r="E90" t="n">
-        <v>28148</v>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>28148</t>
+        </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -18263,8 +18205,10 @@
         </is>
       </c>
       <c r="G90" t="inlineStr"/>
-      <c r="H90" t="n">
-        <v>94.59999999999999</v>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>94.6</t>
+        </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
@@ -18283,91 +18227,147 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N90" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="O90" t="n">
-        <v>0.01</v>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
       </c>
       <c r="P90" t="inlineStr"/>
-      <c r="Q90" t="n">
-        <v>1.6358</v>
-      </c>
-      <c r="R90" t="n">
-        <v>0.1983</v>
-      </c>
-      <c r="S90" t="n">
-        <v>5.8141</v>
-      </c>
-      <c r="T90" t="n">
-        <v>0.033</v>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>1.6358</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>0.1983</t>
+        </is>
+      </c>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>5.8141</t>
+        </is>
+      </c>
+      <c r="T90" t="inlineStr">
+        <is>
+          <t>0.033</t>
+        </is>
       </c>
       <c r="U90" t="inlineStr"/>
-      <c r="V90" t="n">
-        <v>767</v>
-      </c>
-      <c r="W90" t="n">
-        <v>242</v>
-      </c>
-      <c r="X90" t="n">
-        <v>3.1061</v>
-      </c>
-      <c r="Y90" t="n">
-        <v>22</v>
-      </c>
-      <c r="Z90" t="n">
-        <v>205</v>
-      </c>
-      <c r="AA90" t="n">
-        <v>540</v>
-      </c>
-      <c r="AB90" t="n">
-        <v>2.6312</v>
-      </c>
-      <c r="AC90" t="n">
-        <v>6.931</v>
-      </c>
-      <c r="AD90" t="n">
-        <v>77.9111</v>
-      </c>
-      <c r="AE90" t="n">
-        <v>18</v>
-      </c>
-      <c r="AF90" t="n">
-        <v>20</v>
-      </c>
-      <c r="AG90" t="n">
-        <v>0.1809</v>
-      </c>
-      <c r="AH90" t="n">
-        <v>0.8567</v>
-      </c>
-      <c r="AI90" t="n">
-        <v>0.0513</v>
-      </c>
-      <c r="AJ90" t="n">
-        <v>-0.0344</v>
-      </c>
-      <c r="AK90" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL90" t="n">
-        <v>0.785</v>
-      </c>
-      <c r="AM90" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN90" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO90" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP90" t="n">
-        <v>1</v>
-      </c>
-      <c r="AQ90" t="n">
-        <v>1</v>
+      <c r="V90" t="inlineStr">
+        <is>
+          <t>767</t>
+        </is>
+      </c>
+      <c r="W90" t="inlineStr">
+        <is>
+          <t>242</t>
+        </is>
+      </c>
+      <c r="X90" t="inlineStr">
+        <is>
+          <t>3.1061</t>
+        </is>
+      </c>
+      <c r="Y90" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="Z90" t="inlineStr">
+        <is>
+          <t>205</t>
+        </is>
+      </c>
+      <c r="AA90" t="inlineStr">
+        <is>
+          <t>540</t>
+        </is>
+      </c>
+      <c r="AB90" t="inlineStr">
+        <is>
+          <t>2.6312</t>
+        </is>
+      </c>
+      <c r="AC90" t="inlineStr">
+        <is>
+          <t>6.931</t>
+        </is>
+      </c>
+      <c r="AD90" t="inlineStr">
+        <is>
+          <t>77.9111</t>
+        </is>
+      </c>
+      <c r="AE90" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="AF90" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="AG90" t="inlineStr">
+        <is>
+          <t>0.1809</t>
+        </is>
+      </c>
+      <c r="AH90" t="inlineStr">
+        <is>
+          <t>0.8567</t>
+        </is>
+      </c>
+      <c r="AI90" t="inlineStr">
+        <is>
+          <t>0.0513</t>
+        </is>
+      </c>
+      <c r="AJ90" t="inlineStr">
+        <is>
+          <t>-0.0344</t>
+        </is>
+      </c>
+      <c r="AK90" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL90" t="inlineStr">
+        <is>
+          <t>0.785</t>
+        </is>
+      </c>
+      <c r="AM90" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN90" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO90" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AP90" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AQ90" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
     </row>
     <row r="91">
@@ -19983,8 +19983,10 @@
           <t>leviathan</t>
         </is>
       </c>
-      <c r="E99" t="n">
-        <v>86412</v>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>86412</t>
+        </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -19992,8 +19994,10 @@
         </is>
       </c>
       <c r="G99" t="inlineStr"/>
-      <c r="H99" t="n">
-        <v>97.7</v>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>97.7</t>
+        </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
@@ -20012,91 +20016,147 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N99" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="O99" t="n">
-        <v>0.002</v>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>0.002</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>0.002</t>
+        </is>
       </c>
       <c r="P99" t="inlineStr"/>
-      <c r="Q99" t="n">
-        <v>1.4402</v>
-      </c>
-      <c r="R99" t="n">
-        <v>0.1709</v>
-      </c>
-      <c r="S99" t="n">
-        <v>4.5164</v>
-      </c>
-      <c r="T99" t="n">
-        <v>0.0925</v>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>1.4402</t>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>0.1709</t>
+        </is>
+      </c>
+      <c r="S99" t="inlineStr">
+        <is>
+          <t>4.5164</t>
+        </is>
+      </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>0.0925</t>
+        </is>
       </c>
       <c r="U99" t="inlineStr"/>
-      <c r="V99" t="n">
-        <v>1784</v>
-      </c>
-      <c r="W99" t="n">
-        <v>247</v>
-      </c>
-      <c r="X99" t="n">
-        <v>2.2347</v>
-      </c>
-      <c r="Y99" t="n">
-        <v>34</v>
-      </c>
-      <c r="Z99" t="n">
-        <v>142</v>
-      </c>
-      <c r="AA99" t="n">
-        <v>1608</v>
-      </c>
-      <c r="AB99" t="n">
-        <v>1.2847</v>
-      </c>
-      <c r="AC99" t="n">
-        <v>14.5482</v>
-      </c>
-      <c r="AD99" t="n">
-        <v>110.529</v>
-      </c>
-      <c r="AE99" t="n">
-        <v>4</v>
-      </c>
-      <c r="AF99" t="n">
-        <v>19</v>
-      </c>
-      <c r="AG99" t="n">
-        <v>0.2652</v>
-      </c>
-      <c r="AH99" t="n">
-        <v>0.8561</v>
-      </c>
-      <c r="AI99" t="n">
-        <v>0.0601</v>
-      </c>
-      <c r="AJ99" t="n">
-        <v>0.1499</v>
-      </c>
-      <c r="AK99" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL99" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM99" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN99" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO99" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP99" t="n">
-        <v>0.848</v>
-      </c>
-      <c r="AQ99" t="n">
-        <v>1</v>
+      <c r="V99" t="inlineStr">
+        <is>
+          <t>1784</t>
+        </is>
+      </c>
+      <c r="W99" t="inlineStr">
+        <is>
+          <t>247</t>
+        </is>
+      </c>
+      <c r="X99" t="inlineStr">
+        <is>
+          <t>2.2347</t>
+        </is>
+      </c>
+      <c r="Y99" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="Z99" t="inlineStr">
+        <is>
+          <t>142</t>
+        </is>
+      </c>
+      <c r="AA99" t="inlineStr">
+        <is>
+          <t>1608</t>
+        </is>
+      </c>
+      <c r="AB99" t="inlineStr">
+        <is>
+          <t>1.2847</t>
+        </is>
+      </c>
+      <c r="AC99" t="inlineStr">
+        <is>
+          <t>14.5482</t>
+        </is>
+      </c>
+      <c r="AD99" t="inlineStr">
+        <is>
+          <t>110.529</t>
+        </is>
+      </c>
+      <c r="AE99" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AF99" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="AG99" t="inlineStr">
+        <is>
+          <t>0.2652</t>
+        </is>
+      </c>
+      <c r="AH99" t="inlineStr">
+        <is>
+          <t>0.8561</t>
+        </is>
+      </c>
+      <c r="AI99" t="inlineStr">
+        <is>
+          <t>0.0601</t>
+        </is>
+      </c>
+      <c r="AJ99" t="inlineStr">
+        <is>
+          <t>0.1499</t>
+        </is>
+      </c>
+      <c r="AK99" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL99" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AM99" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN99" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO99" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AP99" t="inlineStr">
+        <is>
+          <t>0.848</t>
+        </is>
+      </c>
+      <c r="AQ99" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
     </row>
     <row r="100">
@@ -23133,7 +23193,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>55236</t>
+          <t>67060</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -23166,49 +23226,49 @@
       </c>
       <c r="N115" t="inlineStr">
         <is>
-          <t>0.013</t>
+          <t>0.006</t>
         </is>
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>0.029</t>
+          <t>0.009</t>
         </is>
       </c>
       <c r="P115" t="inlineStr"/>
       <c r="Q115" t="inlineStr">
         <is>
-          <t>2.4311</t>
+          <t>2.4227</t>
         </is>
       </c>
       <c r="R115" t="inlineStr">
         <is>
-          <t>0.2018</t>
+          <t>0.2322</t>
         </is>
       </c>
       <c r="S115" t="inlineStr">
         <is>
-          <t>6.0667</t>
+          <t>7.9931</t>
         </is>
       </c>
       <c r="T115" t="inlineStr">
         <is>
-          <t>0.199</t>
+          <t>0.1979</t>
         </is>
       </c>
       <c r="U115" t="inlineStr"/>
       <c r="V115" t="inlineStr">
         <is>
-          <t>1550</t>
+          <t>1757</t>
         </is>
       </c>
       <c r="W115" t="inlineStr">
         <is>
-          <t>159</t>
+          <t>204</t>
         </is>
       </c>
       <c r="X115" t="inlineStr">
         <is>
-          <t>0.7494</t>
+          <t>0.8792</t>
         </is>
       </c>
       <c r="Y115" t="inlineStr">
@@ -23218,32 +23278,32 @@
       </c>
       <c r="Z115" t="inlineStr">
         <is>
-          <t>471</t>
+          <t>551</t>
         </is>
       </c>
       <c r="AA115" t="inlineStr">
         <is>
-          <t>1060</t>
+          <t>1187</t>
         </is>
       </c>
       <c r="AB115" t="inlineStr">
         <is>
-          <t>2.2199</t>
+          <t>2.3748</t>
         </is>
       </c>
       <c r="AC115" t="inlineStr">
         <is>
-          <t>4.996</t>
+          <t>5.1159</t>
         </is>
       </c>
       <c r="AD115" t="inlineStr">
         <is>
-          <t>212.1676</t>
+          <t>232.0215</t>
         </is>
       </c>
       <c r="AE115" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="AF115" t="inlineStr">
@@ -23253,7 +23313,7 @@
       </c>
       <c r="AG115" t="inlineStr">
         <is>
-          <t>0.2828</t>
+          <t>0.2786</t>
         </is>
       </c>
       <c r="AH115" t="inlineStr">
@@ -23263,12 +23323,12 @@
       </c>
       <c r="AI115" t="inlineStr">
         <is>
-          <t>0.0368</t>
+          <t>0.0344</t>
         </is>
       </c>
       <c r="AJ115" t="inlineStr">
         <is>
-          <t>0.1436</t>
+          <t>0.1293</t>
         </is>
       </c>
       <c r="AK115" t="inlineStr">
@@ -24317,8 +24377,10 @@
           <t>nyx</t>
         </is>
       </c>
-      <c r="E121" t="n">
-        <v>17028</v>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>17028</t>
+        </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
@@ -24326,8 +24388,10 @@
         </is>
       </c>
       <c r="G121" t="inlineStr"/>
-      <c r="H121" t="n">
-        <v>93.5</v>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>93.5</t>
+        </is>
       </c>
       <c r="I121" t="inlineStr">
         <is>
@@ -24346,91 +24410,147 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N121" t="n">
-        <v>0.008999999999999999</v>
-      </c>
-      <c r="O121" t="n">
-        <v>0.01</v>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>0.009</t>
+        </is>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
       </c>
       <c r="P121" t="inlineStr"/>
-      <c r="Q121" t="n">
-        <v>1.3616</v>
-      </c>
-      <c r="R121" t="n">
-        <v>0.0988</v>
-      </c>
-      <c r="S121" t="n">
-        <v>2.2773</v>
-      </c>
-      <c r="T121" t="n">
-        <v>0.0342</v>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t>1.3616</t>
+        </is>
+      </c>
+      <c r="R121" t="inlineStr">
+        <is>
+          <t>0.0988</t>
+        </is>
+      </c>
+      <c r="S121" t="inlineStr">
+        <is>
+          <t>2.2773</t>
+        </is>
+      </c>
+      <c r="T121" t="inlineStr">
+        <is>
+          <t>0.0342</t>
+        </is>
       </c>
       <c r="U121" t="inlineStr"/>
-      <c r="V121" t="n">
-        <v>526</v>
-      </c>
-      <c r="W121" t="n">
-        <v>110</v>
-      </c>
-      <c r="X121" t="n">
-        <v>1.2705</v>
-      </c>
-      <c r="Y121" t="n">
-        <v>23</v>
-      </c>
-      <c r="Z121" t="n">
-        <v>103</v>
-      </c>
-      <c r="AA121" t="n">
-        <v>400</v>
-      </c>
-      <c r="AB121" t="n">
-        <v>1.1897</v>
-      </c>
-      <c r="AC121" t="n">
-        <v>4.62</v>
-      </c>
-      <c r="AD121" t="n">
-        <v>86.57940000000001</v>
-      </c>
-      <c r="AE121" t="n">
-        <v>8</v>
-      </c>
-      <c r="AF121" t="n">
-        <v>14</v>
-      </c>
-      <c r="AG121" t="n">
-        <v>0.3047</v>
-      </c>
-      <c r="AH121" t="n">
-        <v>0.8975</v>
-      </c>
-      <c r="AI121" t="n">
-        <v>0.0668</v>
-      </c>
-      <c r="AJ121" t="n">
-        <v>0.1516</v>
-      </c>
-      <c r="AK121" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL121" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM121" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN121" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO121" t="n">
-        <v>0.864</v>
-      </c>
-      <c r="AP121" t="n">
-        <v>0.748</v>
-      </c>
-      <c r="AQ121" t="n">
-        <v>1</v>
+      <c r="V121" t="inlineStr">
+        <is>
+          <t>526</t>
+        </is>
+      </c>
+      <c r="W121" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="X121" t="inlineStr">
+        <is>
+          <t>1.2705</t>
+        </is>
+      </c>
+      <c r="Y121" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="Z121" t="inlineStr">
+        <is>
+          <t>103</t>
+        </is>
+      </c>
+      <c r="AA121" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="AB121" t="inlineStr">
+        <is>
+          <t>1.1897</t>
+        </is>
+      </c>
+      <c r="AC121" t="inlineStr">
+        <is>
+          <t>4.62</t>
+        </is>
+      </c>
+      <c r="AD121" t="inlineStr">
+        <is>
+          <t>86.5794</t>
+        </is>
+      </c>
+      <c r="AE121" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AF121" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="AG121" t="inlineStr">
+        <is>
+          <t>0.3047</t>
+        </is>
+      </c>
+      <c r="AH121" t="inlineStr">
+        <is>
+          <t>0.8975</t>
+        </is>
+      </c>
+      <c r="AI121" t="inlineStr">
+        <is>
+          <t>0.0668</t>
+        </is>
+      </c>
+      <c r="AJ121" t="inlineStr">
+        <is>
+          <t>0.1516</t>
+        </is>
+      </c>
+      <c r="AK121" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL121" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AM121" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN121" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO121" t="inlineStr">
+        <is>
+          <t>0.864</t>
+        </is>
+      </c>
+      <c r="AP121" t="inlineStr">
+        <is>
+          <t>0.748</t>
+        </is>
+      </c>
+      <c r="AQ121" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
     </row>
     <row r="122">
@@ -27457,8 +27577,10 @@
           <t>scylla</t>
         </is>
       </c>
-      <c r="E137" t="n">
-        <v>28994</v>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>28994</t>
+        </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
@@ -27466,8 +27588,10 @@
         </is>
       </c>
       <c r="G137" t="inlineStr"/>
-      <c r="H137" t="n">
-        <v>97.59999999999999</v>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>97.6</t>
+        </is>
       </c>
       <c r="I137" t="inlineStr">
         <is>
@@ -27486,91 +27610,147 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N137" t="n">
-        <v>0.006</v>
-      </c>
-      <c r="O137" t="n">
-        <v>0.006</v>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t>0.006</t>
+        </is>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>0.006</t>
+        </is>
       </c>
       <c r="P137" t="inlineStr"/>
-      <c r="Q137" t="n">
-        <v>1.5953</v>
-      </c>
-      <c r="R137" t="n">
-        <v>0.1467</v>
-      </c>
-      <c r="S137" t="n">
-        <v>4.2824</v>
-      </c>
-      <c r="T137" t="n">
-        <v>0.026</v>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>1.5953</t>
+        </is>
+      </c>
+      <c r="R137" t="inlineStr">
+        <is>
+          <t>0.1467</t>
+        </is>
+      </c>
+      <c r="S137" t="inlineStr">
+        <is>
+          <t>4.2824</t>
+        </is>
+      </c>
+      <c r="T137" t="inlineStr">
+        <is>
+          <t>0.026</t>
+        </is>
       </c>
       <c r="U137" t="inlineStr"/>
-      <c r="V137" t="n">
-        <v>723</v>
-      </c>
-      <c r="W137" t="n">
-        <v>145</v>
-      </c>
-      <c r="X137" t="n">
-        <v>1.5206</v>
-      </c>
-      <c r="Y137" t="n">
-        <v>22</v>
-      </c>
-      <c r="Z137" t="n">
-        <v>107</v>
-      </c>
-      <c r="AA137" t="n">
-        <v>594</v>
-      </c>
-      <c r="AB137" t="n">
-        <v>1.1221</v>
-      </c>
-      <c r="AC137" t="n">
-        <v>6.2294</v>
-      </c>
-      <c r="AD137" t="n">
-        <v>95.354</v>
-      </c>
-      <c r="AE137" t="n">
-        <v>10</v>
-      </c>
-      <c r="AF137" t="n">
-        <v>16</v>
-      </c>
-      <c r="AG137" t="n">
-        <v>0.2877</v>
-      </c>
-      <c r="AH137" t="n">
-        <v>0.879</v>
-      </c>
-      <c r="AI137" t="n">
-        <v>0.0558</v>
-      </c>
-      <c r="AJ137" t="n">
-        <v>0.168</v>
-      </c>
-      <c r="AK137" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL137" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM137" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN137" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO137" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP137" t="n">
-        <v>0.837</v>
-      </c>
-      <c r="AQ137" t="n">
-        <v>1</v>
+      <c r="V137" t="inlineStr">
+        <is>
+          <t>723</t>
+        </is>
+      </c>
+      <c r="W137" t="inlineStr">
+        <is>
+          <t>145</t>
+        </is>
+      </c>
+      <c r="X137" t="inlineStr">
+        <is>
+          <t>1.5206</t>
+        </is>
+      </c>
+      <c r="Y137" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="Z137" t="inlineStr">
+        <is>
+          <t>107</t>
+        </is>
+      </c>
+      <c r="AA137" t="inlineStr">
+        <is>
+          <t>594</t>
+        </is>
+      </c>
+      <c r="AB137" t="inlineStr">
+        <is>
+          <t>1.1221</t>
+        </is>
+      </c>
+      <c r="AC137" t="inlineStr">
+        <is>
+          <t>6.2294</t>
+        </is>
+      </c>
+      <c r="AD137" t="inlineStr">
+        <is>
+          <t>95.354</t>
+        </is>
+      </c>
+      <c r="AE137" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AF137" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="AG137" t="inlineStr">
+        <is>
+          <t>0.2877</t>
+        </is>
+      </c>
+      <c r="AH137" t="inlineStr">
+        <is>
+          <t>0.879</t>
+        </is>
+      </c>
+      <c r="AI137" t="inlineStr">
+        <is>
+          <t>0.0558</t>
+        </is>
+      </c>
+      <c r="AJ137" t="inlineStr">
+        <is>
+          <t>0.168</t>
+        </is>
+      </c>
+      <c r="AK137" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL137" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AM137" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN137" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO137" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AP137" t="inlineStr">
+        <is>
+          <t>0.837</t>
+        </is>
+      </c>
+      <c r="AQ137" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
     </row>
     <row r="138">
@@ -29190,8 +29370,10 @@
           <t>silver_bug</t>
         </is>
       </c>
-      <c r="E146" t="n">
-        <v>58220</v>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>58220</t>
+        </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
@@ -29199,8 +29381,10 @@
         </is>
       </c>
       <c r="G146" t="inlineStr"/>
-      <c r="H146" t="n">
-        <v>92.90000000000001</v>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>92.9</t>
+        </is>
       </c>
       <c r="I146" t="inlineStr">
         <is>
@@ -29219,91 +29403,147 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N146" t="n">
-        <v>0.027</v>
-      </c>
-      <c r="O146" t="n">
-        <v>0.027</v>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>0.027</t>
+        </is>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>0.027</t>
+        </is>
       </c>
       <c r="P146" t="inlineStr"/>
-      <c r="Q146" t="n">
-        <v>1.5926</v>
-      </c>
-      <c r="R146" t="n">
-        <v>0.2285</v>
-      </c>
-      <c r="S146" t="n">
-        <v>7.7112</v>
-      </c>
-      <c r="T146" t="n">
-        <v>0.0226</v>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>1.5926</t>
+        </is>
+      </c>
+      <c r="R146" t="inlineStr">
+        <is>
+          <t>0.2285</t>
+        </is>
+      </c>
+      <c r="S146" t="inlineStr">
+        <is>
+          <t>7.7112</t>
+        </is>
+      </c>
+      <c r="T146" t="inlineStr">
+        <is>
+          <t>0.0226</t>
+        </is>
       </c>
       <c r="U146" t="inlineStr"/>
-      <c r="V146" t="n">
-        <v>1299</v>
-      </c>
-      <c r="W146" t="n">
-        <v>318</v>
-      </c>
-      <c r="X146" t="n">
-        <v>2.3291</v>
-      </c>
-      <c r="Y146" t="n">
-        <v>52</v>
-      </c>
-      <c r="Z146" t="n">
-        <v>233</v>
-      </c>
-      <c r="AA146" t="n">
-        <v>1014</v>
-      </c>
-      <c r="AB146" t="n">
-        <v>1.7066</v>
-      </c>
-      <c r="AC146" t="n">
-        <v>7.4269</v>
-      </c>
-      <c r="AD146" t="n">
-        <v>136.5308</v>
-      </c>
-      <c r="AE146" t="n">
-        <v>19</v>
-      </c>
-      <c r="AF146" t="n">
-        <v>17</v>
-      </c>
-      <c r="AG146" t="n">
-        <v>0.1881</v>
-      </c>
-      <c r="AH146" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI146" t="n">
-        <v>0.1171</v>
-      </c>
-      <c r="AJ146" t="n">
-        <v>0.0169</v>
-      </c>
-      <c r="AK146" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL146" t="n">
-        <v>0.716</v>
-      </c>
-      <c r="AM146" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN146" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO146" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP146" t="n">
-        <v>1</v>
-      </c>
-      <c r="AQ146" t="n">
-        <v>1</v>
+      <c r="V146" t="inlineStr">
+        <is>
+          <t>1299</t>
+        </is>
+      </c>
+      <c r="W146" t="inlineStr">
+        <is>
+          <t>318</t>
+        </is>
+      </c>
+      <c r="X146" t="inlineStr">
+        <is>
+          <t>2.3291</t>
+        </is>
+      </c>
+      <c r="Y146" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="Z146" t="inlineStr">
+        <is>
+          <t>233</t>
+        </is>
+      </c>
+      <c r="AA146" t="inlineStr">
+        <is>
+          <t>1014</t>
+        </is>
+      </c>
+      <c r="AB146" t="inlineStr">
+        <is>
+          <t>1.7066</t>
+        </is>
+      </c>
+      <c r="AC146" t="inlineStr">
+        <is>
+          <t>7.4269</t>
+        </is>
+      </c>
+      <c r="AD146" t="inlineStr">
+        <is>
+          <t>136.5308</t>
+        </is>
+      </c>
+      <c r="AE146" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="AF146" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="AG146" t="inlineStr">
+        <is>
+          <t>0.1881</t>
+        </is>
+      </c>
+      <c r="AH146" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AI146" t="inlineStr">
+        <is>
+          <t>0.1171</t>
+        </is>
+      </c>
+      <c r="AJ146" t="inlineStr">
+        <is>
+          <t>0.0169</t>
+        </is>
+      </c>
+      <c r="AK146" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL146" t="inlineStr">
+        <is>
+          <t>0.716</t>
+        </is>
+      </c>
+      <c r="AM146" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN146" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO146" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AP146" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AQ146" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
     </row>
     <row r="147">
@@ -29323,8 +29563,10 @@
         </is>
       </c>
       <c r="D147" t="inlineStr"/>
-      <c r="E147" t="n">
-        <v>60090</v>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>60090</t>
+        </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
@@ -29336,8 +29578,10 @@
           <t>parts: missing base, walls</t>
         </is>
       </c>
-      <c r="H147" t="n">
-        <v>66.59999999999999</v>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>66.6</t>
+        </is>
       </c>
       <c r="I147" t="inlineStr">
         <is>
@@ -29356,91 +29600,147 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N147" t="n">
-        <v>0.023</v>
-      </c>
-      <c r="O147" t="n">
-        <v>0.024</v>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>0.023</t>
+        </is>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>0.024</t>
+        </is>
       </c>
       <c r="P147" t="inlineStr"/>
-      <c r="Q147" t="n">
-        <v>1.3848</v>
-      </c>
-      <c r="R147" t="n">
-        <v>0.0914</v>
-      </c>
-      <c r="S147" t="n">
-        <v>2.7648</v>
-      </c>
-      <c r="T147" t="n">
-        <v>0.1028</v>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>1.3848</t>
+        </is>
+      </c>
+      <c r="R147" t="inlineStr">
+        <is>
+          <t>0.0914</t>
+        </is>
+      </c>
+      <c r="S147" t="inlineStr">
+        <is>
+          <t>2.7648</t>
+        </is>
+      </c>
+      <c r="T147" t="inlineStr">
+        <is>
+          <t>0.1028</t>
+        </is>
       </c>
       <c r="U147" t="inlineStr"/>
-      <c r="V147" t="n">
-        <v>1387</v>
-      </c>
-      <c r="W147" t="n">
-        <v>370</v>
-      </c>
-      <c r="X147" t="n">
-        <v>2.966</v>
-      </c>
-      <c r="Y147" t="n">
-        <v>27</v>
-      </c>
-      <c r="Z147" t="n">
-        <v>203</v>
-      </c>
-      <c r="AA147" t="n">
-        <v>1157</v>
-      </c>
-      <c r="AB147" t="n">
-        <v>1.6273</v>
-      </c>
-      <c r="AC147" t="n">
-        <v>9.274800000000001</v>
-      </c>
-      <c r="AD147" t="n">
-        <v>124.7461</v>
-      </c>
-      <c r="AE147" t="n">
-        <v>19</v>
-      </c>
-      <c r="AF147" t="n">
-        <v>18</v>
-      </c>
-      <c r="AG147" t="n">
-        <v>0.1366</v>
-      </c>
-      <c r="AH147" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI147" t="n">
-        <v>0.1041</v>
-      </c>
-      <c r="AJ147" t="n">
-        <v>0.0283</v>
-      </c>
-      <c r="AK147" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL147" t="n">
-        <v>0.266</v>
-      </c>
-      <c r="AM147" t="n">
-        <v>0.569</v>
-      </c>
-      <c r="AN147" t="n">
-        <v>0.426</v>
-      </c>
-      <c r="AO147" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP147" t="n">
-        <v>1</v>
-      </c>
-      <c r="AQ147" t="n">
-        <v>1</v>
+      <c r="V147" t="inlineStr">
+        <is>
+          <t>1387</t>
+        </is>
+      </c>
+      <c r="W147" t="inlineStr">
+        <is>
+          <t>370</t>
+        </is>
+      </c>
+      <c r="X147" t="inlineStr">
+        <is>
+          <t>2.966</t>
+        </is>
+      </c>
+      <c r="Y147" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="Z147" t="inlineStr">
+        <is>
+          <t>203</t>
+        </is>
+      </c>
+      <c r="AA147" t="inlineStr">
+        <is>
+          <t>1157</t>
+        </is>
+      </c>
+      <c r="AB147" t="inlineStr">
+        <is>
+          <t>1.6273</t>
+        </is>
+      </c>
+      <c r="AC147" t="inlineStr">
+        <is>
+          <t>9.2748</t>
+        </is>
+      </c>
+      <c r="AD147" t="inlineStr">
+        <is>
+          <t>124.7461</t>
+        </is>
+      </c>
+      <c r="AE147" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="AF147" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="AG147" t="inlineStr">
+        <is>
+          <t>0.1366</t>
+        </is>
+      </c>
+      <c r="AH147" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AI147" t="inlineStr">
+        <is>
+          <t>0.1041</t>
+        </is>
+      </c>
+      <c r="AJ147" t="inlineStr">
+        <is>
+          <t>0.0283</t>
+        </is>
+      </c>
+      <c r="AK147" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL147" t="inlineStr">
+        <is>
+          <t>0.266</t>
+        </is>
+      </c>
+      <c r="AM147" t="inlineStr">
+        <is>
+          <t>0.569</t>
+        </is>
+      </c>
+      <c r="AN147" t="inlineStr">
+        <is>
+          <t>0.426</t>
+        </is>
+      </c>
+      <c r="AO147" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AP147" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AQ147" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
     </row>
     <row r="148">

</xml_diff>

<commit_message>
Play-test 14 sea bosses: new AA guns, launchers, stern gun, liveries
Scylla +2 AK-230 +2 2M-7 +2 Uran banks, Nyx +2 Millennium +VLS, Typhon stern 57 mm, Hydra smaller guns and launcher;
six sea bosses in bespoke naval liveries. DECISIONS "Play-test 14 sea bosses after R4 (lane sea)", CHANGES PT14-SEA.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/models/quality_report.xlsx
+++ b/Docs/models/quality_report.xlsx
@@ -6656,8 +6656,10 @@
           <t>coeus</t>
         </is>
       </c>
-      <c r="E32" t="n">
-        <v>30614</v>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>30614</t>
+        </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -6665,8 +6667,10 @@
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" t="n">
-        <v>82.7</v>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>82.7</t>
+        </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -6685,91 +6689,147 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N32" t="n">
-        <v>0.021</v>
-      </c>
-      <c r="O32" t="n">
-        <v>0.011</v>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>0.021</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>0.011</t>
+        </is>
       </c>
       <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="n">
-        <v>1.5477</v>
-      </c>
-      <c r="R32" t="n">
-        <v>0.1041</v>
-      </c>
-      <c r="S32" t="n">
-        <v>2.4142</v>
-      </c>
-      <c r="T32" t="n">
-        <v>0.0157</v>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>1.5477</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>0.1041</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>2.4142</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>0.0157</t>
+        </is>
       </c>
       <c r="U32" t="inlineStr"/>
-      <c r="V32" t="n">
-        <v>461</v>
-      </c>
-      <c r="W32" t="n">
-        <v>157</v>
-      </c>
-      <c r="X32" t="n">
-        <v>1.2426</v>
-      </c>
-      <c r="Y32" t="n">
-        <v>11</v>
-      </c>
-      <c r="Z32" t="n">
-        <v>126</v>
-      </c>
-      <c r="AA32" t="n">
-        <v>324</v>
-      </c>
-      <c r="AB32" t="n">
-        <v>0.9972</v>
-      </c>
-      <c r="AC32" t="n">
-        <v>2.5643</v>
-      </c>
-      <c r="AD32" t="n">
-        <v>126.3493</v>
-      </c>
-      <c r="AE32" t="n">
-        <v>13</v>
-      </c>
-      <c r="AF32" t="n">
-        <v>13</v>
-      </c>
-      <c r="AG32" t="n">
-        <v>0.4299</v>
-      </c>
-      <c r="AH32" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI32" t="n">
-        <v>0.2416</v>
-      </c>
-      <c r="AJ32" t="n">
-        <v>-0.0009</v>
-      </c>
-      <c r="AK32" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL32" t="n">
-        <v>0.676</v>
-      </c>
-      <c r="AM32" t="n">
-        <v>0.953</v>
-      </c>
-      <c r="AN32" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="AO32" t="n">
-        <v>0.993</v>
-      </c>
-      <c r="AP32" t="n">
-        <v>0.631</v>
-      </c>
-      <c r="AQ32" t="n">
-        <v>1</v>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>461</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>157</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>1.2426</t>
+        </is>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>126</t>
+        </is>
+      </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>324</t>
+        </is>
+      </c>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>0.9972</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>2.5643</t>
+        </is>
+      </c>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>126.3493</t>
+        </is>
+      </c>
+      <c r="AE32" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="AF32" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="AG32" t="inlineStr">
+        <is>
+          <t>0.4299</t>
+        </is>
+      </c>
+      <c r="AH32" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AI32" t="inlineStr">
+        <is>
+          <t>0.2416</t>
+        </is>
+      </c>
+      <c r="AJ32" t="inlineStr">
+        <is>
+          <t>-0.0009</t>
+        </is>
+      </c>
+      <c r="AK32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL32" t="inlineStr">
+        <is>
+          <t>0.676</t>
+        </is>
+      </c>
+      <c r="AM32" t="inlineStr">
+        <is>
+          <t>0.953</t>
+        </is>
+      </c>
+      <c r="AN32" t="inlineStr">
+        <is>
+          <t>0.81</t>
+        </is>
+      </c>
+      <c r="AO32" t="inlineStr">
+        <is>
+          <t>0.993</t>
+        </is>
+      </c>
+      <c r="AP32" t="inlineStr">
+        <is>
+          <t>0.631</t>
+        </is>
+      </c>
+      <c r="AQ32" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -17998,7 +18058,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>20080</v>
+        <v>18804</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
@@ -18007,16 +18067,16 @@
       </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="n">
-        <v>99.7</v>
+        <v>73.7</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Tốt</t>
+          <t>Cần sửa</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="K89" t="inlineStr"/>
@@ -18027,87 +18087,87 @@
         </is>
       </c>
       <c r="N89" t="n">
-        <v>0.024</v>
+        <v>0.021</v>
       </c>
       <c r="O89" t="n">
-        <v>0.02</v>
+        <v>0.017</v>
       </c>
       <c r="P89" t="inlineStr"/>
       <c r="Q89" t="n">
-        <v>1.2665</v>
+        <v>1.2698</v>
       </c>
       <c r="R89" t="n">
-        <v>0.1022</v>
+        <v>0.0086</v>
       </c>
       <c r="S89" t="n">
-        <v>2.703</v>
+        <v>0.384</v>
       </c>
       <c r="T89" t="n">
         <v>0.0364</v>
       </c>
       <c r="U89" t="inlineStr"/>
       <c r="V89" t="n">
-        <v>526</v>
+        <v>383</v>
       </c>
       <c r="W89" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="X89" t="n">
-        <v>2.3108</v>
+        <v>2.3323</v>
       </c>
       <c r="Y89" t="n">
         <v>13</v>
       </c>
       <c r="Z89" t="n">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="AA89" t="n">
-        <v>451</v>
+        <v>319</v>
       </c>
       <c r="AB89" t="n">
-        <v>1.6098</v>
+        <v>1.3517</v>
       </c>
       <c r="AC89" t="n">
-        <v>11.7097</v>
+        <v>8.454499999999999</v>
       </c>
       <c r="AD89" t="n">
-        <v>38.5152</v>
+        <v>37.7315</v>
       </c>
       <c r="AE89" t="n">
         <v>40</v>
       </c>
       <c r="AF89" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AG89" t="n">
-        <v>0.2661</v>
+        <v>0.2565</v>
       </c>
       <c r="AH89" t="n">
-        <v>0.7985</v>
+        <v>0.8064</v>
       </c>
       <c r="AI89" t="n">
-        <v>0.0202</v>
+        <v>0.0394</v>
       </c>
       <c r="AJ89" t="n">
-        <v>0.1366</v>
+        <v>0.08890000000000001</v>
       </c>
       <c r="AK89" t="n">
         <v>0</v>
       </c>
       <c r="AL89" t="n">
-        <v>0.987</v>
+        <v>0.999</v>
       </c>
       <c r="AM89" t="n">
-        <v>1</v>
+        <v>0.105</v>
       </c>
       <c r="AN89" t="n">
-        <v>1</v>
+        <v>0.226</v>
       </c>
       <c r="AO89" t="n">
         <v>1</v>
       </c>
       <c r="AP89" t="n">
-        <v>0.999</v>
+        <v>0.919</v>
       </c>
       <c r="AQ89" t="n">
         <v>1</v>
@@ -18134,8 +18194,10 @@
           <t>hyperion</t>
         </is>
       </c>
-      <c r="E90" t="n">
-        <v>67352</v>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>67352</t>
+        </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -18143,8 +18205,10 @@
         </is>
       </c>
       <c r="G90" t="inlineStr"/>
-      <c r="H90" t="n">
-        <v>85.8</v>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>85.8</t>
+        </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
@@ -18163,91 +18227,147 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N90" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="O90" t="n">
-        <v>0.006</v>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>0.015</t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>0.006</t>
+        </is>
       </c>
       <c r="P90" t="inlineStr"/>
-      <c r="Q90" t="n">
-        <v>1.3784</v>
-      </c>
-      <c r="R90" t="n">
-        <v>0.1388</v>
-      </c>
-      <c r="S90" t="n">
-        <v>3.3947</v>
-      </c>
-      <c r="T90" t="n">
-        <v>0.0143</v>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>1.3784</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>0.1388</t>
+        </is>
+      </c>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>3.3947</t>
+        </is>
+      </c>
+      <c r="T90" t="inlineStr">
+        <is>
+          <t>0.0143</t>
+        </is>
       </c>
       <c r="U90" t="inlineStr"/>
-      <c r="V90" t="n">
-        <v>934</v>
-      </c>
-      <c r="W90" t="n">
-        <v>212</v>
-      </c>
-      <c r="X90" t="n">
-        <v>1.4989</v>
-      </c>
-      <c r="Y90" t="n">
-        <v>10</v>
-      </c>
-      <c r="Z90" t="n">
-        <v>171</v>
-      </c>
-      <c r="AA90" t="n">
-        <v>753</v>
-      </c>
-      <c r="AB90" t="n">
-        <v>1.209</v>
-      </c>
-      <c r="AC90" t="n">
-        <v>5.3238</v>
-      </c>
-      <c r="AD90" t="n">
-        <v>141.4408</v>
-      </c>
-      <c r="AE90" t="n">
-        <v>11</v>
-      </c>
-      <c r="AF90" t="n">
-        <v>13</v>
-      </c>
-      <c r="AG90" t="n">
-        <v>0.4412</v>
-      </c>
-      <c r="AH90" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI90" t="n">
-        <v>0.2461</v>
-      </c>
-      <c r="AJ90" t="n">
-        <v>0.0159</v>
-      </c>
-      <c r="AK90" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL90" t="n">
-        <v>0.467</v>
-      </c>
-      <c r="AM90" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN90" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO90" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP90" t="n">
-        <v>0.9409999999999999</v>
-      </c>
-      <c r="AQ90" t="n">
-        <v>1</v>
+      <c r="V90" t="inlineStr">
+        <is>
+          <t>934</t>
+        </is>
+      </c>
+      <c r="W90" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
+      <c r="X90" t="inlineStr">
+        <is>
+          <t>1.4989</t>
+        </is>
+      </c>
+      <c r="Y90" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="Z90" t="inlineStr">
+        <is>
+          <t>171</t>
+        </is>
+      </c>
+      <c r="AA90" t="inlineStr">
+        <is>
+          <t>753</t>
+        </is>
+      </c>
+      <c r="AB90" t="inlineStr">
+        <is>
+          <t>1.209</t>
+        </is>
+      </c>
+      <c r="AC90" t="inlineStr">
+        <is>
+          <t>5.3238</t>
+        </is>
+      </c>
+      <c r="AD90" t="inlineStr">
+        <is>
+          <t>141.4408</t>
+        </is>
+      </c>
+      <c r="AE90" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="AF90" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="AG90" t="inlineStr">
+        <is>
+          <t>0.4412</t>
+        </is>
+      </c>
+      <c r="AH90" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AI90" t="inlineStr">
+        <is>
+          <t>0.2461</t>
+        </is>
+      </c>
+      <c r="AJ90" t="inlineStr">
+        <is>
+          <t>0.0159</t>
+        </is>
+      </c>
+      <c r="AK90" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL90" t="inlineStr">
+        <is>
+          <t>0.467</t>
+        </is>
+      </c>
+      <c r="AM90" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN90" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO90" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AP90" t="inlineStr">
+        <is>
+          <t>0.941</t>
+        </is>
+      </c>
+      <c r="AQ90" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
     </row>
     <row r="91">
@@ -19063,10 +19183,8 @@
           <t>kraken</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>61644</t>
-        </is>
+      <c r="E95" t="n">
+        <v>75770</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
@@ -19074,10 +19192,8 @@
         </is>
       </c>
       <c r="G95" t="inlineStr"/>
-      <c r="H95" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
+      <c r="H95" t="n">
+        <v>100</v>
       </c>
       <c r="I95" t="inlineStr">
         <is>
@@ -19096,151 +19212,91 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N95" t="inlineStr">
-        <is>
-          <t>0.107</t>
-        </is>
-      </c>
-      <c r="O95" t="inlineStr">
-        <is>
-          <t>0.102</t>
-        </is>
-      </c>
-      <c r="P95" t="inlineStr">
-        <is>
-          <t>leviathan</t>
-        </is>
-      </c>
-      <c r="Q95" t="inlineStr">
-        <is>
-          <t>1.2757</t>
-        </is>
-      </c>
-      <c r="R95" t="inlineStr">
-        <is>
-          <t>0.1255</t>
-        </is>
-      </c>
-      <c r="S95" t="inlineStr">
-        <is>
-          <t>3.2459</t>
-        </is>
-      </c>
-      <c r="T95" t="inlineStr">
-        <is>
-          <t>0.045</t>
-        </is>
+      <c r="N95" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="O95" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="P95" t="inlineStr"/>
+      <c r="Q95" t="n">
+        <v>1.3111</v>
+      </c>
+      <c r="R95" t="n">
+        <v>0.1244</v>
+      </c>
+      <c r="S95" t="n">
+        <v>3.3347</v>
+      </c>
+      <c r="T95" t="n">
+        <v>0.0397</v>
       </c>
       <c r="U95" t="inlineStr"/>
-      <c r="V95" t="inlineStr">
-        <is>
-          <t>1624</t>
-        </is>
-      </c>
-      <c r="W95" t="inlineStr">
-        <is>
-          <t>224</t>
-        </is>
-      </c>
-      <c r="X95" t="inlineStr">
-        <is>
-          <t>2.501</t>
-        </is>
-      </c>
-      <c r="Y95" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="Z95" t="inlineStr">
-        <is>
-          <t>169</t>
-        </is>
-      </c>
-      <c r="AA95" t="inlineStr">
-        <is>
-          <t>1429</t>
-        </is>
-      </c>
-      <c r="AB95" t="inlineStr">
-        <is>
-          <t>1.8869</t>
-        </is>
-      </c>
-      <c r="AC95" t="inlineStr">
-        <is>
-          <t>15.9553</t>
-        </is>
-      </c>
-      <c r="AD95" t="inlineStr">
-        <is>
-          <t>89.5626</t>
-        </is>
-      </c>
-      <c r="AE95" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="AF95" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="AG95" t="inlineStr">
-        <is>
-          <t>0.2705</t>
-        </is>
-      </c>
-      <c r="AH95" t="inlineStr">
-        <is>
-          <t>0.8731</t>
-        </is>
-      </c>
-      <c r="AI95" t="inlineStr">
-        <is>
-          <t>0.0611</t>
-        </is>
-      </c>
-      <c r="AJ95" t="inlineStr">
-        <is>
-          <t>0.0731</t>
-        </is>
-      </c>
-      <c r="AK95" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AL95" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AM95" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AN95" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AO95" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AP95" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AQ95" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="V95" t="n">
+        <v>2012</v>
+      </c>
+      <c r="W95" t="n">
+        <v>251</v>
+      </c>
+      <c r="X95" t="n">
+        <v>2.8557</v>
+      </c>
+      <c r="Y95" t="n">
+        <v>26</v>
+      </c>
+      <c r="Z95" t="n">
+        <v>160</v>
+      </c>
+      <c r="AA95" t="n">
+        <v>1826</v>
+      </c>
+      <c r="AB95" t="n">
+        <v>1.8203</v>
+      </c>
+      <c r="AC95" t="n">
+        <v>20.7747</v>
+      </c>
+      <c r="AD95" t="n">
+        <v>87.8952</v>
+      </c>
+      <c r="AE95" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF95" t="n">
+        <v>18</v>
+      </c>
+      <c r="AG95" t="n">
+        <v>0.2688</v>
+      </c>
+      <c r="AH95" t="n">
+        <v>0.8172</v>
+      </c>
+      <c r="AI95" t="n">
+        <v>0.0471</v>
+      </c>
+      <c r="AJ95" t="n">
+        <v>0.1224</v>
+      </c>
+      <c r="AK95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL95" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM95" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN95" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO95" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP95" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ95" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="96">
@@ -20060,10 +20116,8 @@
           <t>leviathan</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>86412</t>
-        </is>
+      <c r="E100" t="n">
+        <v>86412</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
@@ -20071,10 +20125,8 @@
         </is>
       </c>
       <c r="G100" t="inlineStr"/>
-      <c r="H100" t="inlineStr">
-        <is>
-          <t>97.7</t>
-        </is>
+      <c r="H100" t="n">
+        <v>97.7</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
@@ -20093,147 +20145,91 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N100" t="inlineStr">
-        <is>
-          <t>0.002</t>
-        </is>
-      </c>
-      <c r="O100" t="inlineStr">
-        <is>
-          <t>0.002</t>
-        </is>
+      <c r="N100" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="O100" t="n">
+        <v>0.008</v>
       </c>
       <c r="P100" t="inlineStr"/>
-      <c r="Q100" t="inlineStr">
-        <is>
-          <t>1.4402</t>
-        </is>
-      </c>
-      <c r="R100" t="inlineStr">
-        <is>
-          <t>0.1709</t>
-        </is>
-      </c>
-      <c r="S100" t="inlineStr">
-        <is>
-          <t>4.5164</t>
-        </is>
-      </c>
-      <c r="T100" t="inlineStr">
-        <is>
-          <t>0.0925</t>
-        </is>
+      <c r="Q100" t="n">
+        <v>1.4402</v>
+      </c>
+      <c r="R100" t="n">
+        <v>0.1464</v>
+      </c>
+      <c r="S100" t="n">
+        <v>3.9035</v>
+      </c>
+      <c r="T100" t="n">
+        <v>0.0925</v>
       </c>
       <c r="U100" t="inlineStr"/>
-      <c r="V100" t="inlineStr">
-        <is>
-          <t>1784</t>
-        </is>
-      </c>
-      <c r="W100" t="inlineStr">
-        <is>
-          <t>247</t>
-        </is>
-      </c>
-      <c r="X100" t="inlineStr">
-        <is>
-          <t>2.2347</t>
-        </is>
-      </c>
-      <c r="Y100" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="Z100" t="inlineStr">
-        <is>
-          <t>142</t>
-        </is>
-      </c>
-      <c r="AA100" t="inlineStr">
-        <is>
-          <t>1608</t>
-        </is>
-      </c>
-      <c r="AB100" t="inlineStr">
-        <is>
-          <t>1.2847</t>
-        </is>
-      </c>
-      <c r="AC100" t="inlineStr">
-        <is>
-          <t>14.5482</t>
-        </is>
-      </c>
-      <c r="AD100" t="inlineStr">
-        <is>
-          <t>110.529</t>
-        </is>
-      </c>
-      <c r="AE100" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="AF100" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="AG100" t="inlineStr">
-        <is>
-          <t>0.2652</t>
-        </is>
-      </c>
-      <c r="AH100" t="inlineStr">
-        <is>
-          <t>0.8561</t>
-        </is>
-      </c>
-      <c r="AI100" t="inlineStr">
-        <is>
-          <t>0.0601</t>
-        </is>
-      </c>
-      <c r="AJ100" t="inlineStr">
-        <is>
-          <t>0.1499</t>
-        </is>
-      </c>
-      <c r="AK100" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AL100" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AM100" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AN100" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AO100" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AP100" t="inlineStr">
-        <is>
-          <t>0.848</t>
-        </is>
-      </c>
-      <c r="AQ100" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="V100" t="n">
+        <v>1784</v>
+      </c>
+      <c r="W100" t="n">
+        <v>247</v>
+      </c>
+      <c r="X100" t="n">
+        <v>2.2347</v>
+      </c>
+      <c r="Y100" t="n">
+        <v>34</v>
+      </c>
+      <c r="Z100" t="n">
+        <v>142</v>
+      </c>
+      <c r="AA100" t="n">
+        <v>1608</v>
+      </c>
+      <c r="AB100" t="n">
+        <v>1.2847</v>
+      </c>
+      <c r="AC100" t="n">
+        <v>14.5482</v>
+      </c>
+      <c r="AD100" t="n">
+        <v>110.529</v>
+      </c>
+      <c r="AE100" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF100" t="n">
+        <v>20</v>
+      </c>
+      <c r="AG100" t="n">
+        <v>0.2522</v>
+      </c>
+      <c r="AH100" t="n">
+        <v>0.8486</v>
+      </c>
+      <c r="AI100" t="n">
+        <v>0.0575</v>
+      </c>
+      <c r="AJ100" t="n">
+        <v>0.1457</v>
+      </c>
+      <c r="AK100" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL100" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM100" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN100" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO100" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP100" t="n">
+        <v>0.848</v>
+      </c>
+      <c r="AQ100" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="101">
@@ -24455,7 +24451,7 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>23034</v>
+        <v>26854</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
@@ -24464,7 +24460,7 @@
       </c>
       <c r="G122" t="inlineStr"/>
       <c r="H122" t="n">
-        <v>98.5</v>
+        <v>91.3</v>
       </c>
       <c r="I122" t="inlineStr">
         <is>
@@ -24484,87 +24480,87 @@
         </is>
       </c>
       <c r="N122" t="n">
-        <v>0.025</v>
+        <v>0.032</v>
       </c>
       <c r="O122" t="n">
-        <v>0.026</v>
+        <v>0.023</v>
       </c>
       <c r="P122" t="inlineStr"/>
       <c r="Q122" t="n">
-        <v>1.3584</v>
+        <v>1.3363</v>
       </c>
       <c r="R122" t="n">
-        <v>0.1021</v>
+        <v>0.07149999999999999</v>
       </c>
       <c r="S122" t="n">
-        <v>2.3914</v>
+        <v>1.5475</v>
       </c>
       <c r="T122" t="n">
         <v>0.0342</v>
       </c>
       <c r="U122" t="inlineStr"/>
       <c r="V122" t="n">
-        <v>769</v>
+        <v>852</v>
       </c>
       <c r="W122" t="n">
-        <v>128</v>
+        <v>143</v>
       </c>
       <c r="X122" t="n">
-        <v>1.4512</v>
+        <v>1.602</v>
       </c>
       <c r="Y122" t="n">
         <v>23</v>
       </c>
       <c r="Z122" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="AA122" t="n">
-        <v>641</v>
+        <v>722</v>
       </c>
       <c r="AB122" t="n">
-        <v>1.1904</v>
+        <v>1.1987</v>
       </c>
       <c r="AC122" t="n">
-        <v>7.2674</v>
+        <v>8.0886</v>
       </c>
       <c r="AD122" t="n">
-        <v>88.20229999999999</v>
+        <v>89.2611</v>
       </c>
       <c r="AE122" t="n">
         <v>8</v>
       </c>
       <c r="AF122" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="AG122" t="n">
-        <v>0.2844</v>
+        <v>0.2562</v>
       </c>
       <c r="AH122" t="n">
-        <v>0.8308</v>
+        <v>0.8721</v>
       </c>
       <c r="AI122" t="n">
-        <v>0.05</v>
+        <v>0.07240000000000001</v>
       </c>
       <c r="AJ122" t="n">
-        <v>0.0997</v>
+        <v>0.15</v>
       </c>
       <c r="AK122" t="n">
         <v>0</v>
       </c>
       <c r="AL122" t="n">
-        <v>0.994</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="AM122" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="AN122" t="n">
+        <v>0.8070000000000001</v>
+      </c>
+      <c r="AO122" t="n">
         <v>1</v>
       </c>
-      <c r="AN122" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO122" t="n">
-        <v>0.987</v>
-      </c>
       <c r="AP122" t="n">
-        <v>0.929</v>
+        <v>0.9360000000000001</v>
       </c>
       <c r="AQ122" t="n">
         <v>1</v>
@@ -27594,10 +27590,8 @@
           <t>scylla</t>
         </is>
       </c>
-      <c r="E138" t="inlineStr">
-        <is>
-          <t>28994</t>
-        </is>
+      <c r="E138" t="n">
+        <v>45394</v>
       </c>
       <c r="F138" t="inlineStr">
         <is>
@@ -27605,10 +27599,8 @@
         </is>
       </c>
       <c r="G138" t="inlineStr"/>
-      <c r="H138" t="inlineStr">
-        <is>
-          <t>97.6</t>
-        </is>
+      <c r="H138" t="n">
+        <v>97.59999999999999</v>
       </c>
       <c r="I138" t="inlineStr">
         <is>
@@ -27627,147 +27619,91 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N138" t="inlineStr">
-        <is>
-          <t>0.006</t>
-        </is>
-      </c>
-      <c r="O138" t="inlineStr">
-        <is>
-          <t>0.006</t>
-        </is>
+      <c r="N138" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="O138" t="n">
+        <v>0.013</v>
       </c>
       <c r="P138" t="inlineStr"/>
-      <c r="Q138" t="inlineStr">
-        <is>
-          <t>1.5953</t>
-        </is>
-      </c>
-      <c r="R138" t="inlineStr">
-        <is>
-          <t>0.1467</t>
-        </is>
-      </c>
-      <c r="S138" t="inlineStr">
-        <is>
-          <t>4.2824</t>
-        </is>
-      </c>
-      <c r="T138" t="inlineStr">
-        <is>
-          <t>0.026</t>
-        </is>
+      <c r="Q138" t="n">
+        <v>1.6363</v>
+      </c>
+      <c r="R138" t="n">
+        <v>0.1178</v>
+      </c>
+      <c r="S138" t="n">
+        <v>3.382</v>
+      </c>
+      <c r="T138" t="n">
+        <v>0.026</v>
       </c>
       <c r="U138" t="inlineStr"/>
-      <c r="V138" t="inlineStr">
-        <is>
-          <t>723</t>
-        </is>
-      </c>
-      <c r="W138" t="inlineStr">
-        <is>
-          <t>145</t>
-        </is>
-      </c>
-      <c r="X138" t="inlineStr">
-        <is>
-          <t>1.5206</t>
-        </is>
-      </c>
-      <c r="Y138" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="Z138" t="inlineStr">
-        <is>
-          <t>107</t>
-        </is>
-      </c>
-      <c r="AA138" t="inlineStr">
-        <is>
-          <t>594</t>
-        </is>
-      </c>
-      <c r="AB138" t="inlineStr">
-        <is>
-          <t>1.1221</t>
-        </is>
-      </c>
-      <c r="AC138" t="inlineStr">
-        <is>
-          <t>6.2294</t>
-        </is>
-      </c>
-      <c r="AD138" t="inlineStr">
-        <is>
-          <t>95.354</t>
-        </is>
-      </c>
-      <c r="AE138" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AF138" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="AG138" t="inlineStr">
-        <is>
-          <t>0.2877</t>
-        </is>
-      </c>
-      <c r="AH138" t="inlineStr">
-        <is>
-          <t>0.879</t>
-        </is>
-      </c>
-      <c r="AI138" t="inlineStr">
-        <is>
-          <t>0.0558</t>
-        </is>
-      </c>
-      <c r="AJ138" t="inlineStr">
-        <is>
-          <t>0.168</t>
-        </is>
-      </c>
-      <c r="AK138" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AL138" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AM138" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AN138" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AO138" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AP138" t="inlineStr">
-        <is>
-          <t>0.837</t>
-        </is>
-      </c>
-      <c r="AQ138" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="V138" t="n">
+        <v>1053</v>
+      </c>
+      <c r="W138" t="n">
+        <v>185</v>
+      </c>
+      <c r="X138" t="n">
+        <v>1.9063</v>
+      </c>
+      <c r="Y138" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z138" t="n">
+        <v>107</v>
+      </c>
+      <c r="AA138" t="n">
+        <v>924</v>
+      </c>
+      <c r="AB138" t="n">
+        <v>1.1026</v>
+      </c>
+      <c r="AC138" t="n">
+        <v>9.5214</v>
+      </c>
+      <c r="AD138" t="n">
+        <v>97.0449</v>
+      </c>
+      <c r="AE138" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF138" t="n">
+        <v>19</v>
+      </c>
+      <c r="AG138" t="n">
+        <v>0.2833</v>
+      </c>
+      <c r="AH138" t="n">
+        <v>0.8933</v>
+      </c>
+      <c r="AI138" t="n">
+        <v>0.0665</v>
+      </c>
+      <c r="AJ138" t="n">
+        <v>0.1572</v>
+      </c>
+      <c r="AK138" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL138" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM138" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN138" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO138" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP138" t="n">
+        <v>0.842</v>
+      </c>
+      <c r="AQ138" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="139">
@@ -31960,8 +31896,10 @@
           <t>theia</t>
         </is>
       </c>
-      <c r="E160" t="n">
-        <v>30454</v>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>30454</t>
+        </is>
       </c>
       <c r="F160" t="inlineStr">
         <is>
@@ -31969,8 +31907,10 @@
         </is>
       </c>
       <c r="G160" t="inlineStr"/>
-      <c r="H160" t="n">
-        <v>81.5</v>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>81.5</t>
+        </is>
       </c>
       <c r="I160" t="inlineStr">
         <is>
@@ -31989,91 +31929,147 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N160" t="n">
-        <v>0.008</v>
-      </c>
-      <c r="O160" t="n">
-        <v>0.008</v>
+      <c r="N160" t="inlineStr">
+        <is>
+          <t>0.008</t>
+        </is>
+      </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>0.008</t>
+        </is>
       </c>
       <c r="P160" t="inlineStr"/>
-      <c r="Q160" t="n">
-        <v>1.4545</v>
-      </c>
-      <c r="R160" t="n">
-        <v>0.1296</v>
-      </c>
-      <c r="S160" t="n">
-        <v>3.2355</v>
-      </c>
-      <c r="T160" t="n">
-        <v>0.0214</v>
+      <c r="Q160" t="inlineStr">
+        <is>
+          <t>1.4545</t>
+        </is>
+      </c>
+      <c r="R160" t="inlineStr">
+        <is>
+          <t>0.1296</t>
+        </is>
+      </c>
+      <c r="S160" t="inlineStr">
+        <is>
+          <t>3.2355</t>
+        </is>
+      </c>
+      <c r="T160" t="inlineStr">
+        <is>
+          <t>0.0214</t>
+        </is>
       </c>
       <c r="U160" t="inlineStr"/>
-      <c r="V160" t="n">
-        <v>449</v>
-      </c>
-      <c r="W160" t="n">
-        <v>151</v>
-      </c>
-      <c r="X160" t="n">
-        <v>1.177</v>
-      </c>
-      <c r="Y160" t="n">
-        <v>8</v>
-      </c>
-      <c r="Z160" t="n">
-        <v>107</v>
-      </c>
-      <c r="AA160" t="n">
-        <v>334</v>
-      </c>
-      <c r="AB160" t="n">
-        <v>0.834</v>
-      </c>
-      <c r="AC160" t="n">
-        <v>2.6034</v>
-      </c>
-      <c r="AD160" t="n">
-        <v>128.2948</v>
-      </c>
-      <c r="AE160" t="n">
-        <v>9</v>
-      </c>
-      <c r="AF160" t="n">
-        <v>14</v>
-      </c>
-      <c r="AG160" t="n">
-        <v>0.4393</v>
-      </c>
-      <c r="AH160" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI160" t="n">
-        <v>0.2216</v>
-      </c>
-      <c r="AJ160" t="n">
-        <v>0.0256</v>
-      </c>
-      <c r="AK160" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL160" t="n">
-        <v>0.5610000000000001</v>
-      </c>
-      <c r="AM160" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN160" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO160" t="n">
-        <v>0.9409999999999999</v>
-      </c>
-      <c r="AP160" t="n">
-        <v>0.576</v>
-      </c>
-      <c r="AQ160" t="n">
-        <v>1</v>
+      <c r="V160" t="inlineStr">
+        <is>
+          <t>449</t>
+        </is>
+      </c>
+      <c r="W160" t="inlineStr">
+        <is>
+          <t>151</t>
+        </is>
+      </c>
+      <c r="X160" t="inlineStr">
+        <is>
+          <t>1.177</t>
+        </is>
+      </c>
+      <c r="Y160" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="Z160" t="inlineStr">
+        <is>
+          <t>107</t>
+        </is>
+      </c>
+      <c r="AA160" t="inlineStr">
+        <is>
+          <t>334</t>
+        </is>
+      </c>
+      <c r="AB160" t="inlineStr">
+        <is>
+          <t>0.834</t>
+        </is>
+      </c>
+      <c r="AC160" t="inlineStr">
+        <is>
+          <t>2.6034</t>
+        </is>
+      </c>
+      <c r="AD160" t="inlineStr">
+        <is>
+          <t>128.2948</t>
+        </is>
+      </c>
+      <c r="AE160" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="AF160" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="AG160" t="inlineStr">
+        <is>
+          <t>0.4393</t>
+        </is>
+      </c>
+      <c r="AH160" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AI160" t="inlineStr">
+        <is>
+          <t>0.2216</t>
+        </is>
+      </c>
+      <c r="AJ160" t="inlineStr">
+        <is>
+          <t>0.0256</t>
+        </is>
+      </c>
+      <c r="AK160" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL160" t="inlineStr">
+        <is>
+          <t>0.561</t>
+        </is>
+      </c>
+      <c r="AM160" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN160" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO160" t="inlineStr">
+        <is>
+          <t>0.941</t>
+        </is>
+      </c>
+      <c r="AP160" t="inlineStr">
+        <is>
+          <t>0.576</t>
+        </is>
+      </c>
+      <c r="AQ160" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
     </row>
     <row r="161">
@@ -32889,10 +32885,8 @@
           <t>typhon</t>
         </is>
       </c>
-      <c r="E165" t="inlineStr">
-        <is>
-          <t>13260</t>
-        </is>
+      <c r="E165" t="n">
+        <v>32624</v>
       </c>
       <c r="F165" t="inlineStr">
         <is>
@@ -32900,19 +32894,17 @@
         </is>
       </c>
       <c r="G165" t="inlineStr"/>
-      <c r="H165" t="inlineStr">
-        <is>
-          <t>81.4</t>
-        </is>
+      <c r="H165" t="n">
+        <v>70.09999999999999</v>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>Tốt</t>
+          <t>Cần sửa</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="K165" t="inlineStr"/>
@@ -32922,147 +32914,91 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N165" t="inlineStr">
-        <is>
-          <t>0.053</t>
-        </is>
-      </c>
-      <c r="O165" t="inlineStr">
-        <is>
-          <t>0.045</t>
-        </is>
+      <c r="N165" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="O165" t="n">
+        <v>0.013</v>
       </c>
       <c r="P165" t="inlineStr"/>
-      <c r="Q165" t="inlineStr">
-        <is>
-          <t>1.2921</t>
-        </is>
-      </c>
-      <c r="R165" t="inlineStr">
-        <is>
-          <t>0.0506</t>
-        </is>
-      </c>
-      <c r="S165" t="inlineStr">
-        <is>
-          <t>1.495</t>
-        </is>
-      </c>
-      <c r="T165" t="inlineStr">
-        <is>
-          <t>0.0056</t>
-        </is>
+      <c r="Q165" t="n">
+        <v>1.2501</v>
+      </c>
+      <c r="R165" t="n">
+        <v>0.0046</v>
+      </c>
+      <c r="S165" t="n">
+        <v>0.1219</v>
+      </c>
+      <c r="T165" t="n">
+        <v>0.0202</v>
       </c>
       <c r="U165" t="inlineStr"/>
-      <c r="V165" t="inlineStr">
-        <is>
-          <t>474</t>
-        </is>
-      </c>
-      <c r="W165" t="inlineStr">
-        <is>
-          <t>70</t>
-        </is>
-      </c>
-      <c r="X165" t="inlineStr">
-        <is>
-          <t>1.2689</t>
-        </is>
-      </c>
-      <c r="Y165" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="Z165" t="inlineStr">
-        <is>
-          <t>55</t>
-        </is>
-      </c>
-      <c r="AA165" t="inlineStr">
-        <is>
-          <t>412</t>
-        </is>
-      </c>
-      <c r="AB165" t="inlineStr">
-        <is>
-          <t>0.997</t>
-        </is>
-      </c>
-      <c r="AC165" t="inlineStr">
-        <is>
-          <t>7.4684</t>
-        </is>
-      </c>
-      <c r="AD165" t="inlineStr">
-        <is>
-          <t>55.1655</t>
-        </is>
-      </c>
-      <c r="AE165" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="AF165" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AG165" t="inlineStr">
-        <is>
-          <t>0.168</t>
-        </is>
-      </c>
-      <c r="AH165" t="inlineStr">
-        <is>
-          <t>0.7985</t>
-        </is>
-      </c>
-      <c r="AI165" t="inlineStr">
-        <is>
-          <t>0.0225</t>
-        </is>
-      </c>
-      <c r="AJ165" t="inlineStr">
-        <is>
-          <t>0.0426</t>
-        </is>
-      </c>
-      <c r="AK165" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AL165" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AM165" t="inlineStr">
-        <is>
-          <t>0.619</t>
-        </is>
-      </c>
-      <c r="AN165" t="inlineStr">
-        <is>
-          <t>0.879</t>
-        </is>
-      </c>
-      <c r="AO165" t="inlineStr">
-        <is>
-          <t>0.841</t>
-        </is>
-      </c>
-      <c r="AP165" t="inlineStr">
-        <is>
-          <t>0.809</t>
-        </is>
-      </c>
-      <c r="AQ165" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="V165" t="n">
+        <v>889</v>
+      </c>
+      <c r="W165" t="n">
+        <v>150</v>
+      </c>
+      <c r="X165" t="n">
+        <v>2.9821</v>
+      </c>
+      <c r="Y165" t="n">
+        <v>11</v>
+      </c>
+      <c r="Z165" t="n">
+        <v>85</v>
+      </c>
+      <c r="AA165" t="n">
+        <v>793</v>
+      </c>
+      <c r="AB165" t="n">
+        <v>1.6899</v>
+      </c>
+      <c r="AC165" t="n">
+        <v>15.7653</v>
+      </c>
+      <c r="AD165" t="n">
+        <v>50.3003</v>
+      </c>
+      <c r="AE165" t="n">
+        <v>21</v>
+      </c>
+      <c r="AF165" t="n">
+        <v>17</v>
+      </c>
+      <c r="AG165" t="n">
+        <v>0.2582</v>
+      </c>
+      <c r="AH165" t="n">
+        <v>0.8319</v>
+      </c>
+      <c r="AI165" t="n">
+        <v>0.0505</v>
+      </c>
+      <c r="AJ165" t="n">
+        <v>0.1131</v>
+      </c>
+      <c r="AK165" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL165" t="n">
+        <v>0.926</v>
+      </c>
+      <c r="AM165" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="AN165" t="n">
+        <v>0.07199999999999999</v>
+      </c>
+      <c r="AO165" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP165" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ165" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="166">

</xml_diff>

<commit_message>
Play-test 14 space ships: ventral guns, missiles, no railguns, own paint
Icarus/Mk.0/Daedalus ventral guns; Hyperion/Theia/Coeus 155/203 mm, VLS, pods, Spike.
Data CHANGES PT14-SP-1..32; DECISIONS 'Play-test 14 space ships after R4 (lane space)'.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/models/quality_report.xlsx
+++ b/Docs/models/quality_report.xlsx
@@ -6657,7 +6657,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>30614</v>
+        <v>34364</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>82.7</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -6686,87 +6686,87 @@
         </is>
       </c>
       <c r="N32" t="n">
-        <v>0.021</v>
+        <v>0.014</v>
       </c>
       <c r="O32" t="n">
-        <v>0.011</v>
+        <v>0.006</v>
       </c>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="n">
-        <v>1.5477</v>
+        <v>1.5767</v>
       </c>
       <c r="R32" t="n">
-        <v>0.1041</v>
+        <v>0.1108</v>
       </c>
       <c r="S32" t="n">
-        <v>2.4142</v>
+        <v>2.7949</v>
       </c>
       <c r="T32" t="n">
-        <v>0.0157</v>
+        <v>0.0191</v>
       </c>
       <c r="U32" t="inlineStr"/>
       <c r="V32" t="n">
-        <v>461</v>
+        <v>523</v>
       </c>
       <c r="W32" t="n">
-        <v>157</v>
+        <v>178</v>
       </c>
       <c r="X32" t="n">
-        <v>1.2426</v>
+        <v>1.4227</v>
       </c>
       <c r="Y32" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Z32" t="n">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="AA32" t="n">
-        <v>324</v>
+        <v>371</v>
       </c>
       <c r="AB32" t="n">
-        <v>0.9972</v>
+        <v>1.119</v>
       </c>
       <c r="AC32" t="n">
-        <v>2.5643</v>
+        <v>2.9654</v>
       </c>
       <c r="AD32" t="n">
-        <v>126.3493</v>
+        <v>125.1106</v>
       </c>
       <c r="AE32" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="AF32" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AG32" t="n">
-        <v>0.4299</v>
+        <v>0.381</v>
       </c>
       <c r="AH32" t="n">
         <v>1</v>
       </c>
       <c r="AI32" t="n">
-        <v>0.2416</v>
+        <v>0.2175</v>
       </c>
       <c r="AJ32" t="n">
-        <v>-0.0009</v>
+        <v>0.0548</v>
       </c>
       <c r="AK32" t="n">
         <v>0</v>
       </c>
       <c r="AL32" t="n">
-        <v>0.676</v>
+        <v>0.712</v>
       </c>
       <c r="AM32" t="n">
-        <v>0.953</v>
+        <v>1</v>
       </c>
       <c r="AN32" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="AO32" t="n">
-        <v>0.993</v>
+        <v>1</v>
       </c>
       <c r="AP32" t="n">
-        <v>0.631</v>
+        <v>0.717</v>
       </c>
       <c r="AQ32" t="n">
         <v>1</v>
@@ -7999,10 +7999,8 @@
           <t>daedalus</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>28160</t>
-        </is>
+      <c r="E39" t="n">
+        <v>33636</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -8010,10 +8008,8 @@
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>86.4</t>
-        </is>
+      <c r="H39" t="n">
+        <v>89</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
@@ -8032,147 +8028,91 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>0.016</t>
-        </is>
-      </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>0.017</t>
-        </is>
+      <c r="N39" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0.025</v>
       </c>
       <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr">
-        <is>
-          <t>1.4197</t>
-        </is>
-      </c>
-      <c r="R39" t="inlineStr">
-        <is>
-          <t>0.1861</t>
-        </is>
-      </c>
-      <c r="S39" t="inlineStr">
-        <is>
-          <t>5.1808</t>
-        </is>
-      </c>
-      <c r="T39" t="inlineStr">
-        <is>
-          <t>0.0362</t>
-        </is>
+      <c r="Q39" t="n">
+        <v>1.4976</v>
+      </c>
+      <c r="R39" t="n">
+        <v>0.1726</v>
+      </c>
+      <c r="S39" t="n">
+        <v>4.7997</v>
+      </c>
+      <c r="T39" t="n">
+        <v>0.0362</v>
       </c>
       <c r="U39" t="inlineStr"/>
-      <c r="V39" t="inlineStr">
-        <is>
-          <t>1134</t>
-        </is>
-      </c>
-      <c r="W39" t="inlineStr">
-        <is>
-          <t>275</t>
-        </is>
-      </c>
-      <c r="X39" t="inlineStr">
-        <is>
-          <t>1.8311</t>
-        </is>
-      </c>
-      <c r="Y39" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="Z39" t="inlineStr">
-        <is>
-          <t>181</t>
-        </is>
-      </c>
-      <c r="AA39" t="inlineStr">
-        <is>
-          <t>937</t>
-        </is>
-      </c>
-      <c r="AB39" t="inlineStr">
-        <is>
-          <t>1.2052</t>
-        </is>
-      </c>
-      <c r="AC39" t="inlineStr">
-        <is>
-          <t>6.2391</t>
-        </is>
-      </c>
-      <c r="AD39" t="inlineStr">
-        <is>
-          <t>150.1808</t>
-        </is>
-      </c>
-      <c r="AE39" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="AF39" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="AG39" t="inlineStr">
-        <is>
-          <t>0.2193</t>
-        </is>
-      </c>
-      <c r="AH39" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AI39" t="inlineStr">
-        <is>
-          <t>0.1705</t>
-        </is>
-      </c>
-      <c r="AJ39" t="inlineStr">
-        <is>
-          <t>0.0733</t>
-        </is>
-      </c>
-      <c r="AK39" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AL39" t="inlineStr">
-        <is>
-          <t>0.528</t>
-        </is>
-      </c>
-      <c r="AM39" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AN39" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AO39" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AP39" t="inlineStr">
-        <is>
-          <t>0.881</t>
-        </is>
-      </c>
-      <c r="AQ39" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="V39" t="n">
+        <v>1226</v>
+      </c>
+      <c r="W39" t="n">
+        <v>296</v>
+      </c>
+      <c r="X39" t="n">
+        <v>1.9158</v>
+      </c>
+      <c r="Y39" t="n">
+        <v>16</v>
+      </c>
+      <c r="Z39" t="n">
+        <v>191</v>
+      </c>
+      <c r="AA39" t="n">
+        <v>1019</v>
+      </c>
+      <c r="AB39" t="n">
+        <v>1.2362</v>
+      </c>
+      <c r="AC39" t="n">
+        <v>6.5952</v>
+      </c>
+      <c r="AD39" t="n">
+        <v>154.5063</v>
+      </c>
+      <c r="AE39" t="n">
+        <v>23</v>
+      </c>
+      <c r="AF39" t="n">
+        <v>15</v>
+      </c>
+      <c r="AG39" t="n">
+        <v>0.223</v>
+      </c>
+      <c r="AH39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI39" t="n">
+        <v>0.1585</v>
+      </c>
+      <c r="AJ39" t="n">
+        <v>0.1006</v>
+      </c>
+      <c r="AK39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL39" t="n">
+        <v>0.626</v>
+      </c>
+      <c r="AM39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP39" t="n">
+        <v>0.891</v>
+      </c>
+      <c r="AQ39" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -17997,8 +17937,10 @@
           <t>hydra</t>
         </is>
       </c>
-      <c r="E89" t="n">
-        <v>20080</v>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>20080</t>
+        </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
@@ -18006,8 +17948,10 @@
         </is>
       </c>
       <c r="G89" t="inlineStr"/>
-      <c r="H89" t="n">
-        <v>99.7</v>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>99.7</t>
+        </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
@@ -18026,91 +17970,147 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N89" t="n">
-        <v>0.024</v>
-      </c>
-      <c r="O89" t="n">
-        <v>0.02</v>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>0.024</t>
+        </is>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
       </c>
       <c r="P89" t="inlineStr"/>
-      <c r="Q89" t="n">
-        <v>1.2665</v>
-      </c>
-      <c r="R89" t="n">
-        <v>0.1022</v>
-      </c>
-      <c r="S89" t="n">
-        <v>2.703</v>
-      </c>
-      <c r="T89" t="n">
-        <v>0.0364</v>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>1.2665</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>0.1022</t>
+        </is>
+      </c>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t>2.703</t>
+        </is>
+      </c>
+      <c r="T89" t="inlineStr">
+        <is>
+          <t>0.0364</t>
+        </is>
       </c>
       <c r="U89" t="inlineStr"/>
-      <c r="V89" t="n">
-        <v>526</v>
-      </c>
-      <c r="W89" t="n">
-        <v>89</v>
-      </c>
-      <c r="X89" t="n">
-        <v>2.3108</v>
-      </c>
-      <c r="Y89" t="n">
-        <v>13</v>
-      </c>
-      <c r="Z89" t="n">
-        <v>62</v>
-      </c>
-      <c r="AA89" t="n">
-        <v>451</v>
-      </c>
-      <c r="AB89" t="n">
-        <v>1.6098</v>
-      </c>
-      <c r="AC89" t="n">
-        <v>11.7097</v>
-      </c>
-      <c r="AD89" t="n">
-        <v>38.5152</v>
-      </c>
-      <c r="AE89" t="n">
-        <v>40</v>
-      </c>
-      <c r="AF89" t="n">
-        <v>11</v>
-      </c>
-      <c r="AG89" t="n">
-        <v>0.2661</v>
-      </c>
-      <c r="AH89" t="n">
-        <v>0.7985</v>
-      </c>
-      <c r="AI89" t="n">
-        <v>0.0202</v>
-      </c>
-      <c r="AJ89" t="n">
-        <v>0.1366</v>
-      </c>
-      <c r="AK89" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL89" t="n">
-        <v>0.987</v>
-      </c>
-      <c r="AM89" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN89" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO89" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP89" t="n">
-        <v>0.999</v>
-      </c>
-      <c r="AQ89" t="n">
-        <v>1</v>
+      <c r="V89" t="inlineStr">
+        <is>
+          <t>526</t>
+        </is>
+      </c>
+      <c r="W89" t="inlineStr">
+        <is>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="X89" t="inlineStr">
+        <is>
+          <t>2.3108</t>
+        </is>
+      </c>
+      <c r="Y89" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="Z89" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="AA89" t="inlineStr">
+        <is>
+          <t>451</t>
+        </is>
+      </c>
+      <c r="AB89" t="inlineStr">
+        <is>
+          <t>1.6098</t>
+        </is>
+      </c>
+      <c r="AC89" t="inlineStr">
+        <is>
+          <t>11.7097</t>
+        </is>
+      </c>
+      <c r="AD89" t="inlineStr">
+        <is>
+          <t>38.5152</t>
+        </is>
+      </c>
+      <c r="AE89" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="AF89" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="AG89" t="inlineStr">
+        <is>
+          <t>0.2661</t>
+        </is>
+      </c>
+      <c r="AH89" t="inlineStr">
+        <is>
+          <t>0.7985</t>
+        </is>
+      </c>
+      <c r="AI89" t="inlineStr">
+        <is>
+          <t>0.0202</t>
+        </is>
+      </c>
+      <c r="AJ89" t="inlineStr">
+        <is>
+          <t>0.1366</t>
+        </is>
+      </c>
+      <c r="AK89" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL89" t="inlineStr">
+        <is>
+          <t>0.987</t>
+        </is>
+      </c>
+      <c r="AM89" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN89" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO89" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AP89" t="inlineStr">
+        <is>
+          <t>0.999</t>
+        </is>
+      </c>
+      <c r="AQ89" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
     </row>
     <row r="90">
@@ -18135,7 +18135,7 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>67352</v>
+        <v>71400</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -18144,7 +18144,7 @@
       </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="n">
-        <v>85.8</v>
+        <v>88</v>
       </c>
       <c r="I90" t="inlineStr">
         <is>
@@ -18164,75 +18164,75 @@
         </is>
       </c>
       <c r="N90" t="n">
-        <v>0.015</v>
+        <v>0.022</v>
       </c>
       <c r="O90" t="n">
-        <v>0.006</v>
+        <v>0.014</v>
       </c>
       <c r="P90" t="inlineStr"/>
       <c r="Q90" t="n">
-        <v>1.3784</v>
+        <v>1.437</v>
       </c>
       <c r="R90" t="n">
-        <v>0.1388</v>
+        <v>0.1396</v>
       </c>
       <c r="S90" t="n">
-        <v>3.3947</v>
+        <v>3.7001</v>
       </c>
       <c r="T90" t="n">
-        <v>0.0143</v>
+        <v>0.0149</v>
       </c>
       <c r="U90" t="inlineStr"/>
       <c r="V90" t="n">
-        <v>934</v>
+        <v>1016</v>
       </c>
       <c r="W90" t="n">
-        <v>212</v>
+        <v>236</v>
       </c>
       <c r="X90" t="n">
-        <v>1.4989</v>
+        <v>1.6527</v>
       </c>
       <c r="Y90" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="Z90" t="n">
-        <v>171</v>
+        <v>183</v>
       </c>
       <c r="AA90" t="n">
-        <v>753</v>
+        <v>819</v>
       </c>
       <c r="AB90" t="n">
-        <v>1.209</v>
+        <v>1.2815</v>
       </c>
       <c r="AC90" t="n">
-        <v>5.3238</v>
+        <v>5.7353</v>
       </c>
       <c r="AD90" t="n">
-        <v>141.4408</v>
+        <v>142.8004</v>
       </c>
       <c r="AE90" t="n">
         <v>11</v>
       </c>
       <c r="AF90" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="AG90" t="n">
-        <v>0.4412</v>
+        <v>0.402</v>
       </c>
       <c r="AH90" t="n">
         <v>1</v>
       </c>
       <c r="AI90" t="n">
-        <v>0.2461</v>
+        <v>0.2081</v>
       </c>
       <c r="AJ90" t="n">
-        <v>0.0159</v>
+        <v>-0.0107</v>
       </c>
       <c r="AK90" t="n">
         <v>0</v>
       </c>
       <c r="AL90" t="n">
-        <v>0.467</v>
+        <v>0.539</v>
       </c>
       <c r="AM90" t="n">
         <v>1</v>
@@ -18244,7 +18244,7 @@
         <v>1</v>
       </c>
       <c r="AP90" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.967</v>
       </c>
       <c r="AQ90" t="n">
         <v>1</v>
@@ -18271,10 +18271,8 @@
           <t>icarus_mk0</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>28148</t>
-        </is>
+      <c r="E91" t="n">
+        <v>31652</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -18282,10 +18280,8 @@
         </is>
       </c>
       <c r="G91" t="inlineStr"/>
-      <c r="H91" t="inlineStr">
-        <is>
-          <t>94.6</t>
-        </is>
+      <c r="H91" t="n">
+        <v>99</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>
@@ -18304,147 +18300,91 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N91" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
-      <c r="O91" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
+      <c r="N91" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="O91" t="n">
+        <v>0.012</v>
       </c>
       <c r="P91" t="inlineStr"/>
-      <c r="Q91" t="inlineStr">
-        <is>
-          <t>1.6358</t>
-        </is>
-      </c>
-      <c r="R91" t="inlineStr">
-        <is>
-          <t>0.1983</t>
-        </is>
-      </c>
-      <c r="S91" t="inlineStr">
-        <is>
-          <t>5.8141</t>
-        </is>
-      </c>
-      <c r="T91" t="inlineStr">
-        <is>
-          <t>0.033</t>
-        </is>
+      <c r="Q91" t="n">
+        <v>1.7781</v>
+      </c>
+      <c r="R91" t="n">
+        <v>0.1991</v>
+      </c>
+      <c r="S91" t="n">
+        <v>5.9064</v>
+      </c>
+      <c r="T91" t="n">
+        <v>0.033</v>
       </c>
       <c r="U91" t="inlineStr"/>
-      <c r="V91" t="inlineStr">
-        <is>
-          <t>767</t>
-        </is>
-      </c>
-      <c r="W91" t="inlineStr">
-        <is>
-          <t>242</t>
-        </is>
-      </c>
-      <c r="X91" t="inlineStr">
-        <is>
-          <t>3.1061</t>
-        </is>
-      </c>
-      <c r="Y91" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="Z91" t="inlineStr">
-        <is>
-          <t>205</t>
-        </is>
-      </c>
-      <c r="AA91" t="inlineStr">
-        <is>
-          <t>540</t>
-        </is>
-      </c>
-      <c r="AB91" t="inlineStr">
-        <is>
-          <t>2.6312</t>
-        </is>
-      </c>
-      <c r="AC91" t="inlineStr">
-        <is>
-          <t>6.931</t>
-        </is>
-      </c>
-      <c r="AD91" t="inlineStr">
-        <is>
-          <t>77.9111</t>
-        </is>
-      </c>
-      <c r="AE91" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="AF91" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="AG91" t="inlineStr">
-        <is>
-          <t>0.1809</t>
-        </is>
-      </c>
-      <c r="AH91" t="inlineStr">
-        <is>
-          <t>0.8567</t>
-        </is>
-      </c>
-      <c r="AI91" t="inlineStr">
-        <is>
-          <t>0.0513</t>
-        </is>
-      </c>
-      <c r="AJ91" t="inlineStr">
-        <is>
-          <t>-0.0344</t>
-        </is>
-      </c>
-      <c r="AK91" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AL91" t="inlineStr">
-        <is>
-          <t>0.785</t>
-        </is>
-      </c>
-      <c r="AM91" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AN91" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AO91" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AP91" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AQ91" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="V91" t="n">
+        <v>843</v>
+      </c>
+      <c r="W91" t="n">
+        <v>258</v>
+      </c>
+      <c r="X91" t="n">
+        <v>3.2651</v>
+      </c>
+      <c r="Y91" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z91" t="n">
+        <v>207</v>
+      </c>
+      <c r="AA91" t="n">
+        <v>614</v>
+      </c>
+      <c r="AB91" t="n">
+        <v>2.6197</v>
+      </c>
+      <c r="AC91" t="n">
+        <v>7.7704</v>
+      </c>
+      <c r="AD91" t="n">
+        <v>79.0179</v>
+      </c>
+      <c r="AE91" t="n">
+        <v>18</v>
+      </c>
+      <c r="AF91" t="n">
+        <v>22</v>
+      </c>
+      <c r="AG91" t="n">
+        <v>0.1527</v>
+      </c>
+      <c r="AH91" t="n">
+        <v>0.8399</v>
+      </c>
+      <c r="AI91" t="n">
+        <v>0.0505</v>
+      </c>
+      <c r="AJ91" t="n">
+        <v>0.0706</v>
+      </c>
+      <c r="AK91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL91" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="AM91" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN91" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO91" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP91" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ91" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="92">
@@ -24454,8 +24394,10 @@
           <t>nyx</t>
         </is>
       </c>
-      <c r="E122" t="n">
-        <v>23034</v>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>23034</t>
+        </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
@@ -24463,8 +24405,10 @@
         </is>
       </c>
       <c r="G122" t="inlineStr"/>
-      <c r="H122" t="n">
-        <v>98.5</v>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>98.5</t>
+        </is>
       </c>
       <c r="I122" t="inlineStr">
         <is>
@@ -24483,91 +24427,147 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N122" t="n">
-        <v>0.025</v>
-      </c>
-      <c r="O122" t="n">
-        <v>0.026</v>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>0.025</t>
+        </is>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>0.026</t>
+        </is>
       </c>
       <c r="P122" t="inlineStr"/>
-      <c r="Q122" t="n">
-        <v>1.3584</v>
-      </c>
-      <c r="R122" t="n">
-        <v>0.1021</v>
-      </c>
-      <c r="S122" t="n">
-        <v>2.3914</v>
-      </c>
-      <c r="T122" t="n">
-        <v>0.0342</v>
+      <c r="Q122" t="inlineStr">
+        <is>
+          <t>1.3584</t>
+        </is>
+      </c>
+      <c r="R122" t="inlineStr">
+        <is>
+          <t>0.1021</t>
+        </is>
+      </c>
+      <c r="S122" t="inlineStr">
+        <is>
+          <t>2.3914</t>
+        </is>
+      </c>
+      <c r="T122" t="inlineStr">
+        <is>
+          <t>0.0342</t>
+        </is>
       </c>
       <c r="U122" t="inlineStr"/>
-      <c r="V122" t="n">
-        <v>769</v>
-      </c>
-      <c r="W122" t="n">
-        <v>128</v>
-      </c>
-      <c r="X122" t="n">
-        <v>1.4512</v>
-      </c>
-      <c r="Y122" t="n">
-        <v>23</v>
-      </c>
-      <c r="Z122" t="n">
-        <v>105</v>
-      </c>
-      <c r="AA122" t="n">
-        <v>641</v>
-      </c>
-      <c r="AB122" t="n">
-        <v>1.1904</v>
-      </c>
-      <c r="AC122" t="n">
-        <v>7.2674</v>
-      </c>
-      <c r="AD122" t="n">
-        <v>88.20229999999999</v>
-      </c>
-      <c r="AE122" t="n">
-        <v>8</v>
-      </c>
-      <c r="AF122" t="n">
-        <v>15</v>
-      </c>
-      <c r="AG122" t="n">
-        <v>0.2844</v>
-      </c>
-      <c r="AH122" t="n">
-        <v>0.8308</v>
-      </c>
-      <c r="AI122" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="AJ122" t="n">
-        <v>0.0997</v>
-      </c>
-      <c r="AK122" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL122" t="n">
-        <v>0.994</v>
-      </c>
-      <c r="AM122" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN122" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO122" t="n">
-        <v>0.987</v>
-      </c>
-      <c r="AP122" t="n">
-        <v>0.929</v>
-      </c>
-      <c r="AQ122" t="n">
-        <v>1</v>
+      <c r="V122" t="inlineStr">
+        <is>
+          <t>769</t>
+        </is>
+      </c>
+      <c r="W122" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
+      <c r="X122" t="inlineStr">
+        <is>
+          <t>1.4512</t>
+        </is>
+      </c>
+      <c r="Y122" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="Z122" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="AA122" t="inlineStr">
+        <is>
+          <t>641</t>
+        </is>
+      </c>
+      <c r="AB122" t="inlineStr">
+        <is>
+          <t>1.1904</t>
+        </is>
+      </c>
+      <c r="AC122" t="inlineStr">
+        <is>
+          <t>7.2674</t>
+        </is>
+      </c>
+      <c r="AD122" t="inlineStr">
+        <is>
+          <t>88.2023</t>
+        </is>
+      </c>
+      <c r="AE122" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AF122" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="AG122" t="inlineStr">
+        <is>
+          <t>0.2844</t>
+        </is>
+      </c>
+      <c r="AH122" t="inlineStr">
+        <is>
+          <t>0.8308</t>
+        </is>
+      </c>
+      <c r="AI122" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="AJ122" t="inlineStr">
+        <is>
+          <t>0.0997</t>
+        </is>
+      </c>
+      <c r="AK122" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AL122" t="inlineStr">
+        <is>
+          <t>0.994</t>
+        </is>
+      </c>
+      <c r="AM122" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN122" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO122" t="inlineStr">
+        <is>
+          <t>0.987</t>
+        </is>
+      </c>
+      <c r="AP122" t="inlineStr">
+        <is>
+          <t>0.929</t>
+        </is>
+      </c>
+      <c r="AQ122" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
     </row>
     <row r="123">
@@ -29387,10 +29387,8 @@
           <t>silver_bug</t>
         </is>
       </c>
-      <c r="E147" t="inlineStr">
-        <is>
-          <t>58220</t>
-        </is>
+      <c r="E147" t="n">
+        <v>67592</v>
       </c>
       <c r="F147" t="inlineStr">
         <is>
@@ -29398,10 +29396,8 @@
         </is>
       </c>
       <c r="G147" t="inlineStr"/>
-      <c r="H147" t="inlineStr">
-        <is>
-          <t>92.9</t>
-        </is>
+      <c r="H147" t="n">
+        <v>95.3</v>
       </c>
       <c r="I147" t="inlineStr">
         <is>
@@ -29420,147 +29416,91 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N147" t="inlineStr">
-        <is>
-          <t>0.027</t>
-        </is>
-      </c>
-      <c r="O147" t="inlineStr">
-        <is>
-          <t>0.027</t>
-        </is>
+      <c r="N147" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="O147" t="n">
+        <v>0.022</v>
       </c>
       <c r="P147" t="inlineStr"/>
-      <c r="Q147" t="inlineStr">
-        <is>
-          <t>1.5926</t>
-        </is>
-      </c>
-      <c r="R147" t="inlineStr">
-        <is>
-          <t>0.2285</t>
-        </is>
-      </c>
-      <c r="S147" t="inlineStr">
-        <is>
-          <t>7.7112</t>
-        </is>
-      </c>
-      <c r="T147" t="inlineStr">
-        <is>
-          <t>0.0226</t>
-        </is>
+      <c r="Q147" t="n">
+        <v>1.671</v>
+      </c>
+      <c r="R147" t="n">
+        <v>0.2256</v>
+      </c>
+      <c r="S147" t="n">
+        <v>7.4384</v>
+      </c>
+      <c r="T147" t="n">
+        <v>0.0224</v>
       </c>
       <c r="U147" t="inlineStr"/>
-      <c r="V147" t="inlineStr">
-        <is>
-          <t>1299</t>
-        </is>
-      </c>
-      <c r="W147" t="inlineStr">
-        <is>
-          <t>318</t>
-        </is>
-      </c>
-      <c r="X147" t="inlineStr">
-        <is>
-          <t>2.3291</t>
-        </is>
-      </c>
-      <c r="Y147" t="inlineStr">
-        <is>
-          <t>52</t>
-        </is>
-      </c>
-      <c r="Z147" t="inlineStr">
-        <is>
-          <t>233</t>
-        </is>
-      </c>
-      <c r="AA147" t="inlineStr">
-        <is>
-          <t>1014</t>
-        </is>
-      </c>
-      <c r="AB147" t="inlineStr">
-        <is>
-          <t>1.7066</t>
-        </is>
-      </c>
-      <c r="AC147" t="inlineStr">
-        <is>
-          <t>7.4269</t>
-        </is>
-      </c>
-      <c r="AD147" t="inlineStr">
-        <is>
-          <t>136.5308</t>
-        </is>
-      </c>
-      <c r="AE147" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="AF147" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="AG147" t="inlineStr">
-        <is>
-          <t>0.1881</t>
-        </is>
-      </c>
-      <c r="AH147" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AI147" t="inlineStr">
-        <is>
-          <t>0.1171</t>
-        </is>
-      </c>
-      <c r="AJ147" t="inlineStr">
-        <is>
-          <t>0.0169</t>
-        </is>
-      </c>
-      <c r="AK147" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AL147" t="inlineStr">
-        <is>
-          <t>0.716</t>
-        </is>
-      </c>
-      <c r="AM147" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AN147" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AO147" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AP147" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AQ147" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="V147" t="n">
+        <v>1407</v>
+      </c>
+      <c r="W147" t="n">
+        <v>345</v>
+      </c>
+      <c r="X147" t="n">
+        <v>2.3859</v>
+      </c>
+      <c r="Y147" t="n">
+        <v>52</v>
+      </c>
+      <c r="Z147" t="n">
+        <v>259</v>
+      </c>
+      <c r="AA147" t="n">
+        <v>1096</v>
+      </c>
+      <c r="AB147" t="n">
+        <v>1.7912</v>
+      </c>
+      <c r="AC147" t="n">
+        <v>7.5797</v>
+      </c>
+      <c r="AD147" t="n">
+        <v>144.5972</v>
+      </c>
+      <c r="AE147" t="n">
+        <v>16</v>
+      </c>
+      <c r="AF147" t="n">
+        <v>20</v>
+      </c>
+      <c r="AG147" t="n">
+        <v>0.1914</v>
+      </c>
+      <c r="AH147" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI147" t="n">
+        <v>0.1088</v>
+      </c>
+      <c r="AJ147" t="n">
+        <v>0.0638</v>
+      </c>
+      <c r="AK147" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL147" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="AM147" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN147" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO147" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP147" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ147" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="148">
@@ -29582,7 +29522,7 @@
       <c r="D148" t="inlineStr"/>
       <c r="E148" t="inlineStr">
         <is>
-          <t>60090</t>
+          <t>69462</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -29597,7 +29537,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>66.6</t>
+          <t>66.5</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -29619,28 +29559,28 @@
       </c>
       <c r="N148" t="inlineStr">
         <is>
-          <t>0.023</t>
+          <t>0.019</t>
         </is>
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>0.024</t>
+          <t>0.02</t>
         </is>
       </c>
       <c r="P148" t="inlineStr"/>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>1.3848</t>
+          <t>1.4018</t>
         </is>
       </c>
       <c r="R148" t="inlineStr">
         <is>
-          <t>0.0914</t>
+          <t>0.0897</t>
         </is>
       </c>
       <c r="S148" t="inlineStr">
         <is>
-          <t>2.7648</t>
+          <t>2.67</t>
         </is>
       </c>
       <c r="T148" t="inlineStr">
@@ -29651,17 +29591,17 @@
       <c r="U148" t="inlineStr"/>
       <c r="V148" t="inlineStr">
         <is>
-          <t>1387</t>
+          <t>1495</t>
         </is>
       </c>
       <c r="W148" t="inlineStr">
         <is>
-          <t>370</t>
+          <t>396</t>
         </is>
       </c>
       <c r="X148" t="inlineStr">
         <is>
-          <t>2.966</t>
+          <t>3.0514</t>
         </is>
       </c>
       <c r="Y148" t="inlineStr">
@@ -29671,42 +29611,42 @@
       </c>
       <c r="Z148" t="inlineStr">
         <is>
-          <t>203</t>
+          <t>225</t>
         </is>
       </c>
       <c r="AA148" t="inlineStr">
         <is>
-          <t>1157</t>
+          <t>1243</t>
         </is>
       </c>
       <c r="AB148" t="inlineStr">
         <is>
-          <t>1.6273</t>
+          <t>1.7337</t>
         </is>
       </c>
       <c r="AC148" t="inlineStr">
         <is>
-          <t>9.2748</t>
+          <t>9.5779</t>
         </is>
       </c>
       <c r="AD148" t="inlineStr">
         <is>
-          <t>124.7461</t>
+          <t>129.7781</t>
         </is>
       </c>
       <c r="AE148" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>16</t>
         </is>
       </c>
       <c r="AF148" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>21</t>
         </is>
       </c>
       <c r="AG148" t="inlineStr">
         <is>
-          <t>0.1366</t>
+          <t>0.1347</t>
         </is>
       </c>
       <c r="AH148" t="inlineStr">
@@ -29716,12 +29656,12 @@
       </c>
       <c r="AI148" t="inlineStr">
         <is>
-          <t>0.1041</t>
+          <t>0.092</t>
         </is>
       </c>
       <c r="AJ148" t="inlineStr">
         <is>
-          <t>0.0283</t>
+          <t>0.1172</t>
         </is>
       </c>
       <c r="AK148" t="inlineStr">
@@ -29731,17 +29671,17 @@
       </c>
       <c r="AL148" t="inlineStr">
         <is>
-          <t>0.266</t>
+          <t>0.278</t>
         </is>
       </c>
       <c r="AM148" t="inlineStr">
         <is>
-          <t>0.569</t>
+          <t>0.559</t>
         </is>
       </c>
       <c r="AN148" t="inlineStr">
         <is>
-          <t>0.426</t>
+          <t>0.412</t>
         </is>
       </c>
       <c r="AO148" t="inlineStr">
@@ -31961,7 +31901,7 @@
         </is>
       </c>
       <c r="E160" t="n">
-        <v>30454</v>
+        <v>36650</v>
       </c>
       <c r="F160" t="inlineStr">
         <is>
@@ -31970,7 +31910,7 @@
       </c>
       <c r="G160" t="inlineStr"/>
       <c r="H160" t="n">
-        <v>81.5</v>
+        <v>81.2</v>
       </c>
       <c r="I160" t="inlineStr">
         <is>
@@ -31990,75 +31930,75 @@
         </is>
       </c>
       <c r="N160" t="n">
-        <v>0.008</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="O160" t="n">
-        <v>0.008</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="P160" t="inlineStr"/>
       <c r="Q160" t="n">
-        <v>1.4545</v>
+        <v>1.4938</v>
       </c>
       <c r="R160" t="n">
-        <v>0.1296</v>
+        <v>0.1345</v>
       </c>
       <c r="S160" t="n">
-        <v>3.2355</v>
+        <v>3.4213</v>
       </c>
       <c r="T160" t="n">
-        <v>0.0214</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="U160" t="inlineStr"/>
       <c r="V160" t="n">
-        <v>449</v>
+        <v>573</v>
       </c>
       <c r="W160" t="n">
-        <v>151</v>
+        <v>178</v>
       </c>
       <c r="X160" t="n">
-        <v>1.177</v>
+        <v>1.331</v>
       </c>
       <c r="Y160" t="n">
         <v>8</v>
       </c>
       <c r="Z160" t="n">
-        <v>107</v>
+        <v>149</v>
       </c>
       <c r="AA160" t="n">
-        <v>334</v>
+        <v>416</v>
       </c>
       <c r="AB160" t="n">
-        <v>0.834</v>
+        <v>1.1141</v>
       </c>
       <c r="AC160" t="n">
-        <v>2.6034</v>
+        <v>3.1106</v>
       </c>
       <c r="AD160" t="n">
-        <v>128.2948</v>
+        <v>133.7366</v>
       </c>
       <c r="AE160" t="n">
         <v>9</v>
       </c>
       <c r="AF160" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="AG160" t="n">
-        <v>0.4393</v>
+        <v>0.3609</v>
       </c>
       <c r="AH160" t="n">
         <v>1</v>
       </c>
       <c r="AI160" t="n">
-        <v>0.2216</v>
+        <v>0.2215</v>
       </c>
       <c r="AJ160" t="n">
-        <v>0.0256</v>
+        <v>0.0667</v>
       </c>
       <c r="AK160" t="n">
         <v>0</v>
       </c>
       <c r="AL160" t="n">
-        <v>0.5610000000000001</v>
+        <v>0.609</v>
       </c>
       <c r="AM160" t="n">
         <v>1</v>
@@ -32067,13 +32007,13 @@
         <v>1</v>
       </c>
       <c r="AO160" t="n">
-        <v>0.9409999999999999</v>
+        <v>1</v>
       </c>
       <c r="AP160" t="n">
-        <v>0.576</v>
+        <v>0.731</v>
       </c>
       <c r="AQ160" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="161">

</xml_diff>

<commit_message>
Naval models A: frigate AK-100 larger, torpedo tubes in team paint
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/models/quality_report.xlsx
+++ b/Docs/models/quality_report.xlsx
@@ -12244,8 +12244,10 @@
           <t>ew_corvette</t>
         </is>
       </c>
-      <c r="E60" t="n">
-        <v>8700</v>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>8700</t>
+        </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
@@ -12253,8 +12255,10 @@
         </is>
       </c>
       <c r="G60" t="inlineStr"/>
-      <c r="H60" t="n">
-        <v>83.09999999999999</v>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>83.1</t>
+        </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
@@ -12273,94 +12277,150 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N60" t="n">
-        <v>0.122</v>
-      </c>
-      <c r="O60" t="n">
-        <v>0.185</v>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>0.122</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>0.185</t>
+        </is>
       </c>
       <c r="P60" t="inlineStr">
         <is>
           <t>ciws_escort_ship</t>
         </is>
       </c>
-      <c r="Q60" t="n">
-        <v>1.4251</v>
-      </c>
-      <c r="R60" t="n">
-        <v>0.1276</v>
-      </c>
-      <c r="S60" t="n">
-        <v>3.9934</v>
-      </c>
-      <c r="T60" t="n">
-        <v>0.0348</v>
-      </c>
-      <c r="U60" t="n">
-        <v>308</v>
-      </c>
-      <c r="V60" t="n">
-        <v>113</v>
-      </c>
-      <c r="W60" t="n">
-        <v>2.1477</v>
-      </c>
-      <c r="X60" t="n">
-        <v>12</v>
-      </c>
-      <c r="Y60" t="n">
-        <v>63</v>
-      </c>
-      <c r="Z60" t="n">
-        <v>233</v>
-      </c>
-      <c r="AA60" t="n">
-        <v>1.1974</v>
-      </c>
-      <c r="AB60" t="n">
-        <v>4.4284</v>
-      </c>
-      <c r="AC60" t="n">
-        <v>52.6146</v>
-      </c>
-      <c r="AD60" t="n">
-        <v>7</v>
-      </c>
-      <c r="AE60" t="n">
-        <v>15</v>
-      </c>
-      <c r="AF60" t="n">
-        <v>0.223</v>
-      </c>
-      <c r="AG60" t="n">
-        <v>0.8137</v>
-      </c>
-      <c r="AH60" t="n">
-        <v>0.0311</v>
-      </c>
-      <c r="AI60" t="n">
-        <v>0.2254</v>
-      </c>
-      <c r="AJ60" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK60" t="n">
-        <v>0.695</v>
-      </c>
-      <c r="AL60" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="AM60" t="n">
-        <v>0.629</v>
-      </c>
-      <c r="AN60" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO60" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP60" t="n">
-        <v>1</v>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>1.4251</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>0.1276</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>3.9934</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>0.0348</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>308</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>113</t>
+        </is>
+      </c>
+      <c r="W60" t="inlineStr">
+        <is>
+          <t>2.1477</t>
+        </is>
+      </c>
+      <c r="X60" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="Y60" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="Z60" t="inlineStr">
+        <is>
+          <t>233</t>
+        </is>
+      </c>
+      <c r="AA60" t="inlineStr">
+        <is>
+          <t>1.1974</t>
+        </is>
+      </c>
+      <c r="AB60" t="inlineStr">
+        <is>
+          <t>4.4284</t>
+        </is>
+      </c>
+      <c r="AC60" t="inlineStr">
+        <is>
+          <t>52.6146</t>
+        </is>
+      </c>
+      <c r="AD60" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AE60" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="AF60" t="inlineStr">
+        <is>
+          <t>0.223</t>
+        </is>
+      </c>
+      <c r="AG60" t="inlineStr">
+        <is>
+          <t>0.8137</t>
+        </is>
+      </c>
+      <c r="AH60" t="inlineStr">
+        <is>
+          <t>0.0311</t>
+        </is>
+      </c>
+      <c r="AI60" t="inlineStr">
+        <is>
+          <t>0.2254</t>
+        </is>
+      </c>
+      <c r="AJ60" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK60" t="inlineStr">
+        <is>
+          <t>0.695</t>
+        </is>
+      </c>
+      <c r="AL60" t="inlineStr">
+        <is>
+          <t>0.751</t>
+        </is>
+      </c>
+      <c r="AM60" t="inlineStr">
+        <is>
+          <t>0.629</t>
+        </is>
+      </c>
+      <c r="AN60" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO60" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AP60" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
       <c r="AQ60" t="inlineStr"/>
     </row>
@@ -14785,10 +14845,8 @@
           <t>frigate</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>12460</t>
-        </is>
+      <c r="E73" t="n">
+        <v>12460</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -14796,10 +14854,8 @@
         </is>
       </c>
       <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>80.8</t>
-        </is>
+      <c r="H73" t="n">
+        <v>80.40000000000001</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
@@ -14818,150 +14874,94 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N73" t="inlineStr">
-        <is>
-          <t>0.129</t>
-        </is>
-      </c>
-      <c r="O73" t="inlineStr">
-        <is>
-          <t>0.202</t>
-        </is>
+      <c r="N73" t="n">
+        <v>0.129</v>
+      </c>
+      <c r="O73" t="n">
+        <v>0.202</v>
       </c>
       <c r="P73" t="inlineStr">
         <is>
           <t>missile_frigate</t>
         </is>
       </c>
-      <c r="Q73" t="inlineStr">
-        <is>
-          <t>1.4094</t>
-        </is>
-      </c>
-      <c r="R73" t="inlineStr">
-        <is>
-          <t>0.1227</t>
-        </is>
-      </c>
-      <c r="S73" t="inlineStr">
-        <is>
-          <t>3.5001</t>
-        </is>
-      </c>
-      <c r="T73" t="inlineStr">
-        <is>
-          <t>0.0379</t>
-        </is>
-      </c>
-      <c r="U73" t="inlineStr">
-        <is>
-          <t>458</t>
-        </is>
-      </c>
-      <c r="V73" t="inlineStr">
-        <is>
-          <t>149</t>
-        </is>
-      </c>
-      <c r="W73" t="inlineStr">
-        <is>
-          <t>2.9453</t>
-        </is>
-      </c>
-      <c r="X73" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="Y73" t="inlineStr">
-        <is>
-          <t>46</t>
-        </is>
-      </c>
-      <c r="Z73" t="inlineStr">
-        <is>
-          <t>400</t>
-        </is>
-      </c>
-      <c r="AA73" t="inlineStr">
-        <is>
-          <t>0.9093</t>
-        </is>
-      </c>
-      <c r="AB73" t="inlineStr">
-        <is>
-          <t>7.9067</t>
-        </is>
-      </c>
-      <c r="AC73" t="inlineStr">
-        <is>
-          <t>50.5897</t>
-        </is>
-      </c>
-      <c r="AD73" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="AE73" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="AF73" t="inlineStr">
-        <is>
-          <t>0.2193</t>
-        </is>
-      </c>
-      <c r="AG73" t="inlineStr">
-        <is>
-          <t>0.8137</t>
-        </is>
-      </c>
-      <c r="AH73" t="inlineStr">
-        <is>
-          <t>0.0365</t>
-        </is>
-      </c>
-      <c r="AI73" t="inlineStr">
-        <is>
-          <t>0.2351</t>
-        </is>
-      </c>
-      <c r="AJ73" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AK73" t="inlineStr">
-        <is>
-          <t>0.669</t>
-        </is>
-      </c>
-      <c r="AL73" t="inlineStr">
-        <is>
-          <t>0.723</t>
-        </is>
-      </c>
-      <c r="AM73" t="inlineStr">
-        <is>
-          <t>0.551</t>
-        </is>
-      </c>
-      <c r="AN73" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AO73" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AP73" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="Q73" t="n">
+        <v>1.3959</v>
+      </c>
+      <c r="R73" t="n">
+        <v>0.1241</v>
+      </c>
+      <c r="S73" t="n">
+        <v>3.5048</v>
+      </c>
+      <c r="T73" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="U73" t="n">
+        <v>458</v>
+      </c>
+      <c r="V73" t="n">
+        <v>149</v>
+      </c>
+      <c r="W73" t="n">
+        <v>2.9135</v>
+      </c>
+      <c r="X73" t="n">
+        <v>12</v>
+      </c>
+      <c r="Y73" t="n">
+        <v>46</v>
+      </c>
+      <c r="Z73" t="n">
+        <v>400</v>
+      </c>
+      <c r="AA73" t="n">
+        <v>0.8995</v>
+      </c>
+      <c r="AB73" t="n">
+        <v>7.8214</v>
+      </c>
+      <c r="AC73" t="n">
+        <v>51.1416</v>
+      </c>
+      <c r="AD73" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE73" t="n">
+        <v>15</v>
+      </c>
+      <c r="AF73" t="n">
+        <v>0.2193</v>
+      </c>
+      <c r="AG73" t="n">
+        <v>0.8137</v>
+      </c>
+      <c r="AH73" t="n">
+        <v>0.0363</v>
+      </c>
+      <c r="AI73" t="n">
+        <v>0.2351</v>
+      </c>
+      <c r="AJ73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK73" t="n">
+        <v>0.647</v>
+      </c>
+      <c r="AL73" t="n">
+        <v>0.731</v>
+      </c>
+      <c r="AM73" t="n">
+        <v>0.552</v>
+      </c>
+      <c r="AN73" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO73" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP73" t="n">
+        <v>1</v>
       </c>
       <c r="AQ73" t="inlineStr"/>
     </row>
@@ -24196,8 +24196,10 @@
           <t>missile_boat</t>
         </is>
       </c>
-      <c r="E120" t="n">
-        <v>5752</v>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>5752</t>
+        </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
@@ -24205,8 +24207,10 @@
         </is>
       </c>
       <c r="G120" t="inlineStr"/>
-      <c r="H120" t="n">
-        <v>87.59999999999999</v>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>87.6</t>
+        </is>
       </c>
       <c r="I120" t="inlineStr">
         <is>
@@ -24225,90 +24229,146 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N120" t="n">
-        <v>0.055</v>
-      </c>
-      <c r="O120" t="n">
-        <v>0.036</v>
+      <c r="N120" t="inlineStr">
+        <is>
+          <t>0.055</t>
+        </is>
+      </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>0.036</t>
+        </is>
       </c>
       <c r="P120" t="inlineStr"/>
-      <c r="Q120" t="n">
-        <v>1.7201</v>
-      </c>
-      <c r="R120" t="n">
-        <v>0.2122</v>
-      </c>
-      <c r="S120" t="n">
-        <v>7.9378</v>
-      </c>
-      <c r="T120" t="n">
-        <v>0.0366</v>
-      </c>
-      <c r="U120" t="n">
-        <v>214</v>
-      </c>
-      <c r="V120" t="n">
-        <v>89</v>
-      </c>
-      <c r="W120" t="n">
-        <v>1.2542</v>
-      </c>
-      <c r="X120" t="n">
-        <v>17</v>
-      </c>
-      <c r="Y120" t="n">
-        <v>56</v>
-      </c>
-      <c r="Z120" t="n">
-        <v>141</v>
-      </c>
-      <c r="AA120" t="n">
-        <v>0.7892</v>
-      </c>
-      <c r="AB120" t="n">
-        <v>1.987</v>
-      </c>
-      <c r="AC120" t="n">
-        <v>70.9598</v>
-      </c>
-      <c r="AD120" t="n">
-        <v>12</v>
-      </c>
-      <c r="AE120" t="n">
-        <v>13</v>
-      </c>
-      <c r="AF120" t="n">
-        <v>0.2084</v>
-      </c>
-      <c r="AG120" t="n">
-        <v>0.8216</v>
-      </c>
-      <c r="AH120" t="n">
-        <v>0.0484</v>
-      </c>
-      <c r="AI120" t="n">
-        <v>0.0968</v>
-      </c>
-      <c r="AJ120" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK120" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL120" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM120" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN120" t="n">
-        <v>0.831</v>
-      </c>
-      <c r="AO120" t="n">
-        <v>0.401</v>
-      </c>
-      <c r="AP120" t="n">
-        <v>1</v>
+      <c r="Q120" t="inlineStr">
+        <is>
+          <t>1.7201</t>
+        </is>
+      </c>
+      <c r="R120" t="inlineStr">
+        <is>
+          <t>0.2122</t>
+        </is>
+      </c>
+      <c r="S120" t="inlineStr">
+        <is>
+          <t>7.9378</t>
+        </is>
+      </c>
+      <c r="T120" t="inlineStr">
+        <is>
+          <t>0.0366</t>
+        </is>
+      </c>
+      <c r="U120" t="inlineStr">
+        <is>
+          <t>214</t>
+        </is>
+      </c>
+      <c r="V120" t="inlineStr">
+        <is>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="W120" t="inlineStr">
+        <is>
+          <t>1.2542</t>
+        </is>
+      </c>
+      <c r="X120" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="Y120" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="Z120" t="inlineStr">
+        <is>
+          <t>141</t>
+        </is>
+      </c>
+      <c r="AA120" t="inlineStr">
+        <is>
+          <t>0.7892</t>
+        </is>
+      </c>
+      <c r="AB120" t="inlineStr">
+        <is>
+          <t>1.987</t>
+        </is>
+      </c>
+      <c r="AC120" t="inlineStr">
+        <is>
+          <t>70.9598</t>
+        </is>
+      </c>
+      <c r="AD120" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="AE120" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="AF120" t="inlineStr">
+        <is>
+          <t>0.2084</t>
+        </is>
+      </c>
+      <c r="AG120" t="inlineStr">
+        <is>
+          <t>0.8216</t>
+        </is>
+      </c>
+      <c r="AH120" t="inlineStr">
+        <is>
+          <t>0.0484</t>
+        </is>
+      </c>
+      <c r="AI120" t="inlineStr">
+        <is>
+          <t>0.0968</t>
+        </is>
+      </c>
+      <c r="AJ120" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK120" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AL120" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AM120" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AN120" t="inlineStr">
+        <is>
+          <t>0.831</t>
+        </is>
+      </c>
+      <c r="AO120" t="inlineStr">
+        <is>
+          <t>0.401</t>
+        </is>
+      </c>
+      <c r="AP120" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
       <c r="AQ120" t="inlineStr"/>
     </row>
@@ -27710,8 +27770,10 @@
           <t>rocket_artillery_ship</t>
         </is>
       </c>
-      <c r="E138" t="n">
-        <v>9262</v>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>9262</t>
+        </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
@@ -27719,8 +27781,10 @@
         </is>
       </c>
       <c r="G138" t="inlineStr"/>
-      <c r="H138" t="n">
-        <v>83.40000000000001</v>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>83.4</t>
+        </is>
       </c>
       <c r="I138" t="inlineStr">
         <is>
@@ -27739,90 +27803,146 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N138" t="n">
-        <v>0.039</v>
-      </c>
-      <c r="O138" t="n">
-        <v>0.05</v>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>0.039</t>
+        </is>
+      </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
       </c>
       <c r="P138" t="inlineStr"/>
-      <c r="Q138" t="n">
-        <v>1.5025</v>
-      </c>
-      <c r="R138" t="n">
-        <v>0.1084</v>
-      </c>
-      <c r="S138" t="n">
-        <v>3.5042</v>
-      </c>
-      <c r="T138" t="n">
-        <v>0.0244</v>
-      </c>
-      <c r="U138" t="n">
-        <v>331</v>
-      </c>
-      <c r="V138" t="n">
-        <v>92</v>
-      </c>
-      <c r="W138" t="n">
-        <v>1.7287</v>
-      </c>
-      <c r="X138" t="n">
-        <v>13</v>
-      </c>
-      <c r="Y138" t="n">
-        <v>50</v>
-      </c>
-      <c r="Z138" t="n">
-        <v>268</v>
-      </c>
-      <c r="AA138" t="n">
-        <v>0.9395</v>
-      </c>
-      <c r="AB138" t="n">
-        <v>5.0357</v>
-      </c>
-      <c r="AC138" t="n">
-        <v>53.2203</v>
-      </c>
-      <c r="AD138" t="n">
-        <v>5</v>
-      </c>
-      <c r="AE138" t="n">
-        <v>15</v>
-      </c>
-      <c r="AF138" t="n">
-        <v>0.2048</v>
-      </c>
-      <c r="AG138" t="n">
-        <v>0.8222</v>
-      </c>
-      <c r="AH138" t="n">
-        <v>0.0485</v>
-      </c>
-      <c r="AI138" t="n">
-        <v>0.2177</v>
-      </c>
-      <c r="AJ138" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK138" t="n">
-        <v>0.821</v>
-      </c>
-      <c r="AL138" t="n">
-        <v>0.638</v>
-      </c>
-      <c r="AM138" t="n">
-        <v>0.552</v>
-      </c>
-      <c r="AN138" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO138" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP138" t="n">
-        <v>1</v>
+      <c r="Q138" t="inlineStr">
+        <is>
+          <t>1.5025</t>
+        </is>
+      </c>
+      <c r="R138" t="inlineStr">
+        <is>
+          <t>0.1084</t>
+        </is>
+      </c>
+      <c r="S138" t="inlineStr">
+        <is>
+          <t>3.5042</t>
+        </is>
+      </c>
+      <c r="T138" t="inlineStr">
+        <is>
+          <t>0.0244</t>
+        </is>
+      </c>
+      <c r="U138" t="inlineStr">
+        <is>
+          <t>331</t>
+        </is>
+      </c>
+      <c r="V138" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="W138" t="inlineStr">
+        <is>
+          <t>1.7287</t>
+        </is>
+      </c>
+      <c r="X138" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="Y138" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="Z138" t="inlineStr">
+        <is>
+          <t>268</t>
+        </is>
+      </c>
+      <c r="AA138" t="inlineStr">
+        <is>
+          <t>0.9395</t>
+        </is>
+      </c>
+      <c r="AB138" t="inlineStr">
+        <is>
+          <t>5.0357</t>
+        </is>
+      </c>
+      <c r="AC138" t="inlineStr">
+        <is>
+          <t>53.2203</t>
+        </is>
+      </c>
+      <c r="AD138" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AE138" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="AF138" t="inlineStr">
+        <is>
+          <t>0.2048</t>
+        </is>
+      </c>
+      <c r="AG138" t="inlineStr">
+        <is>
+          <t>0.8222</t>
+        </is>
+      </c>
+      <c r="AH138" t="inlineStr">
+        <is>
+          <t>0.0485</t>
+        </is>
+      </c>
+      <c r="AI138" t="inlineStr">
+        <is>
+          <t>0.2177</t>
+        </is>
+      </c>
+      <c r="AJ138" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK138" t="inlineStr">
+        <is>
+          <t>0.821</t>
+        </is>
+      </c>
+      <c r="AL138" t="inlineStr">
+        <is>
+          <t>0.638</t>
+        </is>
+      </c>
+      <c r="AM138" t="inlineStr">
+        <is>
+          <t>0.552</t>
+        </is>
+      </c>
+      <c r="AN138" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO138" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AP138" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
       <c r="AQ138" t="inlineStr"/>
     </row>
@@ -29447,8 +29567,10 @@
           <t>sea_corvette</t>
         </is>
       </c>
-      <c r="E147" t="n">
-        <v>7638</v>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>7638</t>
+        </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
@@ -29456,8 +29578,10 @@
         </is>
       </c>
       <c r="G147" t="inlineStr"/>
-      <c r="H147" t="n">
-        <v>91.90000000000001</v>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>91.9</t>
+        </is>
       </c>
       <c r="I147" t="inlineStr">
         <is>
@@ -29476,90 +29600,146 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N147" t="n">
-        <v>0.031</v>
-      </c>
-      <c r="O147" t="n">
-        <v>0.038</v>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>0.031</t>
+        </is>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>0.038</t>
+        </is>
       </c>
       <c r="P147" t="inlineStr"/>
-      <c r="Q147" t="n">
-        <v>1.5631</v>
-      </c>
-      <c r="R147" t="n">
-        <v>0.1412</v>
-      </c>
-      <c r="S147" t="n">
-        <v>4.8445</v>
-      </c>
-      <c r="T147" t="n">
-        <v>0.0288</v>
-      </c>
-      <c r="U147" t="n">
-        <v>343</v>
-      </c>
-      <c r="V147" t="n">
-        <v>113</v>
-      </c>
-      <c r="W147" t="n">
-        <v>1.5427</v>
-      </c>
-      <c r="X147" t="n">
-        <v>13</v>
-      </c>
-      <c r="Y147" t="n">
-        <v>71</v>
-      </c>
-      <c r="Z147" t="n">
-        <v>259</v>
-      </c>
-      <c r="AA147" t="n">
-        <v>0.9693000000000001</v>
-      </c>
-      <c r="AB147" t="n">
-        <v>3.536</v>
-      </c>
-      <c r="AC147" t="n">
-        <v>73.247</v>
-      </c>
-      <c r="AD147" t="n">
-        <v>10</v>
-      </c>
-      <c r="AE147" t="n">
-        <v>10</v>
-      </c>
-      <c r="AF147" t="n">
-        <v>0.2048</v>
-      </c>
-      <c r="AG147" t="n">
-        <v>0.8137</v>
-      </c>
-      <c r="AH147" t="n">
-        <v>0.0346</v>
-      </c>
-      <c r="AI147" t="n">
-        <v>0.2941</v>
-      </c>
-      <c r="AJ147" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK147" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="AL147" t="n">
-        <v>0.832</v>
-      </c>
-      <c r="AM147" t="n">
-        <v>0.763</v>
-      </c>
-      <c r="AN147" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO147" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP147" t="n">
-        <v>1</v>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>1.5631</t>
+        </is>
+      </c>
+      <c r="R147" t="inlineStr">
+        <is>
+          <t>0.1412</t>
+        </is>
+      </c>
+      <c r="S147" t="inlineStr">
+        <is>
+          <t>4.8445</t>
+        </is>
+      </c>
+      <c r="T147" t="inlineStr">
+        <is>
+          <t>0.0288</t>
+        </is>
+      </c>
+      <c r="U147" t="inlineStr">
+        <is>
+          <t>343</t>
+        </is>
+      </c>
+      <c r="V147" t="inlineStr">
+        <is>
+          <t>113</t>
+        </is>
+      </c>
+      <c r="W147" t="inlineStr">
+        <is>
+          <t>1.5427</t>
+        </is>
+      </c>
+      <c r="X147" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="Y147" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="Z147" t="inlineStr">
+        <is>
+          <t>259</t>
+        </is>
+      </c>
+      <c r="AA147" t="inlineStr">
+        <is>
+          <t>0.9693</t>
+        </is>
+      </c>
+      <c r="AB147" t="inlineStr">
+        <is>
+          <t>3.536</t>
+        </is>
+      </c>
+      <c r="AC147" t="inlineStr">
+        <is>
+          <t>73.247</t>
+        </is>
+      </c>
+      <c r="AD147" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AE147" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AF147" t="inlineStr">
+        <is>
+          <t>0.2048</t>
+        </is>
+      </c>
+      <c r="AG147" t="inlineStr">
+        <is>
+          <t>0.8137</t>
+        </is>
+      </c>
+      <c r="AH147" t="inlineStr">
+        <is>
+          <t>0.0346</t>
+        </is>
+      </c>
+      <c r="AI147" t="inlineStr">
+        <is>
+          <t>0.2941</t>
+        </is>
+      </c>
+      <c r="AJ147" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK147" t="inlineStr">
+        <is>
+          <t>0.92</t>
+        </is>
+      </c>
+      <c r="AL147" t="inlineStr">
+        <is>
+          <t>0.832</t>
+        </is>
+      </c>
+      <c r="AM147" t="inlineStr">
+        <is>
+          <t>0.763</t>
+        </is>
+      </c>
+      <c r="AN147" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO147" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AP147" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
       <c r="AQ147" t="inlineStr"/>
     </row>
@@ -29584,8 +29764,10 @@
           <t>sea_cruiser aa_destroyer battlecruiser</t>
         </is>
       </c>
-      <c r="E148" t="n">
-        <v>14150</v>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>14150</t>
+        </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
@@ -29593,8 +29775,10 @@
         </is>
       </c>
       <c r="G148" t="inlineStr"/>
-      <c r="H148" t="n">
-        <v>75.8</v>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>75.8</t>
+        </is>
       </c>
       <c r="I148" t="inlineStr">
         <is>
@@ -29613,90 +29797,146 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N148" t="n">
-        <v>0.022</v>
-      </c>
-      <c r="O148" t="n">
-        <v>0.025</v>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>0.022</t>
+        </is>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>0.025</t>
+        </is>
       </c>
       <c r="P148" t="inlineStr"/>
-      <c r="Q148" t="n">
-        <v>1.4163</v>
-      </c>
-      <c r="R148" t="n">
-        <v>0.0956</v>
-      </c>
-      <c r="S148" t="n">
-        <v>2.2835</v>
-      </c>
-      <c r="T148" t="n">
-        <v>0.036</v>
-      </c>
-      <c r="U148" t="n">
-        <v>701</v>
-      </c>
-      <c r="V148" t="n">
-        <v>142</v>
-      </c>
-      <c r="W148" t="n">
-        <v>2.1673</v>
-      </c>
-      <c r="X148" t="n">
-        <v>18</v>
-      </c>
-      <c r="Y148" t="n">
-        <v>107</v>
-      </c>
-      <c r="Z148" t="n">
-        <v>576</v>
-      </c>
-      <c r="AA148" t="n">
-        <v>1.6331</v>
-      </c>
-      <c r="AB148" t="n">
-        <v>8.7912</v>
-      </c>
-      <c r="AC148" t="n">
-        <v>65.5198</v>
-      </c>
-      <c r="AD148" t="n">
-        <v>8</v>
-      </c>
-      <c r="AE148" t="n">
-        <v>14</v>
-      </c>
-      <c r="AF148" t="n">
-        <v>0.1468</v>
-      </c>
-      <c r="AG148" t="n">
-        <v>0.8143</v>
-      </c>
-      <c r="AH148" t="n">
-        <v>0.0446</v>
-      </c>
-      <c r="AI148" t="n">
-        <v>0.2699</v>
-      </c>
-      <c r="AJ148" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK148" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="AL148" t="n">
-        <v>0.5629999999999999</v>
-      </c>
-      <c r="AM148" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="AN148" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO148" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP148" t="n">
-        <v>1</v>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>1.4163</t>
+        </is>
+      </c>
+      <c r="R148" t="inlineStr">
+        <is>
+          <t>0.0956</t>
+        </is>
+      </c>
+      <c r="S148" t="inlineStr">
+        <is>
+          <t>2.2835</t>
+        </is>
+      </c>
+      <c r="T148" t="inlineStr">
+        <is>
+          <t>0.036</t>
+        </is>
+      </c>
+      <c r="U148" t="inlineStr">
+        <is>
+          <t>701</t>
+        </is>
+      </c>
+      <c r="V148" t="inlineStr">
+        <is>
+          <t>142</t>
+        </is>
+      </c>
+      <c r="W148" t="inlineStr">
+        <is>
+          <t>2.1673</t>
+        </is>
+      </c>
+      <c r="X148" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="Y148" t="inlineStr">
+        <is>
+          <t>107</t>
+        </is>
+      </c>
+      <c r="Z148" t="inlineStr">
+        <is>
+          <t>576</t>
+        </is>
+      </c>
+      <c r="AA148" t="inlineStr">
+        <is>
+          <t>1.6331</t>
+        </is>
+      </c>
+      <c r="AB148" t="inlineStr">
+        <is>
+          <t>8.7912</t>
+        </is>
+      </c>
+      <c r="AC148" t="inlineStr">
+        <is>
+          <t>65.5198</t>
+        </is>
+      </c>
+      <c r="AD148" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="AE148" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="AF148" t="inlineStr">
+        <is>
+          <t>0.1468</t>
+        </is>
+      </c>
+      <c r="AG148" t="inlineStr">
+        <is>
+          <t>0.8143</t>
+        </is>
+      </c>
+      <c r="AH148" t="inlineStr">
+        <is>
+          <t>0.0446</t>
+        </is>
+      </c>
+      <c r="AI148" t="inlineStr">
+        <is>
+          <t>0.2699</t>
+        </is>
+      </c>
+      <c r="AJ148" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK148" t="inlineStr">
+        <is>
+          <t>0.68</t>
+        </is>
+      </c>
+      <c r="AL148" t="inlineStr">
+        <is>
+          <t>0.563</t>
+        </is>
+      </c>
+      <c r="AM148" t="inlineStr">
+        <is>
+          <t>0.36</t>
+        </is>
+      </c>
+      <c r="AN148" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO148" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AP148" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
       <c r="AQ148" t="inlineStr"/>
     </row>
@@ -33904,7 +34144,7 @@
       </c>
       <c r="G170" t="inlineStr"/>
       <c r="H170" t="n">
-        <v>92</v>
+        <v>95.3</v>
       </c>
       <c r="I170" t="inlineStr">
         <is>
@@ -33934,10 +34174,10 @@
         <v>1.4971</v>
       </c>
       <c r="R170" t="n">
-        <v>0.1505</v>
+        <v>0.1913</v>
       </c>
       <c r="S170" t="n">
-        <v>5.6864</v>
+        <v>6.7863</v>
       </c>
       <c r="T170" t="n">
         <v>0.0135</v>
@@ -33994,10 +34234,10 @@
         <v>0.8120000000000001</v>
       </c>
       <c r="AL170" t="n">
-        <v>0.887</v>
+        <v>1</v>
       </c>
       <c r="AM170" t="n">
-        <v>0.895</v>
+        <v>1</v>
       </c>
       <c r="AN170" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Barrels: narrow to the battleship triple turrets, audit report only
Other units' data, models and the Sim change reverted (owner); naval_406_bs 3 x 200,
kit rise flag for the battleship only; BARREL_AUDIT.md lists the rest.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/models/quality_report.xlsx
+++ b/Docs/models/quality_report.xlsx
@@ -5269,8 +5269,10 @@
           <t>battlecruiser</t>
         </is>
       </c>
-      <c r="E25" t="n">
-        <v>17586</v>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>17586</t>
+        </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -5278,8 +5280,10 @@
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" t="n">
-        <v>83.09999999999999</v>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>83.1</t>
+        </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -5298,90 +5302,146 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N25" t="n">
-        <v>0.075</v>
-      </c>
-      <c r="O25" t="n">
-        <v>0.099</v>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>0.075</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>0.099</t>
+        </is>
       </c>
       <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="n">
-        <v>1.4493</v>
-      </c>
-      <c r="R25" t="n">
-        <v>0.1362</v>
-      </c>
-      <c r="S25" t="n">
-        <v>3.2662</v>
-      </c>
-      <c r="T25" t="n">
-        <v>0.049</v>
-      </c>
-      <c r="U25" t="n">
-        <v>812</v>
-      </c>
-      <c r="V25" t="n">
-        <v>164</v>
-      </c>
-      <c r="W25" t="n">
-        <v>2.9855</v>
-      </c>
-      <c r="X25" t="n">
-        <v>22</v>
-      </c>
-      <c r="Y25" t="n">
-        <v>105</v>
-      </c>
-      <c r="Z25" t="n">
-        <v>685</v>
-      </c>
-      <c r="AA25" t="n">
-        <v>1.9114</v>
-      </c>
-      <c r="AB25" t="n">
-        <v>12.4697</v>
-      </c>
-      <c r="AC25" t="n">
-        <v>54.933</v>
-      </c>
-      <c r="AD25" t="n">
-        <v>10</v>
-      </c>
-      <c r="AE25" t="n">
-        <v>19</v>
-      </c>
-      <c r="AF25" t="n">
-        <v>0.2013</v>
-      </c>
-      <c r="AG25" t="n">
-        <v>0.8137</v>
-      </c>
-      <c r="AH25" t="n">
-        <v>0.0435</v>
-      </c>
-      <c r="AI25" t="n">
-        <v>0.141</v>
-      </c>
-      <c r="AJ25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK25" t="n">
-        <v>0.734</v>
-      </c>
-      <c r="AL25" t="n">
-        <v>0.802</v>
-      </c>
-      <c r="AM25" t="n">
-        <v>0.514</v>
-      </c>
-      <c r="AN25" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO25" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP25" t="n">
-        <v>1</v>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>1.4493</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>0.1362</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>3.2662</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>0.049</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>812</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>164</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>2.9855</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>685</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>1.9114</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>12.4697</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>54.933</t>
+        </is>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AE25" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>0.2013</t>
+        </is>
+      </c>
+      <c r="AG25" t="inlineStr">
+        <is>
+          <t>0.8137</t>
+        </is>
+      </c>
+      <c r="AH25" t="inlineStr">
+        <is>
+          <t>0.0435</t>
+        </is>
+      </c>
+      <c r="AI25" t="inlineStr">
+        <is>
+          <t>0.141</t>
+        </is>
+      </c>
+      <c r="AJ25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK25" t="inlineStr">
+        <is>
+          <t>0.734</t>
+        </is>
+      </c>
+      <c r="AL25" t="inlineStr">
+        <is>
+          <t>0.802</t>
+        </is>
+      </c>
+      <c r="AM25" t="inlineStr">
+        <is>
+          <t>0.514</t>
+        </is>
+      </c>
+      <c r="AN25" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO25" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AP25" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
       <c r="AQ25" t="inlineStr"/>
     </row>
@@ -17732,8 +17792,10 @@
           <t>heavy_monitor</t>
         </is>
       </c>
-      <c r="E88" t="n">
-        <v>10564</v>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>10564</t>
+        </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
@@ -17741,8 +17803,10 @@
         </is>
       </c>
       <c r="G88" t="inlineStr"/>
-      <c r="H88" t="n">
-        <v>88.3</v>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>88.3</t>
+        </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
@@ -17761,94 +17825,150 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N88" t="n">
-        <v>0.095</v>
-      </c>
-      <c r="O88" t="n">
-        <v>0.11</v>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>0.095</t>
+        </is>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>0.11</t>
+        </is>
       </c>
       <c r="P88" t="inlineStr">
         <is>
           <t>battlecruiser</t>
         </is>
       </c>
-      <c r="Q88" t="n">
-        <v>1.5174</v>
-      </c>
-      <c r="R88" t="n">
-        <v>0.1499</v>
-      </c>
-      <c r="S88" t="n">
-        <v>3.7615</v>
-      </c>
-      <c r="T88" t="n">
-        <v>0.0271</v>
-      </c>
-      <c r="U88" t="n">
-        <v>482</v>
-      </c>
-      <c r="V88" t="n">
-        <v>123</v>
-      </c>
-      <c r="W88" t="n">
-        <v>2.138</v>
-      </c>
-      <c r="X88" t="n">
-        <v>21</v>
-      </c>
-      <c r="Y88" t="n">
-        <v>88</v>
-      </c>
-      <c r="Z88" t="n">
-        <v>373</v>
-      </c>
-      <c r="AA88" t="n">
-        <v>1.5297</v>
-      </c>
-      <c r="AB88" t="n">
-        <v>6.4837</v>
-      </c>
-      <c r="AC88" t="n">
-        <v>57.5292</v>
-      </c>
-      <c r="AD88" t="n">
-        <v>7</v>
-      </c>
-      <c r="AE88" t="n">
-        <v>16</v>
-      </c>
-      <c r="AF88" t="n">
-        <v>0.212</v>
-      </c>
-      <c r="AG88" t="n">
-        <v>0.8222</v>
-      </c>
-      <c r="AH88" t="n">
-        <v>0.0494</v>
-      </c>
-      <c r="AI88" t="n">
-        <v>0.2097</v>
-      </c>
-      <c r="AJ88" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK88" t="n">
-        <v>0.845</v>
-      </c>
-      <c r="AL88" t="n">
-        <v>0.883</v>
-      </c>
-      <c r="AM88" t="n">
-        <v>0.592</v>
-      </c>
-      <c r="AN88" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO88" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP88" t="n">
-        <v>1</v>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>1.5174</t>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>0.1499</t>
+        </is>
+      </c>
+      <c r="S88" t="inlineStr">
+        <is>
+          <t>3.7615</t>
+        </is>
+      </c>
+      <c r="T88" t="inlineStr">
+        <is>
+          <t>0.0271</t>
+        </is>
+      </c>
+      <c r="U88" t="inlineStr">
+        <is>
+          <t>482</t>
+        </is>
+      </c>
+      <c r="V88" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="W88" t="inlineStr">
+        <is>
+          <t>2.138</t>
+        </is>
+      </c>
+      <c r="X88" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="Y88" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="Z88" t="inlineStr">
+        <is>
+          <t>373</t>
+        </is>
+      </c>
+      <c r="AA88" t="inlineStr">
+        <is>
+          <t>1.5297</t>
+        </is>
+      </c>
+      <c r="AB88" t="inlineStr">
+        <is>
+          <t>6.4837</t>
+        </is>
+      </c>
+      <c r="AC88" t="inlineStr">
+        <is>
+          <t>57.5292</t>
+        </is>
+      </c>
+      <c r="AD88" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AE88" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="AF88" t="inlineStr">
+        <is>
+          <t>0.212</t>
+        </is>
+      </c>
+      <c r="AG88" t="inlineStr">
+        <is>
+          <t>0.8222</t>
+        </is>
+      </c>
+      <c r="AH88" t="inlineStr">
+        <is>
+          <t>0.0494</t>
+        </is>
+      </c>
+      <c r="AI88" t="inlineStr">
+        <is>
+          <t>0.2097</t>
+        </is>
+      </c>
+      <c r="AJ88" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AK88" t="inlineStr">
+        <is>
+          <t>0.845</t>
+        </is>
+      </c>
+      <c r="AL88" t="inlineStr">
+        <is>
+          <t>0.883</t>
+        </is>
+      </c>
+      <c r="AM88" t="inlineStr">
+        <is>
+          <t>0.592</t>
+        </is>
+      </c>
+      <c r="AN88" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AO88" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AP88" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
       <c r="AQ88" t="inlineStr"/>
     </row>

</xml_diff>